<commit_message>
vault backup: 2026-02-26 20:22:55
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -1333,7 +1333,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr filterMode="1"/>
+  <sheetPr/>
   <dimension ref="A1:K73"/>
   <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
   <cols>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="2" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A2" s="6">
         <v>600410</v>
       </c>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="K2"/>
     </row>
-    <row r="3" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="3" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A3" s="6">
         <v>600745</v>
       </c>
@@ -1447,7 +1447,7 @@
       </c>
       <c r="K3"/>
     </row>
-    <row r="4" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="4" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A4" s="6">
         <v>600745</v>
       </c>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="K4"/>
     </row>
-    <row r="5" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="5" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A5" s="6">
         <v>600410</v>
       </c>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="K5"/>
     </row>
-    <row r="6" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="6" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A6" s="6">
         <v>600745</v>
       </c>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="K6"/>
     </row>
-    <row r="7" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="7" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A7" s="6">
         <v>600276</v>
       </c>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="K7"/>
     </row>
-    <row r="8" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="8" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A8" s="6">
         <v>600745</v>
       </c>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="K8"/>
     </row>
-    <row r="9" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="9" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A9" s="6">
         <v>600745</v>
       </c>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="K9"/>
     </row>
-    <row r="10" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="10" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A10" s="6">
         <v>600276</v>
       </c>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="K10"/>
     </row>
-    <row r="11" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="11" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A11" s="6">
         <v>600036</v>
       </c>
@@ -1727,7 +1727,7 @@
       </c>
       <c r="K11"/>
     </row>
-    <row r="12" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="12" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A12" s="6">
         <v>605358</v>
       </c>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="K12"/>
     </row>
-    <row r="13" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="13" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A13" s="6">
         <v>601138</v>
       </c>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="K13"/>
     </row>
-    <row r="14" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="14" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A14" s="6">
         <v>601138</v>
       </c>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="K14"/>
     </row>
-    <row r="15" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="15" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A15" s="6">
         <v>601138</v>
       </c>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="K15"/>
     </row>
-    <row r="16" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="16" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A16" s="6">
         <v>600745</v>
       </c>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="K16"/>
     </row>
-    <row r="17" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="17" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A17" s="6">
         <v>600745</v>
       </c>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="K17"/>
     </row>
-    <row r="18" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="18" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A18" s="6">
         <v>600745</v>
       </c>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="K18"/>
     </row>
-    <row r="19" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="19" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A19" s="6">
         <v>603986</v>
       </c>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="K19"/>
     </row>
-    <row r="20" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="20" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A20" s="6">
         <v>601138</v>
       </c>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="K20"/>
     </row>
-    <row r="21" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="21" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A21" s="6">
         <v>600111</v>
       </c>
@@ -2077,7 +2077,7 @@
       </c>
       <c r="K21"/>
     </row>
-    <row r="22" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="22" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A22" s="6">
         <v>600111</v>
       </c>
@@ -2112,7 +2112,7 @@
       </c>
       <c r="K22"/>
     </row>
-    <row r="23" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="23" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A23" s="6">
         <v>601138</v>
       </c>
@@ -2147,7 +2147,7 @@
       </c>
       <c r="K23"/>
     </row>
-    <row r="24" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="24" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A24" s="6">
         <v>603986</v>
       </c>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="K24"/>
     </row>
-    <row r="25" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="25" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A25" s="6">
         <v>600111</v>
       </c>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="K25"/>
     </row>
-    <row r="26" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="26" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A26" s="6">
         <v>600745</v>
       </c>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="K26"/>
     </row>
-    <row r="27" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="27" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A27" s="6" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="K27"/>
     </row>
-    <row r="28" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="28" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A28" s="6">
         <v>603259</v>
       </c>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="K28"/>
     </row>
-    <row r="29" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="29" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A29" s="6" t="str">
         <f>"002371"</f>
         <v>002371</v>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="K29"/>
     </row>
-    <row r="30" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="30" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A30" s="6" t="str">
         <f>"002281"</f>
         <v>002281</v>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="K30"/>
     </row>
-    <row r="31" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="31" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A31" s="6">
         <v>603259</v>
       </c>
@@ -2430,7 +2430,7 @@
       </c>
       <c r="K31"/>
     </row>
-    <row r="32" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="32" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A32" s="6" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="K32"/>
     </row>
-    <row r="33" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="33" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A33" s="6">
         <v>603986</v>
       </c>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="K33"/>
     </row>
-    <row r="34" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="34" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A34" s="6" t="str">
         <f>"002371"</f>
         <v>002371</v>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="K34"/>
     </row>
-    <row r="35" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="35" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A35" s="6" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="K35"/>
     </row>
-    <row r="36" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="36" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A36" s="6">
         <v>603986</v>
       </c>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="K36"/>
     </row>
-    <row r="37" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="37" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A37" s="6" t="str">
         <f>"002281"</f>
         <v>002281</v>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="K37"/>
     </row>
-    <row r="38" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="38" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A38" s="6">
         <v>603083</v>
       </c>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="K38"/>
     </row>
-    <row r="39" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="39" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A39" s="6">
         <v>603083</v>
       </c>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="K39"/>
     </row>
-    <row r="40" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="40" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A40" s="6">
         <v>603986</v>
       </c>
@@ -2749,7 +2749,7 @@
       </c>
       <c r="K40"/>
     </row>
-    <row r="41" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="41" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A41" s="6">
         <v>603799</v>
       </c>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="K41"/>
     </row>
-    <row r="42" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="42" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A42" s="6">
         <v>603986</v>
       </c>
@@ -2819,7 +2819,7 @@
       </c>
       <c r="K42"/>
     </row>
-    <row r="43" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="43" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A43" s="6">
         <v>603099</v>
       </c>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="K43"/>
     </row>
-    <row r="44" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="44" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A44" s="6">
         <v>603099</v>
       </c>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="K44"/>
     </row>
-    <row r="45" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="45" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A45" s="6">
         <v>603799</v>
       </c>
@@ -2924,7 +2924,7 @@
       </c>
       <c r="K45"/>
     </row>
-    <row r="46" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="46" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A46" s="6">
         <v>603099</v>
       </c>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="K47"/>
     </row>
-    <row r="48" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="48" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A48" s="6">
         <v>601179</v>
       </c>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="K49"/>
     </row>
-    <row r="50" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="50" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A50" s="6">
         <v>603986</v>
       </c>
@@ -3173,7 +3173,7 @@
       </c>
       <c r="K52"/>
     </row>
-    <row r="53" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="53" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A53" s="6">
         <v>600584</v>
       </c>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="K53"/>
     </row>
-    <row r="54" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="54" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A54" s="6">
         <v>601179</v>
       </c>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="K54"/>
     </row>
-    <row r="55" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="55" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A55" s="6">
         <v>600584</v>
       </c>
@@ -3278,7 +3278,7 @@
       </c>
       <c r="K55"/>
     </row>
-    <row r="56" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="56" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A56" s="6" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="K57"/>
     </row>
-    <row r="58" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="58" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A58" s="6" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -3386,7 +3386,7 @@
       </c>
       <c r="K58"/>
     </row>
-    <row r="59" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="59" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A59" s="6">
         <v>600584</v>
       </c>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="K59"/>
     </row>
-    <row r="60" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="60" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A60" s="6" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -3493,7 +3493,7 @@
       </c>
       <c r="K61"/>
     </row>
-    <row r="62" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="62" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A62" s="6">
         <v>601179</v>
       </c>
@@ -3564,7 +3564,7 @@
       </c>
       <c r="K63"/>
     </row>
-    <row r="64" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="64" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A64" s="6" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="K64"/>
     </row>
-    <row r="65" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="65" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A65" s="6">
         <v>600584</v>
       </c>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="K65"/>
     </row>
-    <row r="66" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="66" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A66" s="6">
         <v>601179</v>
       </c>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="K67"/>
     </row>
-    <row r="68" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="68" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A68" s="6" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -3850,7 +3850,7 @@
       </c>
       <c r="K71"/>
     </row>
-    <row r="72" s="2" customFormat="1" ht="20.4" hidden="1" customHeight="1" spans="1:11">
+    <row r="72" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A72" s="6">
         <v>600584</v>
       </c>
@@ -3923,11 +3923,6 @@
     </row>
   </sheetData>
   <autoFilter ref="B1:B73">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="思源电气"/>
-      </filters>
-    </filterColumn>
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-02-26 20:37:27
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交易记录" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'交易记录'!$B$1:$B$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'交易记录'!$A$1:$J$60</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -44,8 +44,8 @@
     <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <b val="1"/>
-      <sz val="11"/>
+      <color theme="1"/>
+      <sz val="14"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -191,9 +191,6 @@
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="34">
@@ -672,15 +669,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="21" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1280,15 +1273,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:N63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
   <cols>
     <col width="14.6153846153846" customWidth="1" style="3" min="1" max="1"/>
     <col width="14.6153846153846" customWidth="1" style="4" min="2" max="2"/>
     <col width="35.4615384615385" customWidth="1" style="4" min="3" max="3"/>
     <col width="14.6153846153846" customWidth="1" style="4" min="4" max="10"/>
-    <col width="14" customWidth="1" style="4" min="11" max="11"/>
-    <col width="14" customWidth="1" style="4" min="12" max="12"/>
+    <col width="14.6153846153846" customWidth="1" style="4" min="11" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="23.2" customFormat="1" customHeight="1" s="1">
@@ -1342,106 +1334,110 @@
           <t>剩余仓位</t>
         </is>
       </c>
-      <c r="K1" s="8" t="n"/>
-      <c r="L1" s="9" t="inlineStr">
-        <is>
-          <t>未实现利润</t>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>买入逻辑</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>计划止盈</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>计划止损</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>清仓逻辑</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A2" s="6" t="n">
-        <v>600410</v>
+        <v>600276</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>华胜天成</t>
+          <t>恒瑞医药</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>20250901</v>
-      </c>
-      <c r="E2" s="7" t="n">
-        <v>0.3998148148148148</v>
+        <v>20250902</v>
+      </c>
+      <c r="E2" s="8" t="n">
+        <v>0.3959837962962963</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>22.5</v>
+        <v>69.43000000000001</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-500</v>
+        <v>200</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>11250</v>
+        <v>13886</v>
       </c>
       <c r="I2" s="2">
-        <f>IF(AND($C2="卖出",SUMIFS($G$2:G2,$A$2:A2,$A2)=0),SUMIFS($H$2:H2,$A$2:A2,$A2,$C$2:C2,"卖出")-SUMIFS($H$2:H2,$A$2:A2,$A2,$C$2:C2,"买入"),"")</f>
+        <f>IF(AND($C2="卖出",SUMIFS($G$2:G4,$A$2:A4,$A2)=0),SUMIFS($H$2:H4,$A$2:A4,$A2,$C$2:C4,"卖出")-SUMIFS($H$2:H4,$A$2:A4,$A2,$C$2:C4,"买入"),"")</f>
         <v/>
       </c>
       <c r="J2" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A2)=COUNTIF($A$2:A2,$A2),SUMIFS($G$2:$G$73,$A$2:$A$73,$A2),"")</f>
-        <v/>
-      </c>
-      <c r="K2" s="0" t="n"/>
-      <c r="L2">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A2)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A2,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A2,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A2),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A2,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A2,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A2)))</f>
+        <f>SUMIFS($G$2:G2,$A$2:A2,$A2)</f>
         <v/>
       </c>
     </row>
     <row r="3" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A3" s="6" t="n">
-        <v>600745</v>
+        <v>600276</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>恒瑞医药</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>20250902</v>
-      </c>
-      <c r="E3" s="7" t="n">
-        <v>0.4647222222222222</v>
+        <v>20250903</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>0.4002893518518518</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>41.1</v>
+        <v>69.09</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>100</v>
+        <v>-200</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>4110</v>
+        <v>13818</v>
       </c>
       <c r="I3" s="2">
-        <f>IF(AND($C3="卖出",SUMIFS($G$2:G3,$A$2:A3,$A3)=0),SUMIFS($H$2:H3,$A$2:A3,$A3,$C$2:C3,"卖出")-SUMIFS($H$2:H3,$A$2:A3,$A3,$C$2:C3,"买入"),"")</f>
+        <f>IF(AND($C3="卖出",SUMIFS($G$2:G4,$A$2:A4,$A3)=0),SUMIFS($H$2:H4,$A$2:A4,$A3,$C$2:C4,"卖出")-SUMIFS($H$2:H4,$A$2:A4,$A3,$C$2:C4,"买入"),"")</f>
         <v/>
       </c>
       <c r="J3" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A3)=COUNTIF($A$2:A3,$A3),SUMIFS($G$2:$G$73,$A$2:$A$73,$A3),"")</f>
-        <v/>
-      </c>
-      <c r="K3" s="0" t="n"/>
-      <c r="L3">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A3)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A3,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A3,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A3),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A3,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A3,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A3)))</f>
+        <f>SUMIFS($G$2:G3,$A$2:A3,$A3)</f>
         <v/>
       </c>
     </row>
     <row r="4" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A4" s="6" t="n">
-        <v>600745</v>
+        <v>601138</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>工业富联</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1450,84 +1446,74 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>20250902</v>
-      </c>
-      <c r="E4" s="7" t="n">
-        <v>0.4569560185185185</v>
+        <v>20250912</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>0.4076388888888889</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>41.3</v>
+        <v>61</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>8260</v>
+        <v>24400</v>
       </c>
       <c r="I4" s="2">
         <f>IF(AND($C4="卖出",SUMIFS($G$2:G4,$A$2:A4,$A4)=0),SUMIFS($H$2:H4,$A$2:A4,$A4,$C$2:C4,"卖出")-SUMIFS($H$2:H4,$A$2:A4,$A4,$C$2:C4,"买入"),"")</f>
         <v/>
       </c>
       <c r="J4" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A4)=COUNTIF($A$2:A4,$A4),SUMIFS($G$2:$G$73,$A$2:$A$73,$A4),"")</f>
-        <v/>
-      </c>
-      <c r="K4" s="0" t="n"/>
-      <c r="L4">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A4)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A4,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A4,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A4),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A4,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A4,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A4)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" ht="20.4" customFormat="1" customHeight="1" s="2">
+        <f>SUMIFS($G$2:G4,$A$2:A4,$A4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="20" customFormat="1" customHeight="1" s="2">
       <c r="A5" s="6" t="n">
-        <v>600410</v>
+        <v>601138</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>华胜天成</t>
+          <t>工业富联</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>20250902</v>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>0.4403703703703704</v>
+        <v>20250915</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>0.5917824074074074</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>23</v>
+        <v>59.5</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>-500</v>
+        <v>100</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>11500</v>
+        <v>5950</v>
       </c>
       <c r="I5" s="2">
         <f>IF(AND($C5="卖出",SUMIFS($G$2:G5,$A$2:A5,$A5)=0),SUMIFS($H$2:H5,$A$2:A5,$A5,$C$2:C5,"卖出")-SUMIFS($H$2:H5,$A$2:A5,$A5,$C$2:C5,"买入"),"")</f>
         <v/>
       </c>
       <c r="J5" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A5)=COUNTIF($A$2:A5,$A5),SUMIFS($G$2:$G$73,$A$2:$A$73,$A5),"")</f>
-        <v/>
-      </c>
-      <c r="K5" s="0" t="n"/>
-      <c r="L5">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A5)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A5,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A5,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A5),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A5,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A5,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A5)))</f>
+        <f>SUMIFS($G$2:G5,$A$2:A5,$A5)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A6" s="6" t="n">
-        <v>600745</v>
+        <v>601138</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>工业富联</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1536,41 +1522,36 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>20250902</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>0.420462962962963</v>
+        <v>20250915</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0.3993634259259259</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>41.91</v>
+        <v>60.5</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>8382</v>
+        <v>6050</v>
       </c>
       <c r="I6" s="2">
         <f>IF(AND($C6="卖出",SUMIFS($G$2:G6,$A$2:A6,$A6)=0),SUMIFS($H$2:H6,$A$2:A6,$A6,$C$2:C6,"卖出")-SUMIFS($H$2:H6,$A$2:A6,$A6,$C$2:C6,"买入"),"")</f>
         <v/>
       </c>
       <c r="J6" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A6)=COUNTIF($A$2:A6,$A6),SUMIFS($G$2:$G$73,$A$2:$A$73,$A6),"")</f>
-        <v/>
-      </c>
-      <c r="K6" s="0" t="n"/>
-      <c r="L6">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A6)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A6,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A6,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A6),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A6,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A6,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A6)))</f>
+        <f>SUMIFS($G$2:G6,$A$2:A6,$A6)</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A7" s="6" t="n">
-        <v>600276</v>
+        <v>603986</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>恒瑞医药</t>
+          <t>兆易创新</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1579,84 +1560,74 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>20250902</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>0.3959837962962963</v>
+        <v>20250925</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0.6093402777777778</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>69.43000000000001</v>
+        <v>198</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>13886</v>
+        <v>19800</v>
       </c>
       <c r="I7" s="2">
-        <f>IF(AND($C7="卖出",SUMIFS($G$2:G7,$A$2:A7,$A7)=0),SUMIFS($H$2:H7,$A$2:A7,$A7,$C$2:C7,"卖出")-SUMIFS($H$2:H7,$A$2:A7,$A7,$C$2:C7,"买入"),"")</f>
+        <f>IF(AND($C7="卖出",SUMIFS($G$2:G11,$A$2:A11,$A7)=0),SUMIFS($H$2:H11,$A$2:A11,$A7,$C$2:C11,"卖出")-SUMIFS($H$2:H11,$A$2:A11,$A7,$C$2:C11,"买入"),"")</f>
         <v/>
       </c>
       <c r="J7" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A7)=COUNTIF($A$2:A7,$A7),SUMIFS($G$2:$G$73,$A$2:$A$73,$A7),"")</f>
-        <v/>
-      </c>
-      <c r="K7" s="0" t="n"/>
-      <c r="L7">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A7)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A7,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A7,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A7),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A7,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A7,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A7)))</f>
+        <f>SUMIFS($G$2:G7,$A$2:A7,$A7)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A8" s="6" t="n">
-        <v>600745</v>
+        <v>601138</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>工业富联</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>20250903</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>0.474537037037037</v>
+        <v>20251009</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>0.4468518518518518</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>41.2</v>
+        <v>70</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>100</v>
+        <v>-200</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>4120</v>
+        <v>14000</v>
       </c>
       <c r="I8" s="2">
-        <f>IF(AND($C8="卖出",SUMIFS($G$2:G8,$A$2:A8,$A8)=0),SUMIFS($H$2:H8,$A$2:A8,$A8,$C$2:C8,"卖出")-SUMIFS($H$2:H8,$A$2:A8,$A8,$C$2:C8,"买入"),"")</f>
+        <f>IF(AND($C8="卖出",SUMIFS($G$2:G11,$A$2:A11,$A8)=0),SUMIFS($H$2:H11,$A$2:A11,$A8,$C$2:C11,"卖出")-SUMIFS($H$2:H11,$A$2:A11,$A8,$C$2:C11,"买入"),"")</f>
         <v/>
       </c>
       <c r="J8" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A8)=COUNTIF($A$2:A8,$A8),SUMIFS($G$2:$G$73,$A$2:$A$73,$A8),"")</f>
-        <v/>
-      </c>
-      <c r="K8" s="0" t="n"/>
-      <c r="L8">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A8)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A8,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A8,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A8),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A8,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A8,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A8)))</f>
+        <f>SUMIFS($G$2:G8,$A$2:A8,$A8)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A9" s="6" t="n">
-        <v>600745</v>
+        <v>600111</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>北方稀土</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1665,84 +1636,74 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>20250903</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>0.4695254629629629</v>
+        <v>20251010</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>0.4173379629629629</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>41.3</v>
+        <v>53.5</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>4130</v>
+        <v>10700</v>
       </c>
       <c r="I9" s="2">
-        <f>IF(AND($C9="卖出",SUMIFS($G$2:G9,$A$2:A9,$A9)=0),SUMIFS($H$2:H9,$A$2:A9,$A9,$C$2:C9,"卖出")-SUMIFS($H$2:H9,$A$2:A9,$A9,$C$2:C9,"买入"),"")</f>
+        <f>IF(AND($C9="卖出",SUMIFS($G$2:G11,$A$2:A11,$A9)=0),SUMIFS($H$2:H11,$A$2:A11,$A9,$C$2:C11,"卖出")-SUMIFS($H$2:H11,$A$2:A11,$A9,$C$2:C11,"买入"),"")</f>
         <v/>
       </c>
       <c r="J9" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A9)=COUNTIF($A$2:A9,$A9),SUMIFS($G$2:$G$73,$A$2:$A$73,$A9),"")</f>
-        <v/>
-      </c>
-      <c r="K9" s="0" t="n"/>
-      <c r="L9">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A9)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A9,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A9,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A9),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A9,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A9,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A9)))</f>
+        <f>SUMIFS($G$2:G9,$A$2:A9,$A9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A10" s="6" t="n">
-        <v>600276</v>
+        <v>600111</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>恒瑞医药</t>
+          <t>北方稀土</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>20250903</v>
-      </c>
-      <c r="E10" s="7" t="n">
-        <v>0.4002893518518518</v>
+        <v>20251010</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0.3965740740740741</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>69.09</v>
+        <v>53.98</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>-200</v>
+        <v>300</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>13818</v>
+        <v>16194</v>
       </c>
       <c r="I10" s="2">
-        <f>IF(AND($C10="卖出",SUMIFS($G$2:G10,$A$2:A10,$A10)=0),SUMIFS($H$2:H10,$A$2:A10,$A10,$C$2:C10,"卖出")-SUMIFS($H$2:H10,$A$2:A10,$A10,$C$2:C10,"买入"),"")</f>
+        <f>IF(AND($C10="卖出",SUMIFS($G$2:G11,$A$2:A11,$A10)=0),SUMIFS($H$2:H11,$A$2:A11,$A10,$C$2:C11,"卖出")-SUMIFS($H$2:H11,$A$2:A11,$A10,$C$2:C11,"买入"),"")</f>
         <v/>
       </c>
       <c r="J10" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A10)=COUNTIF($A$2:A10,$A10),SUMIFS($G$2:$G$73,$A$2:$A$73,$A10),"")</f>
-        <v/>
-      </c>
-      <c r="K10" s="0" t="n"/>
-      <c r="L10">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A10)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A10,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A10,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A10),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A10,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A10,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A10)))</f>
+        <f>SUMIFS($G$2:G10,$A$2:A10,$A10)</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A11" s="6" t="n">
-        <v>600036</v>
+        <v>601138</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>招商银行</t>
+          <t>工业富联</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1751,41 +1712,36 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>20250911</v>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>0.6034722222222222</v>
+        <v>20251015</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>0.453912037037037</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>43.14</v>
+        <v>60.75</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>-400</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>17256</v>
+        <v>24300</v>
       </c>
       <c r="I11" s="2">
         <f>IF(AND($C11="卖出",SUMIFS($G$2:G11,$A$2:A11,$A11)=0),SUMIFS($H$2:H11,$A$2:A11,$A11,$C$2:C11,"卖出")-SUMIFS($H$2:H11,$A$2:A11,$A11,$C$2:C11,"买入"),"")</f>
         <v/>
       </c>
       <c r="J11" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A11)=COUNTIF($A$2:A11,$A11),SUMIFS($G$2:$G$73,$A$2:$A$73,$A11),"")</f>
-        <v/>
-      </c>
-      <c r="K11" s="0" t="n"/>
-      <c r="L11">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A11)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A11,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A11,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A11),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A11,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A11,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A11)))</f>
+        <f>SUMIFS($G$2:G11,$A$2:A11,$A11)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A12" s="6" t="n">
-        <v>605358</v>
+        <v>603986</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>立昂微</t>
+          <t>兆易创新</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1794,84 +1750,75 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>20250912</v>
-      </c>
-      <c r="E12" s="7" t="n">
-        <v>0.4733912037037037</v>
+        <v>20251015</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>0.4537847222222222</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>26</v>
+        <v>193.75</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>-400</v>
+        <v>-100</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>10400</v>
+        <v>19375</v>
       </c>
       <c r="I12" s="2">
         <f>IF(AND($C12="卖出",SUMIFS($G$2:G12,$A$2:A12,$A12)=0),SUMIFS($H$2:H12,$A$2:A12,$A12,$C$2:C12,"卖出")-SUMIFS($H$2:H12,$A$2:A12,$A12,$C$2:C12,"买入"),"")</f>
         <v/>
       </c>
       <c r="J12" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A12)=COUNTIF($A$2:A12,$A12),SUMIFS($G$2:$G$73,$A$2:$A$73,$A12),"")</f>
-        <v/>
-      </c>
-      <c r="K12" s="0" t="n"/>
-      <c r="L12">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A12)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A12,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A12,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A12),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A12,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A12,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A12)))</f>
+        <f>SUMIFS($G$2:G12,$A$2:A12,$A12)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A13" s="6" t="n">
-        <v>601138</v>
+        <v>600111</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>工业富联</t>
+          <t>北方稀土</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>20250912</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>0.4076388888888889</v>
+        <v>20251015</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>0.4226967592592593</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>61</v>
+        <v>54.82</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>400</v>
+        <v>-500</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>24400</v>
+        <v>27410</v>
       </c>
       <c r="I13" s="2">
         <f>IF(AND($C13="卖出",SUMIFS($G$2:G13,$A$2:A13,$A13)=0),SUMIFS($H$2:H13,$A$2:A13,$A13,$C$2:C13,"卖出")-SUMIFS($H$2:H13,$A$2:A13,$A13,$C$2:C13,"买入"),"")</f>
         <v/>
       </c>
       <c r="J13" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A13)=COUNTIF($A$2:A13,$A13),SUMIFS($G$2:$G$73,$A$2:$A$73,$A13),"")</f>
-        <v/>
-      </c>
-      <c r="K13" s="0" t="n"/>
-      <c r="L13">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A13)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A13,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A13,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A13),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A13,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A13,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A13)))</f>
+        <f>SUMIFS($G$2:G13,$A$2:A13,$A13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A14" s="6" t="n">
-        <v>601138</v>
+      <c r="A14" s="6">
+        <f>"002475"</f>
+        <v/>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>工业富联</t>
+          <t>立讯精密</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1880,41 +1827,36 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>20250915</v>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>0.5917824074074074</v>
+        <v>20251016</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>0.5604745370370371</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>59.5</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>5950</v>
+        <v>35700</v>
       </c>
       <c r="I14" s="2">
-        <f>IF(AND($C14="卖出",SUMIFS($G$2:G14,$A$2:A14,$A14)=0),SUMIFS($H$2:H14,$A$2:A14,$A14,$C$2:C14,"卖出")-SUMIFS($H$2:H14,$A$2:A14,$A14,$C$2:C14,"买入"),"")</f>
+        <f>IF(AND($C14="卖出",SUMIFS($G$2:G19,$A$2:A19,$A14)=0),SUMIFS($H$2:H19,$A$2:A19,$A14,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A14,$C$2:C19,"买入"),"")</f>
         <v/>
       </c>
       <c r="J14" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A14)=COUNTIF($A$2:A14,$A14),SUMIFS($G$2:$G$73,$A$2:$A$73,$A14),"")</f>
-        <v/>
-      </c>
-      <c r="K14" s="0" t="n"/>
-      <c r="L14">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A14)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A14,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A14,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A14),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A14,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A14,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A14)))</f>
+        <f>SUMIFS($G$2:G14,$A$2:A14,$A14)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A15" s="6" t="n">
-        <v>601138</v>
+        <v>603259</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>工业富联</t>
+          <t>药明康德</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1923,342 +1865,307 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>20250915</v>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>0.3993634259259259</v>
+        <v>20251016</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>0.4585300925925926</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>60.5</v>
+        <v>101.12</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>100</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>6050</v>
+        <v>10112</v>
       </c>
       <c r="I15" s="2">
-        <f>IF(AND($C15="卖出",SUMIFS($G$2:G15,$A$2:A15,$A15)=0),SUMIFS($H$2:H15,$A$2:A15,$A15,$C$2:C15,"卖出")-SUMIFS($H$2:H15,$A$2:A15,$A15,$C$2:C15,"买入"),"")</f>
+        <f>IF(AND($C15="卖出",SUMIFS($G$2:G19,$A$2:A19,$A15)=0),SUMIFS($H$2:H19,$A$2:A19,$A15,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A15,$C$2:C19,"买入"),"")</f>
         <v/>
       </c>
       <c r="J15" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A15)=COUNTIF($A$2:A15,$A15),SUMIFS($G$2:$G$73,$A$2:$A$73,$A15),"")</f>
-        <v/>
-      </c>
-      <c r="K15" s="0" t="n"/>
-      <c r="L15">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A15)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A15,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A15,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A15),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A15,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A15,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A15)))</f>
+        <f>SUMIFS($G$2:G15,$A$2:A15,$A15)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A16" s="6" t="n">
-        <v>600745</v>
+      <c r="A16" s="6">
+        <f>"002371"</f>
+        <v/>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>北方华创</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>20250916</v>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>0.6060069444444445</v>
+        <v>20251017</v>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>0.625</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>43.2283</v>
+        <v>399.43</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>-1200</v>
+        <v>100</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>51874</v>
+        <v>39943</v>
       </c>
       <c r="I16" s="2">
-        <f>IF(AND($C16="卖出",SUMIFS($G$2:G16,$A$2:A16,$A16)=0),SUMIFS($H$2:H16,$A$2:A16,$A16,$C$2:C16,"卖出")-SUMIFS($H$2:H16,$A$2:A16,$A16,$C$2:C16,"买入"),"")</f>
+        <f>IF(AND($C16="卖出",SUMIFS($G$2:G19,$A$2:A19,$A16)=0),SUMIFS($H$2:H19,$A$2:A19,$A16,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A16,$C$2:C19,"买入"),"")</f>
         <v/>
       </c>
       <c r="J16" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A16)=COUNTIF($A$2:A16,$A16),SUMIFS($G$2:$G$73,$A$2:$A$73,$A16),"")</f>
-        <v/>
-      </c>
-      <c r="K16" s="0" t="n"/>
-      <c r="L16">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A16)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A16,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A16,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A16),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A16,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A16,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A16)))</f>
+        <f>SUMIFS($G$2:G16,$A$2:A16,$A16)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A17" s="6" t="n">
-        <v>600745</v>
+      <c r="A17" s="6">
+        <f>"002281"</f>
+        <v/>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>光迅科技</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>市买1（对手方最优价格）</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>20250916</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>0.6037847222222222</v>
+        <v>20251021</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>0.621550925925926</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>43.2</v>
+        <v>61.37</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>8640</v>
+        <v>18411</v>
       </c>
       <c r="I17" s="2">
-        <f>IF(AND($C17="卖出",SUMIFS($G$2:G17,$A$2:A17,$A17)=0),SUMIFS($H$2:H17,$A$2:A17,$A17,$C$2:C17,"卖出")-SUMIFS($H$2:H17,$A$2:A17,$A17,$C$2:C17,"买入"),"")</f>
+        <f>IF(AND($C17="卖出",SUMIFS($G$2:G19,$A$2:A19,$A17)=0),SUMIFS($H$2:H19,$A$2:A19,$A17,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A17,$C$2:C19,"买入"),"")</f>
         <v/>
       </c>
       <c r="J17" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A17)=COUNTIF($A$2:A17,$A17),SUMIFS($G$2:$G$73,$A$2:$A$73,$A17),"")</f>
-        <v/>
-      </c>
-      <c r="K17" s="0" t="n"/>
-      <c r="L17">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A17)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A17,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A17,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A17),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A17,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A17,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A17)))</f>
+        <f>SUMIFS($G$2:G17,$A$2:A17,$A17)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A18" s="6" t="n">
-        <v>600745</v>
+        <v>603259</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>药明康德</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>20250919</v>
-      </c>
-      <c r="E18" s="7" t="n">
-        <v>0.4050462962962963</v>
+        <v>20251021</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>0.4680671296296297</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>47.5</v>
+        <v>101.48</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>200</v>
+        <v>-100</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>9500</v>
+        <v>10148</v>
       </c>
       <c r="I18" s="2">
-        <f>IF(AND($C18="卖出",SUMIFS($G$2:G18,$A$2:A18,$A18)=0),SUMIFS($H$2:H18,$A$2:A18,$A18,$C$2:C18,"卖出")-SUMIFS($H$2:H18,$A$2:A18,$A18,$C$2:C18,"买入"),"")</f>
+        <f>IF(AND($C18="卖出",SUMIFS($G$2:G19,$A$2:A19,$A18)=0),SUMIFS($H$2:H19,$A$2:A19,$A18,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A18,$C$2:C19,"买入"),"")</f>
         <v/>
       </c>
       <c r="J18" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A18)=COUNTIF($A$2:A18,$A18),SUMIFS($G$2:$G$73,$A$2:$A$73,$A18),"")</f>
-        <v/>
-      </c>
-      <c r="K18" s="0" t="n"/>
-      <c r="L18">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A18)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A18,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A18,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A18),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A18,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A18,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A18)))</f>
+        <f>SUMIFS($G$2:G18,$A$2:A18,$A18)</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A19" s="6" t="n">
-        <v>603986</v>
+      <c r="A19" s="6">
+        <f>"002475"</f>
+        <v/>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>兆易创新</t>
+          <t>立讯精密</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>20250925</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>0.6093402777777778</v>
+        <v>20251021</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>0.4185185185185185</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>198</v>
+        <v>60.07</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>100</v>
+        <v>-200</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>19800</v>
+        <v>12014</v>
       </c>
       <c r="I19" s="2">
         <f>IF(AND($C19="卖出",SUMIFS($G$2:G19,$A$2:A19,$A19)=0),SUMIFS($H$2:H19,$A$2:A19,$A19,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A19,$C$2:C19,"买入"),"")</f>
         <v/>
       </c>
       <c r="J19" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A19)=COUNTIF($A$2:A19,$A19),SUMIFS($G$2:$G$73,$A$2:$A$73,$A19),"")</f>
-        <v/>
-      </c>
-      <c r="K19" s="0" t="n"/>
-      <c r="L19">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A19)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A19,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A19,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A19),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A19,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A19,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A19)))</f>
+        <f>SUMIFS($G$2:G19,$A$2:A19,$A19)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A20" s="6" t="n">
-        <v>601138</v>
+        <v>603986</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>工业富联</t>
+          <t>兆易创新</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>20251009</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>0.4468518518518518</v>
+        <v>20251023</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>0.6177777777777778</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>70</v>
+        <v>208.04</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>-200</v>
+        <v>200</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>14000</v>
+        <v>41608</v>
       </c>
       <c r="I20" s="2">
         <f>IF(AND($C20="卖出",SUMIFS($G$2:G20,$A$2:A20,$A20)=0),SUMIFS($H$2:H20,$A$2:A20,$A20,$C$2:C20,"卖出")-SUMIFS($H$2:H20,$A$2:A20,$A20,$C$2:C20,"买入"),"")</f>
         <v/>
       </c>
       <c r="J20" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A20)=COUNTIF($A$2:A20,$A20),SUMIFS($G$2:$G$73,$A$2:$A$73,$A20),"")</f>
-        <v/>
-      </c>
-      <c r="K20" s="0" t="n"/>
-      <c r="L20">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A20)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A20,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A20,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A20),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A20,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A20,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A20)))</f>
+        <f>SUMIFS($G$2:G20,$A$2:A20,$A20)</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A21" s="6" t="n">
-        <v>600111</v>
+      <c r="A21" s="6">
+        <f>"002371"</f>
+        <v/>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>北方稀土</t>
+          <t>北方华创</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>市卖1（对手方最优价格）</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>20251010</v>
-      </c>
-      <c r="E21" s="7" t="n">
-        <v>0.4173379629629629</v>
+        <v>20251023</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>0.6161111111111112</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>53.5</v>
+        <v>402.9</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>200</v>
+        <v>-100</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>10700</v>
+        <v>40290</v>
       </c>
       <c r="I21" s="2">
         <f>IF(AND($C21="卖出",SUMIFS($G$2:G21,$A$2:A21,$A21)=0),SUMIFS($H$2:H21,$A$2:A21,$A21,$C$2:C21,"卖出")-SUMIFS($H$2:H21,$A$2:A21,$A21,$C$2:C21,"买入"),"")</f>
         <v/>
       </c>
       <c r="J21" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A21)=COUNTIF($A$2:A21,$A21),SUMIFS($G$2:$G$73,$A$2:$A$73,$A21),"")</f>
-        <v/>
-      </c>
-      <c r="K21" s="0" t="n"/>
-      <c r="L21">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A21)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A21,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A21,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A21),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A21,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A21,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A21)))</f>
+        <f>SUMIFS($G$2:G21,$A$2:A21,$A21)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A22" s="6" t="n">
-        <v>600111</v>
+      <c r="A22" s="6">
+        <f>"002475"</f>
+        <v/>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>北方稀土</t>
+          <t>立讯精密</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>20251010</v>
-      </c>
-      <c r="E22" s="7" t="n">
-        <v>0.3965740740740741</v>
+        <v>20251024</v>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>0.6010069444444445</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>53.98</v>
+        <v>63.72</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>300</v>
+        <v>-100</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>16194</v>
+        <v>6372</v>
       </c>
       <c r="I22" s="2">
         <f>IF(AND($C22="卖出",SUMIFS($G$2:G22,$A$2:A22,$A22)=0),SUMIFS($H$2:H22,$A$2:A22,$A22,$C$2:C22,"卖出")-SUMIFS($H$2:H22,$A$2:A22,$A22,$C$2:C22,"买入"),"")</f>
         <v/>
       </c>
       <c r="J22" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A22)=COUNTIF($A$2:A22,$A22),SUMIFS($G$2:$G$73,$A$2:$A$73,$A22),"")</f>
-        <v/>
-      </c>
-      <c r="K22" s="0" t="n"/>
-      <c r="L22">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A22)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A22,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A22,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A22),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A22,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A22,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A22)))</f>
+        <f>SUMIFS($G$2:G22,$A$2:A22,$A22)</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A23" s="6" t="n">
-        <v>601138</v>
+        <v>603986</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>工业富联</t>
+          <t>兆易创新</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2267,127 +2174,113 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>20251015</v>
-      </c>
-      <c r="E23" s="7" t="n">
-        <v>0.453912037037037</v>
+        <v>20251024</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>0.589212962962963</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>60.75</v>
+        <v>220</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>-400</v>
+        <v>-100</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>24300</v>
+        <v>22000</v>
       </c>
       <c r="I23" s="2">
         <f>IF(AND($C23="卖出",SUMIFS($G$2:G23,$A$2:A23,$A23)=0),SUMIFS($H$2:H23,$A$2:A23,$A23,$C$2:C23,"卖出")-SUMIFS($H$2:H23,$A$2:A23,$A23,$C$2:C23,"买入"),"")</f>
         <v/>
       </c>
       <c r="J23" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A23)=COUNTIF($A$2:A23,$A23),SUMIFS($G$2:$G$73,$A$2:$A$73,$A23),"")</f>
-        <v/>
-      </c>
-      <c r="K23" s="0" t="n"/>
-      <c r="L23">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A23)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A23,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A23,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A23),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A23,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A23,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A23)))</f>
+        <f>SUMIFS($G$2:G23,$A$2:A23,$A23)</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A24" s="6" t="n">
-        <v>603986</v>
+      <c r="A24" s="6">
+        <f>"002281"</f>
+        <v/>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>兆易创新</t>
+          <t>光迅科技</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>市卖2（本手方最优价格）</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>20251015</v>
-      </c>
-      <c r="E24" s="7" t="n">
-        <v>0.4537847222222222</v>
+        <v>20251024</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>0.4184259259259259</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>193.75</v>
+        <v>61.31</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>-100</v>
+        <v>-300</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>19375</v>
+        <v>18393</v>
       </c>
       <c r="I24" s="2">
         <f>IF(AND($C24="卖出",SUMIFS($G$2:G24,$A$2:A24,$A24)=0),SUMIFS($H$2:H24,$A$2:A24,$A24,$C$2:C24,"卖出")-SUMIFS($H$2:H24,$A$2:A24,$A24,$C$2:C24,"买入"),"")</f>
         <v/>
       </c>
       <c r="J24" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A24)=COUNTIF($A$2:A24,$A24),SUMIFS($G$2:$G$73,$A$2:$A$73,$A24),"")</f>
-        <v/>
-      </c>
-      <c r="K24" s="0" t="n"/>
-      <c r="L24">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A24)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A24,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A24,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A24),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A24,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A24,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A24)))</f>
+        <f>SUMIFS($G$2:G24,$A$2:A24,$A24)</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A25" s="6" t="n">
-        <v>600111</v>
+        <v>603083</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>北方稀土</t>
+          <t>剑桥科技</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>市买2（本手方最优价格）</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>20251015</v>
-      </c>
-      <c r="E25" s="7" t="n">
-        <v>0.4226967592592593</v>
+        <v>20251027</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>0.3990740740740741</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>54.82</v>
+        <v>122.95</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>-500</v>
+        <v>200</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>27410</v>
+        <v>24590</v>
       </c>
       <c r="I25" s="2">
         <f>IF(AND($C25="卖出",SUMIFS($G$2:G25,$A$2:A25,$A25)=0),SUMIFS($H$2:H25,$A$2:A25,$A25,$C$2:C25,"卖出")-SUMIFS($H$2:H25,$A$2:A25,$A25,$C$2:C25,"买入"),"")</f>
         <v/>
       </c>
       <c r="J25" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A25)=COUNTIF($A$2:A25,$A25),SUMIFS($G$2:$G$73,$A$2:$A$73,$A25),"")</f>
-        <v/>
-      </c>
-      <c r="K25" s="0" t="n"/>
-      <c r="L25">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A25)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A25,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A25,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A25),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A25,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A25,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A25)))</f>
+        <f>SUMIFS($G$2:G25,$A$2:A25,$A25)</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A26" s="6" t="n">
-        <v>600745</v>
+        <v>603083</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>闻泰科技</t>
+          <t>剑桥科技</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2396,85 +2289,74 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>20251015</v>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>0.3923611111111111</v>
+        <v>20251028</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>0.625</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>34.5</v>
+        <v>119.28</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>-400</v>
+        <v>-200</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>13800</v>
+        <v>23856</v>
       </c>
       <c r="I26" s="2">
         <f>IF(AND($C26="卖出",SUMIFS($G$2:G26,$A$2:A26,$A26)=0),SUMIFS($H$2:H26,$A$2:A26,$A26,$C$2:C26,"卖出")-SUMIFS($H$2:H26,$A$2:A26,$A26,$C$2:C26,"买入"),"")</f>
         <v/>
       </c>
       <c r="J26" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A26)=COUNTIF($A$2:A26,$A26),SUMIFS($G$2:$G$73,$A$2:$A$73,$A26),"")</f>
-        <v/>
-      </c>
-      <c r="K26" s="0" t="n"/>
-      <c r="L26">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A26)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A26,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A26,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A26),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A26,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A26,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A26)))</f>
+        <f>SUMIFS($G$2:G26,$A$2:A26,$A26)</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A27" s="6">
-        <f>"002475"</f>
-        <v/>
+      <c r="A27" s="6" t="n">
+        <v>603986</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>立讯精密</t>
+          <t>兆易创新</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>20251016</v>
-      </c>
-      <c r="E27" s="7" t="n">
-        <v>0.5604745370370371</v>
+        <v>20251029</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>0.4415509259259259</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>59.5</v>
+        <v>236.41</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>600</v>
+        <v>-100</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>35700</v>
+        <v>23641</v>
       </c>
       <c r="I27" s="2">
         <f>IF(AND($C27="卖出",SUMIFS($G$2:G27,$A$2:A27,$A27)=0),SUMIFS($H$2:H27,$A$2:A27,$A27,$C$2:C27,"卖出")-SUMIFS($H$2:H27,$A$2:A27,$A27,$C$2:C27,"买入"),"")</f>
         <v/>
       </c>
       <c r="J27" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A27)=COUNTIF($A$2:A27,$A27),SUMIFS($G$2:$G$73,$A$2:$A$73,$A27),"")</f>
-        <v/>
-      </c>
-      <c r="K27" s="0" t="n"/>
-      <c r="L27">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A27)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A27,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A27,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A27),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A27,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A27,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A27)))</f>
+        <f>SUMIFS($G$2:G27,$A$2:A27,$A27)</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A28" s="6" t="n">
-        <v>603259</v>
+        <v>603799</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>药明康德</t>
+          <t>华友钴业</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2483,42 +2365,36 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>20251016</v>
-      </c>
-      <c r="E28" s="7" t="n">
-        <v>0.4585300925925926</v>
+        <v>20251030</v>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>0.5655902777777778</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>101.12</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>10112</v>
+        <v>19830</v>
       </c>
       <c r="I28" s="2">
         <f>IF(AND($C28="卖出",SUMIFS($G$2:G28,$A$2:A28,$A28)=0),SUMIFS($H$2:H28,$A$2:A28,$A28,$C$2:C28,"卖出")-SUMIFS($H$2:H28,$A$2:A28,$A28,$C$2:C28,"买入"),"")</f>
         <v/>
       </c>
       <c r="J28" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A28)=COUNTIF($A$2:A28,$A28),SUMIFS($G$2:$G$73,$A$2:$A$73,$A28),"")</f>
-        <v/>
-      </c>
-      <c r="K28" s="0" t="n"/>
-      <c r="L28">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A28)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A28,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A28,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A28),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A28,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A28,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A28)))</f>
+        <f>SUMIFS($G$2:G28,$A$2:A28,$A28)</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A29" s="6">
-        <f>"002371"</f>
-        <v/>
+      <c r="A29" s="6" t="n">
+        <v>603986</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>北方华创</t>
+          <t>兆易创新</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2527,129 +2403,112 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>20251017</v>
-      </c>
-      <c r="E29" s="7" t="n">
-        <v>0.625</v>
+        <v>20251030</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>0.5449884259259259</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>399.43</v>
+        <v>236</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>100</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>39943</v>
+        <v>23600</v>
       </c>
       <c r="I29" s="2">
         <f>IF(AND($C29="卖出",SUMIFS($G$2:G29,$A$2:A29,$A29)=0),SUMIFS($H$2:H29,$A$2:A29,$A29,$C$2:C29,"卖出")-SUMIFS($H$2:H29,$A$2:A29,$A29,$C$2:C29,"买入"),"")</f>
         <v/>
       </c>
       <c r="J29" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A29)=COUNTIF($A$2:A29,$A29),SUMIFS($G$2:$G$73,$A$2:$A$73,$A29),"")</f>
-        <v/>
-      </c>
-      <c r="K29" s="0" t="n"/>
-      <c r="L29">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A29)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A29,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A29,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A29),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A29,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A29,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A29)))</f>
+        <f>SUMIFS($G$2:G29,$A$2:A29,$A29)</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A30" s="6">
-        <f>"002281"</f>
-        <v/>
+      <c r="A30" s="6" t="n">
+        <v>603099</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>光迅科技</t>
+          <t>长白山</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>市买1（对手方最优价格）</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>20251021</v>
-      </c>
-      <c r="E30" s="7" t="n">
-        <v>0.621550925925926</v>
+        <v>20251104</v>
+      </c>
+      <c r="E30" s="8" t="n">
+        <v>0.625</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>61.37</v>
+        <v>57.91</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>18411</v>
+        <v>5791</v>
       </c>
       <c r="I30" s="2">
         <f>IF(AND($C30="卖出",SUMIFS($G$2:G30,$A$2:A30,$A30)=0),SUMIFS($H$2:H30,$A$2:A30,$A30,$C$2:C30,"卖出")-SUMIFS($H$2:H30,$A$2:A30,$A30,$C$2:C30,"买入"),"")</f>
         <v/>
       </c>
       <c r="J30" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A30)=COUNTIF($A$2:A30,$A30),SUMIFS($G$2:$G$73,$A$2:$A$73,$A30),"")</f>
-        <v/>
-      </c>
-      <c r="K30" s="0" t="n"/>
-      <c r="L30">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A30)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A30,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A30,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A30),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A30,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A30,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A30)))</f>
+        <f>SUMIFS($G$2:G30,$A$2:A30,$A30)</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A31" s="6" t="n">
-        <v>603259</v>
+        <v>603099</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>药明康德</t>
+          <t>长白山</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>20251021</v>
-      </c>
-      <c r="E31" s="7" t="n">
-        <v>0.4680671296296297</v>
+        <v>20251104</v>
+      </c>
+      <c r="E31" s="8" t="n">
+        <v>0.625</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>101.48</v>
+        <v>57.91</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>10148</v>
+        <v>5791</v>
       </c>
       <c r="I31" s="2">
         <f>IF(AND($C31="卖出",SUMIFS($G$2:G31,$A$2:A31,$A31)=0),SUMIFS($H$2:H31,$A$2:A31,$A31,$C$2:C31,"卖出")-SUMIFS($H$2:H31,$A$2:A31,$A31,$C$2:C31,"买入"),"")</f>
         <v/>
       </c>
       <c r="J31" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A31)=COUNTIF($A$2:A31,$A31),SUMIFS($G$2:$G$73,$A$2:$A$73,$A31),"")</f>
-        <v/>
-      </c>
-      <c r="K31" s="0" t="n"/>
-      <c r="L31">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A31)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A31,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A31,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A31),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A31,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A31,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A31)))</f>
+        <f>SUMIFS($G$2:G31,$A$2:A31,$A31)</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A32" s="6">
-        <f>"002475"</f>
-        <v/>
+      <c r="A32" s="6" t="n">
+        <v>603799</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>立讯精密</t>
+          <t>华友钴业</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2658,431 +2517,382 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>20251021</v>
-      </c>
-      <c r="E32" s="7" t="n">
-        <v>0.4185185185185185</v>
+        <v>20251104</v>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>0.625</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>60.07</v>
+        <v>59.9</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>-200</v>
+        <v>-300</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>12014</v>
+        <v>17970</v>
       </c>
       <c r="I32" s="2">
         <f>IF(AND($C32="卖出",SUMIFS($G$2:G32,$A$2:A32,$A32)=0),SUMIFS($H$2:H32,$A$2:A32,$A32,$C$2:C32,"卖出")-SUMIFS($H$2:H32,$A$2:A32,$A32,$C$2:C32,"买入"),"")</f>
         <v/>
       </c>
       <c r="J32" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A32)=COUNTIF($A$2:A32,$A32),SUMIFS($G$2:$G$73,$A$2:$A$73,$A32),"")</f>
-        <v/>
-      </c>
-      <c r="K32" s="0" t="n"/>
-      <c r="L32">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A32)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A32,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A32,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A32),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A32,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A32,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A32)))</f>
+        <f>SUMIFS($G$2:G32,$A$2:A32,$A32)</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A33" s="6" t="n">
-        <v>603986</v>
+        <v>603099</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>兆易创新</t>
+          <t>长白山</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>市卖1（对手方最优价格）</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>20251023</v>
-      </c>
-      <c r="E33" s="7" t="n">
-        <v>0.6177777777777778</v>
+        <v>20251105</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>0.4134722222222222</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>208.04</v>
+        <v>56.04</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>200</v>
+        <v>-200</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>41608</v>
+        <v>11208</v>
       </c>
       <c r="I33" s="2">
         <f>IF(AND($C33="卖出",SUMIFS($G$2:G33,$A$2:A33,$A33)=0),SUMIFS($H$2:H33,$A$2:A33,$A33,$C$2:C33,"卖出")-SUMIFS($H$2:H33,$A$2:A33,$A33,$C$2:C33,"买入"),"")</f>
         <v/>
       </c>
       <c r="J33" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A33)=COUNTIF($A$2:A33,$A33),SUMIFS($G$2:$G$73,$A$2:$A$73,$A33),"")</f>
-        <v/>
-      </c>
-      <c r="K33" s="0" t="n"/>
-      <c r="L33">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A33)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A33,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A33,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A33),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A33,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A33,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A33)))</f>
+        <f>SUMIFS($G$2:G33,$A$2:A33,$A33)</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A34" s="6">
-        <f>"002371"</f>
+        <f>"002028"</f>
         <v/>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>北方华创</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>市卖1（对手方最优价格）</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>20251023</v>
-      </c>
-      <c r="E34" s="7" t="n">
-        <v>0.6161111111111112</v>
+        <v>20260119</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>0.4225347222222222</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>402.9</v>
+        <v>199</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>40290</v>
+        <v>19900</v>
       </c>
       <c r="I34" s="2">
         <f>IF(AND($C34="卖出",SUMIFS($G$2:G34,$A$2:A34,$A34)=0),SUMIFS($H$2:H34,$A$2:A34,$A34,$C$2:C34,"卖出")-SUMIFS($H$2:H34,$A$2:A34,$A34,$C$2:C34,"买入"),"")</f>
         <v/>
       </c>
       <c r="J34" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A34)=COUNTIF($A$2:A34,$A34),SUMIFS($G$2:$G$73,$A$2:$A$73,$A34),"")</f>
-        <v/>
-      </c>
-      <c r="K34" s="0" t="n"/>
-      <c r="L34">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A34)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A34,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A34,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A34),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A34,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A34,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A34)))</f>
+        <f>SUMIFS($G$2:G34,$A$2:A34,$A34)</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A35" s="6">
-        <f>"002475"</f>
-        <v/>
+      <c r="A35" s="6" t="n">
+        <v>601179</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>立讯精密</t>
+          <t>中国西电</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>20251024</v>
-      </c>
-      <c r="E35" s="7" t="n">
-        <v>0.6010069444444445</v>
+        <v>20260119</v>
+      </c>
+      <c r="E35" s="8" t="n">
+        <v>0.4008912037037037</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>63.72</v>
+        <v>14.19</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>-100</v>
+        <v>1400</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>6372</v>
+        <v>19866</v>
       </c>
       <c r="I35" s="2">
         <f>IF(AND($C35="卖出",SUMIFS($G$2:G35,$A$2:A35,$A35)=0),SUMIFS($H$2:H35,$A$2:A35,$A35,$C$2:C35,"卖出")-SUMIFS($H$2:H35,$A$2:A35,$A35,$C$2:C35,"买入"),"")</f>
         <v/>
       </c>
       <c r="J35" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A35)=COUNTIF($A$2:A35,$A35),SUMIFS($G$2:$G$73,$A$2:$A$73,$A35),"")</f>
-        <v/>
-      </c>
-      <c r="K35" s="0" t="n"/>
-      <c r="L35">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A35)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A35,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A35,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A35),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A35,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A35,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A35)))</f>
+        <f>SUMIFS($G$2:G35,$A$2:A35,$A35)</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A36" s="6" t="n">
-        <v>603986</v>
+      <c r="A36" s="6">
+        <f>"002028"</f>
+        <v/>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>兆易创新</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>20251024</v>
-      </c>
-      <c r="E36" s="7" t="n">
-        <v>0.589212962962963</v>
+        <v>20260119</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>0.3984837962962963</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>220</v>
+        <v>194</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>22000</v>
+        <v>19400</v>
       </c>
       <c r="I36" s="2">
         <f>IF(AND($C36="卖出",SUMIFS($G$2:G36,$A$2:A36,$A36)=0),SUMIFS($H$2:H36,$A$2:A36,$A36,$C$2:C36,"卖出")-SUMIFS($H$2:H36,$A$2:A36,$A36,$C$2:C36,"买入"),"")</f>
         <v/>
       </c>
       <c r="J36" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A36)=COUNTIF($A$2:A36,$A36),SUMIFS($G$2:$G$73,$A$2:$A$73,$A36),"")</f>
-        <v/>
-      </c>
-      <c r="K36" s="0" t="n"/>
-      <c r="L36">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A36)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A36,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A36,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A36),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A36,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A36,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A36)))</f>
+        <f>SUMIFS($G$2:G36,$A$2:A36,$A36)</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A37" s="6">
-        <f>"002281"</f>
-        <v/>
+      <c r="A37" s="6" t="n">
+        <v>603986</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>光迅科技</t>
+          <t>兆易创新</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>市卖2（本手方最优价格）</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>20251024</v>
-      </c>
-      <c r="E37" s="7" t="n">
-        <v>0.4184259259259259</v>
+        <v>20260119</v>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>0.3960300925925926</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>61.31</v>
+        <v>280.6</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>-300</v>
+        <v>-100</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>18393</v>
+        <v>28060</v>
       </c>
       <c r="I37" s="2">
         <f>IF(AND($C37="卖出",SUMIFS($G$2:G37,$A$2:A37,$A37)=0),SUMIFS($H$2:H37,$A$2:A37,$A37,$C$2:C37,"卖出")-SUMIFS($H$2:H37,$A$2:A37,$A37,$C$2:C37,"买入"),"")</f>
         <v/>
       </c>
       <c r="J37" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A37)=COUNTIF($A$2:A37,$A37),SUMIFS($G$2:$G$73,$A$2:$A$73,$A37),"")</f>
-        <v/>
-      </c>
-      <c r="K37" s="0" t="n"/>
-      <c r="L37">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A37)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A37,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A37,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A37),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A37,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A37,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A37)))</f>
+        <f>SUMIFS($G$2:G37,$A$2:A37,$A37)</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A38" s="6" t="n">
-        <v>603083</v>
+      <c r="A38" s="6">
+        <f>"002028"</f>
+        <v/>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>剑桥科技</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>市买2（本手方最优价格）</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>20251027</v>
-      </c>
-      <c r="E38" s="7" t="n">
-        <v>0.3990740740740741</v>
+        <v>20260121</v>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>0.3973842592592592</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>122.95</v>
+        <v>189</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>24590</v>
+        <v>18900</v>
       </c>
       <c r="I38" s="2">
         <f>IF(AND($C38="卖出",SUMIFS($G$2:G38,$A$2:A38,$A38)=0),SUMIFS($H$2:H38,$A$2:A38,$A38,$C$2:C38,"卖出")-SUMIFS($H$2:H38,$A$2:A38,$A38,$C$2:C38,"买入"),"")</f>
         <v/>
       </c>
       <c r="J38" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A38)=COUNTIF($A$2:A38,$A38),SUMIFS($G$2:$G$73,$A$2:$A$73,$A38),"")</f>
-        <v/>
-      </c>
-      <c r="K38" s="0" t="n"/>
-      <c r="L38">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A38)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A38,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A38,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A38),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A38,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A38,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A38)))</f>
+        <f>SUMIFS($G$2:G38,$A$2:A38,$A38)</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A39" s="6" t="n">
-        <v>603083</v>
+      <c r="A39" s="6">
+        <f>"002028"</f>
+        <v/>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>剑桥科技</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>20251028</v>
-      </c>
-      <c r="E39" s="7" t="n">
-        <v>0.625</v>
+        <v>20260122</v>
+      </c>
+      <c r="E39" s="8" t="n">
+        <v>0.4448611111111111</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>119.28</v>
+        <v>189</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>-200</v>
+        <v>100</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>23856</v>
+        <v>18900</v>
       </c>
       <c r="I39" s="2">
         <f>IF(AND($C39="卖出",SUMIFS($G$2:G39,$A$2:A39,$A39)=0),SUMIFS($H$2:H39,$A$2:A39,$A39,$C$2:C39,"卖出")-SUMIFS($H$2:H39,$A$2:A39,$A39,$C$2:C39,"买入"),"")</f>
         <v/>
       </c>
       <c r="J39" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A39)=COUNTIF($A$2:A39,$A39),SUMIFS($G$2:$G$73,$A$2:$A$73,$A39),"")</f>
-        <v/>
-      </c>
-      <c r="K39" s="0" t="n"/>
-      <c r="L39">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A39)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A39,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A39,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A39),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A39,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A39,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A39)))</f>
+        <f>SUMIFS($G$2:G39,$A$2:A39,$A39)</f>
         <v/>
       </c>
     </row>
     <row r="40" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A40" s="6" t="n">
-        <v>603986</v>
+        <v>600584</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>兆易创新</t>
+          <t>长电科技</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>20251029</v>
-      </c>
-      <c r="E40" s="7" t="n">
-        <v>0.4415509259259259</v>
+        <v>20260122</v>
+      </c>
+      <c r="E40" s="8" t="n">
+        <v>0.4079513888888889</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>236.41</v>
+        <v>50</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>-100</v>
+        <v>400</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>23641</v>
+        <v>20000</v>
       </c>
       <c r="I40" s="2">
         <f>IF(AND($C40="卖出",SUMIFS($G$2:G40,$A$2:A40,$A40)=0),SUMIFS($H$2:H40,$A$2:A40,$A40,$C$2:C40,"卖出")-SUMIFS($H$2:H40,$A$2:A40,$A40,$C$2:C40,"买入"),"")</f>
         <v/>
       </c>
       <c r="J40" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A40)=COUNTIF($A$2:A40,$A40),SUMIFS($G$2:$G$73,$A$2:$A$73,$A40),"")</f>
-        <v/>
-      </c>
-      <c r="K40" s="0" t="n"/>
-      <c r="L40">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A40)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A40,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A40,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A40),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A40,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A40,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A40)))</f>
+        <f>SUMIFS($G$2:G40,$A$2:A40,$A40)</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A41" s="6" t="n">
-        <v>603799</v>
+        <v>601179</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>华友钴业</t>
+          <t>中国西电</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>20251030</v>
-      </c>
-      <c r="E41" s="7" t="n">
-        <v>0.5655902777777778</v>
+        <v>20260126</v>
+      </c>
+      <c r="E41" s="8" t="n">
+        <v>0.622175925925926</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>66.09999999999999</v>
+        <v>16.16</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>300</v>
+        <v>-700</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>19830</v>
+        <v>11312</v>
       </c>
       <c r="I41" s="2">
         <f>IF(AND($C41="卖出",SUMIFS($G$2:G41,$A$2:A41,$A41)=0),SUMIFS($H$2:H41,$A$2:A41,$A41,$C$2:C41,"卖出")-SUMIFS($H$2:H41,$A$2:A41,$A41,$C$2:C41,"买入"),"")</f>
         <v/>
       </c>
       <c r="J41" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A41)=COUNTIF($A$2:A41,$A41),SUMIFS($G$2:$G$73,$A$2:$A$73,$A41),"")</f>
-        <v/>
-      </c>
-      <c r="K41" s="0" t="n"/>
-      <c r="L41">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A41)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A41,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A41,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A41),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A41,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A41,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A41)))</f>
+        <f>SUMIFS($G$2:G41,$A$2:A41,$A41)</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A42" s="6" t="n">
-        <v>603986</v>
+        <v>600584</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>兆易创新</t>
+          <t>长电科技</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -3091,41 +2901,37 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>20251030</v>
-      </c>
-      <c r="E42" s="7" t="n">
-        <v>0.5449884259259259</v>
+        <v>20260127</v>
+      </c>
+      <c r="E42" s="8" t="n">
+        <v>0.5894791666666667</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>236</v>
+        <v>48.3</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>23600</v>
+        <v>9660</v>
       </c>
       <c r="I42" s="2">
         <f>IF(AND($C42="卖出",SUMIFS($G$2:G42,$A$2:A42,$A42)=0),SUMIFS($H$2:H42,$A$2:A42,$A42,$C$2:C42,"卖出")-SUMIFS($H$2:H42,$A$2:A42,$A42,$C$2:C42,"买入"),"")</f>
         <v/>
       </c>
       <c r="J42" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A42)=COUNTIF($A$2:A42,$A42),SUMIFS($G$2:$G$73,$A$2:$A$73,$A42),"")</f>
-        <v/>
-      </c>
-      <c r="K42" s="0" t="n"/>
-      <c r="L42">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A42)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A42,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A42,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A42),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A42,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A42,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A42)))</f>
+        <f>SUMIFS($G$2:G42,$A$2:A42,$A42)</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A43" s="6" t="n">
-        <v>603099</v>
+      <c r="A43" s="6">
+        <f>"002475"</f>
+        <v/>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>长白山</t>
+          <t>立讯精密</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -3134,41 +2940,37 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>20251104</v>
-      </c>
-      <c r="E43" s="7" t="n">
-        <v>0.625</v>
+        <v>20260127</v>
+      </c>
+      <c r="E43" s="8" t="n">
+        <v>0.4139699074074074</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>57.91</v>
+        <v>53.2</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>5791</v>
+        <v>10640</v>
       </c>
       <c r="I43" s="2">
         <f>IF(AND($C43="卖出",SUMIFS($G$2:G43,$A$2:A43,$A43)=0),SUMIFS($H$2:H43,$A$2:A43,$A43,$C$2:C43,"卖出")-SUMIFS($H$2:H43,$A$2:A43,$A43,$C$2:C43,"买入"),"")</f>
         <v/>
       </c>
       <c r="J43" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A43)=COUNTIF($A$2:A43,$A43),SUMIFS($G$2:$G$73,$A$2:$A$73,$A43),"")</f>
-        <v/>
-      </c>
-      <c r="K43" s="0" t="n"/>
-      <c r="L43">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A43)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A43,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A43,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A43),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A43,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A43,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A43)))</f>
+        <f>SUMIFS($G$2:G43,$A$2:A43,$A43)</f>
         <v/>
       </c>
     </row>
     <row r="44" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A44" s="6" t="n">
-        <v>603099</v>
+      <c r="A44" s="6">
+        <f>"002028"</f>
+        <v/>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>长白山</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -3177,41 +2979,37 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>20251104</v>
-      </c>
-      <c r="E44" s="7" t="n">
-        <v>0.625</v>
+        <v>20260129</v>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>0.5778125</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>57.91</v>
+        <v>186.2</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>100</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>5791</v>
+        <v>18620</v>
       </c>
       <c r="I44" s="2">
         <f>IF(AND($C44="卖出",SUMIFS($G$2:G44,$A$2:A44,$A44)=0),SUMIFS($H$2:H44,$A$2:A44,$A44,$C$2:C44,"卖出")-SUMIFS($H$2:H44,$A$2:A44,$A44,$C$2:C44,"买入"),"")</f>
         <v/>
       </c>
       <c r="J44" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A44)=COUNTIF($A$2:A44,$A44),SUMIFS($G$2:$G$73,$A$2:$A$73,$A44),"")</f>
-        <v/>
-      </c>
-      <c r="K44" s="0" t="n"/>
-      <c r="L44">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A44)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A44,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A44,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A44),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A44,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A44,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A44)))</f>
+        <f>SUMIFS($G$2:G44,$A$2:A44,$A44)</f>
         <v/>
       </c>
     </row>
     <row r="45" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A45" s="6" t="n">
-        <v>603799</v>
+      <c r="A45" s="6">
+        <f>"002475"</f>
+        <v/>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>华友钴业</t>
+          <t>立讯精密</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3220,85 +3018,75 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>20251104</v>
-      </c>
-      <c r="E45" s="7" t="n">
-        <v>0.625</v>
+        <v>20260129</v>
+      </c>
+      <c r="E45" s="8" t="n">
+        <v>0.5719907407407407</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>59.9</v>
+        <v>52.2</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>-300</v>
+        <v>-100</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>17970</v>
+        <v>5220</v>
       </c>
       <c r="I45" s="2">
         <f>IF(AND($C45="卖出",SUMIFS($G$2:G45,$A$2:A45,$A45)=0),SUMIFS($H$2:H45,$A$2:A45,$A45,$C$2:C45,"卖出")-SUMIFS($H$2:H45,$A$2:A45,$A45,$C$2:C45,"买入"),"")</f>
         <v/>
       </c>
       <c r="J45" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A45)=COUNTIF($A$2:A45,$A45),SUMIFS($G$2:$G$73,$A$2:$A$73,$A45),"")</f>
-        <v/>
-      </c>
-      <c r="K45" s="0" t="n"/>
-      <c r="L45">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A45)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A45,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A45,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A45),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A45,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A45,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A45)))</f>
+        <f>SUMIFS($G$2:G45,$A$2:A45,$A45)</f>
         <v/>
       </c>
     </row>
     <row r="46" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A46" s="6" t="n">
-        <v>603099</v>
+        <v>600584</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>长白山</t>
+          <t>长电科技</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>市卖1（对手方最优价格）</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>20251105</v>
-      </c>
-      <c r="E46" s="7" t="n">
-        <v>0.4134722222222222</v>
+        <v>20260129</v>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>0.5709953703703704</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>56.04</v>
+        <v>49.2</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>-200</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>11208</v>
+        <v>9840</v>
       </c>
       <c r="I46" s="2">
         <f>IF(AND($C46="卖出",SUMIFS($G$2:G46,$A$2:A46,$A46)=0),SUMIFS($H$2:H46,$A$2:A46,$A46,$C$2:C46,"卖出")-SUMIFS($H$2:H46,$A$2:A46,$A46,$C$2:C46,"买入"),"")</f>
         <v/>
       </c>
       <c r="J46" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A46)=COUNTIF($A$2:A46,$A46),SUMIFS($G$2:$G$73,$A$2:$A$73,$A46),"")</f>
-        <v/>
-      </c>
-      <c r="K46" s="0" t="n"/>
-      <c r="L46">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A46)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A46,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A46,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A46),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A46,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A46,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A46)))</f>
+        <f>SUMIFS($G$2:G46,$A$2:A46,$A46)</f>
         <v/>
       </c>
     </row>
     <row r="47" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A47" s="6">
-        <f>"002028"</f>
+        <f>"002475"</f>
         <v/>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>思源电气</t>
+          <t>立讯精密</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3307,41 +3095,37 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>20260119</v>
-      </c>
-      <c r="E47" s="7" t="n">
-        <v>0.4225347222222222</v>
+        <v>20260129</v>
+      </c>
+      <c r="E47" s="8" t="n">
+        <v>0.5454629629629629</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>199</v>
+        <v>51.9</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>100</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>19900</v>
+        <v>5190</v>
       </c>
       <c r="I47" s="2">
         <f>IF(AND($C47="卖出",SUMIFS($G$2:G47,$A$2:A47,$A47)=0),SUMIFS($H$2:H47,$A$2:A47,$A47,$C$2:C47,"卖出")-SUMIFS($H$2:H47,$A$2:A47,$A47,$C$2:C47,"买入"),"")</f>
         <v/>
       </c>
       <c r="J47" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A47)=COUNTIF($A$2:A47,$A47),SUMIFS($G$2:$G$73,$A$2:$A$73,$A47),"")</f>
-        <v/>
-      </c>
-      <c r="K47" s="0" t="n"/>
-      <c r="L47">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A47)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A47,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A47,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A47),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A47,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A47,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A47)))</f>
+        <f>SUMIFS($G$2:G47,$A$2:A47,$A47)</f>
         <v/>
       </c>
     </row>
     <row r="48" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A48" s="6" t="n">
-        <v>601179</v>
+      <c r="A48" s="6">
+        <f>"002028"</f>
+        <v/>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>中国西电</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3350,42 +3134,36 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>20260119</v>
-      </c>
-      <c r="E48" s="7" t="n">
-        <v>0.4008912037037037</v>
+        <v>20260129</v>
+      </c>
+      <c r="E48" s="8" t="n">
+        <v>0.5423958333333333</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>14.19</v>
+        <v>188</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>1400</v>
+        <v>100</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>19866</v>
+        <v>18800</v>
       </c>
       <c r="I48" s="2">
         <f>IF(AND($C48="卖出",SUMIFS($G$2:G48,$A$2:A48,$A48)=0),SUMIFS($H$2:H48,$A$2:A48,$A48,$C$2:C48,"卖出")-SUMIFS($H$2:H48,$A$2:A48,$A48,$C$2:C48,"买入"),"")</f>
         <v/>
       </c>
       <c r="J48" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A48)=COUNTIF($A$2:A48,$A48),SUMIFS($G$2:$G$73,$A$2:$A$73,$A48),"")</f>
-        <v/>
-      </c>
-      <c r="K48" s="0" t="n"/>
-      <c r="L48">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A48)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A48,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A48,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A48),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A48,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A48,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A48)))</f>
+        <f>SUMIFS($G$2:G48,$A$2:A48,$A48)</f>
         <v/>
       </c>
     </row>
     <row r="49" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A49" s="6">
-        <f>"002028"</f>
-        <v/>
+      <c r="A49" s="6" t="n">
+        <v>601179</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>思源电气</t>
+          <t>中国西电</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3394,129 +3172,114 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>20260119</v>
-      </c>
-      <c r="E49" s="7" t="n">
-        <v>0.3984837962962963</v>
+        <v>20260130</v>
+      </c>
+      <c r="E49" s="8" t="n">
+        <v>0.4404398148148148</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>194</v>
+        <v>14</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>19400</v>
+        <v>5600</v>
       </c>
       <c r="I49" s="2">
         <f>IF(AND($C49="卖出",SUMIFS($G$2:G49,$A$2:A49,$A49)=0),SUMIFS($H$2:H49,$A$2:A49,$A49,$C$2:C49,"卖出")-SUMIFS($H$2:H49,$A$2:A49,$A49,$C$2:C49,"买入"),"")</f>
         <v/>
       </c>
       <c r="J49" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A49)=COUNTIF($A$2:A49,$A49),SUMIFS($G$2:$G$73,$A$2:$A$73,$A49),"")</f>
-        <v/>
-      </c>
-      <c r="K49" s="0" t="n"/>
-      <c r="L49">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A49)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A49,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A49,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A49),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A49,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A49,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A49)))</f>
+        <f>SUMIFS($G$2:G49,$A$2:A49,$A49)</f>
         <v/>
       </c>
     </row>
     <row r="50" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A50" s="6" t="n">
-        <v>603986</v>
+      <c r="A50" s="6">
+        <f>"002028"</f>
+        <v/>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>兆易创新</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>20260119</v>
-      </c>
-      <c r="E50" s="7" t="n">
-        <v>0.3960300925925926</v>
+        <v>20260130</v>
+      </c>
+      <c r="E50" s="8" t="n">
+        <v>0.4310300925925926</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>280.6</v>
+        <v>180</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>28060</v>
+        <v>18000</v>
       </c>
       <c r="I50" s="2">
         <f>IF(AND($C50="卖出",SUMIFS($G$2:G50,$A$2:A50,$A50)=0),SUMIFS($H$2:H50,$A$2:A50,$A50,$C$2:C50,"卖出")-SUMIFS($H$2:H50,$A$2:A50,$A50,$C$2:C50,"买入"),"")</f>
         <v/>
       </c>
       <c r="J50" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A50)=COUNTIF($A$2:A50,$A50),SUMIFS($G$2:$G$73,$A$2:$A$73,$A50),"")</f>
-        <v/>
-      </c>
-      <c r="K50" s="0" t="n"/>
-      <c r="L50">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A50)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A50,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A50,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A50),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A50,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A50,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A50)))</f>
+        <f>SUMIFS($G$2:G50,$A$2:A50,$A50)</f>
         <v/>
       </c>
     </row>
     <row r="51" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A51" s="6">
-        <f>"002028"</f>
+        <f>"002475"</f>
         <v/>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>思源电气</t>
+          <t>立讯精密</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>20260121</v>
-      </c>
-      <c r="E51" s="7" t="n">
-        <v>0.3973842592592592</v>
+        <v>20260202</v>
+      </c>
+      <c r="E51" s="8" t="n">
+        <v>0.6189930555555555</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>189</v>
+        <v>52.08</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>100</v>
+        <v>-300</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>18900</v>
+        <v>15624</v>
       </c>
       <c r="I51" s="2">
         <f>IF(AND($C51="卖出",SUMIFS($G$2:G51,$A$2:A51,$A51)=0),SUMIFS($H$2:H51,$A$2:A51,$A51,$C$2:C51,"卖出")-SUMIFS($H$2:H51,$A$2:A51,$A51,$C$2:C51,"买入"),"")</f>
         <v/>
       </c>
       <c r="J51" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A51)=COUNTIF($A$2:A51,$A51),SUMIFS($G$2:$G$73,$A$2:$A$73,$A51),"")</f>
-        <v/>
-      </c>
-      <c r="K51" s="0" t="n"/>
-      <c r="L51">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A51)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A51,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A51,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A51),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A51,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A51,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A51)))</f>
+        <f>SUMIFS($G$2:G51,$A$2:A51,$A51)</f>
         <v/>
       </c>
     </row>
     <row r="52" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A52" s="6">
-        <f>"002028"</f>
-        <v/>
+      <c r="A52" s="6" t="n">
+        <v>600584</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>思源电气</t>
+          <t>长电科技</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3525,84 +3288,75 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>20260122</v>
-      </c>
-      <c r="E52" s="7" t="n">
-        <v>0.4448611111111111</v>
+        <v>20260202</v>
+      </c>
+      <c r="E52" s="8" t="n">
+        <v>0.5656944444444445</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>189</v>
+        <v>46.8</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>100</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>18900</v>
+        <v>4680</v>
       </c>
       <c r="I52" s="2">
         <f>IF(AND($C52="卖出",SUMIFS($G$2:G52,$A$2:A52,$A52)=0),SUMIFS($H$2:H52,$A$2:A52,$A52,$C$2:C52,"卖出")-SUMIFS($H$2:H52,$A$2:A52,$A52,$C$2:C52,"买入"),"")</f>
         <v/>
       </c>
       <c r="J52" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A52)=COUNTIF($A$2:A52,$A52),SUMIFS($G$2:$G$73,$A$2:$A$73,$A52),"")</f>
-        <v/>
-      </c>
-      <c r="K52" s="0" t="n"/>
-      <c r="L52">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A52)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A52,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A52,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A52),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A52,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A52,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A52)))</f>
+        <f>SUMIFS($G$2:G52,$A$2:A52,$A52)</f>
         <v/>
       </c>
     </row>
     <row r="53" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A53" s="6" t="n">
-        <v>600584</v>
+        <v>601179</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>长电科技</t>
+          <t>中国西电</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>20260122</v>
-      </c>
-      <c r="E53" s="7" t="n">
-        <v>0.4079513888888889</v>
+        <v>20260202</v>
+      </c>
+      <c r="E53" s="8" t="n">
+        <v>0.5599421296296296</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>50</v>
+        <v>15.7</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>400</v>
+        <v>-1100</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>20000</v>
+        <v>17270</v>
       </c>
       <c r="I53" s="2">
         <f>IF(AND($C53="卖出",SUMIFS($G$2:G53,$A$2:A53,$A53)=0),SUMIFS($H$2:H53,$A$2:A53,$A53,$C$2:C53,"卖出")-SUMIFS($H$2:H53,$A$2:A53,$A53,$C$2:C53,"买入"),"")</f>
         <v/>
       </c>
       <c r="J53" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A53)=COUNTIF($A$2:A53,$A53),SUMIFS($G$2:$G$73,$A$2:$A$73,$A53),"")</f>
-        <v/>
-      </c>
-      <c r="K53" s="0" t="n"/>
-      <c r="L53">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A53)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A53,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A53,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A53),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A53,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A53,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A53)))</f>
+        <f>SUMIFS($G$2:G53,$A$2:A53,$A53)</f>
         <v/>
       </c>
     </row>
     <row r="54" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A54" s="6" t="n">
-        <v>601179</v>
+      <c r="A54" s="6">
+        <f>"002028"</f>
+        <v/>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>中国西电</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3611,118 +3365,104 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>20260126</v>
-      </c>
-      <c r="E54" s="7" t="n">
-        <v>0.622175925925926</v>
+        <v>20260202</v>
+      </c>
+      <c r="E54" s="8" t="n">
+        <v>0.4467476851851852</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>16.16</v>
+        <v>191</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>-700</v>
+        <v>-100</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>11312</v>
+        <v>19100</v>
       </c>
       <c r="I54" s="2">
         <f>IF(AND($C54="卖出",SUMIFS($G$2:G54,$A$2:A54,$A54)=0),SUMIFS($H$2:H54,$A$2:A54,$A54,$C$2:C54,"卖出")-SUMIFS($H$2:H54,$A$2:A54,$A54,$C$2:C54,"买入"),"")</f>
         <v/>
       </c>
       <c r="J54" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A54)=COUNTIF($A$2:A54,$A54),SUMIFS($G$2:$G$73,$A$2:$A$73,$A54),"")</f>
-        <v/>
-      </c>
-      <c r="K54" s="0" t="n"/>
-      <c r="L54">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A54)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A54,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A54,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A54),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A54,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A54,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A54)))</f>
+        <f>SUMIFS($G$2:G54,$A$2:A54,$A54)</f>
         <v/>
       </c>
     </row>
     <row r="55" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A55" s="6" t="n">
-        <v>600584</v>
+      <c r="A55" s="6">
+        <f>"002475"</f>
+        <v/>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>长电科技</t>
+          <t>立讯精密</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>20260127</v>
-      </c>
-      <c r="E55" s="7" t="n">
-        <v>0.5894791666666667</v>
+        <v>20260202</v>
+      </c>
+      <c r="E55" s="8" t="n">
+        <v>0.4406712962962963</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>48.3</v>
+        <v>53.09</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>200</v>
+        <v>-200</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>9660</v>
+        <v>10618</v>
       </c>
       <c r="I55" s="2">
         <f>IF(AND($C55="卖出",SUMIFS($G$2:G55,$A$2:A55,$A55)=0),SUMIFS($H$2:H55,$A$2:A55,$A55,$C$2:C55,"卖出")-SUMIFS($H$2:H55,$A$2:A55,$A55,$C$2:C55,"买入"),"")</f>
         <v/>
       </c>
       <c r="J55" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A55)=COUNTIF($A$2:A55,$A55),SUMIFS($G$2:$G$73,$A$2:$A$73,$A55),"")</f>
-        <v/>
-      </c>
-      <c r="K55" s="0" t="n"/>
-      <c r="L55">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A55)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A55,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A55,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A55),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A55,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A55,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A55)))</f>
+        <f>SUMIFS($G$2:G55,$A$2:A55,$A55)</f>
         <v/>
       </c>
     </row>
     <row r="56" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A56" s="6">
-        <f>"002475"</f>
+        <f>"002028"</f>
         <v/>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>立讯精密</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>20260127</v>
-      </c>
-      <c r="E56" s="7" t="n">
-        <v>0.4139699074074074</v>
+        <v>20260203</v>
+      </c>
+      <c r="E56" s="8" t="n">
+        <v>0.4091782407407407</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>53.2</v>
+        <v>194</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>200</v>
+        <v>-100</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>10640</v>
+        <v>19400</v>
       </c>
       <c r="I56" s="2">
         <f>IF(AND($C56="卖出",SUMIFS($G$2:G56,$A$2:A56,$A56)=0),SUMIFS($H$2:H56,$A$2:A56,$A56,$C$2:C56,"卖出")-SUMIFS($H$2:H56,$A$2:A56,$A56,$C$2:C56,"买入"),"")</f>
         <v/>
       </c>
       <c r="J56" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A56)=COUNTIF($A$2:A56,$A56),SUMIFS($G$2:$G$73,$A$2:$A$73,$A56),"")</f>
-        <v/>
-      </c>
-      <c r="K56" s="0" t="n"/>
-      <c r="L56">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A56)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A56,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A56,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A56),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A56,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A56,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A56)))</f>
+        <f>SUMIFS($G$2:G56,$A$2:A56,$A56)</f>
         <v/>
       </c>
     </row>
@@ -3742,75 +3482,65 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>20260129</v>
-      </c>
-      <c r="E57" s="7" t="n">
-        <v>0.5778125</v>
+        <v>20260205</v>
+      </c>
+      <c r="E57" s="8" t="n">
+        <v>0.4043634259259259</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>186.2</v>
+        <v>195</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>100</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>18620</v>
+        <v>19500</v>
       </c>
       <c r="I57" s="2">
         <f>IF(AND($C57="卖出",SUMIFS($G$2:G57,$A$2:A57,$A57)=0),SUMIFS($H$2:H57,$A$2:A57,$A57,$C$2:C57,"卖出")-SUMIFS($H$2:H57,$A$2:A57,$A57,$C$2:C57,"买入"),"")</f>
         <v/>
       </c>
       <c r="J57" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A57)=COUNTIF($A$2:A57,$A57),SUMIFS($G$2:$G$73,$A$2:$A$73,$A57),"")</f>
-        <v/>
-      </c>
-      <c r="K57" s="0" t="n"/>
-      <c r="L57">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A57)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A57,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A57,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A57),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A57,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A57,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A57)))</f>
+        <f>SUMIFS($G$2:G57,$A$2:A57,$A57)</f>
         <v/>
       </c>
     </row>
     <row r="58" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A58" s="6">
-        <f>"002475"</f>
+        <f>"002028"</f>
         <v/>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>立讯精密</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>20260129</v>
-      </c>
-      <c r="E58" s="7" t="n">
-        <v>0.5719907407407407</v>
+        <v>20260209</v>
+      </c>
+      <c r="E58" s="8" t="n">
+        <v>0.4454861111111111</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>52.2</v>
+        <v>198.73</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>5220</v>
+        <v>19873</v>
       </c>
       <c r="I58" s="2">
         <f>IF(AND($C58="卖出",SUMIFS($G$2:G58,$A$2:A58,$A58)=0),SUMIFS($H$2:H58,$A$2:A58,$A58,$C$2:C58,"卖出")-SUMIFS($H$2:H58,$A$2:A58,$A58,$C$2:C58,"买入"),"")</f>
         <v/>
       </c>
       <c r="J58" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A58)=COUNTIF($A$2:A58,$A58),SUMIFS($G$2:$G$73,$A$2:$A$73,$A58),"")</f>
-        <v/>
-      </c>
-      <c r="K58" s="0" t="n"/>
-      <c r="L58">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A58)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A58,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A58,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A58),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A58,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A58,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A58)))</f>
+        <f>SUMIFS($G$2:G58,$A$2:A58,$A58)</f>
         <v/>
       </c>
     </row>
@@ -3825,90 +3555,79 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>卖出</t>
+          <t>买入</t>
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>20260129</v>
-      </c>
-      <c r="E59" s="7" t="n">
-        <v>0.5709953703703704</v>
+        <v>20260209</v>
+      </c>
+      <c r="E59" s="8" t="n">
+        <v>0.4388657407407408</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>49.2</v>
+        <v>46.09</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>-200</v>
+        <v>200</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>9840</v>
+        <v>9218</v>
       </c>
       <c r="I59" s="2">
         <f>IF(AND($C59="卖出",SUMIFS($G$2:G59,$A$2:A59,$A59)=0),SUMIFS($H$2:H59,$A$2:A59,$A59,$C$2:C59,"卖出")-SUMIFS($H$2:H59,$A$2:A59,$A59,$C$2:C59,"买入"),"")</f>
         <v/>
       </c>
       <c r="J59" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A59)=COUNTIF($A$2:A59,$A59),SUMIFS($G$2:$G$73,$A$2:$A$73,$A59),"")</f>
-        <v/>
-      </c>
-      <c r="K59" s="0" t="n"/>
-      <c r="L59">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A59)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A59,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A59,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A59),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A59,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A59,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A59)))</f>
+        <f>SUMIFS($G$2:G59,$A$2:A59,$A59)</f>
         <v/>
       </c>
     </row>
     <row r="60" ht="20.4" customFormat="1" customHeight="1" s="2">
       <c r="A60" s="6">
-        <f>"002475"</f>
+        <f>"002028"</f>
         <v/>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>立讯精密</t>
+          <t>思源电气</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>买入</t>
+          <t>卖出</t>
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>20260129</v>
-      </c>
-      <c r="E60" s="7" t="n">
-        <v>0.5454629629629629</v>
+        <v>20260209</v>
+      </c>
+      <c r="E60" s="8" t="n">
+        <v>0.4105902777777778</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>51.9</v>
+        <v>192.5</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>100</v>
+        <v>-200</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>5190</v>
+        <v>38500</v>
       </c>
       <c r="I60" s="2">
         <f>IF(AND($C60="卖出",SUMIFS($G$2:G60,$A$2:A60,$A60)=0),SUMIFS($H$2:H60,$A$2:A60,$A60,$C$2:C60,"卖出")-SUMIFS($H$2:H60,$A$2:A60,$A60,$C$2:C60,"买入"),"")</f>
         <v/>
       </c>
       <c r="J60" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A60)=COUNTIF($A$2:A60,$A60),SUMIFS($G$2:$G$73,$A$2:$A$73,$A60),"")</f>
-        <v/>
-      </c>
-      <c r="K60" s="0" t="n"/>
-      <c r="L60">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A60)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A60,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A60,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A60),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A60,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A60,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A60)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A61" s="6">
-        <f>"002028"</f>
-        <v/>
+        <f>SUMIFS($G$2:G60,$A$2:A60,$A60)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="20.4" customHeight="1" s="4">
+      <c r="A61" s="6" t="n">
+        <v>600584</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>思源电气</t>
+          <t>长电科技</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -3916,561 +3635,41 @@
           <t>买入</t>
         </is>
       </c>
-      <c r="D61" s="2" t="n">
-        <v>20260129</v>
-      </c>
-      <c r="E61" s="7" t="n">
-        <v>0.5423958333333333</v>
+      <c r="D61" s="7" t="n">
+        <v>20260226</v>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>0.549131944444444</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>188</v>
+        <v>48.3</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>18800</v>
-      </c>
-      <c r="I61" s="2">
-        <f>IF(AND($C61="卖出",SUMIFS($G$2:G61,$A$2:A61,$A61)=0),SUMIFS($H$2:H61,$A$2:A61,$A61,$C$2:C61,"卖出")-SUMIFS($H$2:H61,$A$2:A61,$A61,$C$2:C61,"买入"),"")</f>
-        <v/>
+        <v>19320</v>
       </c>
       <c r="J61" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A61)=COUNTIF($A$2:A61,$A61),SUMIFS($G$2:$G$73,$A$2:$A$73,$A61),"")</f>
-        <v/>
-      </c>
-      <c r="K61" s="0" t="n"/>
-      <c r="L61">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A61)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A61,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A61,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A61),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A61,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A61,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A61)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A62" s="6" t="n">
-        <v>601179</v>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>中国西电</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>买入</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="n">
-        <v>20260130</v>
-      </c>
-      <c r="E62" s="7" t="n">
-        <v>0.4404398148148148</v>
-      </c>
-      <c r="F62" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="G62" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="H62" s="2" t="n">
-        <v>5600</v>
-      </c>
-      <c r="I62" s="2">
-        <f>IF(AND($C62="卖出",SUMIFS($G$2:G62,$A$2:A62,$A62)=0),SUMIFS($H$2:H62,$A$2:A62,$A62,$C$2:C62,"卖出")-SUMIFS($H$2:H62,$A$2:A62,$A62,$C$2:C62,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J62" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A62)=COUNTIF($A$2:A62,$A62),SUMIFS($G$2:$G$73,$A$2:$A$73,$A62),"")</f>
-        <v/>
-      </c>
-      <c r="K62" s="0" t="n"/>
-      <c r="L62">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A62)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A62,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A62,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A62),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A62,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A62,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A62)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A63" s="6">
-        <f>"002028"</f>
-        <v/>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>思源电气</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>买入</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="n">
-        <v>20260130</v>
-      </c>
-      <c r="E63" s="7" t="n">
-        <v>0.4310300925925926</v>
-      </c>
-      <c r="F63" s="2" t="n">
-        <v>180</v>
-      </c>
-      <c r="G63" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="H63" s="2" t="n">
-        <v>18000</v>
-      </c>
-      <c r="I63" s="2">
-        <f>IF(AND($C63="卖出",SUMIFS($G$2:G63,$A$2:A63,$A63)=0),SUMIFS($H$2:H63,$A$2:A63,$A63,$C$2:C63,"卖出")-SUMIFS($H$2:H63,$A$2:A63,$A63,$C$2:C63,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J63" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A63)=COUNTIF($A$2:A63,$A63),SUMIFS($G$2:$G$73,$A$2:$A$73,$A63),"")</f>
-        <v/>
-      </c>
-      <c r="K63" s="0" t="n"/>
-      <c r="L63">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A63)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A63,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A63,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A63),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A63,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A63,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A63)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A64" s="6">
-        <f>"002475"</f>
-        <v/>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>立讯精密</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>卖出</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="n">
-        <v>20260202</v>
-      </c>
-      <c r="E64" s="7" t="n">
-        <v>0.6189930555555555</v>
-      </c>
-      <c r="F64" s="2" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="G64" s="2" t="n">
-        <v>-300</v>
-      </c>
-      <c r="H64" s="2" t="n">
-        <v>15624</v>
-      </c>
-      <c r="I64" s="2">
-        <f>IF(AND($C64="卖出",SUMIFS($G$2:G64,$A$2:A64,$A64)=0),SUMIFS($H$2:H64,$A$2:A64,$A64,$C$2:C64,"卖出")-SUMIFS($H$2:H64,$A$2:A64,$A64,$C$2:C64,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J64" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A64)=COUNTIF($A$2:A64,$A64),SUMIFS($G$2:$G$73,$A$2:$A$73,$A64),"")</f>
-        <v/>
-      </c>
-      <c r="K64" s="0" t="n"/>
-      <c r="L64">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A64)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A64,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A64,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A64),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A64,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A64,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A64)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A65" s="6" t="n">
-        <v>600584</v>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>长电科技</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>买入</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="n">
-        <v>20260202</v>
-      </c>
-      <c r="E65" s="7" t="n">
-        <v>0.5656944444444445</v>
-      </c>
-      <c r="F65" s="2" t="n">
-        <v>46.8</v>
-      </c>
-      <c r="G65" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="H65" s="2" t="n">
-        <v>4680</v>
-      </c>
-      <c r="I65" s="2">
-        <f>IF(AND($C65="卖出",SUMIFS($G$2:G65,$A$2:A65,$A65)=0),SUMIFS($H$2:H65,$A$2:A65,$A65,$C$2:C65,"卖出")-SUMIFS($H$2:H65,$A$2:A65,$A65,$C$2:C65,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J65" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A65)=COUNTIF($A$2:A65,$A65),SUMIFS($G$2:$G$73,$A$2:$A$73,$A65),"")</f>
-        <v/>
-      </c>
-      <c r="K65" s="0" t="n"/>
-      <c r="L65">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A65)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A65,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A65,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A65),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A65,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A65,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A65)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A66" s="6" t="n">
-        <v>601179</v>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>中国西电</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>卖出</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="n">
-        <v>20260202</v>
-      </c>
-      <c r="E66" s="7" t="n">
-        <v>0.5599421296296296</v>
-      </c>
-      <c r="F66" s="2" t="n">
-        <v>15.7</v>
-      </c>
-      <c r="G66" s="2" t="n">
-        <v>-1100</v>
-      </c>
-      <c r="H66" s="2" t="n">
-        <v>17270</v>
-      </c>
-      <c r="I66" s="2">
-        <f>IF(AND($C66="卖出",SUMIFS($G$2:G66,$A$2:A66,$A66)=0),SUMIFS($H$2:H66,$A$2:A66,$A66,$C$2:C66,"卖出")-SUMIFS($H$2:H66,$A$2:A66,$A66,$C$2:C66,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J66" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A66)=COUNTIF($A$2:A66,$A66),SUMIFS($G$2:$G$73,$A$2:$A$73,$A66),"")</f>
-        <v/>
-      </c>
-      <c r="K66" s="0" t="n"/>
-      <c r="L66">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A66)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A66,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A66,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A66),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A66,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A66,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A66)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A67" s="6">
-        <f>"002028"</f>
-        <v/>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>思源电气</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>卖出</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="n">
-        <v>20260202</v>
-      </c>
-      <c r="E67" s="7" t="n">
-        <v>0.4467476851851852</v>
-      </c>
-      <c r="F67" s="2" t="n">
-        <v>191</v>
-      </c>
-      <c r="G67" s="2" t="n">
-        <v>-100</v>
-      </c>
-      <c r="H67" s="2" t="n">
-        <v>19100</v>
-      </c>
-      <c r="I67" s="2">
-        <f>IF(AND($C67="卖出",SUMIFS($G$2:G67,$A$2:A67,$A67)=0),SUMIFS($H$2:H67,$A$2:A67,$A67,$C$2:C67,"卖出")-SUMIFS($H$2:H67,$A$2:A67,$A67,$C$2:C67,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J67" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A67)=COUNTIF($A$2:A67,$A67),SUMIFS($G$2:$G$73,$A$2:$A$73,$A67),"")</f>
-        <v/>
-      </c>
-      <c r="K67" s="0" t="n"/>
-      <c r="L67">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A67)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A67,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A67,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A67),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A67,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A67,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A67)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A68" s="6">
-        <f>"002475"</f>
-        <v/>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>立讯精密</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>卖出</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="n">
-        <v>20260202</v>
-      </c>
-      <c r="E68" s="7" t="n">
-        <v>0.4406712962962963</v>
-      </c>
-      <c r="F68" s="2" t="n">
-        <v>53.09</v>
-      </c>
-      <c r="G68" s="2" t="n">
-        <v>-200</v>
-      </c>
-      <c r="H68" s="2" t="n">
-        <v>10618</v>
-      </c>
-      <c r="I68" s="2">
-        <f>IF(AND($C68="卖出",SUMIFS($G$2:G68,$A$2:A68,$A68)=0),SUMIFS($H$2:H68,$A$2:A68,$A68,$C$2:C68,"卖出")-SUMIFS($H$2:H68,$A$2:A68,$A68,$C$2:C68,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J68" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A68)=COUNTIF($A$2:A68,$A68),SUMIFS($G$2:$G$73,$A$2:$A$73,$A68),"")</f>
-        <v/>
-      </c>
-      <c r="K68" s="0" t="n"/>
-      <c r="L68">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A68)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A68,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A68,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A68),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A68,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A68,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A68)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A69" s="6">
-        <f>"002028"</f>
-        <v/>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>思源电气</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>卖出</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="n">
-        <v>20260203</v>
-      </c>
-      <c r="E69" s="7" t="n">
-        <v>0.4091782407407407</v>
-      </c>
-      <c r="F69" s="2" t="n">
-        <v>194</v>
-      </c>
-      <c r="G69" s="2" t="n">
-        <v>-100</v>
-      </c>
-      <c r="H69" s="2" t="n">
-        <v>19400</v>
-      </c>
-      <c r="I69" s="2">
-        <f>IF(AND($C69="卖出",SUMIFS($G$2:G69,$A$2:A69,$A69)=0),SUMIFS($H$2:H69,$A$2:A69,$A69,$C$2:C69,"卖出")-SUMIFS($H$2:H69,$A$2:A69,$A69,$C$2:C69,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J69" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A69)=COUNTIF($A$2:A69,$A69),SUMIFS($G$2:$G$73,$A$2:$A$73,$A69),"")</f>
-        <v/>
-      </c>
-      <c r="K69" s="0" t="n"/>
-      <c r="L69">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A69)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A69,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A69,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A69),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A69,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A69,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A69)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A70" s="6">
-        <f>"002028"</f>
-        <v/>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>思源电气</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>买入</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="n">
-        <v>20260205</v>
-      </c>
-      <c r="E70" s="7" t="n">
-        <v>0.4043634259259259</v>
-      </c>
-      <c r="F70" s="2" t="n">
-        <v>195</v>
-      </c>
-      <c r="G70" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="H70" s="2" t="n">
-        <v>19500</v>
-      </c>
-      <c r="I70" s="2">
-        <f>IF(AND($C70="卖出",SUMIFS($G$2:G70,$A$2:A70,$A70)=0),SUMIFS($H$2:H70,$A$2:A70,$A70,$C$2:C70,"卖出")-SUMIFS($H$2:H70,$A$2:A70,$A70,$C$2:C70,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J70" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A70)=COUNTIF($A$2:A70,$A70),SUMIFS($G$2:$G$73,$A$2:$A$73,$A70),"")</f>
-        <v/>
-      </c>
-      <c r="K70" s="0" t="n"/>
-      <c r="L70">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A70)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A70,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A70,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A70),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A70,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A70,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A70)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A71" s="6">
-        <f>"002028"</f>
-        <v/>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>思源电气</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>买入</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="n">
-        <v>20260209</v>
-      </c>
-      <c r="E71" s="7" t="n">
-        <v>0.4454861111111111</v>
-      </c>
-      <c r="F71" s="2" t="n">
-        <v>198.73</v>
-      </c>
-      <c r="G71" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="H71" s="2" t="n">
-        <v>19873</v>
-      </c>
-      <c r="I71" s="2">
-        <f>IF(AND($C71="卖出",SUMIFS($G$2:G71,$A$2:A71,$A71)=0),SUMIFS($H$2:H71,$A$2:A71,$A71,$C$2:C71,"卖出")-SUMIFS($H$2:H71,$A$2:A71,$A71,$C$2:C71,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J71" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A71)=COUNTIF($A$2:A71,$A71),SUMIFS($G$2:$G$73,$A$2:$A$73,$A71),"")</f>
-        <v/>
-      </c>
-      <c r="K71" s="0" t="n"/>
-      <c r="L71">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A71)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A71,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A71,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A71),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A71,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A71,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A71)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A72" s="6" t="n">
-        <v>600584</v>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>长电科技</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>买入</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="n">
-        <v>20260209</v>
-      </c>
-      <c r="E72" s="7" t="n">
-        <v>0.4388657407407408</v>
-      </c>
-      <c r="F72" s="2" t="n">
-        <v>46.09</v>
-      </c>
-      <c r="G72" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="H72" s="2" t="n">
-        <v>9218</v>
-      </c>
-      <c r="I72" s="2">
-        <f>IF(AND($C72="卖出",SUMIFS($G$2:G72,$A$2:A72,$A72)=0),SUMIFS($H$2:H72,$A$2:A72,$A72,$C$2:C72,"卖出")-SUMIFS($H$2:H72,$A$2:A72,$A72,$C$2:C72,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J72" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A72)=COUNTIF($A$2:A72,$A72),SUMIFS($G$2:$G$73,$A$2:$A$73,$A72),"")</f>
-        <v/>
-      </c>
-      <c r="K72" s="0" t="n"/>
-      <c r="L72">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A72)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A72,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A72,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A72),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A72,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A72,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A72)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73" ht="20.4" customFormat="1" customHeight="1" s="2">
-      <c r="A73" s="6">
-        <f>"002028"</f>
-        <v/>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>思源电气</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>卖出</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="n">
-        <v>20260209</v>
-      </c>
-      <c r="E73" s="7" t="n">
-        <v>0.4105902777777778</v>
-      </c>
-      <c r="F73" s="2" t="n">
-        <v>192.5</v>
-      </c>
-      <c r="G73" s="2" t="n">
-        <v>-200</v>
-      </c>
-      <c r="H73" s="2" t="n">
-        <v>38500</v>
-      </c>
-      <c r="I73" s="2">
-        <f>IF(AND($C73="卖出",SUMIFS($G$2:G73,$A$2:A73,$A73)=0),SUMIFS($H$2:H73,$A$2:A73,$A73,$C$2:C73,"卖出")-SUMIFS($H$2:H73,$A$2:A73,$A73,$C$2:C73,"买入"),"")</f>
-        <v/>
-      </c>
-      <c r="J73" s="2">
-        <f>IF(COUNTIF($A$2:$A$73,$A73)=COUNTIF($A$2:A73,$A73),SUMIFS($G$2:$G$73,$A$2:$A$73,$A73),"")</f>
-        <v/>
-      </c>
-      <c r="K73" s="0" t="n"/>
-      <c r="L73">
-        <f>IF(SUMIFS($G$2:$G$73,$A$2:$A$73,$A73)=0,"",IF(IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A73,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A73,$C$2:$C$73,"买入"),"")="","",(LOOKUP(2,1/($A$2:$A$73=$A73),$F$2:$F$73)-IFERROR(SUMIFS($H$2:$H$73,$A$2:$A$73,$A73,$C$2:$C$73,"买入")/SUMIFS($G$2:$G$73,$A$2:$A$73,$A73,$C$2:$C$73,"买入"),""))*SUMIFS($G$2:$G$73,$A$2:$A$73,$A73)))</f>
+        <f>SUMIFS($G$2:G61,$A$2:A61,$A61)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="J62">
+        <f>SUMIFS($G$2:G62,$A$2:A62,$A62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="20.4" customHeight="1" s="4">
+      <c r="E63" s="9" t="n"/>
+      <c r="J63">
+        <f>SUMIFS($G$2:G63,$A$2:A63,$A63)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B73"/>
+  <autoFilter ref="A1:J60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-03-01 16:48:28
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="22440"/>
+    <workbookView windowWidth="29100" windowHeight="14560"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="40">
   <si>
     <t>证券代码</t>
   </si>
@@ -143,6 +143,16 @@
   </si>
   <si>
     <t>放量跌破30日线全仓止损</t>
+  </si>
+  <si>
+    <t xml:space="preserve">基本面没有改变 思源电气回踩13日线  只是一个短期获利盘的了结  做的不足的地方在于太想抄底了 应该等股价稳稳踩住13日线的时候再进行加仓
+</t>
+  </si>
+  <si>
+    <t>止盈依旧设置在250 止盈半仓</t>
+  </si>
+  <si>
+    <t>放量跌破13日均线且没有收复迹象时全仓离场</t>
   </si>
 </sst>
 </file>
@@ -786,7 +796,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -806,6 +816,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1417,7 +1428,7 @@
       <c r="D2" s="2">
         <v>20250902</v>
       </c>
-      <c r="E2" s="8">
+      <c r="E2" s="9">
         <v>0.395983796296296</v>
       </c>
       <c r="F2" s="2">
@@ -1451,7 +1462,7 @@
       <c r="D3" s="2">
         <v>20250903</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="9">
         <v>0.400289351851852</v>
       </c>
       <c r="F3" s="2">
@@ -1485,7 +1496,7 @@
       <c r="D4" s="2">
         <v>20250912</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="9">
         <v>0.407638888888889</v>
       </c>
       <c r="F4" s="2">
@@ -1519,7 +1530,7 @@
       <c r="D5" s="2">
         <v>20250915</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="9">
         <v>0.591782407407407</v>
       </c>
       <c r="F5" s="2">
@@ -1553,7 +1564,7 @@
       <c r="D6" s="2">
         <v>20250915</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="9">
         <v>0.399363425925926</v>
       </c>
       <c r="F6" s="2">
@@ -1587,7 +1598,7 @@
       <c r="D7" s="2">
         <v>20250925</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="9">
         <v>0.609340277777778</v>
       </c>
       <c r="F7" s="2">
@@ -1621,7 +1632,7 @@
       <c r="D8" s="2">
         <v>20251009</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="9">
         <v>0.446851851851852</v>
       </c>
       <c r="F8" s="2">
@@ -1655,7 +1666,7 @@
       <c r="D9" s="2">
         <v>20251010</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="9">
         <v>0.417337962962963</v>
       </c>
       <c r="F9" s="2">
@@ -1689,7 +1700,7 @@
       <c r="D10" s="2">
         <v>20251010</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="9">
         <v>0.396574074074074</v>
       </c>
       <c r="F10" s="2">
@@ -1723,7 +1734,7 @@
       <c r="D11" s="2">
         <v>20251015</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="9">
         <v>0.453912037037037</v>
       </c>
       <c r="F11" s="2">
@@ -1757,7 +1768,7 @@
       <c r="D12" s="2">
         <v>20251015</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="9">
         <v>0.453784722222222</v>
       </c>
       <c r="F12" s="2">
@@ -1791,7 +1802,7 @@
       <c r="D13" s="2">
         <v>20251015</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="9">
         <v>0.422696759259259</v>
       </c>
       <c r="F13" s="2">
@@ -1826,7 +1837,7 @@
       <c r="D14" s="2">
         <v>20251016</v>
       </c>
-      <c r="E14" s="8">
+      <c r="E14" s="9">
         <v>0.560474537037037</v>
       </c>
       <c r="F14" s="2">
@@ -1860,7 +1871,7 @@
       <c r="D15" s="2">
         <v>20251016</v>
       </c>
-      <c r="E15" s="8">
+      <c r="E15" s="9">
         <v>0.458530092592593</v>
       </c>
       <c r="F15" s="2">
@@ -1895,7 +1906,7 @@
       <c r="D16" s="2">
         <v>20251017</v>
       </c>
-      <c r="E16" s="8">
+      <c r="E16" s="9">
         <v>0.625</v>
       </c>
       <c r="F16" s="2">
@@ -1930,7 +1941,7 @@
       <c r="D17" s="2">
         <v>20251021</v>
       </c>
-      <c r="E17" s="8">
+      <c r="E17" s="9">
         <v>0.621550925925926</v>
       </c>
       <c r="F17" s="2">
@@ -1964,7 +1975,7 @@
       <c r="D18" s="2">
         <v>20251021</v>
       </c>
-      <c r="E18" s="8">
+      <c r="E18" s="9">
         <v>0.46806712962963</v>
       </c>
       <c r="F18" s="2">
@@ -1999,7 +2010,7 @@
       <c r="D19" s="2">
         <v>20251021</v>
       </c>
-      <c r="E19" s="8">
+      <c r="E19" s="9">
         <v>0.418518518518519</v>
       </c>
       <c r="F19" s="2">
@@ -2033,7 +2044,7 @@
       <c r="D20" s="2">
         <v>20251023</v>
       </c>
-      <c r="E20" s="8">
+      <c r="E20" s="9">
         <v>0.617777777777778</v>
       </c>
       <c r="F20" s="2">
@@ -2068,7 +2079,7 @@
       <c r="D21" s="2">
         <v>20251023</v>
       </c>
-      <c r="E21" s="8">
+      <c r="E21" s="9">
         <v>0.616111111111111</v>
       </c>
       <c r="F21" s="2">
@@ -2103,7 +2114,7 @@
       <c r="D22" s="2">
         <v>20251024</v>
       </c>
-      <c r="E22" s="8">
+      <c r="E22" s="9">
         <v>0.601006944444444</v>
       </c>
       <c r="F22" s="2">
@@ -2137,7 +2148,7 @@
       <c r="D23" s="2">
         <v>20251024</v>
       </c>
-      <c r="E23" s="8">
+      <c r="E23" s="9">
         <v>0.589212962962963</v>
       </c>
       <c r="F23" s="2">
@@ -2172,7 +2183,7 @@
       <c r="D24" s="2">
         <v>20251024</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E24" s="9">
         <v>0.418425925925926</v>
       </c>
       <c r="F24" s="2">
@@ -2206,7 +2217,7 @@
       <c r="D25" s="2">
         <v>20251027</v>
       </c>
-      <c r="E25" s="8">
+      <c r="E25" s="9">
         <v>0.399074074074074</v>
       </c>
       <c r="F25" s="2">
@@ -2240,7 +2251,7 @@
       <c r="D26" s="2">
         <v>20251028</v>
       </c>
-      <c r="E26" s="8">
+      <c r="E26" s="9">
         <v>0.625</v>
       </c>
       <c r="F26" s="2">
@@ -2274,7 +2285,7 @@
       <c r="D27" s="2">
         <v>20251029</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E27" s="9">
         <v>0.441550925925926</v>
       </c>
       <c r="F27" s="2">
@@ -2308,7 +2319,7 @@
       <c r="D28" s="2">
         <v>20251030</v>
       </c>
-      <c r="E28" s="8">
+      <c r="E28" s="9">
         <v>0.565590277777778</v>
       </c>
       <c r="F28" s="2">
@@ -2342,7 +2353,7 @@
       <c r="D29" s="2">
         <v>20251030</v>
       </c>
-      <c r="E29" s="8">
+      <c r="E29" s="9">
         <v>0.544988425925926</v>
       </c>
       <c r="F29" s="2">
@@ -2376,7 +2387,7 @@
       <c r="D30" s="2">
         <v>20251104</v>
       </c>
-      <c r="E30" s="8">
+      <c r="E30" s="9">
         <v>0.625</v>
       </c>
       <c r="F30" s="2">
@@ -2410,7 +2421,7 @@
       <c r="D31" s="2">
         <v>20251104</v>
       </c>
-      <c r="E31" s="8">
+      <c r="E31" s="9">
         <v>0.625</v>
       </c>
       <c r="F31" s="2">
@@ -2444,7 +2455,7 @@
       <c r="D32" s="2">
         <v>20251104</v>
       </c>
-      <c r="E32" s="8">
+      <c r="E32" s="9">
         <v>0.625</v>
       </c>
       <c r="F32" s="2">
@@ -2478,7 +2489,7 @@
       <c r="D33" s="2">
         <v>20251105</v>
       </c>
-      <c r="E33" s="8">
+      <c r="E33" s="9">
         <v>0.413472222222222</v>
       </c>
       <c r="F33" s="2">
@@ -2513,7 +2524,7 @@
       <c r="D34" s="2">
         <v>20260119</v>
       </c>
-      <c r="E34" s="8">
+      <c r="E34" s="9">
         <v>0.422534722222222</v>
       </c>
       <c r="F34" s="2">
@@ -2547,7 +2558,7 @@
       <c r="D35" s="2">
         <v>20260119</v>
       </c>
-      <c r="E35" s="8">
+      <c r="E35" s="9">
         <v>0.400891203703704</v>
       </c>
       <c r="F35" s="2">
@@ -2582,7 +2593,7 @@
       <c r="D36" s="2">
         <v>20260119</v>
       </c>
-      <c r="E36" s="8">
+      <c r="E36" s="9">
         <v>0.398483796296296</v>
       </c>
       <c r="F36" s="2">
@@ -2616,7 +2627,7 @@
       <c r="D37" s="2">
         <v>20260119</v>
       </c>
-      <c r="E37" s="8">
+      <c r="E37" s="9">
         <v>0.396030092592593</v>
       </c>
       <c r="F37" s="2">
@@ -2651,7 +2662,7 @@
       <c r="D38" s="2">
         <v>20260121</v>
       </c>
-      <c r="E38" s="8">
+      <c r="E38" s="9">
         <v>0.397384259259259</v>
       </c>
       <c r="F38" s="2">
@@ -2686,7 +2697,7 @@
       <c r="D39" s="2">
         <v>20260122</v>
       </c>
-      <c r="E39" s="8">
+      <c r="E39" s="9">
         <v>0.444861111111111</v>
       </c>
       <c r="F39" s="2">
@@ -2720,7 +2731,7 @@
       <c r="D40" s="2">
         <v>20260122</v>
       </c>
-      <c r="E40" s="8">
+      <c r="E40" s="9">
         <v>0.407951388888889</v>
       </c>
       <c r="F40" s="2">
@@ -2754,7 +2765,7 @@
       <c r="D41" s="2">
         <v>20260126</v>
       </c>
-      <c r="E41" s="8">
+      <c r="E41" s="9">
         <v>0.622175925925926</v>
       </c>
       <c r="F41" s="2">
@@ -2788,7 +2799,7 @@
       <c r="D42" s="2">
         <v>20260127</v>
       </c>
-      <c r="E42" s="8">
+      <c r="E42" s="9">
         <v>0.589479166666667</v>
       </c>
       <c r="F42" s="2">
@@ -2823,7 +2834,7 @@
       <c r="D43" s="2">
         <v>20260127</v>
       </c>
-      <c r="E43" s="8">
+      <c r="E43" s="9">
         <v>0.413969907407407</v>
       </c>
       <c r="F43" s="2">
@@ -2858,7 +2869,7 @@
       <c r="D44" s="2">
         <v>20260129</v>
       </c>
-      <c r="E44" s="8">
+      <c r="E44" s="9">
         <v>0.5778125</v>
       </c>
       <c r="F44" s="2">
@@ -2893,7 +2904,7 @@
       <c r="D45" s="2">
         <v>20260129</v>
       </c>
-      <c r="E45" s="8">
+      <c r="E45" s="9">
         <v>0.571990740740741</v>
       </c>
       <c r="F45" s="2">
@@ -2927,7 +2938,7 @@
       <c r="D46" s="2">
         <v>20260129</v>
       </c>
-      <c r="E46" s="8">
+      <c r="E46" s="9">
         <v>0.57099537037037</v>
       </c>
       <c r="F46" s="2">
@@ -2962,7 +2973,7 @@
       <c r="D47" s="2">
         <v>20260129</v>
       </c>
-      <c r="E47" s="8">
+      <c r="E47" s="9">
         <v>0.545462962962963</v>
       </c>
       <c r="F47" s="2">
@@ -2997,7 +3008,7 @@
       <c r="D48" s="2">
         <v>20260129</v>
       </c>
-      <c r="E48" s="8">
+      <c r="E48" s="9">
         <v>0.542395833333333</v>
       </c>
       <c r="F48" s="2">
@@ -3031,7 +3042,7 @@
       <c r="D49" s="2">
         <v>20260130</v>
       </c>
-      <c r="E49" s="8">
+      <c r="E49" s="9">
         <v>0.440439814814815</v>
       </c>
       <c r="F49" s="2">
@@ -3066,7 +3077,7 @@
       <c r="D50" s="2">
         <v>20260130</v>
       </c>
-      <c r="E50" s="8">
+      <c r="E50" s="9">
         <v>0.431030092592593</v>
       </c>
       <c r="F50" s="2">
@@ -3101,7 +3112,7 @@
       <c r="D51" s="2">
         <v>20260202</v>
       </c>
-      <c r="E51" s="8">
+      <c r="E51" s="9">
         <v>0.618993055555556</v>
       </c>
       <c r="F51" s="2">
@@ -3135,7 +3146,7 @@
       <c r="D52" s="2">
         <v>20260202</v>
       </c>
-      <c r="E52" s="8">
+      <c r="E52" s="9">
         <v>0.565694444444444</v>
       </c>
       <c r="F52" s="2">
@@ -3169,7 +3180,7 @@
       <c r="D53" s="2">
         <v>20260202</v>
       </c>
-      <c r="E53" s="8">
+      <c r="E53" s="9">
         <v>0.55994212962963</v>
       </c>
       <c r="F53" s="2">
@@ -3204,7 +3215,7 @@
       <c r="D54" s="2">
         <v>20260202</v>
       </c>
-      <c r="E54" s="8">
+      <c r="E54" s="9">
         <v>0.446747685185185</v>
       </c>
       <c r="F54" s="2">
@@ -3239,7 +3250,7 @@
       <c r="D55" s="2">
         <v>20260202</v>
       </c>
-      <c r="E55" s="8">
+      <c r="E55" s="9">
         <v>0.440671296296296</v>
       </c>
       <c r="F55" s="2">
@@ -3274,7 +3285,7 @@
       <c r="D56" s="2">
         <v>20260203</v>
       </c>
-      <c r="E56" s="8">
+      <c r="E56" s="9">
         <v>0.409178240740741</v>
       </c>
       <c r="F56" s="2">
@@ -3297,7 +3308,7 @@
     </row>
     <row r="57" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
       <c r="A57" s="6" t="str">
-        <f>"002028"</f>
+        <f t="shared" ref="A57:A62" si="0">"002028"</f>
         <v>002028</v>
       </c>
       <c r="B57" s="2" t="s">
@@ -3309,7 +3320,7 @@
       <c r="D57" s="2">
         <v>20260205</v>
       </c>
-      <c r="E57" s="8">
+      <c r="E57" s="9">
         <v>0.404363425925926</v>
       </c>
       <c r="F57" s="2">
@@ -3332,7 +3343,7 @@
     </row>
     <row r="58" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
       <c r="A58" s="6" t="str">
-        <f>"002028"</f>
+        <f t="shared" si="0"/>
         <v>002028</v>
       </c>
       <c r="B58" s="2" t="s">
@@ -3344,7 +3355,7 @@
       <c r="D58" s="2">
         <v>20260209</v>
       </c>
-      <c r="E58" s="8">
+      <c r="E58" s="9">
         <v>0.445486111111111</v>
       </c>
       <c r="F58" s="2">
@@ -3378,7 +3389,7 @@
       <c r="D59" s="2">
         <v>20260209</v>
       </c>
-      <c r="E59" s="8">
+      <c r="E59" s="9">
         <v>0.438865740740741</v>
       </c>
       <c r="F59" s="2">
@@ -3401,7 +3412,7 @@
     </row>
     <row r="60" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
       <c r="A60" s="6" t="str">
-        <f>"002028"</f>
+        <f t="shared" si="0"/>
         <v>002028</v>
       </c>
       <c r="B60" s="2" t="s">
@@ -3413,7 +3424,7 @@
       <c r="D60" s="2">
         <v>20260209</v>
       </c>
-      <c r="E60" s="8">
+      <c r="E60" s="9">
         <v>0.410590277777778</v>
       </c>
       <c r="F60" s="2">
@@ -3463,7 +3474,7 @@
         <f>SUMIFS($G$2:G61,$A$2:A61,$A61)</f>
         <v>1100</v>
       </c>
-      <c r="K61" s="10" t="s">
+      <c r="K61" s="11" t="s">
         <v>34</v>
       </c>
       <c r="L61" s="4" t="s">
@@ -3473,11 +3484,48 @@
         <v>36</v>
       </c>
     </row>
-    <row r="62" spans="10:10">
-      <c r="J62"/>
+    <row r="62" ht="84" spans="1:13">
+      <c r="A62" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>002028</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D62" s="8">
+        <v>20260227</v>
+      </c>
+      <c r="E62" s="9">
+        <v>0.403645833333333</v>
+      </c>
+      <c r="F62" s="2">
+        <v>218.5</v>
+      </c>
+      <c r="G62" s="2">
+        <v>100</v>
+      </c>
+      <c r="H62" s="2">
+        <v>21850</v>
+      </c>
+      <c r="J62" s="2">
+        <f>SUMIFS($G$2:G62,$A$2:A62,$A62)</f>
+        <v>600</v>
+      </c>
+      <c r="K62" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="L62" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="M62" s="4" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="63" ht="20.4" customHeight="1" spans="5:10">
-      <c r="E63" s="9"/>
+      <c r="E63" s="10"/>
       <c r="J63"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-03-09 17:14:31
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="42">
   <si>
     <t>证券代码</t>
   </si>
@@ -153,6 +153,14 @@
   </si>
   <si>
     <t>放量跌破13日均线且没有收复迹象时全仓离场</t>
+  </si>
+  <si>
+    <t xml:space="preserve">卖出 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+止损了600股 主要原因是长电科技有效跌破30日均线且回收的速度不快，温和回收，同时接近尾盘时又下跌了一点 ，对于这种慢慢的温和的回收 我有两个想法 
+一是主力在边打边撤 悄悄出货 二是主力在底部建仓 怕一下子拉飞股价  同时股价是触及到了 短期的支撑位之后回升 留下了长下影 个人主观上我想博一个反弹 客观上破位就走是我定死的纪律 所以中和二者 半苍止损是比较好的选择了</t>
   </si>
 </sst>
 </file>
@@ -165,7 +173,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -182,13 +190,6 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="14"/>
       <color theme="1"/>
       <name val="宋体"/>
@@ -666,137 +667,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -817,11 +818,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1368,7 +1367,7 @@
     <col min="11" max="11" width="43.9038461538462" style="4" customWidth="1"/>
     <col min="12" max="12" width="27.6923076923077" style="4" customWidth="1"/>
     <col min="13" max="13" width="27.0769230769231" style="4" customWidth="1"/>
-    <col min="14" max="14" width="14.6153846153846" style="4" customWidth="1"/>
+    <col min="14" max="14" width="40.5384615384615" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="23.2" customHeight="1" spans="1:14">
@@ -1428,7 +1427,7 @@
       <c r="D2" s="2">
         <v>20250902</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="8">
         <v>0.395983796296296</v>
       </c>
       <c r="F2" s="2">
@@ -1462,7 +1461,7 @@
       <c r="D3" s="2">
         <v>20250903</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="8">
         <v>0.400289351851852</v>
       </c>
       <c r="F3" s="2">
@@ -1496,7 +1495,7 @@
       <c r="D4" s="2">
         <v>20250912</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="8">
         <v>0.407638888888889</v>
       </c>
       <c r="F4" s="2">
@@ -1530,7 +1529,7 @@
       <c r="D5" s="2">
         <v>20250915</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="8">
         <v>0.591782407407407</v>
       </c>
       <c r="F5" s="2">
@@ -1564,7 +1563,7 @@
       <c r="D6" s="2">
         <v>20250915</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="8">
         <v>0.399363425925926</v>
       </c>
       <c r="F6" s="2">
@@ -1598,7 +1597,7 @@
       <c r="D7" s="2">
         <v>20250925</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="8">
         <v>0.609340277777778</v>
       </c>
       <c r="F7" s="2">
@@ -1632,7 +1631,7 @@
       <c r="D8" s="2">
         <v>20251009</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="8">
         <v>0.446851851851852</v>
       </c>
       <c r="F8" s="2">
@@ -1666,7 +1665,7 @@
       <c r="D9" s="2">
         <v>20251010</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="8">
         <v>0.417337962962963</v>
       </c>
       <c r="F9" s="2">
@@ -1700,7 +1699,7 @@
       <c r="D10" s="2">
         <v>20251010</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="8">
         <v>0.396574074074074</v>
       </c>
       <c r="F10" s="2">
@@ -1734,7 +1733,7 @@
       <c r="D11" s="2">
         <v>20251015</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="8">
         <v>0.453912037037037</v>
       </c>
       <c r="F11" s="2">
@@ -1768,7 +1767,7 @@
       <c r="D12" s="2">
         <v>20251015</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="8">
         <v>0.453784722222222</v>
       </c>
       <c r="F12" s="2">
@@ -1802,7 +1801,7 @@
       <c r="D13" s="2">
         <v>20251015</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="8">
         <v>0.422696759259259</v>
       </c>
       <c r="F13" s="2">
@@ -1837,7 +1836,7 @@
       <c r="D14" s="2">
         <v>20251016</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="8">
         <v>0.560474537037037</v>
       </c>
       <c r="F14" s="2">
@@ -1871,7 +1870,7 @@
       <c r="D15" s="2">
         <v>20251016</v>
       </c>
-      <c r="E15" s="9">
+      <c r="E15" s="8">
         <v>0.458530092592593</v>
       </c>
       <c r="F15" s="2">
@@ -1906,7 +1905,7 @@
       <c r="D16" s="2">
         <v>20251017</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16" s="8">
         <v>0.625</v>
       </c>
       <c r="F16" s="2">
@@ -1941,7 +1940,7 @@
       <c r="D17" s="2">
         <v>20251021</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="8">
         <v>0.621550925925926</v>
       </c>
       <c r="F17" s="2">
@@ -1975,7 +1974,7 @@
       <c r="D18" s="2">
         <v>20251021</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="8">
         <v>0.46806712962963</v>
       </c>
       <c r="F18" s="2">
@@ -2010,7 +2009,7 @@
       <c r="D19" s="2">
         <v>20251021</v>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="8">
         <v>0.418518518518519</v>
       </c>
       <c r="F19" s="2">
@@ -2044,7 +2043,7 @@
       <c r="D20" s="2">
         <v>20251023</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="8">
         <v>0.617777777777778</v>
       </c>
       <c r="F20" s="2">
@@ -2079,7 +2078,7 @@
       <c r="D21" s="2">
         <v>20251023</v>
       </c>
-      <c r="E21" s="9">
+      <c r="E21" s="8">
         <v>0.616111111111111</v>
       </c>
       <c r="F21" s="2">
@@ -2114,7 +2113,7 @@
       <c r="D22" s="2">
         <v>20251024</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="8">
         <v>0.601006944444444</v>
       </c>
       <c r="F22" s="2">
@@ -2148,7 +2147,7 @@
       <c r="D23" s="2">
         <v>20251024</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="8">
         <v>0.589212962962963</v>
       </c>
       <c r="F23" s="2">
@@ -2183,7 +2182,7 @@
       <c r="D24" s="2">
         <v>20251024</v>
       </c>
-      <c r="E24" s="9">
+      <c r="E24" s="8">
         <v>0.418425925925926</v>
       </c>
       <c r="F24" s="2">
@@ -2217,7 +2216,7 @@
       <c r="D25" s="2">
         <v>20251027</v>
       </c>
-      <c r="E25" s="9">
+      <c r="E25" s="8">
         <v>0.399074074074074</v>
       </c>
       <c r="F25" s="2">
@@ -2251,7 +2250,7 @@
       <c r="D26" s="2">
         <v>20251028</v>
       </c>
-      <c r="E26" s="9">
+      <c r="E26" s="8">
         <v>0.625</v>
       </c>
       <c r="F26" s="2">
@@ -2285,7 +2284,7 @@
       <c r="D27" s="2">
         <v>20251029</v>
       </c>
-      <c r="E27" s="9">
+      <c r="E27" s="8">
         <v>0.441550925925926</v>
       </c>
       <c r="F27" s="2">
@@ -2319,7 +2318,7 @@
       <c r="D28" s="2">
         <v>20251030</v>
       </c>
-      <c r="E28" s="9">
+      <c r="E28" s="8">
         <v>0.565590277777778</v>
       </c>
       <c r="F28" s="2">
@@ -2353,7 +2352,7 @@
       <c r="D29" s="2">
         <v>20251030</v>
       </c>
-      <c r="E29" s="9">
+      <c r="E29" s="8">
         <v>0.544988425925926</v>
       </c>
       <c r="F29" s="2">
@@ -2387,7 +2386,7 @@
       <c r="D30" s="2">
         <v>20251104</v>
       </c>
-      <c r="E30" s="9">
+      <c r="E30" s="8">
         <v>0.625</v>
       </c>
       <c r="F30" s="2">
@@ -2421,7 +2420,7 @@
       <c r="D31" s="2">
         <v>20251104</v>
       </c>
-      <c r="E31" s="9">
+      <c r="E31" s="8">
         <v>0.625</v>
       </c>
       <c r="F31" s="2">
@@ -2455,7 +2454,7 @@
       <c r="D32" s="2">
         <v>20251104</v>
       </c>
-      <c r="E32" s="9">
+      <c r="E32" s="8">
         <v>0.625</v>
       </c>
       <c r="F32" s="2">
@@ -2489,7 +2488,7 @@
       <c r="D33" s="2">
         <v>20251105</v>
       </c>
-      <c r="E33" s="9">
+      <c r="E33" s="8">
         <v>0.413472222222222</v>
       </c>
       <c r="F33" s="2">
@@ -2524,7 +2523,7 @@
       <c r="D34" s="2">
         <v>20260119</v>
       </c>
-      <c r="E34" s="9">
+      <c r="E34" s="8">
         <v>0.422534722222222</v>
       </c>
       <c r="F34" s="2">
@@ -2558,7 +2557,7 @@
       <c r="D35" s="2">
         <v>20260119</v>
       </c>
-      <c r="E35" s="9">
+      <c r="E35" s="8">
         <v>0.400891203703704</v>
       </c>
       <c r="F35" s="2">
@@ -2593,7 +2592,7 @@
       <c r="D36" s="2">
         <v>20260119</v>
       </c>
-      <c r="E36" s="9">
+      <c r="E36" s="8">
         <v>0.398483796296296</v>
       </c>
       <c r="F36" s="2">
@@ -2627,7 +2626,7 @@
       <c r="D37" s="2">
         <v>20260119</v>
       </c>
-      <c r="E37" s="9">
+      <c r="E37" s="8">
         <v>0.396030092592593</v>
       </c>
       <c r="F37" s="2">
@@ -2662,7 +2661,7 @@
       <c r="D38" s="2">
         <v>20260121</v>
       </c>
-      <c r="E38" s="9">
+      <c r="E38" s="8">
         <v>0.397384259259259</v>
       </c>
       <c r="F38" s="2">
@@ -2697,7 +2696,7 @@
       <c r="D39" s="2">
         <v>20260122</v>
       </c>
-      <c r="E39" s="9">
+      <c r="E39" s="8">
         <v>0.444861111111111</v>
       </c>
       <c r="F39" s="2">
@@ -2731,7 +2730,7 @@
       <c r="D40" s="2">
         <v>20260122</v>
       </c>
-      <c r="E40" s="9">
+      <c r="E40" s="8">
         <v>0.407951388888889</v>
       </c>
       <c r="F40" s="2">
@@ -2765,7 +2764,7 @@
       <c r="D41" s="2">
         <v>20260126</v>
       </c>
-      <c r="E41" s="9">
+      <c r="E41" s="8">
         <v>0.622175925925926</v>
       </c>
       <c r="F41" s="2">
@@ -2799,7 +2798,7 @@
       <c r="D42" s="2">
         <v>20260127</v>
       </c>
-      <c r="E42" s="9">
+      <c r="E42" s="8">
         <v>0.589479166666667</v>
       </c>
       <c r="F42" s="2">
@@ -2834,7 +2833,7 @@
       <c r="D43" s="2">
         <v>20260127</v>
       </c>
-      <c r="E43" s="9">
+      <c r="E43" s="8">
         <v>0.413969907407407</v>
       </c>
       <c r="F43" s="2">
@@ -2869,7 +2868,7 @@
       <c r="D44" s="2">
         <v>20260129</v>
       </c>
-      <c r="E44" s="9">
+      <c r="E44" s="8">
         <v>0.5778125</v>
       </c>
       <c r="F44" s="2">
@@ -2904,7 +2903,7 @@
       <c r="D45" s="2">
         <v>20260129</v>
       </c>
-      <c r="E45" s="9">
+      <c r="E45" s="8">
         <v>0.571990740740741</v>
       </c>
       <c r="F45" s="2">
@@ -2938,7 +2937,7 @@
       <c r="D46" s="2">
         <v>20260129</v>
       </c>
-      <c r="E46" s="9">
+      <c r="E46" s="8">
         <v>0.57099537037037</v>
       </c>
       <c r="F46" s="2">
@@ -2973,7 +2972,7 @@
       <c r="D47" s="2">
         <v>20260129</v>
       </c>
-      <c r="E47" s="9">
+      <c r="E47" s="8">
         <v>0.545462962962963</v>
       </c>
       <c r="F47" s="2">
@@ -3008,7 +3007,7 @@
       <c r="D48" s="2">
         <v>20260129</v>
       </c>
-      <c r="E48" s="9">
+      <c r="E48" s="8">
         <v>0.542395833333333</v>
       </c>
       <c r="F48" s="2">
@@ -3042,7 +3041,7 @@
       <c r="D49" s="2">
         <v>20260130</v>
       </c>
-      <c r="E49" s="9">
+      <c r="E49" s="8">
         <v>0.440439814814815</v>
       </c>
       <c r="F49" s="2">
@@ -3077,7 +3076,7 @@
       <c r="D50" s="2">
         <v>20260130</v>
       </c>
-      <c r="E50" s="9">
+      <c r="E50" s="8">
         <v>0.431030092592593</v>
       </c>
       <c r="F50" s="2">
@@ -3112,7 +3111,7 @@
       <c r="D51" s="2">
         <v>20260202</v>
       </c>
-      <c r="E51" s="9">
+      <c r="E51" s="8">
         <v>0.618993055555556</v>
       </c>
       <c r="F51" s="2">
@@ -3146,7 +3145,7 @@
       <c r="D52" s="2">
         <v>20260202</v>
       </c>
-      <c r="E52" s="9">
+      <c r="E52" s="8">
         <v>0.565694444444444</v>
       </c>
       <c r="F52" s="2">
@@ -3180,7 +3179,7 @@
       <c r="D53" s="2">
         <v>20260202</v>
       </c>
-      <c r="E53" s="9">
+      <c r="E53" s="8">
         <v>0.55994212962963</v>
       </c>
       <c r="F53" s="2">
@@ -3215,7 +3214,7 @@
       <c r="D54" s="2">
         <v>20260202</v>
       </c>
-      <c r="E54" s="9">
+      <c r="E54" s="8">
         <v>0.446747685185185</v>
       </c>
       <c r="F54" s="2">
@@ -3250,7 +3249,7 @@
       <c r="D55" s="2">
         <v>20260202</v>
       </c>
-      <c r="E55" s="9">
+      <c r="E55" s="8">
         <v>0.440671296296296</v>
       </c>
       <c r="F55" s="2">
@@ -3285,7 +3284,7 @@
       <c r="D56" s="2">
         <v>20260203</v>
       </c>
-      <c r="E56" s="9">
+      <c r="E56" s="8">
         <v>0.409178240740741</v>
       </c>
       <c r="F56" s="2">
@@ -3320,7 +3319,7 @@
       <c r="D57" s="2">
         <v>20260205</v>
       </c>
-      <c r="E57" s="9">
+      <c r="E57" s="8">
         <v>0.404363425925926</v>
       </c>
       <c r="F57" s="2">
@@ -3355,7 +3354,7 @@
       <c r="D58" s="2">
         <v>20260209</v>
       </c>
-      <c r="E58" s="9">
+      <c r="E58" s="8">
         <v>0.445486111111111</v>
       </c>
       <c r="F58" s="2">
@@ -3389,7 +3388,7 @@
       <c r="D59" s="2">
         <v>20260209</v>
       </c>
-      <c r="E59" s="9">
+      <c r="E59" s="8">
         <v>0.438865740740741</v>
       </c>
       <c r="F59" s="2">
@@ -3424,7 +3423,7 @@
       <c r="D60" s="2">
         <v>20260209</v>
       </c>
-      <c r="E60" s="9">
+      <c r="E60" s="8">
         <v>0.410590277777778</v>
       </c>
       <c r="F60" s="2">
@@ -3474,7 +3473,7 @@
         <f>SUMIFS($G$2:G61,$A$2:A61,$A61)</f>
         <v>1100</v>
       </c>
-      <c r="K61" s="11" t="s">
+      <c r="K61" s="9" t="s">
         <v>34</v>
       </c>
       <c r="L61" s="4" t="s">
@@ -3493,12 +3492,12 @@
         <v>31</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D62" s="8">
+        <v>15</v>
+      </c>
+      <c r="D62" s="7">
         <v>20260227</v>
       </c>
-      <c r="E62" s="9">
+      <c r="E62" s="8">
         <v>0.403645833333333</v>
       </c>
       <c r="F62" s="2">
@@ -3514,7 +3513,7 @@
         <f>SUMIFS($G$2:G62,$A$2:A62,$A62)</f>
         <v>600</v>
       </c>
-      <c r="K62" s="11" t="s">
+      <c r="K62" s="9" t="s">
         <v>37</v>
       </c>
       <c r="L62" s="4" t="s">
@@ -3524,9 +3523,38 @@
         <v>39</v>
       </c>
     </row>
-    <row r="63" ht="20.4" customHeight="1" spans="5:10">
-      <c r="E63" s="10"/>
-      <c r="J63"/>
+    <row r="63" ht="77" customHeight="1" spans="1:14">
+      <c r="A63" s="3">
+        <v>600584</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D63" s="2">
+        <v>20260309</v>
+      </c>
+      <c r="E63" s="2">
+        <v>0.620138888888889</v>
+      </c>
+      <c r="F63" s="2">
+        <v>45.03</v>
+      </c>
+      <c r="G63" s="2">
+        <v>-600</v>
+      </c>
+      <c r="H63" s="2">
+        <v>27018</v>
+      </c>
+      <c r="J63" s="2">
+        <f>SUMIFS($G$2:G63,$A$2:A63,$A63)</f>
+        <v>500</v>
+      </c>
+      <c r="N63" s="9" t="s">
+        <v>41</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J63">

</xml_diff>

<commit_message>
vault backup: 2026-03-12 13:09:56
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="14560"/>
+    <workbookView windowWidth="29100" windowHeight="13020"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="43">
   <si>
     <t>证券代码</t>
   </si>
@@ -161,6 +161,9 @@
     <t xml:space="preserve">
 止损了600股 主要原因是长电科技有效跌破30日均线且回收的速度不快，温和回收，同时接近尾盘时又下跌了一点 ，对于这种慢慢的温和的回收 我有两个想法 
 一是主力在边打边撤 悄悄出货 二是主力在底部建仓 怕一下子拉飞股价  同时股价是触及到了 短期的支撑位之后回升 留下了长下影 个人主观上我想博一个反弹 客观上破位就走是我定死的纪律 所以中和二者 半苍止损是比较好的选择了</t>
+  </si>
+  <si>
+    <t>002028</t>
   </si>
 </sst>
 </file>
@@ -824,6 +827,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1357,7 +1361,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N63"/>
+  <dimension ref="A1:N64"/>
   <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="14.6153846153846" style="3" customWidth="1"/>
@@ -3556,6 +3560,20 @@
         <v>41</v>
       </c>
     </row>
+    <row r="64" ht="20.4" spans="1:4">
+      <c r="A64" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D64" s="7">
+        <v>22060312</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J63">
     <extLst/>

</xml_diff>

<commit_message>
vault backup: 2026-03-12 13:25:30
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -10,7 +10,7 @@
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$64</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="45">
   <si>
     <t>证券代码</t>
   </si>
@@ -164,6 +164,12 @@
   </si>
   <si>
     <t>002028</t>
+  </si>
+  <si>
+    <t>当时的心态和想法是 博一个反弹 当时思源电气并没有基本面或者重大利空 我不理解为什么这个时候跌破了13日均线 本来13日均线是我的止损价格 可是我没有执行好我的策略 却真的好像在赌博一样依旧加仓 我受到讨论区的影响也有点大 看到大家都觉得没事 回调 这个也一定程度上影响了我的判断 今天是加仓后的第二天我确认我做错了。</t>
+  </si>
+  <si>
+    <t>有效跌破210 止盈离场 恢复趋势后才能进场</t>
   </si>
 </sst>
 </file>
@@ -3520,10 +3526,10 @@
       <c r="K62" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L62" s="4" t="s">
+      <c r="L62" t="s">
         <v>38</v>
       </c>
-      <c r="M62" s="4" t="s">
+      <c r="M62" t="s">
         <v>39</v>
       </c>
     </row>
@@ -3540,8 +3546,8 @@
       <c r="D63" s="2">
         <v>20260309</v>
       </c>
-      <c r="E63" s="2">
-        <v>0.620138888888889</v>
+      <c r="E63" s="8">
+        <v>0.618055555555556</v>
       </c>
       <c r="F63" s="2">
         <v>45.03</v>
@@ -3560,7 +3566,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="64" ht="20.4" spans="1:4">
+    <row r="64" ht="135" spans="1:13">
       <c r="A64" s="10" t="s">
         <v>42</v>
       </c>
@@ -3573,9 +3579,31 @@
       <c r="D64" s="7">
         <v>22060312</v>
       </c>
+      <c r="E64" s="8">
+        <v>0.618055555555556</v>
+      </c>
+      <c r="F64" s="2">
+        <v>220</v>
+      </c>
+      <c r="G64" s="2">
+        <v>100</v>
+      </c>
+      <c r="H64" s="2">
+        <v>22000</v>
+      </c>
+      <c r="I64" s="2"/>
+      <c r="J64" s="2">
+        <v>700</v>
+      </c>
+      <c r="K64" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="M64" t="s">
+        <v>44</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J63">
+  <autoFilter ref="A1:J64">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-03-16 17:42:24
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="47">
   <si>
     <t>证券代码</t>
   </si>
@@ -170,6 +170,15 @@
   </si>
   <si>
     <t>有效跌破210 止盈离场 恢复趋势后才能进场</t>
+  </si>
+  <si>
+    <t>思源电气跌破210支撑位且最终没有有力的回收
+需要适当规避风险，短期走弱，但会持续关注，企稳30日线后可以入场建仓，但现在不是时候</t>
+  </si>
+  <si>
+    <t>尽管今天盘中爆出关于7nm制成工艺的利好
+依旧走势很弱涨幅小，没有回收47块，判定为
+短暂弱势+封测板块本身没什么涨头遂离场</t>
   </si>
 </sst>
 </file>
@@ -833,7 +842,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1367,7 +1378,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N64"/>
+  <dimension ref="A1:N66"/>
   <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="14.6153846153846" style="3" customWidth="1"/>
@@ -3570,13 +3581,13 @@
       <c r="A64" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B64" s="7" t="s">
+      <c r="B64" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C64" s="7" t="s">
+      <c r="C64" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D64" s="7">
+      <c r="D64" s="2">
         <v>22060312</v>
       </c>
       <c r="E64" s="8">
@@ -3600,6 +3611,71 @@
       </c>
       <c r="M64" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="65" ht="84" spans="1:14">
+      <c r="A65" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D65" s="2">
+        <v>22060316</v>
+      </c>
+      <c r="E65" s="8">
+        <v>0.618055555555556</v>
+      </c>
+      <c r="F65" s="2">
+        <v>208.14</v>
+      </c>
+      <c r="G65" s="8">
+        <v>700</v>
+      </c>
+      <c r="H65" s="2">
+        <v>145698</v>
+      </c>
+      <c r="J65" s="4">
+        <v>0</v>
+      </c>
+      <c r="N65" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="66" ht="101" spans="1:14">
+      <c r="A66" s="6">
+        <v>600584</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D66" s="2">
+        <v>22060316</v>
+      </c>
+      <c r="E66" s="8">
+        <v>0.618055555555556</v>
+      </c>
+      <c r="F66" s="2">
+        <v>45.7</v>
+      </c>
+      <c r="G66" s="8">
+        <v>500</v>
+      </c>
+      <c r="H66" s="2">
+        <v>22850</v>
+      </c>
+      <c r="I66" s="2"/>
+      <c r="J66" s="4">
+        <v>0</v>
+      </c>
+      <c r="N66" s="9" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-03-18 20:30:07
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -10,7 +10,7 @@
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$66</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="52">
   <si>
     <t>证券代码</t>
   </si>
@@ -179,6 +179,22 @@
     <t>尽管今天盘中爆出关于7nm制成工艺的利好
 依旧走势很弱涨幅小，没有回收47块，判定为
 短暂弱势+封测板块本身没什么涨头遂离场</t>
+  </si>
+  <si>
+    <t>思源电气 逻辑还在 今天正式站稳30日线 且上涨幅度达4%强度可延续 今天初步建仓主要为了试仓 最终仓位上限定格在10w</t>
+  </si>
+  <si>
+    <t>跌破30日线离场</t>
+  </si>
+  <si>
+    <t>亨通光电</t>
+  </si>
+  <si>
+    <t>亨通光电作为光纤的人气公司 pe处于低值 同时今天站稳了30日线
+ 做一下左侧交易问题应该不大 轻仓试错中</t>
+  </si>
+  <si>
+    <t>有效跌破30日线离场</t>
   </si>
 </sst>
 </file>
@@ -1378,7 +1394,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N66"/>
+  <dimension ref="A1:N68"/>
   <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="14.6153846153846" style="3" customWidth="1"/>
@@ -3632,7 +3648,7 @@
       <c r="F65" s="2">
         <v>208.14</v>
       </c>
-      <c r="G65" s="8">
+      <c r="G65" s="2">
         <v>700</v>
       </c>
       <c r="H65" s="2">
@@ -3664,7 +3680,7 @@
       <c r="F66" s="2">
         <v>45.7</v>
       </c>
-      <c r="G66" s="8">
+      <c r="G66" s="2">
         <v>500</v>
       </c>
       <c r="H66" s="2">
@@ -3678,8 +3694,79 @@
         <v>46</v>
       </c>
     </row>
+    <row r="67" ht="51" spans="1:13">
+      <c r="A67" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D67" s="2">
+        <v>20260318</v>
+      </c>
+      <c r="E67" s="8">
+        <v>0.618055555555556</v>
+      </c>
+      <c r="F67" s="2">
+        <v>220.183</v>
+      </c>
+      <c r="G67" s="2">
+        <v>100</v>
+      </c>
+      <c r="H67" s="2">
+        <v>22018</v>
+      </c>
+      <c r="I67" s="2"/>
+      <c r="J67" s="2">
+        <v>100</v>
+      </c>
+      <c r="K67" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="M67" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="68" ht="51" spans="1:13">
+      <c r="A68" s="6">
+        <v>600487</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D68" s="2">
+        <v>20260318</v>
+      </c>
+      <c r="E68" s="8">
+        <v>0.618055555555556</v>
+      </c>
+      <c r="F68" s="4">
+        <v>44.53</v>
+      </c>
+      <c r="G68" s="4">
+        <v>600</v>
+      </c>
+      <c r="H68" s="4">
+        <v>26708</v>
+      </c>
+      <c r="J68" s="4">
+        <v>600</v>
+      </c>
+      <c r="K68" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="M68" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J64">
+  <autoFilter ref="A1:J66">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-03-19 18:38:36
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -10,7 +10,7 @@
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$68</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="54">
   <si>
     <t>证券代码</t>
   </si>
@@ -190,11 +190,16 @@
     <t>亨通光电</t>
   </si>
   <si>
-    <t>亨通光电作为光纤的人气公司 pe处于低值 同时今天站稳了30日线
- 做一下左侧交易问题应该不大 轻仓试错中</t>
+    <t>亨通光电作为光纤的人气公司 pe处于低值 同时今天站稳了30日线做一下左侧交易问题应该不大 轻仓试错中</t>
   </si>
   <si>
     <t>有效跌破30日线离场</t>
+  </si>
+  <si>
+    <t>今天在9:57的时候有一波操作 这波操作跟我之前的都不太一样，买点依据当天早上212.8时我看到分时图已经开始反转同时有反弹的趋势，我害怕还像昨天那样错过大反弹+鉴于今天大盘表现不佳 下午拉盘的概率高+思源电气早上反弹的概率大 于是选择买入</t>
+  </si>
+  <si>
+    <t>原本设定的限价单放在了210，直到收盘也没有打到210的位置，我认为今天作为一个普跌行情，反弹是最近的大概率事件，尾盘突然的拉伸正想追进去发现尾盘又砸了，既然稳在30日线 逐步布局加仓也是好的</t>
   </si>
 </sst>
 </file>
@@ -1394,7 +1399,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N68"/>
+  <dimension ref="A1:N70"/>
   <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="14.6153846153846" style="3" customWidth="1"/>
@@ -3654,7 +3659,7 @@
       <c r="H65" s="2">
         <v>145698</v>
       </c>
-      <c r="J65" s="4">
+      <c r="J65" s="2">
         <v>0</v>
       </c>
       <c r="N65" s="9" t="s">
@@ -3687,7 +3692,7 @@
         <v>22850</v>
       </c>
       <c r="I66" s="2"/>
-      <c r="J66" s="4">
+      <c r="J66" s="2">
         <v>0</v>
       </c>
       <c r="N66" s="9" t="s">
@@ -3746,16 +3751,16 @@
       <c r="E68" s="8">
         <v>0.618055555555556</v>
       </c>
-      <c r="F68" s="4">
+      <c r="F68" s="2">
         <v>44.53</v>
       </c>
-      <c r="G68" s="4">
+      <c r="G68" s="2">
         <v>600</v>
       </c>
-      <c r="H68" s="4">
+      <c r="H68" s="2">
         <v>26708</v>
       </c>
-      <c r="J68" s="4">
+      <c r="J68" s="2">
         <v>600</v>
       </c>
       <c r="K68" s="9" t="s">
@@ -3765,8 +3770,72 @@
         <v>51</v>
       </c>
     </row>
+    <row r="69" ht="101" spans="1:11">
+      <c r="A69" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D69" s="2">
+        <v>20260319</v>
+      </c>
+      <c r="E69" s="8">
+        <v>0.414583333333333</v>
+      </c>
+      <c r="F69" s="2">
+        <v>214.5</v>
+      </c>
+      <c r="G69" s="2">
+        <v>100</v>
+      </c>
+      <c r="H69" s="2">
+        <v>21459</v>
+      </c>
+      <c r="J69" s="2">
+        <v>200</v>
+      </c>
+      <c r="K69" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="70" ht="84" spans="1:11">
+      <c r="A70" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D70" s="2">
+        <v>20260319</v>
+      </c>
+      <c r="E70" s="8">
+        <v>0.625</v>
+      </c>
+      <c r="F70" s="2">
+        <v>211.1</v>
+      </c>
+      <c r="G70" s="2">
+        <v>100</v>
+      </c>
+      <c r="H70" s="2">
+        <v>21110</v>
+      </c>
+      <c r="J70" s="2">
+        <v>200</v>
+      </c>
+      <c r="K70" s="9" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J66">
+  <autoFilter ref="A1:J68">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-03-23 23:17:08
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="13020"/>
+    <workbookView windowWidth="29100" windowHeight="14560"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$70</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="55">
   <si>
     <t>证券代码</t>
   </si>
@@ -200,6 +200,10 @@
   </si>
   <si>
     <t>原本设定的限价单放在了210，直到收盘也没有打到210的位置，我认为今天作为一个普跌行情，反弹是最近的大概率事件，尾盘突然的拉伸正想追进去发现尾盘又砸了，既然稳在30日线 逐步布局加仓也是好的</t>
+  </si>
+  <si>
+    <t>认为短期是一个加仓的时期 同时早盘
+走的很强势 于是有点贸然加仓了</t>
   </si>
 </sst>
 </file>
@@ -836,7 +840,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -862,6 +866,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center"/>
@@ -1399,13 +1406,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:N71"/>
   <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="14.6153846153846" style="3" customWidth="1"/>
     <col min="2" max="2" width="14.6153846153846" style="4" customWidth="1"/>
     <col min="3" max="3" width="35.4615384615385" style="4" customWidth="1"/>
-    <col min="4" max="10" width="14.6153846153846" style="4" customWidth="1"/>
+    <col min="4" max="4" width="28.6538461538462" style="4" customWidth="1"/>
+    <col min="5" max="10" width="14.6153846153846" style="4" customWidth="1"/>
     <col min="11" max="11" width="43.9038461538462" style="4" customWidth="1"/>
     <col min="12" max="12" width="27.6923076923077" style="4" customWidth="1"/>
     <col min="13" max="13" width="27.0769230769231" style="4" customWidth="1"/>
@@ -3599,7 +3607,7 @@
       </c>
     </row>
     <row r="64" ht="135" spans="1:13">
-      <c r="A64" s="10" t="s">
+      <c r="A64" s="11" t="s">
         <v>42</v>
       </c>
       <c r="B64" s="2" t="s">
@@ -3635,7 +3643,7 @@
       </c>
     </row>
     <row r="65" ht="84" spans="1:14">
-      <c r="A65" s="10" t="s">
+      <c r="A65" s="11" t="s">
         <v>42</v>
       </c>
       <c r="B65" s="2" t="s">
@@ -3700,7 +3708,7 @@
       </c>
     </row>
     <row r="67" ht="51" spans="1:13">
-      <c r="A67" s="10" t="s">
+      <c r="A67" s="11" t="s">
         <v>42</v>
       </c>
       <c r="B67" s="2" t="s">
@@ -3771,7 +3779,7 @@
       </c>
     </row>
     <row r="69" ht="101" spans="1:11">
-      <c r="A69" s="10" t="s">
+      <c r="A69" s="11" t="s">
         <v>42</v>
       </c>
       <c r="B69" s="2" t="s">
@@ -3803,7 +3811,7 @@
       </c>
     </row>
     <row r="70" ht="84" spans="1:11">
-      <c r="A70" s="10" t="s">
+      <c r="A70" s="11" t="s">
         <v>42</v>
       </c>
       <c r="B70" s="2" t="s">
@@ -3828,14 +3836,46 @@
         <v>21110</v>
       </c>
       <c r="J70" s="2">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="K70" s="9" t="s">
         <v>53</v>
       </c>
     </row>
+    <row r="71" ht="34" spans="1:11">
+      <c r="A71" s="6">
+        <v>600487</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D71" s="10">
+        <v>20260320</v>
+      </c>
+      <c r="E71" s="2">
+        <v>0.425</v>
+      </c>
+      <c r="F71" s="2">
+        <v>45.07</v>
+      </c>
+      <c r="G71" s="2">
+        <v>600</v>
+      </c>
+      <c r="H71" s="2">
+        <v>27042</v>
+      </c>
+      <c r="J71" s="2">
+        <v>1200</v>
+      </c>
+      <c r="K71" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J68">
+  <autoFilter ref="A1:J70">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-03-25 17:14:19
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="14560"/>
+    <workbookView windowWidth="29100" windowHeight="13020"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$71</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="58">
   <si>
     <t>证券代码</t>
   </si>
@@ -204,6 +204,15 @@
   <si>
     <t>认为短期是一个加仓的时期 同时早盘
 走的很强势 于是有点贸然加仓了</t>
+  </si>
+  <si>
+    <t>亨通光电早盘高开低走下午探底回升之后十分强势收复前几天大跌的阴线，且当时均价仍低于成本线，短期支撑位40.96已经明晰，寻求一波追涨</t>
+  </si>
+  <si>
+    <t>002208</t>
+  </si>
+  <si>
+    <t>这一波买入跟昨天买入亨通光电的逻辑是一致的在看到思源电气企稳逐步回到趋势后 同时又低于现在仓位均价加仓是看起来很划算的事情 ，电力走的好 一定程度上也带动了电网，但要开始逐步小心风险了</t>
   </si>
 </sst>
 </file>
@@ -216,7 +225,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,6 +244,14 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -710,137 +727,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -850,25 +867,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center"/>
@@ -1406,18 +1416,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N71"/>
-  <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
+  <dimension ref="A1:N73"/>
+  <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="20.4"/>
   <cols>
-    <col min="1" max="1" width="14.6153846153846" style="3" customWidth="1"/>
-    <col min="2" max="2" width="14.6153846153846" style="4" customWidth="1"/>
-    <col min="3" max="3" width="35.4615384615385" style="4" customWidth="1"/>
-    <col min="4" max="4" width="28.6538461538462" style="4" customWidth="1"/>
-    <col min="5" max="10" width="14.6153846153846" style="4" customWidth="1"/>
-    <col min="11" max="11" width="43.9038461538462" style="4" customWidth="1"/>
-    <col min="12" max="12" width="27.6923076923077" style="4" customWidth="1"/>
-    <col min="13" max="13" width="27.0769230769231" style="4" customWidth="1"/>
-    <col min="14" max="14" width="40.5384615384615" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14.6153846153846" style="2" customWidth="1"/>
+    <col min="2" max="2" width="14.6153846153846" style="3" customWidth="1"/>
+    <col min="3" max="3" width="35.4615384615385" style="2" customWidth="1"/>
+    <col min="4" max="4" width="28.6538461538462" style="2" customWidth="1"/>
+    <col min="5" max="5" width="14.6153846153846" style="4" customWidth="1"/>
+    <col min="6" max="8" width="14.6153846153846" style="2" customWidth="1"/>
+    <col min="9" max="9" width="14.6153846153846" style="3" customWidth="1"/>
+    <col min="10" max="10" width="14.6153846153846" style="2" customWidth="1"/>
+    <col min="11" max="11" width="43.9038461538462" style="3" customWidth="1"/>
+    <col min="12" max="12" width="27.6923076923077" style="3" customWidth="1"/>
+    <col min="13" max="13" width="27.0769230769231" style="3" customWidth="1"/>
+    <col min="14" max="14" width="40.5384615384615" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="23.2" customHeight="1" spans="1:14">
@@ -1427,28 +1440,28 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
@@ -1464,8 +1477,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A2" s="6">
+    <row r="2" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A2" s="2">
         <v>600276</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1477,7 +1490,7 @@
       <c r="D2" s="2">
         <v>20250902</v>
       </c>
-      <c r="E2" s="8">
+      <c r="E2" s="4">
         <v>0.395983796296296</v>
       </c>
       <c r="F2" s="2">
@@ -1498,8 +1511,8 @@
         <v>200</v>
       </c>
     </row>
-    <row r="3" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A3" s="6">
+    <row r="3" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A3" s="2">
         <v>600276</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1511,7 +1524,7 @@
       <c r="D3" s="2">
         <v>20250903</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="4">
         <v>0.400289351851852</v>
       </c>
       <c r="F3" s="2">
@@ -1532,8 +1545,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A4" s="6">
+    <row r="4" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A4" s="2">
         <v>601138</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -1545,7 +1558,7 @@
       <c r="D4" s="2">
         <v>20250912</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="4">
         <v>0.407638888888889</v>
       </c>
       <c r="F4" s="2">
@@ -1567,7 +1580,7 @@
       </c>
     </row>
     <row r="5" s="2" customFormat="1" ht="20" customHeight="1" spans="1:10">
-      <c r="A5" s="6">
+      <c r="A5" s="2">
         <v>601138</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1579,7 +1592,7 @@
       <c r="D5" s="2">
         <v>20250915</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="4">
         <v>0.591782407407407</v>
       </c>
       <c r="F5" s="2">
@@ -1600,8 +1613,8 @@
         <v>500</v>
       </c>
     </row>
-    <row r="6" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A6" s="6">
+    <row r="6" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A6" s="2">
         <v>601138</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -1613,7 +1626,7 @@
       <c r="D6" s="2">
         <v>20250915</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="4">
         <v>0.399363425925926</v>
       </c>
       <c r="F6" s="2">
@@ -1634,8 +1647,8 @@
         <v>600</v>
       </c>
     </row>
-    <row r="7" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A7" s="6">
+    <row r="7" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A7" s="2">
         <v>603986</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1647,7 +1660,7 @@
       <c r="D7" s="2">
         <v>20250925</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="4">
         <v>0.609340277777778</v>
       </c>
       <c r="F7" s="2">
@@ -1668,8 +1681,8 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A8" s="6">
+    <row r="8" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A8" s="2">
         <v>601138</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -1681,7 +1694,7 @@
       <c r="D8" s="2">
         <v>20251009</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="4">
         <v>0.446851851851852</v>
       </c>
       <c r="F8" s="2">
@@ -1702,8 +1715,8 @@
         <v>400</v>
       </c>
     </row>
-    <row r="9" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A9" s="6">
+    <row r="9" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A9" s="2">
         <v>600111</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -1715,7 +1728,7 @@
       <c r="D9" s="2">
         <v>20251010</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="4">
         <v>0.417337962962963</v>
       </c>
       <c r="F9" s="2">
@@ -1736,8 +1749,8 @@
         <v>200</v>
       </c>
     </row>
-    <row r="10" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A10" s="6">
+    <row r="10" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A10" s="2">
         <v>600111</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1749,7 +1762,7 @@
       <c r="D10" s="2">
         <v>20251010</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="4">
         <v>0.396574074074074</v>
       </c>
       <c r="F10" s="2">
@@ -1770,8 +1783,8 @@
         <v>500</v>
       </c>
     </row>
-    <row r="11" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A11" s="6">
+    <row r="11" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A11" s="2">
         <v>601138</v>
       </c>
       <c r="B11" s="2" t="s">
@@ -1783,7 +1796,7 @@
       <c r="D11" s="2">
         <v>20251015</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="4">
         <v>0.453912037037037</v>
       </c>
       <c r="F11" s="2">
@@ -1804,8 +1817,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A12" s="6">
+    <row r="12" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A12" s="2">
         <v>603986</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -1817,7 +1830,7 @@
       <c r="D12" s="2">
         <v>20251015</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="4">
         <v>0.453784722222222</v>
       </c>
       <c r="F12" s="2">
@@ -1838,8 +1851,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A13" s="6">
+    <row r="13" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A13" s="2">
         <v>600111</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -1851,7 +1864,7 @@
       <c r="D13" s="2">
         <v>20251015</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="4">
         <v>0.422696759259259</v>
       </c>
       <c r="F13" s="2">
@@ -1872,8 +1885,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A14" s="6" t="str">
+    <row r="14" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A14" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
@@ -1886,7 +1899,7 @@
       <c r="D14" s="2">
         <v>20251016</v>
       </c>
-      <c r="E14" s="8">
+      <c r="E14" s="4">
         <v>0.560474537037037</v>
       </c>
       <c r="F14" s="2">
@@ -1907,8 +1920,8 @@
         <v>600</v>
       </c>
     </row>
-    <row r="15" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A15" s="6">
+    <row r="15" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A15" s="2">
         <v>603259</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -1920,7 +1933,7 @@
       <c r="D15" s="2">
         <v>20251016</v>
       </c>
-      <c r="E15" s="8">
+      <c r="E15" s="4">
         <v>0.458530092592593</v>
       </c>
       <c r="F15" s="2">
@@ -1941,8 +1954,8 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A16" s="6" t="str">
+    <row r="16" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A16" s="2" t="str">
         <f>"002371"</f>
         <v>002371</v>
       </c>
@@ -1955,7 +1968,7 @@
       <c r="D16" s="2">
         <v>20251017</v>
       </c>
-      <c r="E16" s="8">
+      <c r="E16" s="4">
         <v>0.625</v>
       </c>
       <c r="F16" s="2">
@@ -1976,8 +1989,8 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A17" s="6" t="str">
+    <row r="17" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A17" s="2" t="str">
         <f>"002281"</f>
         <v>002281</v>
       </c>
@@ -1990,7 +2003,7 @@
       <c r="D17" s="2">
         <v>20251021</v>
       </c>
-      <c r="E17" s="8">
+      <c r="E17" s="4">
         <v>0.621550925925926</v>
       </c>
       <c r="F17" s="2">
@@ -2011,8 +2024,8 @@
         <v>300</v>
       </c>
     </row>
-    <row r="18" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A18" s="6">
+    <row r="18" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A18" s="2">
         <v>603259</v>
       </c>
       <c r="B18" s="2" t="s">
@@ -2024,7 +2037,7 @@
       <c r="D18" s="2">
         <v>20251021</v>
       </c>
-      <c r="E18" s="8">
+      <c r="E18" s="4">
         <v>0.46806712962963</v>
       </c>
       <c r="F18" s="2">
@@ -2045,8 +2058,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A19" s="6" t="str">
+    <row r="19" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A19" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
@@ -2059,7 +2072,7 @@
       <c r="D19" s="2">
         <v>20251021</v>
       </c>
-      <c r="E19" s="8">
+      <c r="E19" s="4">
         <v>0.418518518518519</v>
       </c>
       <c r="F19" s="2">
@@ -2080,8 +2093,8 @@
         <v>400</v>
       </c>
     </row>
-    <row r="20" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A20" s="6">
+    <row r="20" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A20" s="2">
         <v>603986</v>
       </c>
       <c r="B20" s="2" t="s">
@@ -2093,7 +2106,7 @@
       <c r="D20" s="2">
         <v>20251023</v>
       </c>
-      <c r="E20" s="8">
+      <c r="E20" s="4">
         <v>0.617777777777778</v>
       </c>
       <c r="F20" s="2">
@@ -2114,8 +2127,8 @@
         <v>200</v>
       </c>
     </row>
-    <row r="21" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A21" s="6" t="str">
+    <row r="21" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A21" s="2" t="str">
         <f>"002371"</f>
         <v>002371</v>
       </c>
@@ -2128,7 +2141,7 @@
       <c r="D21" s="2">
         <v>20251023</v>
       </c>
-      <c r="E21" s="8">
+      <c r="E21" s="4">
         <v>0.616111111111111</v>
       </c>
       <c r="F21" s="2">
@@ -2149,8 +2162,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A22" s="6" t="str">
+    <row r="22" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A22" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
@@ -2163,7 +2176,7 @@
       <c r="D22" s="2">
         <v>20251024</v>
       </c>
-      <c r="E22" s="8">
+      <c r="E22" s="4">
         <v>0.601006944444444</v>
       </c>
       <c r="F22" s="2">
@@ -2184,8 +2197,8 @@
         <v>300</v>
       </c>
     </row>
-    <row r="23" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A23" s="6">
+    <row r="23" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A23" s="2">
         <v>603986</v>
       </c>
       <c r="B23" s="2" t="s">
@@ -2197,7 +2210,7 @@
       <c r="D23" s="2">
         <v>20251024</v>
       </c>
-      <c r="E23" s="8">
+      <c r="E23" s="4">
         <v>0.589212962962963</v>
       </c>
       <c r="F23" s="2">
@@ -2218,8 +2231,8 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A24" s="6" t="str">
+    <row r="24" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A24" s="2" t="str">
         <f>"002281"</f>
         <v>002281</v>
       </c>
@@ -2232,7 +2245,7 @@
       <c r="D24" s="2">
         <v>20251024</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E24" s="4">
         <v>0.418425925925926</v>
       </c>
       <c r="F24" s="2">
@@ -2253,8 +2266,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A25" s="6">
+    <row r="25" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A25" s="2">
         <v>603083</v>
       </c>
       <c r="B25" s="2" t="s">
@@ -2266,7 +2279,7 @@
       <c r="D25" s="2">
         <v>20251027</v>
       </c>
-      <c r="E25" s="8">
+      <c r="E25" s="4">
         <v>0.399074074074074</v>
       </c>
       <c r="F25" s="2">
@@ -2287,8 +2300,8 @@
         <v>200</v>
       </c>
     </row>
-    <row r="26" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A26" s="6">
+    <row r="26" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A26" s="2">
         <v>603083</v>
       </c>
       <c r="B26" s="2" t="s">
@@ -2300,7 +2313,7 @@
       <c r="D26" s="2">
         <v>20251028</v>
       </c>
-      <c r="E26" s="8">
+      <c r="E26" s="4">
         <v>0.625</v>
       </c>
       <c r="F26" s="2">
@@ -2321,8 +2334,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A27" s="6">
+    <row r="27" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A27" s="2">
         <v>603986</v>
       </c>
       <c r="B27" s="2" t="s">
@@ -2334,7 +2347,7 @@
       <c r="D27" s="2">
         <v>20251029</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E27" s="4">
         <v>0.441550925925926</v>
       </c>
       <c r="F27" s="2">
@@ -2355,8 +2368,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A28" s="6">
+    <row r="28" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A28" s="2">
         <v>603799</v>
       </c>
       <c r="B28" s="2" t="s">
@@ -2368,7 +2381,7 @@
       <c r="D28" s="2">
         <v>20251030</v>
       </c>
-      <c r="E28" s="8">
+      <c r="E28" s="4">
         <v>0.565590277777778</v>
       </c>
       <c r="F28" s="2">
@@ -2389,8 +2402,8 @@
         <v>300</v>
       </c>
     </row>
-    <row r="29" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A29" s="6">
+    <row r="29" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A29" s="2">
         <v>603986</v>
       </c>
       <c r="B29" s="2" t="s">
@@ -2402,7 +2415,7 @@
       <c r="D29" s="2">
         <v>20251030</v>
       </c>
-      <c r="E29" s="8">
+      <c r="E29" s="4">
         <v>0.544988425925926</v>
       </c>
       <c r="F29" s="2">
@@ -2423,8 +2436,8 @@
         <v>100</v>
       </c>
     </row>
-    <row r="30" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A30" s="6">
+    <row r="30" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A30" s="2">
         <v>603099</v>
       </c>
       <c r="B30" s="2" t="s">
@@ -2436,7 +2449,7 @@
       <c r="D30" s="2">
         <v>20251104</v>
       </c>
-      <c r="E30" s="8">
+      <c r="E30" s="4">
         <v>0.625</v>
       </c>
       <c r="F30" s="2">
@@ -2457,8 +2470,8 @@
         <v>100</v>
       </c>
     </row>
-    <row r="31" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A31" s="6">
+    <row r="31" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A31" s="2">
         <v>603099</v>
       </c>
       <c r="B31" s="2" t="s">
@@ -2470,7 +2483,7 @@
       <c r="D31" s="2">
         <v>20251104</v>
       </c>
-      <c r="E31" s="8">
+      <c r="E31" s="4">
         <v>0.625</v>
       </c>
       <c r="F31" s="2">
@@ -2491,8 +2504,8 @@
         <v>200</v>
       </c>
     </row>
-    <row r="32" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A32" s="6">
+    <row r="32" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A32" s="2">
         <v>603799</v>
       </c>
       <c r="B32" s="2" t="s">
@@ -2504,7 +2517,7 @@
       <c r="D32" s="2">
         <v>20251104</v>
       </c>
-      <c r="E32" s="8">
+      <c r="E32" s="4">
         <v>0.625</v>
       </c>
       <c r="F32" s="2">
@@ -2525,8 +2538,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A33" s="6">
+    <row r="33" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A33" s="2">
         <v>603099</v>
       </c>
       <c r="B33" s="2" t="s">
@@ -2538,7 +2551,7 @@
       <c r="D33" s="2">
         <v>20251105</v>
       </c>
-      <c r="E33" s="8">
+      <c r="E33" s="4">
         <v>0.413472222222222</v>
       </c>
       <c r="F33" s="2">
@@ -2559,8 +2572,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A34" s="6" t="str">
+    <row r="34" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A34" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
@@ -2573,7 +2586,7 @@
       <c r="D34" s="2">
         <v>20260119</v>
       </c>
-      <c r="E34" s="8">
+      <c r="E34" s="4">
         <v>0.422534722222222</v>
       </c>
       <c r="F34" s="2">
@@ -2594,8 +2607,8 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A35" s="6">
+    <row r="35" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A35" s="2">
         <v>601179</v>
       </c>
       <c r="B35" s="2" t="s">
@@ -2607,7 +2620,7 @@
       <c r="D35" s="2">
         <v>20260119</v>
       </c>
-      <c r="E35" s="8">
+      <c r="E35" s="4">
         <v>0.400891203703704</v>
       </c>
       <c r="F35" s="2">
@@ -2628,8 +2641,8 @@
         <v>1400</v>
       </c>
     </row>
-    <row r="36" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A36" s="6" t="str">
+    <row r="36" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A36" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
@@ -2642,7 +2655,7 @@
       <c r="D36" s="2">
         <v>20260119</v>
       </c>
-      <c r="E36" s="8">
+      <c r="E36" s="4">
         <v>0.398483796296296</v>
       </c>
       <c r="F36" s="2">
@@ -2663,8 +2676,8 @@
         <v>200</v>
       </c>
     </row>
-    <row r="37" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A37" s="6">
+    <row r="37" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A37" s="2">
         <v>603986</v>
       </c>
       <c r="B37" s="2" t="s">
@@ -2676,7 +2689,7 @@
       <c r="D37" s="2">
         <v>20260119</v>
       </c>
-      <c r="E37" s="8">
+      <c r="E37" s="4">
         <v>0.396030092592593</v>
       </c>
       <c r="F37" s="2">
@@ -2697,8 +2710,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A38" s="6" t="str">
+    <row r="38" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A38" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
@@ -2711,7 +2724,7 @@
       <c r="D38" s="2">
         <v>20260121</v>
       </c>
-      <c r="E38" s="8">
+      <c r="E38" s="4">
         <v>0.397384259259259</v>
       </c>
       <c r="F38" s="2">
@@ -2732,8 +2745,8 @@
         <v>300</v>
       </c>
     </row>
-    <row r="39" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A39" s="6" t="str">
+    <row r="39" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A39" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
@@ -2746,7 +2759,7 @@
       <c r="D39" s="2">
         <v>20260122</v>
       </c>
-      <c r="E39" s="8">
+      <c r="E39" s="4">
         <v>0.444861111111111</v>
       </c>
       <c r="F39" s="2">
@@ -2767,8 +2780,8 @@
         <v>400</v>
       </c>
     </row>
-    <row r="40" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A40" s="6">
+    <row r="40" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A40" s="2">
         <v>600584</v>
       </c>
       <c r="B40" s="2" t="s">
@@ -2780,7 +2793,7 @@
       <c r="D40" s="2">
         <v>20260122</v>
       </c>
-      <c r="E40" s="8">
+      <c r="E40" s="4">
         <v>0.407951388888889</v>
       </c>
       <c r="F40" s="2">
@@ -2801,8 +2814,8 @@
         <v>400</v>
       </c>
     </row>
-    <row r="41" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A41" s="6">
+    <row r="41" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A41" s="2">
         <v>601179</v>
       </c>
       <c r="B41" s="2" t="s">
@@ -2814,7 +2827,7 @@
       <c r="D41" s="2">
         <v>20260126</v>
       </c>
-      <c r="E41" s="8">
+      <c r="E41" s="4">
         <v>0.622175925925926</v>
       </c>
       <c r="F41" s="2">
@@ -2835,8 +2848,8 @@
         <v>700</v>
       </c>
     </row>
-    <row r="42" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A42" s="6">
+    <row r="42" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A42" s="2">
         <v>600584</v>
       </c>
       <c r="B42" s="2" t="s">
@@ -2848,7 +2861,7 @@
       <c r="D42" s="2">
         <v>20260127</v>
       </c>
-      <c r="E42" s="8">
+      <c r="E42" s="4">
         <v>0.589479166666667</v>
       </c>
       <c r="F42" s="2">
@@ -2869,8 +2882,8 @@
         <v>600</v>
       </c>
     </row>
-    <row r="43" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A43" s="6" t="str">
+    <row r="43" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A43" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
@@ -2883,7 +2896,7 @@
       <c r="D43" s="2">
         <v>20260127</v>
       </c>
-      <c r="E43" s="8">
+      <c r="E43" s="4">
         <v>0.413969907407407</v>
       </c>
       <c r="F43" s="2">
@@ -2904,8 +2917,8 @@
         <v>500</v>
       </c>
     </row>
-    <row r="44" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A44" s="6" t="str">
+    <row r="44" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A44" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
@@ -2918,7 +2931,7 @@
       <c r="D44" s="2">
         <v>20260129</v>
       </c>
-      <c r="E44" s="8">
+      <c r="E44" s="4">
         <v>0.5778125</v>
       </c>
       <c r="F44" s="2">
@@ -2939,8 +2952,8 @@
         <v>500</v>
       </c>
     </row>
-    <row r="45" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A45" s="6" t="str">
+    <row r="45" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A45" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
@@ -2953,7 +2966,7 @@
       <c r="D45" s="2">
         <v>20260129</v>
       </c>
-      <c r="E45" s="8">
+      <c r="E45" s="4">
         <v>0.571990740740741</v>
       </c>
       <c r="F45" s="2">
@@ -2974,8 +2987,8 @@
         <v>400</v>
       </c>
     </row>
-    <row r="46" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A46" s="6">
+    <row r="46" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A46" s="2">
         <v>600584</v>
       </c>
       <c r="B46" s="2" t="s">
@@ -2987,7 +3000,7 @@
       <c r="D46" s="2">
         <v>20260129</v>
       </c>
-      <c r="E46" s="8">
+      <c r="E46" s="4">
         <v>0.57099537037037</v>
       </c>
       <c r="F46" s="2">
@@ -3008,8 +3021,8 @@
         <v>400</v>
       </c>
     </row>
-    <row r="47" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A47" s="6" t="str">
+    <row r="47" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A47" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
@@ -3022,7 +3035,7 @@
       <c r="D47" s="2">
         <v>20260129</v>
       </c>
-      <c r="E47" s="8">
+      <c r="E47" s="4">
         <v>0.545462962962963</v>
       </c>
       <c r="F47" s="2">
@@ -3043,8 +3056,8 @@
         <v>500</v>
       </c>
     </row>
-    <row r="48" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A48" s="6" t="str">
+    <row r="48" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A48" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
@@ -3057,7 +3070,7 @@
       <c r="D48" s="2">
         <v>20260129</v>
       </c>
-      <c r="E48" s="8">
+      <c r="E48" s="4">
         <v>0.542395833333333</v>
       </c>
       <c r="F48" s="2">
@@ -3078,8 +3091,8 @@
         <v>600</v>
       </c>
     </row>
-    <row r="49" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A49" s="6">
+    <row r="49" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A49" s="2">
         <v>601179</v>
       </c>
       <c r="B49" s="2" t="s">
@@ -3091,7 +3104,7 @@
       <c r="D49" s="2">
         <v>20260130</v>
       </c>
-      <c r="E49" s="8">
+      <c r="E49" s="4">
         <v>0.440439814814815</v>
       </c>
       <c r="F49" s="2">
@@ -3112,8 +3125,8 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="50" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A50" s="6" t="str">
+    <row r="50" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A50" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
@@ -3126,7 +3139,7 @@
       <c r="D50" s="2">
         <v>20260130</v>
       </c>
-      <c r="E50" s="8">
+      <c r="E50" s="4">
         <v>0.431030092592593</v>
       </c>
       <c r="F50" s="2">
@@ -3147,8 +3160,8 @@
         <v>700</v>
       </c>
     </row>
-    <row r="51" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A51" s="6" t="str">
+    <row r="51" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A51" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
@@ -3161,7 +3174,7 @@
       <c r="D51" s="2">
         <v>20260202</v>
       </c>
-      <c r="E51" s="8">
+      <c r="E51" s="4">
         <v>0.618993055555556</v>
       </c>
       <c r="F51" s="2">
@@ -3182,8 +3195,8 @@
         <v>200</v>
       </c>
     </row>
-    <row r="52" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A52" s="6">
+    <row r="52" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A52" s="2">
         <v>600584</v>
       </c>
       <c r="B52" s="2" t="s">
@@ -3195,7 +3208,7 @@
       <c r="D52" s="2">
         <v>20260202</v>
       </c>
-      <c r="E52" s="8">
+      <c r="E52" s="4">
         <v>0.565694444444444</v>
       </c>
       <c r="F52" s="2">
@@ -3216,8 +3229,8 @@
         <v>500</v>
       </c>
     </row>
-    <row r="53" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A53" s="6">
+    <row r="53" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A53" s="2">
         <v>601179</v>
       </c>
       <c r="B53" s="2" t="s">
@@ -3229,7 +3242,7 @@
       <c r="D53" s="2">
         <v>20260202</v>
       </c>
-      <c r="E53" s="8">
+      <c r="E53" s="4">
         <v>0.55994212962963</v>
       </c>
       <c r="F53" s="2">
@@ -3250,8 +3263,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A54" s="6" t="str">
+    <row r="54" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A54" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
@@ -3264,7 +3277,7 @@
       <c r="D54" s="2">
         <v>20260202</v>
       </c>
-      <c r="E54" s="8">
+      <c r="E54" s="4">
         <v>0.446747685185185</v>
       </c>
       <c r="F54" s="2">
@@ -3285,8 +3298,8 @@
         <v>600</v>
       </c>
     </row>
-    <row r="55" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A55" s="6" t="str">
+    <row r="55" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A55" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
@@ -3299,7 +3312,7 @@
       <c r="D55" s="2">
         <v>20260202</v>
       </c>
-      <c r="E55" s="8">
+      <c r="E55" s="4">
         <v>0.440671296296296</v>
       </c>
       <c r="F55" s="2">
@@ -3320,8 +3333,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A56" s="6" t="str">
+    <row r="56" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A56" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
@@ -3334,7 +3347,7 @@
       <c r="D56" s="2">
         <v>20260203</v>
       </c>
-      <c r="E56" s="8">
+      <c r="E56" s="4">
         <v>0.409178240740741</v>
       </c>
       <c r="F56" s="2">
@@ -3355,8 +3368,8 @@
         <v>500</v>
       </c>
     </row>
-    <row r="57" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A57" s="6" t="str">
+    <row r="57" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A57" s="2" t="str">
         <f t="shared" ref="A57:A62" si="0">"002028"</f>
         <v>002028</v>
       </c>
@@ -3369,7 +3382,7 @@
       <c r="D57" s="2">
         <v>20260205</v>
       </c>
-      <c r="E57" s="8">
+      <c r="E57" s="4">
         <v>0.404363425925926</v>
       </c>
       <c r="F57" s="2">
@@ -3390,8 +3403,8 @@
         <v>600</v>
       </c>
     </row>
-    <row r="58" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A58" s="6" t="str">
+    <row r="58" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A58" s="2" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
       </c>
@@ -3404,7 +3417,7 @@
       <c r="D58" s="2">
         <v>20260209</v>
       </c>
-      <c r="E58" s="8">
+      <c r="E58" s="4">
         <v>0.445486111111111</v>
       </c>
       <c r="F58" s="2">
@@ -3425,8 +3438,8 @@
         <v>700</v>
       </c>
     </row>
-    <row r="59" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A59" s="6">
+    <row r="59" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A59" s="2">
         <v>600584</v>
       </c>
       <c r="B59" s="2" t="s">
@@ -3438,7 +3451,7 @@
       <c r="D59" s="2">
         <v>20260209</v>
       </c>
-      <c r="E59" s="8">
+      <c r="E59" s="4">
         <v>0.438865740740741</v>
       </c>
       <c r="F59" s="2">
@@ -3459,8 +3472,8 @@
         <v>700</v>
       </c>
     </row>
-    <row r="60" s="2" customFormat="1" ht="20.4" customHeight="1" spans="1:10">
-      <c r="A60" s="6" t="str">
+    <row r="60" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="A60" s="2" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
       </c>
@@ -3473,7 +3486,7 @@
       <c r="D60" s="2">
         <v>20260209</v>
       </c>
-      <c r="E60" s="8">
+      <c r="E60" s="4">
         <v>0.410590277777778</v>
       </c>
       <c r="F60" s="2">
@@ -3495,7 +3508,7 @@
       </c>
     </row>
     <row r="61" ht="16" customHeight="1" spans="1:13">
-      <c r="A61" s="6">
+      <c r="A61" s="2">
         <v>600584</v>
       </c>
       <c r="B61" s="2" t="s">
@@ -3504,10 +3517,10 @@
       <c r="C61" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D61" s="7">
+      <c r="D61" s="2">
         <v>20260226</v>
       </c>
-      <c r="E61" s="2">
+      <c r="E61" s="4">
         <v>0.549131944444444</v>
       </c>
       <c r="F61" s="2">
@@ -3523,18 +3536,18 @@
         <f>SUMIFS($G$2:G61,$A$2:A61,$A61)</f>
         <v>1100</v>
       </c>
-      <c r="K61" s="9" t="s">
+      <c r="K61" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="L61" s="4" t="s">
+      <c r="L61" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="M61" s="4" t="s">
+      <c r="M61" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="62" ht="84" spans="1:13">
-      <c r="A62" s="6" t="str">
+      <c r="A62" s="2" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
       </c>
@@ -3544,10 +3557,10 @@
       <c r="C62" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D62" s="7">
+      <c r="D62" s="2">
         <v>20260227</v>
       </c>
-      <c r="E62" s="8">
+      <c r="E62" s="4">
         <v>0.403645833333333</v>
       </c>
       <c r="F62" s="2">
@@ -3563,7 +3576,7 @@
         <f>SUMIFS($G$2:G62,$A$2:A62,$A62)</f>
         <v>600</v>
       </c>
-      <c r="K62" s="9" t="s">
+      <c r="K62" s="7" t="s">
         <v>37</v>
       </c>
       <c r="L62" t="s">
@@ -3574,7 +3587,7 @@
       </c>
     </row>
     <row r="63" ht="77" customHeight="1" spans="1:14">
-      <c r="A63" s="3">
+      <c r="A63" s="2">
         <v>600584</v>
       </c>
       <c r="B63" s="2" t="s">
@@ -3586,7 +3599,7 @@
       <c r="D63" s="2">
         <v>20260309</v>
       </c>
-      <c r="E63" s="8">
+      <c r="E63" s="4">
         <v>0.618055555555556</v>
       </c>
       <c r="F63" s="2">
@@ -3602,12 +3615,12 @@
         <f>SUMIFS($G$2:G63,$A$2:A63,$A63)</f>
         <v>500</v>
       </c>
-      <c r="N63" s="9" t="s">
+      <c r="N63" s="7" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="64" ht="135" spans="1:13">
-      <c r="A64" s="11" t="s">
+      <c r="A64" s="8" t="s">
         <v>42</v>
       </c>
       <c r="B64" s="2" t="s">
@@ -3619,7 +3632,7 @@
       <c r="D64" s="2">
         <v>22060312</v>
       </c>
-      <c r="E64" s="8">
+      <c r="E64" s="4">
         <v>0.618055555555556</v>
       </c>
       <c r="F64" s="2">
@@ -3635,7 +3648,7 @@
       <c r="J64" s="2">
         <v>700</v>
       </c>
-      <c r="K64" s="9" t="s">
+      <c r="K64" s="7" t="s">
         <v>43</v>
       </c>
       <c r="M64" t="s">
@@ -3643,7 +3656,7 @@
       </c>
     </row>
     <row r="65" ht="84" spans="1:14">
-      <c r="A65" s="11" t="s">
+      <c r="A65" s="8" t="s">
         <v>42</v>
       </c>
       <c r="B65" s="2" t="s">
@@ -3655,7 +3668,7 @@
       <c r="D65" s="2">
         <v>22060316</v>
       </c>
-      <c r="E65" s="8">
+      <c r="E65" s="4">
         <v>0.618055555555556</v>
       </c>
       <c r="F65" s="2">
@@ -3670,12 +3683,12 @@
       <c r="J65" s="2">
         <v>0</v>
       </c>
-      <c r="N65" s="9" t="s">
+      <c r="N65" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="66" ht="101" spans="1:14">
-      <c r="A66" s="6">
+      <c r="A66" s="2">
         <v>600584</v>
       </c>
       <c r="B66" s="2" t="s">
@@ -3687,7 +3700,7 @@
       <c r="D66" s="2">
         <v>22060316</v>
       </c>
-      <c r="E66" s="8">
+      <c r="E66" s="4">
         <v>0.618055555555556</v>
       </c>
       <c r="F66" s="2">
@@ -3703,12 +3716,12 @@
       <c r="J66" s="2">
         <v>0</v>
       </c>
-      <c r="N66" s="9" t="s">
+      <c r="N66" s="7" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="67" ht="51" spans="1:13">
-      <c r="A67" s="11" t="s">
+      <c r="A67" s="8" t="s">
         <v>42</v>
       </c>
       <c r="B67" s="2" t="s">
@@ -3720,7 +3733,7 @@
       <c r="D67" s="2">
         <v>20260318</v>
       </c>
-      <c r="E67" s="8">
+      <c r="E67" s="4">
         <v>0.618055555555556</v>
       </c>
       <c r="F67" s="2">
@@ -3736,7 +3749,7 @@
       <c r="J67" s="2">
         <v>100</v>
       </c>
-      <c r="K67" s="9" t="s">
+      <c r="K67" s="7" t="s">
         <v>47</v>
       </c>
       <c r="M67" t="s">
@@ -3744,7 +3757,7 @@
       </c>
     </row>
     <row r="68" ht="51" spans="1:13">
-      <c r="A68" s="6">
+      <c r="A68" s="2">
         <v>600487</v>
       </c>
       <c r="B68" s="2" t="s">
@@ -3756,7 +3769,7 @@
       <c r="D68" s="2">
         <v>20260318</v>
       </c>
-      <c r="E68" s="8">
+      <c r="E68" s="4">
         <v>0.618055555555556</v>
       </c>
       <c r="F68" s="2">
@@ -3771,15 +3784,15 @@
       <c r="J68" s="2">
         <v>600</v>
       </c>
-      <c r="K68" s="9" t="s">
+      <c r="K68" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="M68" s="4" t="s">
+      <c r="M68" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="69" ht="101" spans="1:11">
-      <c r="A69" s="11" t="s">
+      <c r="A69" s="8" t="s">
         <v>42</v>
       </c>
       <c r="B69" s="2" t="s">
@@ -3791,7 +3804,7 @@
       <c r="D69" s="2">
         <v>20260319</v>
       </c>
-      <c r="E69" s="8">
+      <c r="E69" s="4">
         <v>0.414583333333333</v>
       </c>
       <c r="F69" s="2">
@@ -3806,12 +3819,12 @@
       <c r="J69" s="2">
         <v>200</v>
       </c>
-      <c r="K69" s="9" t="s">
+      <c r="K69" s="7" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="70" ht="84" spans="1:11">
-      <c r="A70" s="11" t="s">
+      <c r="A70" s="8" t="s">
         <v>42</v>
       </c>
       <c r="B70" s="2" t="s">
@@ -3823,7 +3836,7 @@
       <c r="D70" s="2">
         <v>20260319</v>
       </c>
-      <c r="E70" s="8">
+      <c r="E70" s="4">
         <v>0.625</v>
       </c>
       <c r="F70" s="2">
@@ -3838,12 +3851,12 @@
       <c r="J70" s="2">
         <v>300</v>
       </c>
-      <c r="K70" s="9" t="s">
+      <c r="K70" s="7" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="71" ht="34" spans="1:11">
-      <c r="A71" s="6">
+      <c r="A71" s="2">
         <v>600487</v>
       </c>
       <c r="B71" s="2" t="s">
@@ -3852,10 +3865,10 @@
       <c r="C71" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D71" s="10">
+      <c r="D71" s="2">
         <v>20260320</v>
       </c>
-      <c r="E71" s="2">
+      <c r="E71" s="4">
         <v>0.425</v>
       </c>
       <c r="F71" s="2">
@@ -3870,12 +3883,76 @@
       <c r="J71" s="2">
         <v>1200</v>
       </c>
-      <c r="K71" s="9" t="s">
+      <c r="K71" s="7" t="s">
         <v>54</v>
       </c>
     </row>
+    <row r="72" ht="68" spans="1:11">
+      <c r="A72" s="2">
+        <v>600487</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D72" s="2">
+        <v>20260324</v>
+      </c>
+      <c r="E72" s="4">
+        <v>0.616666666666667</v>
+      </c>
+      <c r="F72" s="2">
+        <v>44</v>
+      </c>
+      <c r="G72" s="2">
+        <v>300</v>
+      </c>
+      <c r="H72" s="2">
+        <v>13200</v>
+      </c>
+      <c r="J72" s="2">
+        <v>1500</v>
+      </c>
+      <c r="K72" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="73" ht="84" spans="1:11">
+      <c r="A73" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D73" s="2">
+        <v>20260325</v>
+      </c>
+      <c r="E73" s="4">
+        <v>0.409027777777778</v>
+      </c>
+      <c r="F73" s="2">
+        <v>213.77</v>
+      </c>
+      <c r="G73" s="2">
+        <v>100</v>
+      </c>
+      <c r="H73" s="2">
+        <v>21377</v>
+      </c>
+      <c r="J73" s="2">
+        <v>400</v>
+      </c>
+      <c r="K73" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J70">
+  <autoFilter ref="A1:J71">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-03-29 23:55:39
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="13020"/>
+    <workbookView windowWidth="29100" windowHeight="14560"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$73</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="61">
   <si>
     <t>证券代码</t>
   </si>
@@ -213,6 +213,17 @@
   </si>
   <si>
     <t>这一波买入跟昨天买入亨通光电的逻辑是一致的在看到思源电气企稳逐步回到趋势后 同时又低于现在仓位均价加仓是看起来很划算的事情 ，电力走的好 一定程度上也带动了电网，但要开始逐步小心风险了</t>
+  </si>
+  <si>
+    <t xml:space="preserve">今天早盘一波放量下杀之后有效回收了涨幅留下了长下影线 作为一个安全的短期支撑位 同时有隐约上冲的势头 于是我选在在208这个位置买入做一个短t 短期这支票的最大容量为我的50%仓位 已经完全打满 奉高做t降低成本 是现在的主要任务 同时连着两日缩量  股价已经在200-210之间得到了企稳 
+</t>
+  </si>
+  <si>
+    <t>3614    （+5.4%）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.三天时间亨通光电累计涨幅达到14个点 但是前一天 在上午走出了当日最高点之后一路回落尾盘 收红 留下长下影线 我将这个信号视作滞涨 + 当晚美股对标股票康宁大跌4% 观察了每天亨通光电早上都有冲高回落迹象且都发生在10点左右 于是决定在这个附近清仓 其实一开始都是和预想到差不多 开盘股价一路下杀最后在10点左右开始反弹到开盘价附近 这个时候对我来说是清仓的好时机 因为本来这个仓位就是以短线为主 快进快出才是正解 开仓前我就思考好什么时候做中线什么时候做长线  亨通光电本来就是我想要用来做短线的一个标的 它的热度更好 辨识度更高 弹性也更好 事实证明确实如此 在反弹中我收到大量获利 。 但是如果回看上周五我其实是卖飞了 我认为自己没有做好的点 1. 太把外盘的走势当回事 虽然外盘股价确实与A股对应标的股价有部分相关关系 但不应该就当作全部 它只是参考 不能成为买卖的关键 。 2.昨天的上影线太明显了所有人都知道这是滞涨的信号 我也被这样的表象所迷惑 但或许也不是迷惑因为最近大盘轮转的很快 获利之后快速抽身也并不是错误 这个决定只能等待时间来检验
+</t>
   </si>
 </sst>
 </file>
@@ -857,7 +868,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -879,6 +890,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center"/>
@@ -1416,7 +1430,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:N75"/>
   <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="20.4"/>
   <cols>
     <col min="1" max="1" width="14.6153846153846" style="2" customWidth="1"/>
@@ -1429,7 +1443,7 @@
     <col min="10" max="10" width="14.6153846153846" style="2" customWidth="1"/>
     <col min="11" max="11" width="43.9038461538462" style="3" customWidth="1"/>
     <col min="12" max="12" width="27.6923076923077" style="3" customWidth="1"/>
-    <col min="13" max="13" width="27.0769230769231" style="3" customWidth="1"/>
+    <col min="13" max="13" width="48.9230769230769" style="3" customWidth="1"/>
     <col min="14" max="14" width="40.5384615384615" style="3" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3620,7 +3634,7 @@
       </c>
     </row>
     <row r="64" ht="135" spans="1:13">
-      <c r="A64" s="8" t="s">
+      <c r="A64" s="9" t="s">
         <v>42</v>
       </c>
       <c r="B64" s="2" t="s">
@@ -3656,7 +3670,7 @@
       </c>
     </row>
     <row r="65" ht="84" spans="1:14">
-      <c r="A65" s="8" t="s">
+      <c r="A65" s="9" t="s">
         <v>42</v>
       </c>
       <c r="B65" s="2" t="s">
@@ -3721,7 +3735,7 @@
       </c>
     </row>
     <row r="67" ht="51" spans="1:13">
-      <c r="A67" s="8" t="s">
+      <c r="A67" s="9" t="s">
         <v>42</v>
       </c>
       <c r="B67" s="2" t="s">
@@ -3792,7 +3806,7 @@
       </c>
     </row>
     <row r="69" ht="101" spans="1:11">
-      <c r="A69" s="8" t="s">
+      <c r="A69" s="9" t="s">
         <v>42</v>
       </c>
       <c r="B69" s="2" t="s">
@@ -3824,7 +3838,7 @@
       </c>
     </row>
     <row r="70" ht="84" spans="1:11">
-      <c r="A70" s="8" t="s">
+      <c r="A70" s="9" t="s">
         <v>42</v>
       </c>
       <c r="B70" s="2" t="s">
@@ -3920,7 +3934,7 @@
       </c>
     </row>
     <row r="73" ht="84" spans="1:11">
-      <c r="A73" s="8" t="s">
+      <c r="A73" s="9" t="s">
         <v>56</v>
       </c>
       <c r="B73" s="2" t="s">
@@ -3951,8 +3965,75 @@
         <v>57</v>
       </c>
     </row>
+    <row r="74" ht="135" spans="1:11">
+      <c r="A74" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D74" s="2">
+        <v>20260327</v>
+      </c>
+      <c r="E74" s="4">
+        <v>0.441666666666667</v>
+      </c>
+      <c r="F74" s="2">
+        <v>208</v>
+      </c>
+      <c r="G74" s="2">
+        <v>100</v>
+      </c>
+      <c r="H74" s="2">
+        <v>20800</v>
+      </c>
+      <c r="J74" s="2">
+        <v>500</v>
+      </c>
+      <c r="K74" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="75" ht="370" spans="1:13">
+      <c r="A75" s="8">
+        <v>600487</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D75" s="2">
+        <v>20260327</v>
+      </c>
+      <c r="E75" s="4">
+        <v>0.410416666666667</v>
+      </c>
+      <c r="F75" s="2">
+        <v>47.08</v>
+      </c>
+      <c r="G75" s="2">
+        <v>1500</v>
+      </c>
+      <c r="H75" s="2">
+        <v>70620</v>
+      </c>
+      <c r="I75" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="J75" s="2">
+        <v>0</v>
+      </c>
+      <c r="M75" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J71">
+  <autoFilter ref="A1:J73">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-03-31 20:29:11
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -10,7 +10,7 @@
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$75</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="62">
   <si>
     <t>证券代码</t>
   </si>
@@ -224,6 +224,9 @@
   <si>
     <t xml:space="preserve">1.三天时间亨通光电累计涨幅达到14个点 但是前一天 在上午走出了当日最高点之后一路回落尾盘 收红 留下长下影线 我将这个信号视作滞涨 + 当晚美股对标股票康宁大跌4% 观察了每天亨通光电早上都有冲高回落迹象且都发生在10点左右 于是决定在这个附近清仓 其实一开始都是和预想到差不多 开盘股价一路下杀最后在10点左右开始反弹到开盘价附近 这个时候对我来说是清仓的好时机 因为本来这个仓位就是以短线为主 快进快出才是正解 开仓前我就思考好什么时候做中线什么时候做长线  亨通光电本来就是我想要用来做短线的一个标的 它的热度更好 辨识度更高 弹性也更好 事实证明确实如此 在反弹中我收到大量获利 。 但是如果回看上周五我其实是卖飞了 我认为自己没有做好的点 1. 太把外盘的走势当回事 虽然外盘股价确实与A股对应标的股价有部分相关关系 但不应该就当作全部 它只是参考 不能成为买卖的关键 。 2.昨天的上影线太明显了所有人都知道这是滞涨的信号 我也被这样的表象所迷惑 但或许也不是迷惑因为最近大盘轮转的很快 获利之后快速抽身也并不是错误 这个决定只能等待时间来检验
 </t>
+  </si>
+  <si>
+    <t>200是思源电气这几日的短期低点这个地方应当有比较好的支撑，事实证明我做对了 两次探底200之后都得到了回收，但大盘抛压太重今天放量跌了2% 还在努力降低成本 有机会就高卖做t</t>
   </si>
 </sst>
 </file>
@@ -1430,7 +1433,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N75"/>
+  <dimension ref="A1:N76"/>
   <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="20.4"/>
   <cols>
     <col min="1" max="1" width="14.6153846153846" style="2" customWidth="1"/>
@@ -4032,8 +4035,40 @@
         <v>60</v>
       </c>
     </row>
+    <row r="76" ht="84" spans="1:11">
+      <c r="A76" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D76" s="2">
+        <v>20260331</v>
+      </c>
+      <c r="E76" s="4">
+        <v>0.565972222222222</v>
+      </c>
+      <c r="F76" s="2">
+        <v>200.5</v>
+      </c>
+      <c r="G76" s="2">
+        <v>100</v>
+      </c>
+      <c r="H76" s="2">
+        <v>20050</v>
+      </c>
+      <c r="J76" s="2">
+        <v>600</v>
+      </c>
+      <c r="K76" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J73">
+  <autoFilter ref="A1:J75">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-07 00:23:41
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="14560"/>
+    <workbookView windowWidth="29100" windowHeight="13060"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">交易记录!$A$1:$J$76</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -4068,7 +4068,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J75">
+  <autoFilter ref="A1:J76">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-07 10:08:28
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="13060"/>
+    <workbookView windowWidth="29100" windowHeight="13020"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -2343,8 +2343,7 @@
         <v>23856</v>
       </c>
       <c r="I26" s="2">
-        <f>IF(AND($C26="卖出",SUMIFS($G$2:G26,$A$2:A26,$A26)=0),SUMIFS($H$2:H26,$A$2:A26,$A26,$C$2:C26,"卖出")-SUMIFS($H$2:H26,$A$2:A26,$A26,$C$2:C26,"买入"),"")</f>
-        <v>23856</v>
+        <v>-700</v>
       </c>
       <c r="J26" s="2">
         <f>SUMIFS($G$2:G26,$A$2:A26,$A26)</f>

</xml_diff>

<commit_message>
vault backup: 2026-04-08 23:00:30
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10328"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDA1F588-494C-B548-85AA-63976641DF7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="13020"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -30,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="74">
   <si>
     <t>证券代码</t>
   </si>
@@ -227,19 +233,62 @@
   </si>
   <si>
     <t>200是思源电气这几日的短期低点这个地方应当有比较好的支撑，事实证明我做对了 两次探底200之后都得到了回收，但大盘抛压太重今天放量跌了2% 还在努力降低成本 有机会就高卖做t</t>
+  </si>
+  <si>
+    <t>思源电气</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>卖出</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>卖出逻辑</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>思源电气在昨天回踩了60日均线且伴随放量但是我并未有发现有什么利空消息在影响股价，一时间难以判断这到底是洗盘还是出货，今天A股全线暴涨思源电气只能说是表现平平，全天仍然缩量为防止踏空+降低风险今天确实应该减仓，这是我从上一次卖飞亨通光电收获的教训，不应该太赌气的清仓留一点悬念和可能性给自己，不要太多的确定性</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>002028</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>000988</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>华工科技</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>买入</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>长远来看华工科技在三月份连跌之后在短期已经出现明显的底部100作为一个短期支撑，同时今天放量收出阳线有反攻事态，总之这个位置是一个盈亏比例较好的位置，前面有前高141，下方有支撑位100，先小仓试错而后加仓。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>002281</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>光迅科技</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>光迅科技在最近的cpo板块里面是更加强势的股票
+鉴于之前在做亨通光电和长飞光纤的时候我选择了更加处于回调上升的亨通光电而错过了长飞的大涨，这让我觉得更应该选择强势的股票 不是看涨的多了就害怕，所以这里也加了2w仓位 决定在华工科技之间优中选优 去弱留强</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="23">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -251,6 +300,7 @@
       <sz val="16"/>
       <color rgb="FFFF0000"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -259,6 +309,7 @@
       <sz val="14"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -267,155 +318,27 @@
       <sz val="14"/>
       <color rgb="FFFF0000"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -428,194 +351,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -623,272 +360,30 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
+  </cellStyleXfs>
+  <cellXfs count="14">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-  </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="21" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="21" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -897,93 +392,172 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <border>
@@ -994,7 +568,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="0"/>
       </font>
       <fill>
@@ -1022,154 +596,40 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39994506668294322"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
+      <tableStyleElement type="pageFieldValues" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1427,30 +887,31 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:N76"/>
-  <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="20.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O79"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="17"/>
   <cols>
-    <col min="1" max="1" width="14.6153846153846" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.6153846153846" style="3" customWidth="1"/>
-    <col min="3" max="3" width="35.4615384615385" style="2" customWidth="1"/>
-    <col min="4" max="4" width="28.6538461538462" style="2" customWidth="1"/>
-    <col min="5" max="5" width="14.6153846153846" style="4" customWidth="1"/>
-    <col min="6" max="8" width="14.6153846153846" style="2" customWidth="1"/>
-    <col min="9" max="9" width="14.6153846153846" style="3" customWidth="1"/>
-    <col min="10" max="10" width="14.6153846153846" style="2" customWidth="1"/>
-    <col min="11" max="11" width="43.9038461538462" style="3" customWidth="1"/>
-    <col min="12" max="12" width="27.6923076923077" style="3" customWidth="1"/>
-    <col min="13" max="13" width="48.9230769230769" style="3" customWidth="1"/>
-    <col min="14" max="14" width="40.5384615384615" style="3" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="35.5" style="2" customWidth="1"/>
+    <col min="4" max="4" width="28.6640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" style="4" customWidth="1"/>
+    <col min="6" max="8" width="14.6640625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="43.83203125" style="3" customWidth="1"/>
+    <col min="12" max="12" width="27.6640625" style="3" customWidth="1"/>
+    <col min="13" max="13" width="49" style="3" customWidth="1"/>
+    <col min="14" max="14" width="40.5" style="3" customWidth="1"/>
+    <col min="15" max="15" width="32.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="23.2" customHeight="1" spans="1:14">
+    <row r="1" spans="1:15" s="1" customFormat="1" ht="23.25" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1493,8 +954,11 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" s="2" customFormat="1" customHeight="1" spans="1:10">
+      <c r="O1" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A2" s="2">
         <v>600276</v>
       </c>
@@ -1508,10 +972,10 @@
         <v>20250902</v>
       </c>
       <c r="E2" s="4">
-        <v>0.395983796296296</v>
+        <v>0.39598379629629599</v>
       </c>
       <c r="F2" s="2">
-        <v>69.43</v>
+        <v>69.430000000000007</v>
       </c>
       <c r="G2" s="2">
         <v>200</v>
@@ -1528,7 +992,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="3" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="3" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A3" s="2">
         <v>600276</v>
       </c>
@@ -1542,7 +1006,7 @@
         <v>20250903</v>
       </c>
       <c r="E3" s="4">
-        <v>0.400289351851852</v>
+        <v>0.40028935185185199</v>
       </c>
       <c r="F3" s="2">
         <v>69.09</v>
@@ -1562,7 +1026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="4" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A4" s="2">
         <v>601138</v>
       </c>
@@ -1576,7 +1040,7 @@
         <v>20250912</v>
       </c>
       <c r="E4" s="4">
-        <v>0.407638888888889</v>
+        <v>0.40763888888888899</v>
       </c>
       <c r="F4" s="2">
         <v>61</v>
@@ -1596,7 +1060,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" s="2" customFormat="1" ht="20" customHeight="1" spans="1:10">
+    <row r="5" spans="1:15" s="2" customFormat="1" ht="20" customHeight="1">
       <c r="A5" s="2">
         <v>601138</v>
       </c>
@@ -1610,7 +1074,7 @@
         <v>20250915</v>
       </c>
       <c r="E5" s="4">
-        <v>0.591782407407407</v>
+        <v>0.59178240740740695</v>
       </c>
       <c r="F5" s="2">
         <v>59.5</v>
@@ -1630,7 +1094,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="6" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="6" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A6" s="2">
         <v>601138</v>
       </c>
@@ -1664,7 +1128,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="7" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="7" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A7" s="2">
         <v>603986</v>
       </c>
@@ -1678,7 +1142,7 @@
         <v>20250925</v>
       </c>
       <c r="E7" s="4">
-        <v>0.609340277777778</v>
+        <v>0.60934027777777799</v>
       </c>
       <c r="F7" s="2">
         <v>198</v>
@@ -1698,7 +1162,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="8" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A8" s="2">
         <v>601138</v>
       </c>
@@ -1732,7 +1196,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="9" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="9" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A9" s="2">
         <v>600111</v>
       </c>
@@ -1746,7 +1210,7 @@
         <v>20251010</v>
       </c>
       <c r="E9" s="4">
-        <v>0.417337962962963</v>
+        <v>0.41733796296296299</v>
       </c>
       <c r="F9" s="2">
         <v>53.5</v>
@@ -1766,7 +1230,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="10" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="10" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A10" s="2">
         <v>600111</v>
       </c>
@@ -1780,7 +1244,7 @@
         <v>20251010</v>
       </c>
       <c r="E10" s="4">
-        <v>0.396574074074074</v>
+        <v>0.39657407407407402</v>
       </c>
       <c r="F10" s="2">
         <v>53.98</v>
@@ -1800,7 +1264,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="11" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="11" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A11" s="2">
         <v>601138</v>
       </c>
@@ -1814,7 +1278,7 @@
         <v>20251015</v>
       </c>
       <c r="E11" s="4">
-        <v>0.453912037037037</v>
+        <v>0.45391203703703698</v>
       </c>
       <c r="F11" s="2">
         <v>60.75</v>
@@ -1834,7 +1298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="12" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A12" s="2">
         <v>603986</v>
       </c>
@@ -1848,7 +1312,7 @@
         <v>20251015</v>
       </c>
       <c r="E12" s="4">
-        <v>0.453784722222222</v>
+        <v>0.45378472222222199</v>
       </c>
       <c r="F12" s="2">
         <v>193.75</v>
@@ -1868,7 +1332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="13" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A13" s="2">
         <v>600111</v>
       </c>
@@ -1882,7 +1346,7 @@
         <v>20251015</v>
       </c>
       <c r="E13" s="4">
-        <v>0.422696759259259</v>
+        <v>0.42269675925925898</v>
       </c>
       <c r="F13" s="2">
         <v>54.82</v>
@@ -1902,7 +1366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="14" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A14" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -1917,7 +1381,7 @@
         <v>20251016</v>
       </c>
       <c r="E14" s="4">
-        <v>0.560474537037037</v>
+        <v>0.56047453703703698</v>
       </c>
       <c r="F14" s="2">
         <v>59.5</v>
@@ -1937,7 +1401,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="15" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="15" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A15" s="2">
         <v>603259</v>
       </c>
@@ -1951,7 +1415,7 @@
         <v>20251016</v>
       </c>
       <c r="E15" s="4">
-        <v>0.458530092592593</v>
+        <v>0.45853009259259297</v>
       </c>
       <c r="F15" s="2">
         <v>101.12</v>
@@ -1971,7 +1435,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="16" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A16" s="2" t="str">
         <f>"002371"</f>
         <v>002371</v>
@@ -2006,7 +1470,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="17" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A17" s="2" t="str">
         <f>"002281"</f>
         <v>002281</v>
@@ -2021,7 +1485,7 @@
         <v>20251021</v>
       </c>
       <c r="E17" s="4">
-        <v>0.621550925925926</v>
+        <v>0.62155092592592598</v>
       </c>
       <c r="F17" s="2">
         <v>61.37</v>
@@ -2041,7 +1505,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="18" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="18" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A18" s="2">
         <v>603259</v>
       </c>
@@ -2055,7 +1519,7 @@
         <v>20251021</v>
       </c>
       <c r="E18" s="4">
-        <v>0.46806712962963</v>
+        <v>0.46806712962962999</v>
       </c>
       <c r="F18" s="2">
         <v>101.48</v>
@@ -2075,7 +1539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="19" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A19" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -2090,7 +1554,7 @@
         <v>20251021</v>
       </c>
       <c r="E19" s="4">
-        <v>0.418518518518519</v>
+        <v>0.41851851851851901</v>
       </c>
       <c r="F19" s="2">
         <v>60.07</v>
@@ -2110,7 +1574,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="20" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="20" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A20" s="2">
         <v>603986</v>
       </c>
@@ -2124,7 +1588,7 @@
         <v>20251023</v>
       </c>
       <c r="E20" s="4">
-        <v>0.617777777777778</v>
+        <v>0.61777777777777798</v>
       </c>
       <c r="F20" s="2">
         <v>208.04</v>
@@ -2144,7 +1608,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="21" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="21" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A21" s="2" t="str">
         <f>"002371"</f>
         <v>002371</v>
@@ -2159,7 +1623,7 @@
         <v>20251023</v>
       </c>
       <c r="E21" s="4">
-        <v>0.616111111111111</v>
+        <v>0.61611111111111105</v>
       </c>
       <c r="F21" s="2">
         <v>402.9</v>
@@ -2179,7 +1643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="22" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A22" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -2194,7 +1658,7 @@
         <v>20251024</v>
       </c>
       <c r="E22" s="4">
-        <v>0.601006944444444</v>
+        <v>0.60100694444444402</v>
       </c>
       <c r="F22" s="2">
         <v>63.72</v>
@@ -2214,7 +1678,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="23" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="23" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A23" s="2">
         <v>603986</v>
       </c>
@@ -2228,7 +1692,7 @@
         <v>20251024</v>
       </c>
       <c r="E23" s="4">
-        <v>0.589212962962963</v>
+        <v>0.58921296296296299</v>
       </c>
       <c r="F23" s="2">
         <v>220</v>
@@ -2248,7 +1712,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="24" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A24" s="2" t="str">
         <f>"002281"</f>
         <v>002281</v>
@@ -2263,7 +1727,7 @@
         <v>20251024</v>
       </c>
       <c r="E24" s="4">
-        <v>0.418425925925926</v>
+        <v>0.41842592592592598</v>
       </c>
       <c r="F24" s="2">
         <v>61.31</v>
@@ -2283,7 +1747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="25" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A25" s="2">
         <v>603083</v>
       </c>
@@ -2297,7 +1761,7 @@
         <v>20251027</v>
       </c>
       <c r="E25" s="4">
-        <v>0.399074074074074</v>
+        <v>0.39907407407407403</v>
       </c>
       <c r="F25" s="2">
         <v>122.95</v>
@@ -2317,7 +1781,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="26" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="26" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A26" s="2">
         <v>603083</v>
       </c>
@@ -2350,7 +1814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="27" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A27" s="2">
         <v>603986</v>
       </c>
@@ -2364,7 +1828,7 @@
         <v>20251029</v>
       </c>
       <c r="E27" s="4">
-        <v>0.441550925925926</v>
+        <v>0.44155092592592599</v>
       </c>
       <c r="F27" s="2">
         <v>236.41</v>
@@ -2384,7 +1848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="28" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A28" s="2">
         <v>603799</v>
       </c>
@@ -2398,10 +1862,10 @@
         <v>20251030</v>
       </c>
       <c r="E28" s="4">
-        <v>0.565590277777778</v>
+        <v>0.56559027777777804</v>
       </c>
       <c r="F28" s="2">
-        <v>66.1</v>
+        <v>66.099999999999994</v>
       </c>
       <c r="G28" s="2">
         <v>300</v>
@@ -2418,7 +1882,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="29" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="29" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A29" s="2">
         <v>603986</v>
       </c>
@@ -2452,7 +1916,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="30" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="30" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A30" s="2">
         <v>603099</v>
       </c>
@@ -2486,7 +1950,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="31" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="31" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A31" s="2">
         <v>603099</v>
       </c>
@@ -2520,7 +1984,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="32" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="32" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A32" s="2">
         <v>603799</v>
       </c>
@@ -2554,7 +2018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="33" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A33" s="2">
         <v>603099</v>
       </c>
@@ -2568,7 +2032,7 @@
         <v>20251105</v>
       </c>
       <c r="E33" s="4">
-        <v>0.413472222222222</v>
+        <v>0.41347222222222202</v>
       </c>
       <c r="F33" s="2">
         <v>56.04</v>
@@ -2588,7 +2052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="34" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A34" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
@@ -2603,7 +2067,7 @@
         <v>20260119</v>
       </c>
       <c r="E34" s="4">
-        <v>0.422534722222222</v>
+        <v>0.42253472222222199</v>
       </c>
       <c r="F34" s="2">
         <v>199</v>
@@ -2623,7 +2087,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="35" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A35" s="2">
         <v>601179</v>
       </c>
@@ -2637,7 +2101,7 @@
         <v>20260119</v>
       </c>
       <c r="E35" s="4">
-        <v>0.400891203703704</v>
+        <v>0.40089120370370401</v>
       </c>
       <c r="F35" s="2">
         <v>14.19</v>
@@ -2657,7 +2121,7 @@
         <v>1400</v>
       </c>
     </row>
-    <row r="36" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="36" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A36" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
@@ -2672,7 +2136,7 @@
         <v>20260119</v>
       </c>
       <c r="E36" s="4">
-        <v>0.398483796296296</v>
+        <v>0.39848379629629599</v>
       </c>
       <c r="F36" s="2">
         <v>194</v>
@@ -2692,7 +2156,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="37" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="37" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A37" s="2">
         <v>603986</v>
       </c>
@@ -2706,10 +2170,10 @@
         <v>20260119</v>
       </c>
       <c r="E37" s="4">
-        <v>0.396030092592593</v>
+        <v>0.39603009259259297</v>
       </c>
       <c r="F37" s="2">
-        <v>280.6</v>
+        <v>280.60000000000002</v>
       </c>
       <c r="G37" s="2">
         <v>-100</v>
@@ -2726,7 +2190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="38" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A38" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
@@ -2741,7 +2205,7 @@
         <v>20260121</v>
       </c>
       <c r="E38" s="4">
-        <v>0.397384259259259</v>
+        <v>0.39738425925925902</v>
       </c>
       <c r="F38" s="2">
         <v>189</v>
@@ -2761,7 +2225,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="39" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="39" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A39" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
@@ -2776,7 +2240,7 @@
         <v>20260122</v>
       </c>
       <c r="E39" s="4">
-        <v>0.444861111111111</v>
+        <v>0.44486111111111099</v>
       </c>
       <c r="F39" s="2">
         <v>189</v>
@@ -2796,7 +2260,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="40" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="40" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A40" s="2">
         <v>600584</v>
       </c>
@@ -2810,7 +2274,7 @@
         <v>20260122</v>
       </c>
       <c r="E40" s="4">
-        <v>0.407951388888889</v>
+        <v>0.40795138888888899</v>
       </c>
       <c r="F40" s="2">
         <v>50</v>
@@ -2830,7 +2294,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="41" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="41" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A41" s="2">
         <v>601179</v>
       </c>
@@ -2844,7 +2308,7 @@
         <v>20260126</v>
       </c>
       <c r="E41" s="4">
-        <v>0.622175925925926</v>
+        <v>0.62217592592592597</v>
       </c>
       <c r="F41" s="2">
         <v>16.16</v>
@@ -2864,7 +2328,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="42" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="42" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A42" s="2">
         <v>600584</v>
       </c>
@@ -2898,7 +2362,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="43" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="43" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A43" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -2913,7 +2377,7 @@
         <v>20260127</v>
       </c>
       <c r="E43" s="4">
-        <v>0.413969907407407</v>
+        <v>0.41396990740740702</v>
       </c>
       <c r="F43" s="2">
         <v>53.2</v>
@@ -2933,7 +2397,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="44" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="44" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A44" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
@@ -2948,7 +2412,7 @@
         <v>20260129</v>
       </c>
       <c r="E44" s="4">
-        <v>0.5778125</v>
+        <v>0.57781249999999995</v>
       </c>
       <c r="F44" s="2">
         <v>186.2</v>
@@ -2968,7 +2432,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="45" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="45" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A45" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -2983,7 +2447,7 @@
         <v>20260129</v>
       </c>
       <c r="E45" s="4">
-        <v>0.571990740740741</v>
+        <v>0.57199074074074097</v>
       </c>
       <c r="F45" s="2">
         <v>52.2</v>
@@ -3003,7 +2467,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="46" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="46" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A46" s="2">
         <v>600584</v>
       </c>
@@ -3017,7 +2481,7 @@
         <v>20260129</v>
       </c>
       <c r="E46" s="4">
-        <v>0.57099537037037</v>
+        <v>0.57099537037036996</v>
       </c>
       <c r="F46" s="2">
         <v>49.2</v>
@@ -3037,7 +2501,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="47" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="47" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A47" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -3052,7 +2516,7 @@
         <v>20260129</v>
       </c>
       <c r="E47" s="4">
-        <v>0.545462962962963</v>
+        <v>0.54546296296296304</v>
       </c>
       <c r="F47" s="2">
         <v>51.9</v>
@@ -3072,7 +2536,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="48" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="48" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A48" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
@@ -3087,7 +2551,7 @@
         <v>20260129</v>
       </c>
       <c r="E48" s="4">
-        <v>0.542395833333333</v>
+        <v>0.54239583333333297</v>
       </c>
       <c r="F48" s="2">
         <v>188</v>
@@ -3107,7 +2571,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="49" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="49" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A49" s="2">
         <v>601179</v>
       </c>
@@ -3121,7 +2585,7 @@
         <v>20260130</v>
       </c>
       <c r="E49" s="4">
-        <v>0.440439814814815</v>
+        <v>0.44043981481481498</v>
       </c>
       <c r="F49" s="2">
         <v>14</v>
@@ -3141,7 +2605,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="50" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="50" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A50" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
@@ -3156,7 +2620,7 @@
         <v>20260130</v>
       </c>
       <c r="E50" s="4">
-        <v>0.431030092592593</v>
+        <v>0.43103009259259301</v>
       </c>
       <c r="F50" s="2">
         <v>180</v>
@@ -3176,7 +2640,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="51" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="51" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A51" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -3191,7 +2655,7 @@
         <v>20260202</v>
       </c>
       <c r="E51" s="4">
-        <v>0.618993055555556</v>
+        <v>0.61899305555555595</v>
       </c>
       <c r="F51" s="2">
         <v>52.08</v>
@@ -3211,7 +2675,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="52" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="52" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A52" s="2">
         <v>600584</v>
       </c>
@@ -3225,7 +2689,7 @@
         <v>20260202</v>
       </c>
       <c r="E52" s="4">
-        <v>0.565694444444444</v>
+        <v>0.56569444444444394</v>
       </c>
       <c r="F52" s="2">
         <v>46.8</v>
@@ -3245,7 +2709,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="53" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="53" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A53" s="2">
         <v>601179</v>
       </c>
@@ -3259,7 +2723,7 @@
         <v>20260202</v>
       </c>
       <c r="E53" s="4">
-        <v>0.55994212962963</v>
+        <v>0.55994212962962997</v>
       </c>
       <c r="F53" s="2">
         <v>15.7</v>
@@ -3279,7 +2743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="54" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A54" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
@@ -3294,7 +2758,7 @@
         <v>20260202</v>
       </c>
       <c r="E54" s="4">
-        <v>0.446747685185185</v>
+        <v>0.44674768518518498</v>
       </c>
       <c r="F54" s="2">
         <v>191</v>
@@ -3314,7 +2778,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="55" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="55" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A55" s="2" t="str">
         <f>"002475"</f>
         <v>002475</v>
@@ -3329,7 +2793,7 @@
         <v>20260202</v>
       </c>
       <c r="E55" s="4">
-        <v>0.440671296296296</v>
+        <v>0.44067129629629598</v>
       </c>
       <c r="F55" s="2">
         <v>53.09</v>
@@ -3349,7 +2813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="56" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A56" s="2" t="str">
         <f>"002028"</f>
         <v>002028</v>
@@ -3364,7 +2828,7 @@
         <v>20260203</v>
       </c>
       <c r="E56" s="4">
-        <v>0.409178240740741</v>
+        <v>0.40917824074074099</v>
       </c>
       <c r="F56" s="2">
         <v>194</v>
@@ -3384,7 +2848,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="57" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="57" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A57" s="2" t="str">
         <f t="shared" ref="A57:A62" si="0">"002028"</f>
         <v>002028</v>
@@ -3419,7 +2883,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="58" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="58" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A58" s="2" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
@@ -3434,7 +2898,7 @@
         <v>20260209</v>
       </c>
       <c r="E58" s="4">
-        <v>0.445486111111111</v>
+        <v>0.44548611111111103</v>
       </c>
       <c r="F58" s="2">
         <v>198.73</v>
@@ -3454,7 +2918,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="59" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="59" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A59" s="2">
         <v>600584</v>
       </c>
@@ -3468,7 +2932,7 @@
         <v>20260209</v>
       </c>
       <c r="E59" s="4">
-        <v>0.438865740740741</v>
+        <v>0.43886574074074097</v>
       </c>
       <c r="F59" s="2">
         <v>46.09</v>
@@ -3488,7 +2952,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="60" s="2" customFormat="1" customHeight="1" spans="1:10">
+    <row r="60" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
       <c r="A60" s="2" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
@@ -3503,7 +2967,7 @@
         <v>20260209</v>
       </c>
       <c r="E60" s="4">
-        <v>0.410590277777778</v>
+        <v>0.41059027777777801</v>
       </c>
       <c r="F60" s="2">
         <v>192.5</v>
@@ -3523,7 +2987,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="61" ht="16" customHeight="1" spans="1:13">
+    <row r="61" spans="1:14" ht="16" customHeight="1">
       <c r="A61" s="2">
         <v>600584</v>
       </c>
@@ -3537,7 +3001,7 @@
         <v>20260226</v>
       </c>
       <c r="E61" s="4">
-        <v>0.549131944444444</v>
+        <v>0.54913194444444402</v>
       </c>
       <c r="F61" s="2">
         <v>48.3</v>
@@ -3562,7 +3026,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="62" ht="84" spans="1:13">
+    <row r="62" spans="1:14" ht="60">
       <c r="A62" s="2" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
@@ -3577,7 +3041,7 @@
         <v>20260227</v>
       </c>
       <c r="E62" s="4">
-        <v>0.403645833333333</v>
+        <v>0.40364583333333298</v>
       </c>
       <c r="F62" s="2">
         <v>218.5</v>
@@ -3602,7 +3066,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="63" ht="77" customHeight="1" spans="1:14">
+    <row r="63" spans="1:14" ht="77" customHeight="1">
       <c r="A63" s="2">
         <v>600584</v>
       </c>
@@ -3616,7 +3080,7 @@
         <v>20260309</v>
       </c>
       <c r="E63" s="4">
-        <v>0.618055555555556</v>
+        <v>0.61805555555555602</v>
       </c>
       <c r="F63" s="2">
         <v>45.03</v>
@@ -3635,7 +3099,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="64" ht="135" spans="1:13">
+    <row r="64" spans="1:14" ht="105">
       <c r="A64" s="9" t="s">
         <v>42</v>
       </c>
@@ -3649,7 +3113,7 @@
         <v>22060312</v>
       </c>
       <c r="E64" s="4">
-        <v>0.618055555555556</v>
+        <v>0.61805555555555602</v>
       </c>
       <c r="F64" s="2">
         <v>220</v>
@@ -3671,7 +3135,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="65" ht="84" spans="1:14">
+    <row r="65" spans="1:15" ht="45">
       <c r="A65" s="9" t="s">
         <v>42</v>
       </c>
@@ -3685,7 +3149,7 @@
         <v>22060316</v>
       </c>
       <c r="E65" s="4">
-        <v>0.618055555555556</v>
+        <v>0.61805555555555602</v>
       </c>
       <c r="F65" s="2">
         <v>208.14</v>
@@ -3703,7 +3167,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="66" ht="101" spans="1:14">
+    <row r="66" spans="1:15" ht="45">
       <c r="A66" s="2">
         <v>600584</v>
       </c>
@@ -3717,7 +3181,7 @@
         <v>22060316</v>
       </c>
       <c r="E66" s="4">
-        <v>0.618055555555556</v>
+        <v>0.61805555555555602</v>
       </c>
       <c r="F66" s="2">
         <v>45.7</v>
@@ -3736,7 +3200,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="67" ht="51" spans="1:13">
+    <row r="67" spans="1:15" ht="45">
       <c r="A67" s="9" t="s">
         <v>42</v>
       </c>
@@ -3750,10 +3214,10 @@
         <v>20260318</v>
       </c>
       <c r="E67" s="4">
-        <v>0.618055555555556</v>
+        <v>0.61805555555555602</v>
       </c>
       <c r="F67" s="2">
-        <v>220.183</v>
+        <v>220.18299999999999</v>
       </c>
       <c r="G67" s="2">
         <v>100</v>
@@ -3772,7 +3236,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="68" ht="51" spans="1:13">
+    <row r="68" spans="1:15" ht="45">
       <c r="A68" s="2">
         <v>600487</v>
       </c>
@@ -3786,7 +3250,7 @@
         <v>20260318</v>
       </c>
       <c r="E68" s="4">
-        <v>0.618055555555556</v>
+        <v>0.61805555555555602</v>
       </c>
       <c r="F68" s="2">
         <v>44.53</v>
@@ -3807,7 +3271,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="69" ht="101" spans="1:11">
+    <row r="69" spans="1:15" ht="75">
       <c r="A69" s="9" t="s">
         <v>42</v>
       </c>
@@ -3821,7 +3285,7 @@
         <v>20260319</v>
       </c>
       <c r="E69" s="4">
-        <v>0.414583333333333</v>
+        <v>0.41458333333333303</v>
       </c>
       <c r="F69" s="2">
         <v>214.5</v>
@@ -3839,7 +3303,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="70" ht="84" spans="1:11">
+    <row r="70" spans="1:15" ht="75">
       <c r="A70" s="9" t="s">
         <v>42</v>
       </c>
@@ -3871,7 +3335,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="71" ht="34" spans="1:11">
+    <row r="71" spans="1:15" ht="30">
       <c r="A71" s="2">
         <v>600487</v>
       </c>
@@ -3885,7 +3349,7 @@
         <v>20260320</v>
       </c>
       <c r="E71" s="4">
-        <v>0.425</v>
+        <v>0.42499999999999999</v>
       </c>
       <c r="F71" s="2">
         <v>45.07</v>
@@ -3903,7 +3367,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="72" ht="68" spans="1:11">
+    <row r="72" spans="1:15" ht="45">
       <c r="A72" s="2">
         <v>600487</v>
       </c>
@@ -3917,7 +3381,7 @@
         <v>20260324</v>
       </c>
       <c r="E72" s="4">
-        <v>0.616666666666667</v>
+        <v>0.61666666666666703</v>
       </c>
       <c r="F72" s="2">
         <v>44</v>
@@ -3935,7 +3399,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="73" ht="84" spans="1:11">
+    <row r="73" spans="1:15" ht="60">
       <c r="A73" s="9" t="s">
         <v>56</v>
       </c>
@@ -3949,7 +3413,7 @@
         <v>20260325</v>
       </c>
       <c r="E73" s="4">
-        <v>0.409027777777778</v>
+        <v>0.40902777777777799</v>
       </c>
       <c r="F73" s="2">
         <v>213.77</v>
@@ -3967,7 +3431,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="74" ht="135" spans="1:11">
+    <row r="74" spans="1:15" ht="105">
       <c r="A74" s="9" t="s">
         <v>42</v>
       </c>
@@ -3981,7 +3445,7 @@
         <v>20260327</v>
       </c>
       <c r="E74" s="4">
-        <v>0.441666666666667</v>
+        <v>0.44166666666666698</v>
       </c>
       <c r="F74" s="2">
         <v>208</v>
@@ -3999,7 +3463,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="75" ht="370" spans="1:13">
+    <row r="75" spans="1:15" ht="285">
       <c r="A75" s="8">
         <v>600487</v>
       </c>
@@ -4013,7 +3477,7 @@
         <v>20260327</v>
       </c>
       <c r="E75" s="4">
-        <v>0.410416666666667</v>
+        <v>0.41041666666666698</v>
       </c>
       <c r="F75" s="2">
         <v>47.08</v>
@@ -4034,11 +3498,11 @@
         <v>60</v>
       </c>
     </row>
-    <row r="76" ht="84" spans="1:11">
+    <row r="76" spans="1:15" ht="60">
       <c r="A76" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B76" s="3" t="s">
+      <c r="B76" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C76" s="2" t="s">
@@ -4048,7 +3512,7 @@
         <v>20260331</v>
       </c>
       <c r="E76" s="4">
-        <v>0.565972222222222</v>
+        <v>0.56597222222222199</v>
       </c>
       <c r="F76" s="2">
         <v>200.5</v>
@@ -4065,12 +3529,108 @@
       <c r="K76" s="7" t="s">
         <v>61</v>
       </c>
+      <c r="O76" s="12"/>
+    </row>
+    <row r="77" spans="1:15" ht="135">
+      <c r="A77" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B77" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D77" s="2">
+        <v>20260408</v>
+      </c>
+      <c r="E77" s="4">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="F77" s="2">
+        <v>205.85</v>
+      </c>
+      <c r="G77" s="2">
+        <v>300</v>
+      </c>
+      <c r="H77" s="2">
+        <v>61755</v>
+      </c>
+      <c r="J77" s="2">
+        <v>300</v>
+      </c>
+      <c r="N77" s="10"/>
+      <c r="O77" s="12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15" ht="75">
+      <c r="A78" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B78" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D78" s="2">
+        <v>20260408</v>
+      </c>
+      <c r="E78" s="4">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="F78" s="2">
+        <v>110.15</v>
+      </c>
+      <c r="G78" s="2">
+        <v>200</v>
+      </c>
+      <c r="H78" s="2">
+        <v>22030</v>
+      </c>
+      <c r="J78" s="2">
+        <v>200</v>
+      </c>
+      <c r="K78" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="79" spans="1:15" ht="90">
+      <c r="A79" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B79" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D79" s="2">
+        <v>20260408</v>
+      </c>
+      <c r="E79" s="4">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="F79" s="2">
+        <v>98.26</v>
+      </c>
+      <c r="G79" s="2">
+        <v>200</v>
+      </c>
+      <c r="H79" s="2">
+        <v>19652</v>
+      </c>
+      <c r="J79" s="2">
+        <v>200</v>
+      </c>
+      <c r="K79" s="13" t="s">
+        <v>73</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J76">
-    <extLst/>
-  </autoFilter>
+  <autoFilter ref="A1:J76" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-04-12 22:21:07
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDA1F588-494C-B548-85AA-63976641DF7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28D497D5-E0EE-A04F-83DE-4B647EAE97A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="77">
   <si>
     <t>证券代码</t>
   </si>
@@ -236,52 +236,65 @@
   </si>
   <si>
     <t>思源电气</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>卖出</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>卖出逻辑</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>思源电气在昨天回踩了60日均线且伴随放量但是我并未有发现有什么利空消息在影响股价，一时间难以判断这到底是洗盘还是出货，今天A股全线暴涨思源电气只能说是表现平平，全天仍然缩量为防止踏空+降低风险今天确实应该减仓，这是我从上一次卖飞亨通光电收获的教训，不应该太赌气的清仓留一点悬念和可能性给自己，不要太多的确定性</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>002028</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>000988</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>华工科技</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>买入</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>长远来看华工科技在三月份连跌之后在短期已经出现明显的底部100作为一个短期支撑，同时今天放量收出阳线有反攻事态，总之这个位置是一个盈亏比例较好的位置，前面有前高141，下方有支撑位100，先小仓试错而后加仓。</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>002281</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>光迅科技</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>光迅科技在最近的cpo板块里面是更加强势的股票
 鉴于之前在做亨通光电和长飞光纤的时候我选择了更加处于回调上升的亨通光电而错过了长飞的大涨，这让我觉得更应该选择强势的股票 不是看涨的多了就害怕，所以这里也加了2w仓位 决定在华工科技之间优中选优 去弱留强</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>今天看到光迅科技在早盘冲高，这时候有一个自我的警示就是等待情绪回落开盘从9:30-10:00这段时间是fomo的时间我认为这里存在着大量的交易噪音，一时间可能会被追涨的人群影响，10点之后继续观察 光迅科技价格仍旧坚挺且还有继续上冲的意图 这里可以大概判断出今天的上涨不是单纯的早盘fomo + 最近利空被消化+ 近期在cpo板块里的强势地位（逆势上涨）-&gt; 果断加仓</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">先买入的是光迅科技这里买入华工科技主要有以下考虑：1.作为同板块的个股 光迅科技的可见强势会在一定程度上带动华工科技 2.华工科技从形态上看比光迅科技更加让人安心 因为在3月份的大跌中 它已经铸成了一个显而易见的100作为低点 同时还站稳了5日线 高点明显+低点明显 盈亏比例在这里差不多有2:1 先把目标价格放在130左右 止损放在100元
+</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>思源电气最近的表现疲软虽然今天是4000家个股下跌，但相对于板块来说这几天的表现远远低于整体板块，伴随着缩量可以解读成买盘萎缩，卖盘也不强劲，预计会在这个箱体内横盘一段时间或者沿着60日支撑震荡，但短期出现行情的概率太低了，之前认为可能是洗盘，但现在来看更像是出货，为了规避风险同时尽可能博一点反弹预期 留了1层底仓 若持续低迷跌破60日均线 可以清仓</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -297,45 +310,41 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
+      <sz val="9"/>
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
+      <sz val="18"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="楷体"/>
       <family val="3"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
+      <color theme="1"/>
+      <name val="楷体"/>
       <family val="3"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="楷体"/>
       <family val="3"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="宋体"/>
+      <b/>
+      <sz val="24"/>
+      <color rgb="FFFF0000"/>
+      <name val="楷体"/>
       <family val="3"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -370,40 +379,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="21" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="21" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="21" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -893,2744 +902,3233 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O79"/>
+  <dimension ref="A1:O82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="17"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="35.5" style="2" customWidth="1"/>
-    <col min="4" max="4" width="28.6640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" style="4" customWidth="1"/>
-    <col min="6" max="8" width="14.6640625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="14.6640625" style="3" customWidth="1"/>
-    <col min="10" max="10" width="14.6640625" style="2" customWidth="1"/>
-    <col min="11" max="11" width="43.83203125" style="3" customWidth="1"/>
-    <col min="12" max="12" width="27.6640625" style="3" customWidth="1"/>
-    <col min="13" max="13" width="49" style="3" customWidth="1"/>
-    <col min="14" max="14" width="40.5" style="3" customWidth="1"/>
-    <col min="15" max="15" width="32.6640625" customWidth="1"/>
+    <col min="1" max="1" width="22.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.1640625" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="22.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.5" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="43.83203125" style="10" customWidth="1"/>
+    <col min="12" max="12" width="27.6640625" style="10" customWidth="1"/>
+    <col min="13" max="13" width="49" style="10" customWidth="1"/>
+    <col min="14" max="14" width="40.5" style="10" customWidth="1"/>
+    <col min="15" max="15" width="32.6640625" style="6" customWidth="1"/>
+    <col min="16" max="16384" width="10.33203125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" ht="23.25" customHeight="1">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:15" s="12" customFormat="1" ht="23.25" customHeight="1">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="12" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A2" s="2">
+    <row r="2" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A2" s="1">
         <v>600276</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="2">
+      <c r="C2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="1">
         <v>20250902</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="2">
         <v>0.39598379629629599</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="1">
         <v>69.430000000000007</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="1">
         <v>200</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>13886</v>
       </c>
-      <c r="I2" s="2" t="str">
+      <c r="I2" s="1" t="str">
         <f>IF(AND($C2="卖出",SUMIFS($G$2:G4,$A$2:A4,$A2)=0),SUMIFS($H$2:H4,$A$2:A4,$A2,$C$2:C4,"卖出")-SUMIFS($H$2:H4,$A$2:A4,$A2,$C$2:C4,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <f>SUMIFS($G$2:G2,$A$2:A2,$A2)</f>
         <v>200</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A3" s="2">
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+    </row>
+    <row r="3" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A3" s="1">
         <v>600276</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>20250903</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="2">
         <v>0.40028935185185199</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>69.09</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>-200</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>13818</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <f>IF(AND($C3="卖出",SUMIFS($G$2:G4,$A$2:A4,$A3)=0),SUMIFS($H$2:H4,$A$2:A4,$A3,$C$2:C4,"卖出")-SUMIFS($H$2:H4,$A$2:A4,$A3,$C$2:C4,"买入"),"")</f>
         <v>-68</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <f>SUMIFS($G$2:G3,$A$2:A3,$A3)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A4" s="2">
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+    </row>
+    <row r="4" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A4" s="1">
         <v>601138</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="2">
+      <c r="C4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="1">
         <v>20250912</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="2">
         <v>0.40763888888888899</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="1">
         <v>61</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <v>400</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>24400</v>
       </c>
-      <c r="I4" s="2" t="str">
+      <c r="I4" s="1" t="str">
         <f>IF(AND($C4="卖出",SUMIFS($G$2:G4,$A$2:A4,$A4)=0),SUMIFS($H$2:H4,$A$2:A4,$A4,$C$2:C4,"卖出")-SUMIFS($H$2:H4,$A$2:A4,$A4,$C$2:C4,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <f>SUMIFS($G$2:G4,$A$2:A4,$A4)</f>
         <v>400</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" s="2" customFormat="1" ht="20" customHeight="1">
-      <c r="A5" s="2">
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+    </row>
+    <row r="5" spans="1:15" s="3" customFormat="1" ht="20" customHeight="1">
+      <c r="A5" s="1">
         <v>601138</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="2">
+      <c r="C5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="1">
         <v>20250915</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <v>0.59178240740740695</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="1">
         <v>59.5</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>100</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>5950</v>
       </c>
-      <c r="I5" s="2" t="str">
+      <c r="I5" s="1" t="str">
         <f>IF(AND($C5="卖出",SUMIFS($G$2:G5,$A$2:A5,$A5)=0),SUMIFS($H$2:H5,$A$2:A5,$A5,$C$2:C5,"卖出")-SUMIFS($H$2:H5,$A$2:A5,$A5,$C$2:C5,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <f>SUMIFS($G$2:G5,$A$2:A5,$A5)</f>
         <v>500</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A6" s="2">
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+    </row>
+    <row r="6" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A6" s="1">
         <v>601138</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="2">
+      <c r="C6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="1">
         <v>20250915</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="2">
         <v>0.399363425925926</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="1">
         <v>60.5</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>100</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>6050</v>
       </c>
-      <c r="I6" s="2" t="str">
+      <c r="I6" s="1" t="str">
         <f>IF(AND($C6="卖出",SUMIFS($G$2:G6,$A$2:A6,$A6)=0),SUMIFS($H$2:H6,$A$2:A6,$A6,$C$2:C6,"卖出")-SUMIFS($H$2:H6,$A$2:A6,$A6,$C$2:C6,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <f>SUMIFS($G$2:G6,$A$2:A6,$A6)</f>
         <v>600</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A7" s="2">
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A7" s="1">
         <v>603986</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="2">
+      <c r="C7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="1">
         <v>20250925</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="2">
         <v>0.60934027777777799</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="1">
         <v>198</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="1">
         <v>100</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>19800</v>
       </c>
-      <c r="I7" s="2" t="str">
+      <c r="I7" s="1" t="str">
         <f>IF(AND($C7="卖出",SUMIFS($G$2:G11,$A$2:A11,$A7)=0),SUMIFS($H$2:H11,$A$2:A11,$A7,$C$2:C11,"卖出")-SUMIFS($H$2:H11,$A$2:A11,$A7,$C$2:C11,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <f>SUMIFS($G$2:G7,$A$2:A7,$A7)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A8" s="2">
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+    </row>
+    <row r="8" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A8" s="1">
         <v>601138</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>20251009</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="2">
         <v>0.446851851851852</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="1">
         <v>70</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="1">
         <v>-200</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>14000</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <f>IF(AND($C8="卖出",SUMIFS($G$2:G11,$A$2:A11,$A8)=0),SUMIFS($H$2:H11,$A$2:A11,$A8,$C$2:C11,"卖出")-SUMIFS($H$2:H11,$A$2:A11,$A8,$C$2:C11,"买入"),"")</f>
         <v>1900</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <f>SUMIFS($G$2:G8,$A$2:A8,$A8)</f>
         <v>400</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A9" s="2">
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+    </row>
+    <row r="9" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A9" s="1">
         <v>600111</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="2">
+      <c r="C9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="1">
         <v>20251010</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="2">
         <v>0.41733796296296299</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="1">
         <v>53.5</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="1">
         <v>200</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>10700</v>
       </c>
-      <c r="I9" s="2" t="str">
+      <c r="I9" s="1" t="str">
         <f>IF(AND($C9="卖出",SUMIFS($G$2:G11,$A$2:A11,$A9)=0),SUMIFS($H$2:H11,$A$2:A11,$A9,$C$2:C11,"卖出")-SUMIFS($H$2:H11,$A$2:A11,$A9,$C$2:C11,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <f>SUMIFS($G$2:G9,$A$2:A9,$A9)</f>
         <v>200</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A10" s="2">
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+    </row>
+    <row r="10" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A10" s="1">
         <v>600111</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="2">
+      <c r="C10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="1">
         <v>20251010</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="2">
         <v>0.39657407407407402</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="1">
         <v>53.98</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>300</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>16194</v>
       </c>
-      <c r="I10" s="2" t="str">
+      <c r="I10" s="1" t="str">
         <f>IF(AND($C10="卖出",SUMIFS($G$2:G11,$A$2:A11,$A10)=0),SUMIFS($H$2:H11,$A$2:A11,$A10,$C$2:C11,"卖出")-SUMIFS($H$2:H11,$A$2:A11,$A10,$C$2:C11,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <f>SUMIFS($G$2:G10,$A$2:A10,$A10)</f>
         <v>500</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A11" s="2">
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+    </row>
+    <row r="11" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A11" s="1">
         <v>601138</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>20251015</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="2">
         <v>0.45391203703703698</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="1">
         <v>60.75</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>-400</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>24300</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <f>IF(AND($C11="卖出",SUMIFS($G$2:G11,$A$2:A11,$A11)=0),SUMIFS($H$2:H11,$A$2:A11,$A11,$C$2:C11,"卖出")-SUMIFS($H$2:H11,$A$2:A11,$A11,$C$2:C11,"买入"),"")</f>
         <v>1900</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <f>SUMIFS($G$2:G11,$A$2:A11,$A11)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A12" s="2">
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+    </row>
+    <row r="12" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A12" s="1">
         <v>603986</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>20251015</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="2">
         <v>0.45378472222222199</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="1">
         <v>193.75</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="1">
         <v>-100</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>19375</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <f>IF(AND($C12="卖出",SUMIFS($G$2:G12,$A$2:A12,$A12)=0),SUMIFS($H$2:H12,$A$2:A12,$A12,$C$2:C12,"卖出")-SUMIFS($H$2:H12,$A$2:A12,$A12,$C$2:C12,"买入"),"")</f>
         <v>-425</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <f>SUMIFS($G$2:G12,$A$2:A12,$A12)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A13" s="2">
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+    </row>
+    <row r="13" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A13" s="1">
         <v>600111</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>20251015</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="2">
         <v>0.42269675925925898</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13" s="1">
         <v>54.82</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="1">
         <v>-500</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>27410</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <f>IF(AND($C13="卖出",SUMIFS($G$2:G13,$A$2:A13,$A13)=0),SUMIFS($H$2:H13,$A$2:A13,$A13,$C$2:C13,"卖出")-SUMIFS($H$2:H13,$A$2:A13,$A13,$C$2:C13,"买入"),"")</f>
         <v>516</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <f>SUMIFS($G$2:G13,$A$2:A13,$A13)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A14" s="2" t="str">
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+    </row>
+    <row r="14" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A14" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="2">
+      <c r="C14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="1">
         <v>20251016</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="2">
         <v>0.56047453703703698</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="1">
         <v>59.5</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>600</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>35700</v>
       </c>
-      <c r="I14" s="2" t="str">
+      <c r="I14" s="1" t="str">
         <f>IF(AND($C14="卖出",SUMIFS($G$2:G19,$A$2:A19,$A14)=0),SUMIFS($H$2:H19,$A$2:A19,$A14,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A14,$C$2:C19,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <f>SUMIFS($G$2:G14,$A$2:A14,$A14)</f>
         <v>600</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A15" s="2">
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+    </row>
+    <row r="15" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A15" s="1">
         <v>603259</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15" s="2">
+      <c r="C15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="1">
         <v>20251016</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="2">
         <v>0.45853009259259297</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="1">
         <v>101.12</v>
       </c>
-      <c r="G15" s="2">
+      <c r="G15" s="1">
         <v>100</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>10112</v>
       </c>
-      <c r="I15" s="2" t="str">
+      <c r="I15" s="1" t="str">
         <f>IF(AND($C15="卖出",SUMIFS($G$2:G19,$A$2:A19,$A15)=0),SUMIFS($H$2:H19,$A$2:A19,$A15,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A15,$C$2:C19,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <f>SUMIFS($G$2:G15,$A$2:A15,$A15)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A16" s="2" t="str">
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+    </row>
+    <row r="16" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A16" s="1" t="str">
         <f>"002371"</f>
         <v>002371</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" s="2">
+      <c r="C16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="1">
         <v>20251017</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="2">
         <v>0.625</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="1">
         <v>399.43</v>
       </c>
-      <c r="G16" s="2">
+      <c r="G16" s="1">
         <v>100</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>39943</v>
       </c>
-      <c r="I16" s="2" t="str">
+      <c r="I16" s="1" t="str">
         <f>IF(AND($C16="卖出",SUMIFS($G$2:G19,$A$2:A19,$A16)=0),SUMIFS($H$2:H19,$A$2:A19,$A16,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A16,$C$2:C19,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <f>SUMIFS($G$2:G16,$A$2:A16,$A16)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A17" s="2" t="str">
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+    </row>
+    <row r="17" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A17" s="1" t="str">
         <f>"002281"</f>
         <v>002281</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>20251021</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="2">
         <v>0.62155092592592598</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="1">
         <v>61.37</v>
       </c>
-      <c r="G17" s="2">
+      <c r="G17" s="1">
         <v>300</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>18411</v>
       </c>
-      <c r="I17" s="2" t="str">
+      <c r="I17" s="1" t="str">
         <f>IF(AND($C17="卖出",SUMIFS($G$2:G19,$A$2:A19,$A17)=0),SUMIFS($H$2:H19,$A$2:A19,$A17,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A17,$C$2:C19,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <f>SUMIFS($G$2:G17,$A$2:A17,$A17)</f>
         <v>300</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A18" s="2">
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+    </row>
+    <row r="18" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A18" s="1">
         <v>603259</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>20251021</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="2">
         <v>0.46806712962962999</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="1">
         <v>101.48</v>
       </c>
-      <c r="G18" s="2">
+      <c r="G18" s="1">
         <v>-100</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>10148</v>
       </c>
-      <c r="I18" s="2">
+      <c r="I18" s="1">
         <f>IF(AND($C18="卖出",SUMIFS($G$2:G19,$A$2:A19,$A18)=0),SUMIFS($H$2:H19,$A$2:A19,$A18,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A18,$C$2:C19,"买入"),"")</f>
         <v>36</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <f>SUMIFS($G$2:G18,$A$2:A18,$A18)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A19" s="2" t="str">
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+    </row>
+    <row r="19" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A19" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>20251021</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="2">
         <v>0.41851851851851901</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19" s="1">
         <v>60.07</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G19" s="1">
         <v>-200</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>12014</v>
       </c>
-      <c r="I19" s="2" t="str">
+      <c r="I19" s="1" t="str">
         <f>IF(AND($C19="卖出",SUMIFS($G$2:G19,$A$2:A19,$A19)=0),SUMIFS($H$2:H19,$A$2:A19,$A19,$C$2:C19,"卖出")-SUMIFS($H$2:H19,$A$2:A19,$A19,$C$2:C19,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <f>SUMIFS($G$2:G19,$A$2:A19,$A19)</f>
         <v>400</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A20" s="2">
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+    </row>
+    <row r="20" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A20" s="1">
         <v>603986</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D20" s="2">
+      <c r="C20" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="1">
         <v>20251023</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="2">
         <v>0.61777777777777798</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F20" s="1">
         <v>208.04</v>
       </c>
-      <c r="G20" s="2">
+      <c r="G20" s="1">
         <v>200</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>41608</v>
       </c>
-      <c r="I20" s="2" t="str">
+      <c r="I20" s="1" t="str">
         <f>IF(AND($C20="卖出",SUMIFS($G$2:G20,$A$2:A20,$A20)=0),SUMIFS($H$2:H20,$A$2:A20,$A20,$C$2:C20,"卖出")-SUMIFS($H$2:H20,$A$2:A20,$A20,$C$2:C20,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <f>SUMIFS($G$2:G20,$A$2:A20,$A20)</f>
         <v>200</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A21" s="2" t="str">
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+    </row>
+    <row r="21" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A21" s="1" t="str">
         <f>"002371"</f>
         <v>002371</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>20251023</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="2">
         <v>0.61611111111111105</v>
       </c>
-      <c r="F21" s="2">
+      <c r="F21" s="1">
         <v>402.9</v>
       </c>
-      <c r="G21" s="2">
+      <c r="G21" s="1">
         <v>-100</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>40290</v>
       </c>
-      <c r="I21" s="2" t="str">
+      <c r="I21" s="1" t="str">
         <f>IF(AND($C21="卖出",SUMIFS($G$2:G21,$A$2:A21,$A21)=0),SUMIFS($H$2:H21,$A$2:A21,$A21,$C$2:C21,"卖出")-SUMIFS($H$2:H21,$A$2:A21,$A21,$C$2:C21,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <f>SUMIFS($G$2:G21,$A$2:A21,$A21)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A22" s="2" t="str">
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+    </row>
+    <row r="22" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A22" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>20251024</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="2">
         <v>0.60100694444444402</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="1">
         <v>63.72</v>
       </c>
-      <c r="G22" s="2">
+      <c r="G22" s="1">
         <v>-100</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>6372</v>
       </c>
-      <c r="I22" s="2" t="str">
+      <c r="I22" s="1" t="str">
         <f>IF(AND($C22="卖出",SUMIFS($G$2:G22,$A$2:A22,$A22)=0),SUMIFS($H$2:H22,$A$2:A22,$A22,$C$2:C22,"卖出")-SUMIFS($H$2:H22,$A$2:A22,$A22,$C$2:C22,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <f>SUMIFS($G$2:G22,$A$2:A22,$A22)</f>
         <v>300</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A23" s="2">
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+    </row>
+    <row r="23" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A23" s="1">
         <v>603986</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>20251024</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="2">
         <v>0.58921296296296299</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="1">
         <v>220</v>
       </c>
-      <c r="G23" s="2">
+      <c r="G23" s="1">
         <v>-100</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>22000</v>
       </c>
-      <c r="I23" s="2" t="str">
+      <c r="I23" s="1" t="str">
         <f>IF(AND($C23="卖出",SUMIFS($G$2:G23,$A$2:A23,$A23)=0),SUMIFS($H$2:H23,$A$2:A23,$A23,$C$2:C23,"卖出")-SUMIFS($H$2:H23,$A$2:A23,$A23,$C$2:C23,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <f>SUMIFS($G$2:G23,$A$2:A23,$A23)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A24" s="2" t="str">
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+    </row>
+    <row r="24" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A24" s="1" t="str">
         <f>"002281"</f>
         <v>002281</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="1">
         <v>20251024</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="2">
         <v>0.41842592592592598</v>
       </c>
-      <c r="F24" s="2">
+      <c r="F24" s="1">
         <v>61.31</v>
       </c>
-      <c r="G24" s="2">
+      <c r="G24" s="1">
         <v>-300</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>18393</v>
       </c>
-      <c r="I24" s="2" t="str">
+      <c r="I24" s="1" t="str">
         <f>IF(AND($C24="卖出",SUMIFS($G$2:G24,$A$2:A24,$A24)=0),SUMIFS($H$2:H24,$A$2:A24,$A24,$C$2:C24,"卖出")-SUMIFS($H$2:H24,$A$2:A24,$A24,$C$2:C24,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <f>SUMIFS($G$2:G24,$A$2:A24,$A24)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A25" s="2">
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+    </row>
+    <row r="25" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A25" s="1">
         <v>603083</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="1">
         <v>20251027</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25" s="2">
         <v>0.39907407407407403</v>
       </c>
-      <c r="F25" s="2">
+      <c r="F25" s="1">
         <v>122.95</v>
       </c>
-      <c r="G25" s="2">
+      <c r="G25" s="1">
         <v>200</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>24590</v>
       </c>
-      <c r="I25" s="2" t="str">
+      <c r="I25" s="1" t="str">
         <f>IF(AND($C25="卖出",SUMIFS($G$2:G25,$A$2:A25,$A25)=0),SUMIFS($H$2:H25,$A$2:A25,$A25,$C$2:C25,"卖出")-SUMIFS($H$2:H25,$A$2:A25,$A25,$C$2:C25,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <f>SUMIFS($G$2:G25,$A$2:A25,$A25)</f>
         <v>200</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A26" s="2">
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+    </row>
+    <row r="26" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A26" s="1">
         <v>603083</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>20251028</v>
       </c>
-      <c r="E26" s="4">
+      <c r="E26" s="2">
         <v>0.625</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F26" s="1">
         <v>119.28</v>
       </c>
-      <c r="G26" s="2">
+      <c r="G26" s="1">
         <v>-200</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>23856</v>
       </c>
-      <c r="I26" s="2">
+      <c r="I26" s="1">
         <v>-700</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <f>SUMIFS($G$2:G26,$A$2:A26,$A26)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A27" s="2">
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+    </row>
+    <row r="27" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A27" s="1">
         <v>603986</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>20251029</v>
       </c>
-      <c r="E27" s="4">
+      <c r="E27" s="2">
         <v>0.44155092592592599</v>
       </c>
-      <c r="F27" s="2">
+      <c r="F27" s="1">
         <v>236.41</v>
       </c>
-      <c r="G27" s="2">
+      <c r="G27" s="1">
         <v>-100</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>23641</v>
       </c>
-      <c r="I27" s="2">
+      <c r="I27" s="1">
         <f>IF(AND($C27="卖出",SUMIFS($G$2:G27,$A$2:A27,$A27)=0),SUMIFS($H$2:H27,$A$2:A27,$A27,$C$2:C27,"卖出")-SUMIFS($H$2:H27,$A$2:A27,$A27,$C$2:C27,"买入"),"")</f>
         <v>3608</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <f>SUMIFS($G$2:G27,$A$2:A27,$A27)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A28" s="2">
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+    </row>
+    <row r="28" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A28" s="1">
         <v>603799</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D28" s="2">
+      <c r="C28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="1">
         <v>20251030</v>
       </c>
-      <c r="E28" s="4">
+      <c r="E28" s="2">
         <v>0.56559027777777804</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F28" s="1">
         <v>66.099999999999994</v>
       </c>
-      <c r="G28" s="2">
+      <c r="G28" s="1">
         <v>300</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>19830</v>
       </c>
-      <c r="I28" s="2" t="str">
+      <c r="I28" s="1" t="str">
         <f>IF(AND($C28="卖出",SUMIFS($G$2:G28,$A$2:A28,$A28)=0),SUMIFS($H$2:H28,$A$2:A28,$A28,$C$2:C28,"卖出")-SUMIFS($H$2:H28,$A$2:A28,$A28,$C$2:C28,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <f>SUMIFS($G$2:G28,$A$2:A28,$A28)</f>
         <v>300</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A29" s="2">
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+    </row>
+    <row r="29" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A29" s="1">
         <v>603986</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D29" s="2">
+      <c r="C29" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="1">
         <v>20251030</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E29" s="2">
         <v>0.544988425925926</v>
       </c>
-      <c r="F29" s="2">
+      <c r="F29" s="1">
         <v>236</v>
       </c>
-      <c r="G29" s="2">
+      <c r="G29" s="1">
         <v>100</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>23600</v>
       </c>
-      <c r="I29" s="2" t="str">
+      <c r="I29" s="1" t="str">
         <f>IF(AND($C29="卖出",SUMIFS($G$2:G29,$A$2:A29,$A29)=0),SUMIFS($H$2:H29,$A$2:A29,$A29,$C$2:C29,"卖出")-SUMIFS($H$2:H29,$A$2:A29,$A29,$C$2:C29,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <f>SUMIFS($G$2:G29,$A$2:A29,$A29)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A30" s="2">
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+    </row>
+    <row r="30" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A30" s="1">
         <v>603099</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D30" s="2">
+      <c r="C30" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" s="1">
         <v>20251104</v>
       </c>
-      <c r="E30" s="4">
+      <c r="E30" s="2">
         <v>0.625</v>
       </c>
-      <c r="F30" s="2">
+      <c r="F30" s="1">
         <v>57.91</v>
       </c>
-      <c r="G30" s="2">
+      <c r="G30" s="1">
         <v>100</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>5791</v>
       </c>
-      <c r="I30" s="2" t="str">
+      <c r="I30" s="1" t="str">
         <f>IF(AND($C30="卖出",SUMIFS($G$2:G30,$A$2:A30,$A30)=0),SUMIFS($H$2:H30,$A$2:A30,$A30,$C$2:C30,"卖出")-SUMIFS($H$2:H30,$A$2:A30,$A30,$C$2:C30,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <f>SUMIFS($G$2:G30,$A$2:A30,$A30)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A31" s="2">
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+    </row>
+    <row r="31" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A31" s="1">
         <v>603099</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D31" s="2">
+      <c r="C31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="1">
         <v>20251104</v>
       </c>
-      <c r="E31" s="4">
+      <c r="E31" s="2">
         <v>0.625</v>
       </c>
-      <c r="F31" s="2">
+      <c r="F31" s="1">
         <v>57.91</v>
       </c>
-      <c r="G31" s="2">
+      <c r="G31" s="1">
         <v>100</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>5791</v>
       </c>
-      <c r="I31" s="2" t="str">
+      <c r="I31" s="1" t="str">
         <f>IF(AND($C31="卖出",SUMIFS($G$2:G31,$A$2:A31,$A31)=0),SUMIFS($H$2:H31,$A$2:A31,$A31,$C$2:C31,"卖出")-SUMIFS($H$2:H31,$A$2:A31,$A31,$C$2:C31,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <f>SUMIFS($G$2:G31,$A$2:A31,$A31)</f>
         <v>200</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A32" s="2">
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+    </row>
+    <row r="32" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A32" s="1">
         <v>603799</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D32" s="2">
+      <c r="D32" s="1">
         <v>20251104</v>
       </c>
-      <c r="E32" s="4">
+      <c r="E32" s="2">
         <v>0.625</v>
       </c>
-      <c r="F32" s="2">
+      <c r="F32" s="1">
         <v>59.9</v>
       </c>
-      <c r="G32" s="2">
+      <c r="G32" s="1">
         <v>-300</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>17970</v>
       </c>
-      <c r="I32" s="2">
+      <c r="I32" s="1">
         <f>IF(AND($C32="卖出",SUMIFS($G$2:G32,$A$2:A32,$A32)=0),SUMIFS($H$2:H32,$A$2:A32,$A32,$C$2:C32,"卖出")-SUMIFS($H$2:H32,$A$2:A32,$A32,$C$2:C32,"买入"),"")</f>
         <v>-1860</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <f>SUMIFS($G$2:G32,$A$2:A32,$A32)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A33" s="2">
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+    </row>
+    <row r="33" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A33" s="1">
         <v>603099</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>20251105</v>
       </c>
-      <c r="E33" s="4">
+      <c r="E33" s="2">
         <v>0.41347222222222202</v>
       </c>
-      <c r="F33" s="2">
+      <c r="F33" s="1">
         <v>56.04</v>
       </c>
-      <c r="G33" s="2">
+      <c r="G33" s="1">
         <v>-200</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>11208</v>
       </c>
-      <c r="I33" s="2" t="str">
+      <c r="I33" s="1" t="str">
         <f>IF(AND($C33="卖出",SUMIFS($G$2:G33,$A$2:A33,$A33)=0),SUMIFS($H$2:H33,$A$2:A33,$A33,$C$2:C33,"卖出")-SUMIFS($H$2:H33,$A$2:A33,$A33,$C$2:C33,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <f>SUMIFS($G$2:G33,$A$2:A33,$A33)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A34" s="2" t="str">
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+    </row>
+    <row r="34" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A34" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D34" s="2">
+      <c r="C34" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" s="1">
         <v>20260119</v>
       </c>
-      <c r="E34" s="4">
+      <c r="E34" s="2">
         <v>0.42253472222222199</v>
       </c>
-      <c r="F34" s="2">
+      <c r="F34" s="1">
         <v>199</v>
       </c>
-      <c r="G34" s="2">
+      <c r="G34" s="1">
         <v>100</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>19900</v>
       </c>
-      <c r="I34" s="2" t="str">
+      <c r="I34" s="1" t="str">
         <f>IF(AND($C34="卖出",SUMIFS($G$2:G34,$A$2:A34,$A34)=0),SUMIFS($H$2:H34,$A$2:A34,$A34,$C$2:C34,"卖出")-SUMIFS($H$2:H34,$A$2:A34,$A34,$C$2:C34,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <f>SUMIFS($G$2:G34,$A$2:A34,$A34)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A35" s="2">
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+    </row>
+    <row r="35" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A35" s="1">
         <v>601179</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D35" s="2">
+      <c r="C35" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" s="1">
         <v>20260119</v>
       </c>
-      <c r="E35" s="4">
+      <c r="E35" s="2">
         <v>0.40089120370370401</v>
       </c>
-      <c r="F35" s="2">
+      <c r="F35" s="1">
         <v>14.19</v>
       </c>
-      <c r="G35" s="2">
+      <c r="G35" s="1">
         <v>1400</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>19866</v>
       </c>
-      <c r="I35" s="2" t="str">
+      <c r="I35" s="1" t="str">
         <f>IF(AND($C35="卖出",SUMIFS($G$2:G35,$A$2:A35,$A35)=0),SUMIFS($H$2:H35,$A$2:A35,$A35,$C$2:C35,"卖出")-SUMIFS($H$2:H35,$A$2:A35,$A35,$C$2:C35,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <f>SUMIFS($G$2:G35,$A$2:A35,$A35)</f>
         <v>1400</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A36" s="2" t="str">
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1"/>
+      <c r="O35" s="1"/>
+    </row>
+    <row r="36" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A36" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D36" s="2">
+      <c r="C36" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D36" s="1">
         <v>20260119</v>
       </c>
-      <c r="E36" s="4">
+      <c r="E36" s="2">
         <v>0.39848379629629599</v>
       </c>
-      <c r="F36" s="2">
+      <c r="F36" s="1">
         <v>194</v>
       </c>
-      <c r="G36" s="2">
+      <c r="G36" s="1">
         <v>100</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>19400</v>
       </c>
-      <c r="I36" s="2" t="str">
+      <c r="I36" s="1" t="str">
         <f>IF(AND($C36="卖出",SUMIFS($G$2:G36,$A$2:A36,$A36)=0),SUMIFS($H$2:H36,$A$2:A36,$A36,$C$2:C36,"卖出")-SUMIFS($H$2:H36,$A$2:A36,$A36,$C$2:C36,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <f>SUMIFS($G$2:G36,$A$2:A36,$A36)</f>
         <v>200</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A37" s="2">
+      <c r="K36" s="1"/>
+      <c r="L36" s="1"/>
+      <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
+      <c r="O36" s="1"/>
+    </row>
+    <row r="37" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A37" s="1">
         <v>603986</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>20260119</v>
       </c>
-      <c r="E37" s="4">
+      <c r="E37" s="2">
         <v>0.39603009259259297</v>
       </c>
-      <c r="F37" s="2">
+      <c r="F37" s="1">
         <v>280.60000000000002</v>
       </c>
-      <c r="G37" s="2">
+      <c r="G37" s="1">
         <v>-100</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>28060</v>
       </c>
-      <c r="I37" s="2">
+      <c r="I37" s="1">
         <f>IF(AND($C37="卖出",SUMIFS($G$2:G37,$A$2:A37,$A37)=0),SUMIFS($H$2:H37,$A$2:A37,$A37,$C$2:C37,"卖出")-SUMIFS($H$2:H37,$A$2:A37,$A37,$C$2:C37,"买入"),"")</f>
         <v>8068</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <f>SUMIFS($G$2:G37,$A$2:A37,$A37)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A38" s="2" t="str">
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1"/>
+      <c r="O37" s="1"/>
+    </row>
+    <row r="38" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A38" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D38" s="2">
+      <c r="C38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D38" s="1">
         <v>20260121</v>
       </c>
-      <c r="E38" s="4">
+      <c r="E38" s="2">
         <v>0.39738425925925902</v>
       </c>
-      <c r="F38" s="2">
+      <c r="F38" s="1">
         <v>189</v>
       </c>
-      <c r="G38" s="2">
+      <c r="G38" s="1">
         <v>100</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>18900</v>
       </c>
-      <c r="I38" s="2" t="str">
+      <c r="I38" s="1" t="str">
         <f>IF(AND($C38="卖出",SUMIFS($G$2:G38,$A$2:A38,$A38)=0),SUMIFS($H$2:H38,$A$2:A38,$A38,$C$2:C38,"卖出")-SUMIFS($H$2:H38,$A$2:A38,$A38,$C$2:C38,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <f>SUMIFS($G$2:G38,$A$2:A38,$A38)</f>
         <v>300</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A39" s="2" t="str">
+      <c r="K38" s="1"/>
+      <c r="L38" s="1"/>
+      <c r="M38" s="1"/>
+      <c r="N38" s="1"/>
+      <c r="O38" s="1"/>
+    </row>
+    <row r="39" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A39" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D39" s="2">
+      <c r="C39" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D39" s="1">
         <v>20260122</v>
       </c>
-      <c r="E39" s="4">
+      <c r="E39" s="2">
         <v>0.44486111111111099</v>
       </c>
-      <c r="F39" s="2">
+      <c r="F39" s="1">
         <v>189</v>
       </c>
-      <c r="G39" s="2">
+      <c r="G39" s="1">
         <v>100</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>18900</v>
       </c>
-      <c r="I39" s="2" t="str">
+      <c r="I39" s="1" t="str">
         <f>IF(AND($C39="卖出",SUMIFS($G$2:G39,$A$2:A39,$A39)=0),SUMIFS($H$2:H39,$A$2:A39,$A39,$C$2:C39,"卖出")-SUMIFS($H$2:H39,$A$2:A39,$A39,$C$2:C39,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <f>SUMIFS($G$2:G39,$A$2:A39,$A39)</f>
         <v>400</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A40" s="2">
+      <c r="K39" s="1"/>
+      <c r="L39" s="1"/>
+      <c r="M39" s="1"/>
+      <c r="N39" s="1"/>
+      <c r="O39" s="1"/>
+    </row>
+    <row r="40" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A40" s="1">
         <v>600584</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D40" s="2">
+      <c r="C40" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D40" s="1">
         <v>20260122</v>
       </c>
-      <c r="E40" s="4">
+      <c r="E40" s="2">
         <v>0.40795138888888899</v>
       </c>
-      <c r="F40" s="2">
+      <c r="F40" s="1">
         <v>50</v>
       </c>
-      <c r="G40" s="2">
+      <c r="G40" s="1">
         <v>400</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>20000</v>
       </c>
-      <c r="I40" s="2" t="str">
+      <c r="I40" s="1" t="str">
         <f>IF(AND($C40="卖出",SUMIFS($G$2:G40,$A$2:A40,$A40)=0),SUMIFS($H$2:H40,$A$2:A40,$A40,$C$2:C40,"卖出")-SUMIFS($H$2:H40,$A$2:A40,$A40,$C$2:C40,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <f>SUMIFS($G$2:G40,$A$2:A40,$A40)</f>
         <v>400</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A41" s="2">
+      <c r="K40" s="1"/>
+      <c r="L40" s="1"/>
+      <c r="M40" s="1"/>
+      <c r="N40" s="1"/>
+      <c r="O40" s="1"/>
+    </row>
+    <row r="41" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A41" s="1">
         <v>601179</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D41" s="2">
+      <c r="D41" s="1">
         <v>20260126</v>
       </c>
-      <c r="E41" s="4">
+      <c r="E41" s="2">
         <v>0.62217592592592597</v>
       </c>
-      <c r="F41" s="2">
+      <c r="F41" s="1">
         <v>16.16</v>
       </c>
-      <c r="G41" s="2">
+      <c r="G41" s="1">
         <v>-700</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>11312</v>
       </c>
-      <c r="I41" s="2" t="str">
+      <c r="I41" s="1" t="str">
         <f>IF(AND($C41="卖出",SUMIFS($G$2:G41,$A$2:A41,$A41)=0),SUMIFS($H$2:H41,$A$2:A41,$A41,$C$2:C41,"卖出")-SUMIFS($H$2:H41,$A$2:A41,$A41,$C$2:C41,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <f>SUMIFS($G$2:G41,$A$2:A41,$A41)</f>
         <v>700</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A42" s="2">
+      <c r="K41" s="1"/>
+      <c r="L41" s="1"/>
+      <c r="M41" s="1"/>
+      <c r="N41" s="1"/>
+      <c r="O41" s="1"/>
+    </row>
+    <row r="42" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A42" s="1">
         <v>600584</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C42" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D42" s="2">
+      <c r="C42" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D42" s="1">
         <v>20260127</v>
       </c>
-      <c r="E42" s="4">
+      <c r="E42" s="2">
         <v>0.589479166666667</v>
       </c>
-      <c r="F42" s="2">
+      <c r="F42" s="1">
         <v>48.3</v>
       </c>
-      <c r="G42" s="2">
+      <c r="G42" s="1">
         <v>200</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>9660</v>
       </c>
-      <c r="I42" s="2" t="str">
+      <c r="I42" s="1" t="str">
         <f>IF(AND($C42="卖出",SUMIFS($G$2:G42,$A$2:A42,$A42)=0),SUMIFS($H$2:H42,$A$2:A42,$A42,$C$2:C42,"卖出")-SUMIFS($H$2:H42,$A$2:A42,$A42,$C$2:C42,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <f>SUMIFS($G$2:G42,$A$2:A42,$A42)</f>
         <v>600</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A43" s="2" t="str">
+      <c r="K42" s="1"/>
+      <c r="L42" s="1"/>
+      <c r="M42" s="1"/>
+      <c r="N42" s="1"/>
+      <c r="O42" s="1"/>
+    </row>
+    <row r="43" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A43" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D43" s="2">
+      <c r="C43" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D43" s="1">
         <v>20260127</v>
       </c>
-      <c r="E43" s="4">
+      <c r="E43" s="2">
         <v>0.41396990740740702</v>
       </c>
-      <c r="F43" s="2">
+      <c r="F43" s="1">
         <v>53.2</v>
       </c>
-      <c r="G43" s="2">
+      <c r="G43" s="1">
         <v>200</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>10640</v>
       </c>
-      <c r="I43" s="2" t="str">
+      <c r="I43" s="1" t="str">
         <f>IF(AND($C43="卖出",SUMIFS($G$2:G43,$A$2:A43,$A43)=0),SUMIFS($H$2:H43,$A$2:A43,$A43,$C$2:C43,"卖出")-SUMIFS($H$2:H43,$A$2:A43,$A43,$C$2:C43,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <f>SUMIFS($G$2:G43,$A$2:A43,$A43)</f>
         <v>500</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A44" s="2" t="str">
+      <c r="K43" s="1"/>
+      <c r="L43" s="1"/>
+      <c r="M43" s="1"/>
+      <c r="N43" s="1"/>
+      <c r="O43" s="1"/>
+    </row>
+    <row r="44" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A44" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D44" s="2">
+      <c r="C44" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D44" s="1">
         <v>20260129</v>
       </c>
-      <c r="E44" s="4">
+      <c r="E44" s="2">
         <v>0.57781249999999995</v>
       </c>
-      <c r="F44" s="2">
+      <c r="F44" s="1">
         <v>186.2</v>
       </c>
-      <c r="G44" s="2">
+      <c r="G44" s="1">
         <v>100</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>18620</v>
       </c>
-      <c r="I44" s="2" t="str">
+      <c r="I44" s="1" t="str">
         <f>IF(AND($C44="卖出",SUMIFS($G$2:G44,$A$2:A44,$A44)=0),SUMIFS($H$2:H44,$A$2:A44,$A44,$C$2:C44,"卖出")-SUMIFS($H$2:H44,$A$2:A44,$A44,$C$2:C44,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <f>SUMIFS($G$2:G44,$A$2:A44,$A44)</f>
         <v>500</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A45" s="2" t="str">
+      <c r="K44" s="1"/>
+      <c r="L44" s="1"/>
+      <c r="M44" s="1"/>
+      <c r="N44" s="1"/>
+      <c r="O44" s="1"/>
+    </row>
+    <row r="45" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A45" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="C45" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>20260129</v>
       </c>
-      <c r="E45" s="4">
+      <c r="E45" s="2">
         <v>0.57199074074074097</v>
       </c>
-      <c r="F45" s="2">
+      <c r="F45" s="1">
         <v>52.2</v>
       </c>
-      <c r="G45" s="2">
+      <c r="G45" s="1">
         <v>-100</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>5220</v>
       </c>
-      <c r="I45" s="2" t="str">
+      <c r="I45" s="1" t="str">
         <f>IF(AND($C45="卖出",SUMIFS($G$2:G45,$A$2:A45,$A45)=0),SUMIFS($H$2:H45,$A$2:A45,$A45,$C$2:C45,"卖出")-SUMIFS($H$2:H45,$A$2:A45,$A45,$C$2:C45,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <f>SUMIFS($G$2:G45,$A$2:A45,$A45)</f>
         <v>400</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A46" s="2">
+      <c r="K45" s="1"/>
+      <c r="L45" s="1"/>
+      <c r="M45" s="1"/>
+      <c r="N45" s="1"/>
+      <c r="O45" s="1"/>
+    </row>
+    <row r="46" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A46" s="1">
         <v>600584</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="C46" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>20260129</v>
       </c>
-      <c r="E46" s="4">
+      <c r="E46" s="2">
         <v>0.57099537037036996</v>
       </c>
-      <c r="F46" s="2">
+      <c r="F46" s="1">
         <v>49.2</v>
       </c>
-      <c r="G46" s="2">
+      <c r="G46" s="1">
         <v>-200</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>9840</v>
       </c>
-      <c r="I46" s="2" t="str">
+      <c r="I46" s="1" t="str">
         <f>IF(AND($C46="卖出",SUMIFS($G$2:G46,$A$2:A46,$A46)=0),SUMIFS($H$2:H46,$A$2:A46,$A46,$C$2:C46,"卖出")-SUMIFS($H$2:H46,$A$2:A46,$A46,$C$2:C46,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <f>SUMIFS($G$2:G46,$A$2:A46,$A46)</f>
         <v>400</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A47" s="2" t="str">
+      <c r="K46" s="1"/>
+      <c r="L46" s="1"/>
+      <c r="M46" s="1"/>
+      <c r="N46" s="1"/>
+      <c r="O46" s="1"/>
+    </row>
+    <row r="47" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A47" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C47" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D47" s="2">
+      <c r="C47" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D47" s="1">
         <v>20260129</v>
       </c>
-      <c r="E47" s="4">
+      <c r="E47" s="2">
         <v>0.54546296296296304</v>
       </c>
-      <c r="F47" s="2">
+      <c r="F47" s="1">
         <v>51.9</v>
       </c>
-      <c r="G47" s="2">
+      <c r="G47" s="1">
         <v>100</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>5190</v>
       </c>
-      <c r="I47" s="2" t="str">
+      <c r="I47" s="1" t="str">
         <f>IF(AND($C47="卖出",SUMIFS($G$2:G47,$A$2:A47,$A47)=0),SUMIFS($H$2:H47,$A$2:A47,$A47,$C$2:C47,"卖出")-SUMIFS($H$2:H47,$A$2:A47,$A47,$C$2:C47,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <f>SUMIFS($G$2:G47,$A$2:A47,$A47)</f>
         <v>500</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A48" s="2" t="str">
+      <c r="K47" s="1"/>
+      <c r="L47" s="1"/>
+      <c r="M47" s="1"/>
+      <c r="N47" s="1"/>
+      <c r="O47" s="1"/>
+    </row>
+    <row r="48" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A48" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C48" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D48" s="2">
+      <c r="C48" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D48" s="1">
         <v>20260129</v>
       </c>
-      <c r="E48" s="4">
+      <c r="E48" s="2">
         <v>0.54239583333333297</v>
       </c>
-      <c r="F48" s="2">
+      <c r="F48" s="1">
         <v>188</v>
       </c>
-      <c r="G48" s="2">
+      <c r="G48" s="1">
         <v>100</v>
       </c>
-      <c r="H48" s="2">
+      <c r="H48" s="1">
         <v>18800</v>
       </c>
-      <c r="I48" s="2" t="str">
+      <c r="I48" s="1" t="str">
         <f>IF(AND($C48="卖出",SUMIFS($G$2:G48,$A$2:A48,$A48)=0),SUMIFS($H$2:H48,$A$2:A48,$A48,$C$2:C48,"卖出")-SUMIFS($H$2:H48,$A$2:A48,$A48,$C$2:C48,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <f>SUMIFS($G$2:G48,$A$2:A48,$A48)</f>
         <v>600</v>
       </c>
-    </row>
-    <row r="49" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A49" s="2">
+      <c r="K48" s="1"/>
+      <c r="L48" s="1"/>
+      <c r="M48" s="1"/>
+      <c r="N48" s="1"/>
+      <c r="O48" s="1"/>
+    </row>
+    <row r="49" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A49" s="1">
         <v>601179</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C49" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D49" s="2">
+      <c r="C49" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D49" s="1">
         <v>20260130</v>
       </c>
-      <c r="E49" s="4">
+      <c r="E49" s="2">
         <v>0.44043981481481498</v>
       </c>
-      <c r="F49" s="2">
+      <c r="F49" s="1">
         <v>14</v>
       </c>
-      <c r="G49" s="2">
+      <c r="G49" s="1">
         <v>400</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>5600</v>
       </c>
-      <c r="I49" s="2" t="str">
+      <c r="I49" s="1" t="str">
         <f>IF(AND($C49="卖出",SUMIFS($G$2:G49,$A$2:A49,$A49)=0),SUMIFS($H$2:H49,$A$2:A49,$A49,$C$2:C49,"卖出")-SUMIFS($H$2:H49,$A$2:A49,$A49,$C$2:C49,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <f>SUMIFS($G$2:G49,$A$2:A49,$A49)</f>
         <v>1100</v>
       </c>
-    </row>
-    <row r="50" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A50" s="2" t="str">
+      <c r="K49" s="1"/>
+      <c r="L49" s="1"/>
+      <c r="M49" s="1"/>
+      <c r="N49" s="1"/>
+      <c r="O49" s="1"/>
+    </row>
+    <row r="50" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A50" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C50" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D50" s="2">
+      <c r="C50" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D50" s="1">
         <v>20260130</v>
       </c>
-      <c r="E50" s="4">
+      <c r="E50" s="2">
         <v>0.43103009259259301</v>
       </c>
-      <c r="F50" s="2">
+      <c r="F50" s="1">
         <v>180</v>
       </c>
-      <c r="G50" s="2">
+      <c r="G50" s="1">
         <v>100</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>18000</v>
       </c>
-      <c r="I50" s="2" t="str">
+      <c r="I50" s="1" t="str">
         <f>IF(AND($C50="卖出",SUMIFS($G$2:G50,$A$2:A50,$A50)=0),SUMIFS($H$2:H50,$A$2:A50,$A50,$C$2:C50,"卖出")-SUMIFS($H$2:H50,$A$2:A50,$A50,$C$2:C50,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <f>SUMIFS($G$2:G50,$A$2:A50,$A50)</f>
         <v>700</v>
       </c>
-    </row>
-    <row r="51" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A51" s="2" t="str">
+      <c r="K50" s="1"/>
+      <c r="L50" s="1"/>
+      <c r="M50" s="1"/>
+      <c r="N50" s="1"/>
+      <c r="O50" s="1"/>
+    </row>
+    <row r="51" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A51" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="C51" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>20260202</v>
       </c>
-      <c r="E51" s="4">
+      <c r="E51" s="2">
         <v>0.61899305555555595</v>
       </c>
-      <c r="F51" s="2">
+      <c r="F51" s="1">
         <v>52.08</v>
       </c>
-      <c r="G51" s="2">
+      <c r="G51" s="1">
         <v>-300</v>
       </c>
-      <c r="H51" s="2">
+      <c r="H51" s="1">
         <v>15624</v>
       </c>
-      <c r="I51" s="2" t="str">
+      <c r="I51" s="1" t="str">
         <f>IF(AND($C51="卖出",SUMIFS($G$2:G51,$A$2:A51,$A51)=0),SUMIFS($H$2:H51,$A$2:A51,$A51,$C$2:C51,"卖出")-SUMIFS($H$2:H51,$A$2:A51,$A51,$C$2:C51,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <f>SUMIFS($G$2:G51,$A$2:A51,$A51)</f>
         <v>200</v>
       </c>
-    </row>
-    <row r="52" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A52" s="2">
+      <c r="K51" s="1"/>
+      <c r="L51" s="1"/>
+      <c r="M51" s="1"/>
+      <c r="N51" s="1"/>
+      <c r="O51" s="1"/>
+    </row>
+    <row r="52" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A52" s="1">
         <v>600584</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C52" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D52" s="2">
+      <c r="C52" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D52" s="1">
         <v>20260202</v>
       </c>
-      <c r="E52" s="4">
+      <c r="E52" s="2">
         <v>0.56569444444444394</v>
       </c>
-      <c r="F52" s="2">
+      <c r="F52" s="1">
         <v>46.8</v>
       </c>
-      <c r="G52" s="2">
+      <c r="G52" s="1">
         <v>100</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>4680</v>
       </c>
-      <c r="I52" s="2" t="str">
+      <c r="I52" s="1" t="str">
         <f>IF(AND($C52="卖出",SUMIFS($G$2:G52,$A$2:A52,$A52)=0),SUMIFS($H$2:H52,$A$2:A52,$A52,$C$2:C52,"卖出")-SUMIFS($H$2:H52,$A$2:A52,$A52,$C$2:C52,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <f>SUMIFS($G$2:G52,$A$2:A52,$A52)</f>
         <v>500</v>
       </c>
-    </row>
-    <row r="53" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A53" s="2">
+      <c r="K52" s="1"/>
+      <c r="L52" s="1"/>
+      <c r="M52" s="1"/>
+      <c r="N52" s="1"/>
+      <c r="O52" s="1"/>
+    </row>
+    <row r="53" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A53" s="1">
         <v>601179</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B53" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="C53" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>20260202</v>
       </c>
-      <c r="E53" s="4">
+      <c r="E53" s="2">
         <v>0.55994212962962997</v>
       </c>
-      <c r="F53" s="2">
+      <c r="F53" s="1">
         <v>15.7</v>
       </c>
-      <c r="G53" s="2">
+      <c r="G53" s="1">
         <v>-1100</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>17270</v>
       </c>
-      <c r="I53" s="2">
+      <c r="I53" s="1">
         <f>IF(AND($C53="卖出",SUMIFS($G$2:G53,$A$2:A53,$A53)=0),SUMIFS($H$2:H53,$A$2:A53,$A53,$C$2:C53,"卖出")-SUMIFS($H$2:H53,$A$2:A53,$A53,$C$2:C53,"买入"),"")</f>
         <v>3116</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <f>SUMIFS($G$2:G53,$A$2:A53,$A53)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A54" s="2" t="str">
+      <c r="K53" s="1"/>
+      <c r="L53" s="1"/>
+      <c r="M53" s="1"/>
+      <c r="N53" s="1"/>
+      <c r="O53" s="1"/>
+    </row>
+    <row r="54" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A54" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="C54" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>20260202</v>
       </c>
-      <c r="E54" s="4">
+      <c r="E54" s="2">
         <v>0.44674768518518498</v>
       </c>
-      <c r="F54" s="2">
+      <c r="F54" s="1">
         <v>191</v>
       </c>
-      <c r="G54" s="2">
+      <c r="G54" s="1">
         <v>-100</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>19100</v>
       </c>
-      <c r="I54" s="2" t="str">
+      <c r="I54" s="1" t="str">
         <f>IF(AND($C54="卖出",SUMIFS($G$2:G54,$A$2:A54,$A54)=0),SUMIFS($H$2:H54,$A$2:A54,$A54,$C$2:C54,"卖出")-SUMIFS($H$2:H54,$A$2:A54,$A54,$C$2:C54,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <f>SUMIFS($G$2:G54,$A$2:A54,$A54)</f>
         <v>600</v>
       </c>
-    </row>
-    <row r="55" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A55" s="2" t="str">
+      <c r="K54" s="1"/>
+      <c r="L54" s="1"/>
+      <c r="M54" s="1"/>
+      <c r="N54" s="1"/>
+      <c r="O54" s="1"/>
+    </row>
+    <row r="55" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A55" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="C55" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D55" s="2">
+      <c r="D55" s="1">
         <v>20260202</v>
       </c>
-      <c r="E55" s="4">
+      <c r="E55" s="2">
         <v>0.44067129629629598</v>
       </c>
-      <c r="F55" s="2">
+      <c r="F55" s="1">
         <v>53.09</v>
       </c>
-      <c r="G55" s="2">
+      <c r="G55" s="1">
         <v>-200</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>10618</v>
       </c>
-      <c r="I55" s="2">
+      <c r="I55" s="1">
         <f>IF(AND($C55="卖出",SUMIFS($G$2:G55,$A$2:A55,$A55)=0),SUMIFS($H$2:H55,$A$2:A55,$A55,$C$2:C55,"卖出")-SUMIFS($H$2:H55,$A$2:A55,$A55,$C$2:C55,"买入"),"")</f>
         <v>-1682</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <f>SUMIFS($G$2:G55,$A$2:A55,$A55)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A56" s="2" t="str">
+      <c r="K55" s="1"/>
+      <c r="L55" s="1"/>
+      <c r="M55" s="1"/>
+      <c r="N55" s="1"/>
+      <c r="O55" s="1"/>
+    </row>
+    <row r="56" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A56" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="C56" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>20260203</v>
       </c>
-      <c r="E56" s="4">
+      <c r="E56" s="2">
         <v>0.40917824074074099</v>
       </c>
-      <c r="F56" s="2">
+      <c r="F56" s="1">
         <v>194</v>
       </c>
-      <c r="G56" s="2">
+      <c r="G56" s="1">
         <v>-100</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>19400</v>
       </c>
-      <c r="I56" s="2" t="str">
+      <c r="I56" s="1" t="str">
         <f>IF(AND($C56="卖出",SUMIFS($G$2:G56,$A$2:A56,$A56)=0),SUMIFS($H$2:H56,$A$2:A56,$A56,$C$2:C56,"卖出")-SUMIFS($H$2:H56,$A$2:A56,$A56,$C$2:C56,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <f>SUMIFS($G$2:G56,$A$2:A56,$A56)</f>
         <v>500</v>
       </c>
-    </row>
-    <row r="57" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A57" s="2" t="str">
+      <c r="K56" s="1"/>
+      <c r="L56" s="1"/>
+      <c r="M56" s="1"/>
+      <c r="N56" s="1"/>
+      <c r="O56" s="1"/>
+    </row>
+    <row r="57" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A57" s="1" t="str">
         <f t="shared" ref="A57:A62" si="0">"002028"</f>
         <v>002028</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C57" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D57" s="2">
+      <c r="C57" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D57" s="1">
         <v>20260205</v>
       </c>
-      <c r="E57" s="4">
+      <c r="E57" s="2">
         <v>0.404363425925926</v>
       </c>
-      <c r="F57" s="2">
+      <c r="F57" s="1">
         <v>195</v>
       </c>
-      <c r="G57" s="2">
+      <c r="G57" s="1">
         <v>100</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>19500</v>
       </c>
-      <c r="I57" s="2" t="str">
+      <c r="I57" s="1" t="str">
         <f>IF(AND($C57="卖出",SUMIFS($G$2:G57,$A$2:A57,$A57)=0),SUMIFS($H$2:H57,$A$2:A57,$A57,$C$2:C57,"卖出")-SUMIFS($H$2:H57,$A$2:A57,$A57,$C$2:C57,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <f>SUMIFS($G$2:G57,$A$2:A57,$A57)</f>
         <v>600</v>
       </c>
-    </row>
-    <row r="58" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A58" s="2" t="str">
+      <c r="K57" s="1"/>
+      <c r="L57" s="1"/>
+      <c r="M57" s="1"/>
+      <c r="N57" s="1"/>
+      <c r="O57" s="1"/>
+    </row>
+    <row r="58" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A58" s="1" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C58" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D58" s="2">
+      <c r="C58" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D58" s="1">
         <v>20260209</v>
       </c>
-      <c r="E58" s="4">
+      <c r="E58" s="2">
         <v>0.44548611111111103</v>
       </c>
-      <c r="F58" s="2">
+      <c r="F58" s="1">
         <v>198.73</v>
       </c>
-      <c r="G58" s="2">
+      <c r="G58" s="1">
         <v>100</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>19873</v>
       </c>
-      <c r="I58" s="2" t="str">
+      <c r="I58" s="1" t="str">
         <f>IF(AND($C58="卖出",SUMIFS($G$2:G58,$A$2:A58,$A58)=0),SUMIFS($H$2:H58,$A$2:A58,$A58,$C$2:C58,"卖出")-SUMIFS($H$2:H58,$A$2:A58,$A58,$C$2:C58,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <f>SUMIFS($G$2:G58,$A$2:A58,$A58)</f>
         <v>700</v>
       </c>
-    </row>
-    <row r="59" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A59" s="2">
+      <c r="K58" s="1"/>
+      <c r="L58" s="1"/>
+      <c r="M58" s="1"/>
+      <c r="N58" s="1"/>
+      <c r="O58" s="1"/>
+    </row>
+    <row r="59" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A59" s="1">
         <v>600584</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B59" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C59" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D59" s="2">
+      <c r="C59" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D59" s="1">
         <v>20260209</v>
       </c>
-      <c r="E59" s="4">
+      <c r="E59" s="2">
         <v>0.43886574074074097</v>
       </c>
-      <c r="F59" s="2">
+      <c r="F59" s="1">
         <v>46.09</v>
       </c>
-      <c r="G59" s="2">
+      <c r="G59" s="1">
         <v>200</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>9218</v>
       </c>
-      <c r="I59" s="2" t="str">
+      <c r="I59" s="1" t="str">
         <f>IF(AND($C59="卖出",SUMIFS($G$2:G59,$A$2:A59,$A59)=0),SUMIFS($H$2:H59,$A$2:A59,$A59,$C$2:C59,"卖出")-SUMIFS($H$2:H59,$A$2:A59,$A59,$C$2:C59,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <f>SUMIFS($G$2:G59,$A$2:A59,$A59)</f>
         <v>700</v>
       </c>
-    </row>
-    <row r="60" spans="1:14" s="2" customFormat="1" ht="20.5" customHeight="1">
-      <c r="A60" s="2" t="str">
+      <c r="K59" s="1"/>
+      <c r="L59" s="1"/>
+      <c r="M59" s="1"/>
+      <c r="N59" s="1"/>
+      <c r="O59" s="1"/>
+    </row>
+    <row r="60" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+      <c r="A60" s="1" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C60" s="2" t="s">
+      <c r="C60" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>20260209</v>
       </c>
-      <c r="E60" s="4">
+      <c r="E60" s="2">
         <v>0.41059027777777801</v>
       </c>
-      <c r="F60" s="2">
+      <c r="F60" s="1">
         <v>192.5</v>
       </c>
-      <c r="G60" s="2">
+      <c r="G60" s="1">
         <v>-200</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>38500</v>
       </c>
-      <c r="I60" s="2" t="str">
+      <c r="I60" s="1" t="str">
         <f>IF(AND($C60="卖出",SUMIFS($G$2:G60,$A$2:A60,$A60)=0),SUMIFS($H$2:H60,$A$2:A60,$A60,$C$2:C60,"卖出")-SUMIFS($H$2:H60,$A$2:A60,$A60,$C$2:C60,"买入"),"")</f>
         <v/>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <f>SUMIFS($G$2:G60,$A$2:A60,$A60)</f>
         <v>500</v>
       </c>
-    </row>
-    <row r="61" spans="1:14" ht="16" customHeight="1">
-      <c r="A61" s="2">
+      <c r="K60" s="1"/>
+      <c r="L60" s="1"/>
+      <c r="M60" s="1"/>
+      <c r="N60" s="1"/>
+      <c r="O60" s="1"/>
+    </row>
+    <row r="61" spans="1:15" ht="16" customHeight="1">
+      <c r="A61" s="1">
         <v>600584</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D61" s="2">
+      <c r="C61" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D61" s="1">
         <v>20260226</v>
       </c>
-      <c r="E61" s="4">
+      <c r="E61" s="2">
         <v>0.54913194444444402</v>
       </c>
-      <c r="F61" s="2">
+      <c r="F61" s="1">
         <v>48.3</v>
       </c>
-      <c r="G61" s="2">
+      <c r="G61" s="1">
         <v>400</v>
       </c>
-      <c r="H61" s="2">
+      <c r="H61" s="1">
         <v>19320</v>
       </c>
-      <c r="J61" s="2">
+      <c r="I61" s="4"/>
+      <c r="J61" s="1">
         <f>SUMIFS($G$2:G61,$A$2:A61,$A61)</f>
         <v>1100</v>
       </c>
-      <c r="K61" s="7" t="s">
+      <c r="K61" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="L61" s="3" t="s">
+      <c r="L61" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M61" s="3" t="s">
+      <c r="M61" s="4" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="62" spans="1:14" ht="60">
-      <c r="A62" s="2" t="str">
+      <c r="N61" s="4"/>
+      <c r="O61" s="1"/>
+    </row>
+    <row r="62" spans="1:15" ht="150">
+      <c r="A62" s="1" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C62" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D62" s="2">
+      <c r="C62" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D62" s="1">
         <v>20260227</v>
       </c>
-      <c r="E62" s="4">
+      <c r="E62" s="2">
         <v>0.40364583333333298</v>
       </c>
-      <c r="F62" s="2">
+      <c r="F62" s="1">
         <v>218.5</v>
       </c>
-      <c r="G62" s="2">
+      <c r="G62" s="1">
         <v>100</v>
       </c>
-      <c r="H62" s="2">
+      <c r="H62" s="1">
         <v>21850</v>
       </c>
-      <c r="J62" s="2">
+      <c r="I62" s="4"/>
+      <c r="J62" s="1">
         <f>SUMIFS($G$2:G62,$A$2:A62,$A62)</f>
         <v>600</v>
       </c>
-      <c r="K62" s="7" t="s">
+      <c r="K62" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="L62" t="s">
+      <c r="L62" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="M62" t="s">
+      <c r="M62" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="63" spans="1:14" ht="77" customHeight="1">
-      <c r="A63" s="2">
+      <c r="N62" s="4"/>
+      <c r="O62" s="1"/>
+    </row>
+    <row r="63" spans="1:15" ht="77" customHeight="1">
+      <c r="A63" s="1">
         <v>600584</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="B63" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C63" s="2" t="s">
+      <c r="C63" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D63" s="2">
+      <c r="D63" s="1">
         <v>20260309</v>
       </c>
-      <c r="E63" s="4">
+      <c r="E63" s="2">
         <v>0.61805555555555602</v>
       </c>
-      <c r="F63" s="2">
+      <c r="F63" s="1">
         <v>45.03</v>
       </c>
-      <c r="G63" s="2">
+      <c r="G63" s="1">
         <v>-600</v>
       </c>
-      <c r="H63" s="2">
+      <c r="H63" s="1">
         <v>27018</v>
       </c>
-      <c r="J63" s="2">
+      <c r="I63" s="4"/>
+      <c r="J63" s="1">
         <f>SUMIFS($G$2:G63,$A$2:A63,$A63)</f>
         <v>500</v>
       </c>
-      <c r="N63" s="7" t="s">
+      <c r="K63" s="4"/>
+      <c r="L63" s="4"/>
+      <c r="M63" s="4"/>
+      <c r="N63" s="5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="64" spans="1:14" ht="105">
-      <c r="A64" s="9" t="s">
+      <c r="O63" s="1"/>
+    </row>
+    <row r="64" spans="1:15" ht="300">
+      <c r="A64" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C64" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D64" s="2">
+      <c r="C64" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D64" s="1">
         <v>22060312</v>
       </c>
-      <c r="E64" s="4">
+      <c r="E64" s="2">
         <v>0.61805555555555602</v>
       </c>
-      <c r="F64" s="2">
+      <c r="F64" s="1">
         <v>220</v>
       </c>
-      <c r="G64" s="2">
+      <c r="G64" s="1">
         <v>100</v>
       </c>
-      <c r="H64" s="2">
+      <c r="H64" s="1">
         <v>22000</v>
       </c>
-      <c r="I64" s="2"/>
-      <c r="J64" s="2">
+      <c r="I64" s="1"/>
+      <c r="J64" s="1">
         <v>700</v>
       </c>
-      <c r="K64" s="7" t="s">
+      <c r="K64" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="M64" t="s">
+      <c r="L64" s="4"/>
+      <c r="M64" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="65" spans="1:15" ht="45">
-      <c r="A65" s="9" t="s">
+      <c r="N64" s="4"/>
+      <c r="O64" s="1"/>
+    </row>
+    <row r="65" spans="1:15" ht="150">
+      <c r="A65" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C65" s="2" t="s">
+      <c r="C65" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>22060316</v>
       </c>
-      <c r="E65" s="4">
+      <c r="E65" s="2">
         <v>0.61805555555555602</v>
       </c>
-      <c r="F65" s="2">
+      <c r="F65" s="1">
         <v>208.14</v>
       </c>
-      <c r="G65" s="2">
+      <c r="G65" s="1">
         <v>700</v>
       </c>
-      <c r="H65" s="2">
+      <c r="H65" s="1">
         <v>145698</v>
       </c>
-      <c r="J65" s="2">
+      <c r="I65" s="4"/>
+      <c r="J65" s="1">
         <v>0</v>
       </c>
-      <c r="N65" s="7" t="s">
+      <c r="K65" s="4"/>
+      <c r="L65" s="4"/>
+      <c r="M65" s="4"/>
+      <c r="N65" s="5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="66" spans="1:15" ht="45">
-      <c r="A66" s="2">
+      <c r="O65" s="1"/>
+    </row>
+    <row r="66" spans="1:15" ht="150">
+      <c r="A66" s="1">
         <v>600584</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="C66" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>22060316</v>
       </c>
-      <c r="E66" s="4">
+      <c r="E66" s="2">
         <v>0.61805555555555602</v>
       </c>
-      <c r="F66" s="2">
+      <c r="F66" s="1">
         <v>45.7</v>
       </c>
-      <c r="G66" s="2">
+      <c r="G66" s="1">
         <v>500</v>
       </c>
-      <c r="H66" s="2">
+      <c r="H66" s="1">
         <v>22850</v>
       </c>
-      <c r="I66" s="2"/>
-      <c r="J66" s="2">
+      <c r="I66" s="1"/>
+      <c r="J66" s="1">
         <v>0</v>
       </c>
-      <c r="N66" s="7" t="s">
+      <c r="K66" s="4"/>
+      <c r="L66" s="4"/>
+      <c r="M66" s="4"/>
+      <c r="N66" s="5" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="67" spans="1:15" ht="45">
-      <c r="A67" s="9" t="s">
+      <c r="O66" s="1"/>
+    </row>
+    <row r="67" spans="1:15" ht="100">
+      <c r="A67" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C67" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D67" s="2">
+      <c r="C67" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D67" s="1">
         <v>20260318</v>
       </c>
-      <c r="E67" s="4">
+      <c r="E67" s="2">
         <v>0.61805555555555602</v>
       </c>
-      <c r="F67" s="2">
+      <c r="F67" s="1">
         <v>220.18299999999999</v>
       </c>
-      <c r="G67" s="2">
+      <c r="G67" s="1">
         <v>100</v>
       </c>
-      <c r="H67" s="2">
+      <c r="H67" s="1">
         <v>22018</v>
       </c>
-      <c r="I67" s="2"/>
-      <c r="J67" s="2">
+      <c r="I67" s="1"/>
+      <c r="J67" s="1">
         <v>100</v>
       </c>
-      <c r="K67" s="7" t="s">
+      <c r="K67" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="M67" t="s">
+      <c r="L67" s="4"/>
+      <c r="M67" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="68" spans="1:15" ht="45">
-      <c r="A68" s="2">
+      <c r="N67" s="4"/>
+      <c r="O67" s="1"/>
+    </row>
+    <row r="68" spans="1:15" ht="100">
+      <c r="A68" s="1">
         <v>600487</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C68" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D68" s="2">
+      <c r="C68" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D68" s="1">
         <v>20260318</v>
       </c>
-      <c r="E68" s="4">
+      <c r="E68" s="2">
         <v>0.61805555555555602</v>
       </c>
-      <c r="F68" s="2">
+      <c r="F68" s="1">
         <v>44.53</v>
       </c>
-      <c r="G68" s="2">
+      <c r="G68" s="1">
         <v>600</v>
       </c>
-      <c r="H68" s="2">
+      <c r="H68" s="1">
         <v>26708</v>
       </c>
-      <c r="J68" s="2">
+      <c r="I68" s="4"/>
+      <c r="J68" s="1">
         <v>600</v>
       </c>
-      <c r="K68" s="7" t="s">
+      <c r="K68" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="M68" s="3" t="s">
+      <c r="L68" s="4"/>
+      <c r="M68" s="4" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="69" spans="1:15" ht="75">
-      <c r="A69" s="9" t="s">
+      <c r="N68" s="4"/>
+      <c r="O68" s="1"/>
+    </row>
+    <row r="69" spans="1:15" ht="225">
+      <c r="A69" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C69" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D69" s="2">
+      <c r="C69" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D69" s="1">
         <v>20260319</v>
       </c>
-      <c r="E69" s="4">
+      <c r="E69" s="2">
         <v>0.41458333333333303</v>
       </c>
-      <c r="F69" s="2">
+      <c r="F69" s="1">
         <v>214.5</v>
       </c>
-      <c r="G69" s="2">
+      <c r="G69" s="1">
         <v>100</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>21459</v>
       </c>
-      <c r="J69" s="2">
+      <c r="I69" s="4"/>
+      <c r="J69" s="1">
         <v>200</v>
       </c>
-      <c r="K69" s="7" t="s">
+      <c r="K69" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="70" spans="1:15" ht="75">
-      <c r="A70" s="9" t="s">
+      <c r="L69" s="4"/>
+      <c r="M69" s="4"/>
+      <c r="N69" s="4"/>
+      <c r="O69" s="1"/>
+    </row>
+    <row r="70" spans="1:15" ht="175">
+      <c r="A70" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C70" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D70" s="2">
+      <c r="C70" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D70" s="1">
         <v>20260319</v>
       </c>
-      <c r="E70" s="4">
+      <c r="E70" s="2">
         <v>0.625</v>
       </c>
-      <c r="F70" s="2">
+      <c r="F70" s="1">
         <v>211.1</v>
       </c>
-      <c r="G70" s="2">
+      <c r="G70" s="1">
         <v>100</v>
       </c>
-      <c r="H70" s="2">
+      <c r="H70" s="1">
         <v>21110</v>
       </c>
-      <c r="J70" s="2">
+      <c r="I70" s="4"/>
+      <c r="J70" s="1">
         <v>300</v>
       </c>
-      <c r="K70" s="7" t="s">
+      <c r="K70" s="5" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="71" spans="1:15" ht="30">
-      <c r="A71" s="2">
+      <c r="L70" s="4"/>
+      <c r="M70" s="4"/>
+      <c r="N70" s="4"/>
+      <c r="O70" s="1"/>
+    </row>
+    <row r="71" spans="1:15" ht="100">
+      <c r="A71" s="1">
         <v>600487</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C71" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D71" s="2">
+      <c r="C71" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D71" s="1">
         <v>20260320</v>
       </c>
-      <c r="E71" s="4">
+      <c r="E71" s="2">
         <v>0.42499999999999999</v>
       </c>
-      <c r="F71" s="2">
+      <c r="F71" s="1">
         <v>45.07</v>
       </c>
-      <c r="G71" s="2">
+      <c r="G71" s="1">
         <v>600</v>
       </c>
-      <c r="H71" s="2">
+      <c r="H71" s="1">
         <v>27042</v>
       </c>
-      <c r="J71" s="2">
+      <c r="I71" s="4"/>
+      <c r="J71" s="1">
         <v>1200</v>
       </c>
-      <c r="K71" s="7" t="s">
+      <c r="K71" s="5" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="72" spans="1:15" ht="45">
-      <c r="A72" s="2">
+      <c r="L71" s="4"/>
+      <c r="M71" s="4"/>
+      <c r="N71" s="4"/>
+      <c r="O71" s="1"/>
+    </row>
+    <row r="72" spans="1:15" ht="125">
+      <c r="A72" s="1">
         <v>600487</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C72" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D72" s="2">
+      <c r="C72" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D72" s="1">
         <v>20260324</v>
       </c>
-      <c r="E72" s="4">
+      <c r="E72" s="2">
         <v>0.61666666666666703</v>
       </c>
-      <c r="F72" s="2">
+      <c r="F72" s="1">
         <v>44</v>
       </c>
-      <c r="G72" s="2">
+      <c r="G72" s="1">
         <v>300</v>
       </c>
-      <c r="H72" s="2">
+      <c r="H72" s="1">
         <v>13200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="I72" s="4"/>
+      <c r="J72" s="1">
         <v>1500</v>
       </c>
-      <c r="K72" s="7" t="s">
+      <c r="K72" s="5" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="73" spans="1:15" ht="60">
-      <c r="A73" s="9" t="s">
+      <c r="L72" s="4"/>
+      <c r="M72" s="4"/>
+      <c r="N72" s="4"/>
+      <c r="O72" s="1"/>
+    </row>
+    <row r="73" spans="1:15" ht="175">
+      <c r="A73" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C73" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D73" s="2">
+      <c r="C73" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D73" s="1">
         <v>20260325</v>
       </c>
-      <c r="E73" s="4">
+      <c r="E73" s="2">
         <v>0.40902777777777799</v>
       </c>
-      <c r="F73" s="2">
+      <c r="F73" s="1">
         <v>213.77</v>
       </c>
-      <c r="G73" s="2">
+      <c r="G73" s="1">
         <v>100</v>
       </c>
-      <c r="H73" s="2">
+      <c r="H73" s="1">
         <v>21377</v>
       </c>
-      <c r="J73" s="2">
+      <c r="I73" s="4"/>
+      <c r="J73" s="1">
         <v>400</v>
       </c>
-      <c r="K73" s="7" t="s">
+      <c r="K73" s="5" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="74" spans="1:15" ht="105">
-      <c r="A74" s="9" t="s">
+      <c r="L73" s="4"/>
+      <c r="M73" s="4"/>
+      <c r="N73" s="4"/>
+      <c r="O73" s="1"/>
+    </row>
+    <row r="74" spans="1:15" ht="275">
+      <c r="A74" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C74" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D74" s="2">
+      <c r="C74" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D74" s="1">
         <v>20260327</v>
       </c>
-      <c r="E74" s="4">
+      <c r="E74" s="2">
         <v>0.44166666666666698</v>
       </c>
-      <c r="F74" s="2">
+      <c r="F74" s="1">
         <v>208</v>
       </c>
-      <c r="G74" s="2">
+      <c r="G74" s="1">
         <v>100</v>
       </c>
-      <c r="H74" s="2">
+      <c r="H74" s="1">
         <v>20800</v>
       </c>
-      <c r="J74" s="2">
+      <c r="I74" s="4"/>
+      <c r="J74" s="1">
         <v>500</v>
       </c>
-      <c r="K74" s="7" t="s">
+      <c r="K74" s="5" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="75" spans="1:15" ht="285">
+      <c r="L74" s="4"/>
+      <c r="M74" s="4"/>
+      <c r="N74" s="4"/>
+      <c r="O74" s="1"/>
+    </row>
+    <row r="75" spans="1:15" ht="409.6">
       <c r="A75" s="8">
         <v>600487</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B75" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="C75" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>20260327</v>
       </c>
-      <c r="E75" s="4">
+      <c r="E75" s="2">
         <v>0.41041666666666698</v>
       </c>
-      <c r="F75" s="2">
+      <c r="F75" s="1">
         <v>47.08</v>
       </c>
-      <c r="G75" s="2">
+      <c r="G75" s="1">
         <v>1500</v>
       </c>
-      <c r="H75" s="2">
+      <c r="H75" s="1">
         <v>70620</v>
       </c>
-      <c r="I75" s="2" t="s">
+      <c r="I75" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>0</v>
       </c>
-      <c r="M75" s="7" t="s">
+      <c r="K75" s="4"/>
+      <c r="L75" s="4"/>
+      <c r="M75" s="5" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="76" spans="1:15" ht="60">
-      <c r="A76" s="9" t="s">
+      <c r="N75" s="4"/>
+      <c r="O75" s="1"/>
+    </row>
+    <row r="76" spans="1:15" ht="175">
+      <c r="A76" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C76" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D76" s="2">
+      <c r="C76" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D76" s="1">
         <v>20260331</v>
       </c>
-      <c r="E76" s="4">
+      <c r="E76" s="2">
         <v>0.56597222222222199</v>
       </c>
-      <c r="F76" s="2">
+      <c r="F76" s="1">
         <v>200.5</v>
       </c>
-      <c r="G76" s="2">
+      <c r="G76" s="1">
         <v>100</v>
       </c>
-      <c r="H76" s="2">
+      <c r="H76" s="1">
         <v>20050</v>
       </c>
-      <c r="J76" s="2">
+      <c r="I76" s="4"/>
+      <c r="J76" s="1">
         <v>600</v>
       </c>
-      <c r="K76" s="7" t="s">
+      <c r="K76" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="O76" s="12"/>
-    </row>
-    <row r="77" spans="1:15" ht="135">
-      <c r="A77" s="9" t="s">
+      <c r="L76" s="4"/>
+      <c r="M76" s="4"/>
+      <c r="N76" s="4"/>
+      <c r="O76" s="9"/>
+    </row>
+    <row r="77" spans="1:15" ht="400">
+      <c r="A77" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B77" s="11" t="s">
+      <c r="B77" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C77" s="2" t="s">
+      <c r="C77" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>20260408</v>
       </c>
-      <c r="E77" s="4">
+      <c r="E77" s="2">
         <v>0.61805555555555558</v>
       </c>
-      <c r="F77" s="2">
+      <c r="F77" s="1">
         <v>205.85</v>
       </c>
-      <c r="G77" s="2">
+      <c r="G77" s="1">
         <v>300</v>
       </c>
-      <c r="H77" s="2">
+      <c r="H77" s="1">
         <v>61755</v>
       </c>
-      <c r="J77" s="2">
+      <c r="I77" s="4"/>
+      <c r="J77" s="1">
         <v>300</v>
       </c>
-      <c r="N77" s="10"/>
-      <c r="O77" s="12" t="s">
+      <c r="K77" s="4"/>
+      <c r="L77" s="4"/>
+      <c r="M77" s="4"/>
+      <c r="N77" s="4"/>
+      <c r="O77" s="9" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="78" spans="1:15" ht="75">
-      <c r="A78" s="9" t="s">
+    <row r="78" spans="1:15" ht="200">
+      <c r="A78" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B78" s="11" t="s">
+      <c r="B78" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="C78" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>20260408</v>
       </c>
-      <c r="E78" s="4">
+      <c r="E78" s="2">
         <v>0.61805555555555558</v>
       </c>
-      <c r="F78" s="2">
+      <c r="F78" s="1">
         <v>110.15</v>
       </c>
-      <c r="G78" s="2">
+      <c r="G78" s="1">
         <v>200</v>
       </c>
-      <c r="H78" s="2">
+      <c r="H78" s="1">
         <v>22030</v>
       </c>
-      <c r="J78" s="2">
+      <c r="I78" s="4"/>
+      <c r="J78" s="1">
         <v>200</v>
       </c>
-      <c r="K78" s="13" t="s">
+      <c r="K78" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="79" spans="1:15" ht="90">
-      <c r="A79" s="9" t="s">
+      <c r="L78" s="4"/>
+      <c r="M78" s="4"/>
+      <c r="N78" s="4"/>
+      <c r="O78" s="1"/>
+    </row>
+    <row r="79" spans="1:15" ht="250">
+      <c r="A79" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B79" s="11" t="s">
+      <c r="B79" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="C79" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>20260408</v>
       </c>
-      <c r="E79" s="4">
+      <c r="E79" s="2">
         <v>0.61805555555555558</v>
       </c>
-      <c r="F79" s="2">
+      <c r="F79" s="1">
         <v>98.26</v>
       </c>
-      <c r="G79" s="2">
+      <c r="G79" s="1">
         <v>200</v>
       </c>
-      <c r="H79" s="2">
+      <c r="H79" s="1">
         <v>19652</v>
       </c>
-      <c r="J79" s="2">
+      <c r="I79" s="4"/>
+      <c r="J79" s="1">
         <v>200</v>
       </c>
-      <c r="K79" s="13" t="s">
+      <c r="K79" s="5" t="s">
         <v>73</v>
+      </c>
+      <c r="L79" s="4"/>
+      <c r="M79" s="4"/>
+      <c r="N79" s="4"/>
+      <c r="O79" s="1"/>
+    </row>
+    <row r="80" spans="1:15" ht="325">
+      <c r="A80" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D80" s="1">
+        <v>20260409</v>
+      </c>
+      <c r="E80" s="2">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="F80" s="1">
+        <v>116</v>
+      </c>
+      <c r="G80" s="1">
+        <v>200</v>
+      </c>
+      <c r="H80" s="1">
+        <v>23200</v>
+      </c>
+      <c r="I80" s="4"/>
+      <c r="J80" s="1">
+        <v>400</v>
+      </c>
+      <c r="K80" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="L80" s="4"/>
+      <c r="M80" s="4"/>
+      <c r="N80" s="4"/>
+      <c r="O80" s="1"/>
+    </row>
+    <row r="81" spans="1:15" ht="325">
+      <c r="A81" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D81" s="1">
+        <v>20260409</v>
+      </c>
+      <c r="E81" s="2">
+        <v>0.4236111111111111</v>
+      </c>
+      <c r="F81" s="1">
+        <v>107.07</v>
+      </c>
+      <c r="G81" s="1">
+        <v>200</v>
+      </c>
+      <c r="H81" s="1">
+        <v>21414</v>
+      </c>
+      <c r="I81" s="4"/>
+      <c r="J81" s="1">
+        <v>400</v>
+      </c>
+      <c r="K81" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="L81" s="4"/>
+      <c r="M81" s="4"/>
+      <c r="N81" s="4"/>
+      <c r="O81" s="1"/>
+    </row>
+    <row r="82" spans="1:15" ht="409.6">
+      <c r="A82" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D82" s="1">
+        <v>20260408</v>
+      </c>
+      <c r="E82" s="2">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="F82" s="1">
+        <v>202.5</v>
+      </c>
+      <c r="G82" s="1">
+        <v>200</v>
+      </c>
+      <c r="H82" s="1">
+        <v>40500</v>
+      </c>
+      <c r="I82" s="4"/>
+      <c r="J82" s="1">
+        <v>100</v>
+      </c>
+      <c r="K82" s="4"/>
+      <c r="L82" s="4"/>
+      <c r="M82" s="4"/>
+      <c r="N82" s="4"/>
+      <c r="O82" s="9" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J76" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-04-13 12:04:30
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28D497D5-E0EE-A04F-83DE-4B647EAE97A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4243FA-DE93-8546-ABDE-D87CBCA76292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="80">
   <si>
     <t>证券代码</t>
   </si>
@@ -294,6 +294,20 @@
   </si>
   <si>
     <t>思源电气最近的表现疲软虽然今天是4000家个股下跌，但相对于板块来说这几天的表现远远低于整体板块，伴随着缩量可以解读成买盘萎缩，卖盘也不强劲，预计会在这个箱体内横盘一段时间或者沿着60日支撑震荡，但短期出现行情的概率太低了，之前认为可能是洗盘，但现在来看更像是出货，为了规避风险同时尽可能博一点反弹预期 留了1层底仓 若持续低迷跌破60日均线 可以清仓</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>当日思源电气低开高走 一改往日颓势 上午我并没有急于追涨 因为想等大众的
+fomo情绪过去之后再入场 到了13:08的时候思源电气依然走强甚至拉高 这时候我认为前几日的杀跌只是洗盘 果断追涨买入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>开盘之后思源电气大幅杀跌 又回到了前几日的低点 这并不符合之前的假设 如果是洗盘 今天不应该是这样杀跌 当然这依然可能是洗盘 我不能排除这样的可能性 但我想说的是自己没做好的一个点 ，那就是太急于下判断 上仓位了 这里我太鲁莽了 应该等到突破阻力位213进行确认再加仓的 我不知道这里到底是牛回了 还是拉高出货 那这个时候就是等价格确认是最好的 今天清仓的逻辑我也说不清楚 感觉是自己在很快的想要摆脱这种亏损 有种在赌气的感觉 操作不理性了 伴随着自己在cpo板块还有盈利今天总体是正盈利的 所以对割肉没有什么心理上的痛觉 只有对这个股票的失望（好奇怪 我不应该有这样的情绪的 为什么要对它失望 它不清楚我买了它 也没有涨的义务 我是来赚钱的 而不是来产生感情的 我感觉自己确实在一只股票上耗费了太大的感情 或者说精力当他不能为我赚钱或者有理由证明不强势的时候我应该离开 而不是死守着逻辑 或者它曾经给我带来过盈利作为借口而抓着不放</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">开盘强势 等fomo情绪退潮在下方接了个114的价位但我觉得接的还是太早了 应该在10点后等待均线确认后加仓 这个时候也消除了大部分开盘期间带来的噪音 现在发现在这种市场情况下 顺势而为 浮盈加仓才是一个让我觉得舒服的交易方式 之前一直跌一直补的做法太煎熬了 我感觉自己也不是一个很坚定的人 这套方法貌似不适合现在的我 
+</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -375,7 +389,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -413,6 +427,9 @@
     </xf>
     <xf numFmtId="21" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -902,7 +919,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O82"/>
+  <dimension ref="A1:O357"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="22.1640625" style="3" bestFit="1" customWidth="1"/>
@@ -916,8 +933,8 @@
     <col min="11" max="11" width="43.83203125" style="10" customWidth="1"/>
     <col min="12" max="12" width="27.6640625" style="10" customWidth="1"/>
     <col min="13" max="13" width="49" style="10" customWidth="1"/>
-    <col min="14" max="14" width="40.5" style="10" customWidth="1"/>
-    <col min="15" max="15" width="32.6640625" style="6" customWidth="1"/>
+    <col min="14" max="14" width="255.83203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="39.1640625" style="6" bestFit="1" customWidth="1"/>
     <col min="16" max="16384" width="10.33203125" style="6"/>
   </cols>
   <sheetData>
@@ -4126,6 +4143,918 @@
         <v>76</v>
       </c>
     </row>
+    <row r="83" spans="1:15" ht="175">
+      <c r="A83" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D83" s="1">
+        <v>20260410</v>
+      </c>
+      <c r="E83" s="2">
+        <v>0.54722222222222228</v>
+      </c>
+      <c r="F83" s="1">
+        <v>211.9</v>
+      </c>
+      <c r="G83" s="1">
+        <v>100</v>
+      </c>
+      <c r="H83" s="1">
+        <v>21190</v>
+      </c>
+      <c r="J83" s="1">
+        <v>200</v>
+      </c>
+      <c r="K83" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15" ht="125">
+      <c r="A84" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D84" s="1">
+        <v>20260413</v>
+      </c>
+      <c r="E84" s="2">
+        <v>0.40208333333333335</v>
+      </c>
+      <c r="F84" s="1">
+        <v>199.36</v>
+      </c>
+      <c r="G84" s="1">
+        <v>200</v>
+      </c>
+      <c r="H84" s="1">
+        <v>39872</v>
+      </c>
+      <c r="J84" s="1">
+        <v>0</v>
+      </c>
+      <c r="N84" s="14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="85" spans="1:15" ht="300">
+      <c r="A85" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D85" s="1">
+        <v>202604013</v>
+      </c>
+      <c r="E85" s="2">
+        <v>0.40486111111111112</v>
+      </c>
+      <c r="F85" s="1">
+        <v>114</v>
+      </c>
+      <c r="G85" s="1">
+        <v>200</v>
+      </c>
+      <c r="H85" s="1">
+        <v>22800</v>
+      </c>
+      <c r="J85" s="1">
+        <v>600</v>
+      </c>
+      <c r="K85" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="86" spans="1:15" ht="24">
+      <c r="C86" s="1"/>
+    </row>
+    <row r="87" spans="1:15" ht="24">
+      <c r="C87" s="1"/>
+    </row>
+    <row r="88" spans="1:15" ht="24">
+      <c r="C88" s="1"/>
+    </row>
+    <row r="89" spans="1:15" ht="24">
+      <c r="C89" s="1"/>
+    </row>
+    <row r="90" spans="1:15" ht="24">
+      <c r="C90" s="1"/>
+    </row>
+    <row r="91" spans="1:15" ht="24">
+      <c r="C91" s="1"/>
+    </row>
+    <row r="92" spans="1:15" ht="24">
+      <c r="C92" s="1"/>
+    </row>
+    <row r="93" spans="1:15" ht="24">
+      <c r="C93" s="1"/>
+    </row>
+    <row r="94" spans="1:15" ht="24">
+      <c r="C94" s="1"/>
+    </row>
+    <row r="95" spans="1:15" ht="24">
+      <c r="C95" s="1"/>
+    </row>
+    <row r="96" spans="1:15" ht="24">
+      <c r="C96" s="1"/>
+    </row>
+    <row r="97" spans="3:3" ht="24">
+      <c r="C97" s="1"/>
+    </row>
+    <row r="98" spans="3:3" ht="24">
+      <c r="C98" s="1"/>
+    </row>
+    <row r="99" spans="3:3" ht="24">
+      <c r="C99" s="1"/>
+    </row>
+    <row r="100" spans="3:3" ht="24">
+      <c r="C100" s="1"/>
+    </row>
+    <row r="101" spans="3:3" ht="24">
+      <c r="C101" s="1"/>
+    </row>
+    <row r="102" spans="3:3" ht="24">
+      <c r="C102" s="1"/>
+    </row>
+    <row r="103" spans="3:3" ht="24">
+      <c r="C103" s="1"/>
+    </row>
+    <row r="104" spans="3:3" ht="24">
+      <c r="C104" s="1"/>
+    </row>
+    <row r="105" spans="3:3" ht="24">
+      <c r="C105" s="1"/>
+    </row>
+    <row r="106" spans="3:3" ht="24">
+      <c r="C106" s="1"/>
+    </row>
+    <row r="107" spans="3:3" ht="24">
+      <c r="C107" s="1"/>
+    </row>
+    <row r="108" spans="3:3" ht="24">
+      <c r="C108" s="1"/>
+    </row>
+    <row r="109" spans="3:3" ht="24">
+      <c r="C109" s="1"/>
+    </row>
+    <row r="110" spans="3:3" ht="24">
+      <c r="C110" s="1"/>
+    </row>
+    <row r="111" spans="3:3" ht="24">
+      <c r="C111" s="1"/>
+    </row>
+    <row r="112" spans="3:3" ht="24">
+      <c r="C112" s="1"/>
+    </row>
+    <row r="113" spans="3:3" ht="24">
+      <c r="C113" s="1"/>
+    </row>
+    <row r="114" spans="3:3" ht="24">
+      <c r="C114" s="1"/>
+    </row>
+    <row r="115" spans="3:3" ht="24">
+      <c r="C115" s="1"/>
+    </row>
+    <row r="116" spans="3:3" ht="24">
+      <c r="C116" s="1"/>
+    </row>
+    <row r="117" spans="3:3" ht="24">
+      <c r="C117" s="1"/>
+    </row>
+    <row r="118" spans="3:3" ht="24">
+      <c r="C118" s="1"/>
+    </row>
+    <row r="119" spans="3:3" ht="24">
+      <c r="C119" s="1"/>
+    </row>
+    <row r="120" spans="3:3" ht="24">
+      <c r="C120" s="1"/>
+    </row>
+    <row r="121" spans="3:3" ht="24">
+      <c r="C121" s="1"/>
+    </row>
+    <row r="122" spans="3:3" ht="24">
+      <c r="C122" s="1"/>
+    </row>
+    <row r="123" spans="3:3" ht="24">
+      <c r="C123" s="1"/>
+    </row>
+    <row r="124" spans="3:3" ht="24">
+      <c r="C124" s="1"/>
+    </row>
+    <row r="125" spans="3:3" ht="24">
+      <c r="C125" s="1"/>
+    </row>
+    <row r="126" spans="3:3" ht="24">
+      <c r="C126" s="1"/>
+    </row>
+    <row r="127" spans="3:3" ht="24">
+      <c r="C127" s="1"/>
+    </row>
+    <row r="128" spans="3:3" ht="24">
+      <c r="C128" s="1"/>
+    </row>
+    <row r="129" spans="3:3" ht="24">
+      <c r="C129" s="1"/>
+    </row>
+    <row r="130" spans="3:3" ht="24">
+      <c r="C130" s="1"/>
+    </row>
+    <row r="131" spans="3:3" ht="24">
+      <c r="C131" s="1"/>
+    </row>
+    <row r="132" spans="3:3" ht="24">
+      <c r="C132" s="1"/>
+    </row>
+    <row r="133" spans="3:3" ht="24">
+      <c r="C133" s="1"/>
+    </row>
+    <row r="134" spans="3:3" ht="24">
+      <c r="C134" s="1"/>
+    </row>
+    <row r="135" spans="3:3" ht="24">
+      <c r="C135" s="1"/>
+    </row>
+    <row r="136" spans="3:3" ht="24">
+      <c r="C136" s="1"/>
+    </row>
+    <row r="137" spans="3:3" ht="24">
+      <c r="C137" s="1"/>
+    </row>
+    <row r="138" spans="3:3" ht="24">
+      <c r="C138" s="1"/>
+    </row>
+    <row r="139" spans="3:3" ht="24">
+      <c r="C139" s="1"/>
+    </row>
+    <row r="140" spans="3:3" ht="24">
+      <c r="C140" s="1"/>
+    </row>
+    <row r="141" spans="3:3" ht="24">
+      <c r="C141" s="1"/>
+    </row>
+    <row r="142" spans="3:3" ht="24">
+      <c r="C142" s="1"/>
+    </row>
+    <row r="143" spans="3:3" ht="24">
+      <c r="C143" s="1"/>
+    </row>
+    <row r="144" spans="3:3" ht="24">
+      <c r="C144" s="1"/>
+    </row>
+    <row r="145" spans="3:3" ht="24">
+      <c r="C145" s="1"/>
+    </row>
+    <row r="146" spans="3:3" ht="24">
+      <c r="C146" s="1"/>
+    </row>
+    <row r="147" spans="3:3" ht="24">
+      <c r="C147" s="1"/>
+    </row>
+    <row r="148" spans="3:3" ht="24">
+      <c r="C148" s="1"/>
+    </row>
+    <row r="149" spans="3:3" ht="24">
+      <c r="C149" s="1"/>
+    </row>
+    <row r="150" spans="3:3" ht="24">
+      <c r="C150" s="1"/>
+    </row>
+    <row r="151" spans="3:3" ht="24">
+      <c r="C151" s="1"/>
+    </row>
+    <row r="152" spans="3:3" ht="24">
+      <c r="C152" s="1"/>
+    </row>
+    <row r="153" spans="3:3" ht="24">
+      <c r="C153" s="1"/>
+    </row>
+    <row r="154" spans="3:3" ht="24">
+      <c r="C154" s="1"/>
+    </row>
+    <row r="155" spans="3:3" ht="24">
+      <c r="C155" s="1"/>
+    </row>
+    <row r="156" spans="3:3" ht="24">
+      <c r="C156" s="1"/>
+    </row>
+    <row r="157" spans="3:3" ht="24">
+      <c r="C157" s="1"/>
+    </row>
+    <row r="158" spans="3:3" ht="24">
+      <c r="C158" s="1"/>
+    </row>
+    <row r="159" spans="3:3" ht="24">
+      <c r="C159" s="1"/>
+    </row>
+    <row r="160" spans="3:3" ht="24">
+      <c r="C160" s="1"/>
+    </row>
+    <row r="161" spans="3:3" ht="24">
+      <c r="C161" s="1"/>
+    </row>
+    <row r="162" spans="3:3" ht="24">
+      <c r="C162" s="1"/>
+    </row>
+    <row r="163" spans="3:3" ht="24">
+      <c r="C163" s="1"/>
+    </row>
+    <row r="164" spans="3:3" ht="24">
+      <c r="C164" s="1"/>
+    </row>
+    <row r="165" spans="3:3" ht="24">
+      <c r="C165" s="1"/>
+    </row>
+    <row r="166" spans="3:3" ht="24">
+      <c r="C166" s="1"/>
+    </row>
+    <row r="167" spans="3:3" ht="24">
+      <c r="C167" s="1"/>
+    </row>
+    <row r="168" spans="3:3" ht="24">
+      <c r="C168" s="1"/>
+    </row>
+    <row r="169" spans="3:3" ht="24">
+      <c r="C169" s="1"/>
+    </row>
+    <row r="170" spans="3:3" ht="24">
+      <c r="C170" s="1"/>
+    </row>
+    <row r="171" spans="3:3" ht="24">
+      <c r="C171" s="1"/>
+    </row>
+    <row r="172" spans="3:3" ht="24">
+      <c r="C172" s="1"/>
+    </row>
+    <row r="173" spans="3:3" ht="24">
+      <c r="C173" s="1"/>
+    </row>
+    <row r="174" spans="3:3" ht="24">
+      <c r="C174" s="1"/>
+    </row>
+    <row r="175" spans="3:3" ht="24">
+      <c r="C175" s="1"/>
+    </row>
+    <row r="176" spans="3:3" ht="24">
+      <c r="C176" s="1"/>
+    </row>
+    <row r="177" spans="3:3" ht="24">
+      <c r="C177" s="1"/>
+    </row>
+    <row r="178" spans="3:3" ht="24">
+      <c r="C178" s="1"/>
+    </row>
+    <row r="179" spans="3:3" ht="24">
+      <c r="C179" s="1"/>
+    </row>
+    <row r="180" spans="3:3" ht="24">
+      <c r="C180" s="1"/>
+    </row>
+    <row r="181" spans="3:3" ht="24">
+      <c r="C181" s="1"/>
+    </row>
+    <row r="182" spans="3:3" ht="24">
+      <c r="C182" s="1"/>
+    </row>
+    <row r="183" spans="3:3" ht="24">
+      <c r="C183" s="1"/>
+    </row>
+    <row r="184" spans="3:3" ht="24">
+      <c r="C184" s="1"/>
+    </row>
+    <row r="185" spans="3:3" ht="24">
+      <c r="C185" s="1"/>
+    </row>
+    <row r="186" spans="3:3" ht="24">
+      <c r="C186" s="1"/>
+    </row>
+    <row r="187" spans="3:3" ht="24">
+      <c r="C187" s="1"/>
+    </row>
+    <row r="188" spans="3:3" ht="24">
+      <c r="C188" s="1"/>
+    </row>
+    <row r="189" spans="3:3" ht="24">
+      <c r="C189" s="1"/>
+    </row>
+    <row r="190" spans="3:3" ht="24">
+      <c r="C190" s="1"/>
+    </row>
+    <row r="191" spans="3:3" ht="24">
+      <c r="C191" s="1"/>
+    </row>
+    <row r="192" spans="3:3" ht="24">
+      <c r="C192" s="1"/>
+    </row>
+    <row r="193" spans="3:3" ht="24">
+      <c r="C193" s="1"/>
+    </row>
+    <row r="194" spans="3:3" ht="24">
+      <c r="C194" s="1"/>
+    </row>
+    <row r="195" spans="3:3" ht="24">
+      <c r="C195" s="1"/>
+    </row>
+    <row r="196" spans="3:3" ht="24">
+      <c r="C196" s="1"/>
+    </row>
+    <row r="197" spans="3:3" ht="24">
+      <c r="C197" s="1"/>
+    </row>
+    <row r="198" spans="3:3" ht="24">
+      <c r="C198" s="1"/>
+    </row>
+    <row r="199" spans="3:3" ht="24">
+      <c r="C199" s="1"/>
+    </row>
+    <row r="200" spans="3:3" ht="24">
+      <c r="C200" s="1"/>
+    </row>
+    <row r="201" spans="3:3" ht="24">
+      <c r="C201" s="1"/>
+    </row>
+    <row r="202" spans="3:3" ht="24">
+      <c r="C202" s="1"/>
+    </row>
+    <row r="203" spans="3:3" ht="24">
+      <c r="C203" s="1"/>
+    </row>
+    <row r="204" spans="3:3" ht="24">
+      <c r="C204" s="1"/>
+    </row>
+    <row r="205" spans="3:3" ht="24">
+      <c r="C205" s="1"/>
+    </row>
+    <row r="206" spans="3:3" ht="24">
+      <c r="C206" s="1"/>
+    </row>
+    <row r="207" spans="3:3" ht="24">
+      <c r="C207" s="1"/>
+    </row>
+    <row r="208" spans="3:3" ht="24">
+      <c r="C208" s="1"/>
+    </row>
+    <row r="209" spans="3:3" ht="24">
+      <c r="C209" s="1"/>
+    </row>
+    <row r="210" spans="3:3" ht="24">
+      <c r="C210" s="1"/>
+    </row>
+    <row r="211" spans="3:3" ht="24">
+      <c r="C211" s="1"/>
+    </row>
+    <row r="212" spans="3:3" ht="24">
+      <c r="C212" s="1"/>
+    </row>
+    <row r="213" spans="3:3" ht="24">
+      <c r="C213" s="1"/>
+    </row>
+    <row r="214" spans="3:3" ht="24">
+      <c r="C214" s="1"/>
+    </row>
+    <row r="215" spans="3:3" ht="24">
+      <c r="C215" s="1"/>
+    </row>
+    <row r="216" spans="3:3" ht="24">
+      <c r="C216" s="1"/>
+    </row>
+    <row r="217" spans="3:3" ht="24">
+      <c r="C217" s="1"/>
+    </row>
+    <row r="218" spans="3:3" ht="24">
+      <c r="C218" s="1"/>
+    </row>
+    <row r="219" spans="3:3" ht="24">
+      <c r="C219" s="1"/>
+    </row>
+    <row r="220" spans="3:3" ht="24">
+      <c r="C220" s="1"/>
+    </row>
+    <row r="221" spans="3:3" ht="24">
+      <c r="C221" s="1"/>
+    </row>
+    <row r="222" spans="3:3" ht="24">
+      <c r="C222" s="1"/>
+    </row>
+    <row r="223" spans="3:3" ht="24">
+      <c r="C223" s="1"/>
+    </row>
+    <row r="224" spans="3:3" ht="24">
+      <c r="C224" s="1"/>
+    </row>
+    <row r="225" spans="3:3" ht="24">
+      <c r="C225" s="1"/>
+    </row>
+    <row r="226" spans="3:3" ht="24">
+      <c r="C226" s="1"/>
+    </row>
+    <row r="227" spans="3:3" ht="24">
+      <c r="C227" s="1"/>
+    </row>
+    <row r="228" spans="3:3" ht="24">
+      <c r="C228" s="1"/>
+    </row>
+    <row r="229" spans="3:3" ht="24">
+      <c r="C229" s="1"/>
+    </row>
+    <row r="230" spans="3:3" ht="24">
+      <c r="C230" s="1"/>
+    </row>
+    <row r="231" spans="3:3" ht="24">
+      <c r="C231" s="1"/>
+    </row>
+    <row r="232" spans="3:3" ht="24">
+      <c r="C232" s="1"/>
+    </row>
+    <row r="233" spans="3:3" ht="24">
+      <c r="C233" s="1"/>
+    </row>
+    <row r="234" spans="3:3" ht="24">
+      <c r="C234" s="1"/>
+    </row>
+    <row r="235" spans="3:3" ht="24">
+      <c r="C235" s="1"/>
+    </row>
+    <row r="236" spans="3:3" ht="24">
+      <c r="C236" s="1"/>
+    </row>
+    <row r="237" spans="3:3" ht="24">
+      <c r="C237" s="1"/>
+    </row>
+    <row r="238" spans="3:3" ht="24">
+      <c r="C238" s="1"/>
+    </row>
+    <row r="239" spans="3:3" ht="24">
+      <c r="C239" s="1"/>
+    </row>
+    <row r="240" spans="3:3" ht="24">
+      <c r="C240" s="1"/>
+    </row>
+    <row r="241" spans="3:3" ht="24">
+      <c r="C241" s="1"/>
+    </row>
+    <row r="242" spans="3:3" ht="24">
+      <c r="C242" s="1"/>
+    </row>
+    <row r="243" spans="3:3" ht="24">
+      <c r="C243" s="1"/>
+    </row>
+    <row r="244" spans="3:3" ht="24">
+      <c r="C244" s="1"/>
+    </row>
+    <row r="245" spans="3:3" ht="24">
+      <c r="C245" s="1"/>
+    </row>
+    <row r="246" spans="3:3" ht="24">
+      <c r="C246" s="1"/>
+    </row>
+    <row r="247" spans="3:3" ht="24">
+      <c r="C247" s="1"/>
+    </row>
+    <row r="248" spans="3:3" ht="24">
+      <c r="C248" s="1"/>
+    </row>
+    <row r="249" spans="3:3" ht="24">
+      <c r="C249" s="1"/>
+    </row>
+    <row r="250" spans="3:3" ht="24">
+      <c r="C250" s="1"/>
+    </row>
+    <row r="251" spans="3:3" ht="24">
+      <c r="C251" s="1"/>
+    </row>
+    <row r="252" spans="3:3" ht="24">
+      <c r="C252" s="1"/>
+    </row>
+    <row r="253" spans="3:3" ht="24">
+      <c r="C253" s="1"/>
+    </row>
+    <row r="254" spans="3:3" ht="24">
+      <c r="C254" s="1"/>
+    </row>
+    <row r="255" spans="3:3" ht="24">
+      <c r="C255" s="1"/>
+    </row>
+    <row r="256" spans="3:3" ht="24">
+      <c r="C256" s="1"/>
+    </row>
+    <row r="257" spans="3:3" ht="24">
+      <c r="C257" s="1"/>
+    </row>
+    <row r="258" spans="3:3" ht="24">
+      <c r="C258" s="1"/>
+    </row>
+    <row r="259" spans="3:3" ht="24">
+      <c r="C259" s="1"/>
+    </row>
+    <row r="260" spans="3:3" ht="24">
+      <c r="C260" s="1"/>
+    </row>
+    <row r="261" spans="3:3" ht="24">
+      <c r="C261" s="1"/>
+    </row>
+    <row r="262" spans="3:3" ht="24">
+      <c r="C262" s="1"/>
+    </row>
+    <row r="263" spans="3:3" ht="24">
+      <c r="C263" s="1"/>
+    </row>
+    <row r="264" spans="3:3" ht="24">
+      <c r="C264" s="1"/>
+    </row>
+    <row r="265" spans="3:3" ht="24">
+      <c r="C265" s="1"/>
+    </row>
+    <row r="266" spans="3:3" ht="24">
+      <c r="C266" s="1"/>
+    </row>
+    <row r="267" spans="3:3" ht="24">
+      <c r="C267" s="1"/>
+    </row>
+    <row r="268" spans="3:3" ht="24">
+      <c r="C268" s="1"/>
+    </row>
+    <row r="269" spans="3:3" ht="24">
+      <c r="C269" s="1"/>
+    </row>
+    <row r="270" spans="3:3" ht="24">
+      <c r="C270" s="1"/>
+    </row>
+    <row r="271" spans="3:3" ht="24">
+      <c r="C271" s="1"/>
+    </row>
+    <row r="272" spans="3:3" ht="24">
+      <c r="C272" s="1"/>
+    </row>
+    <row r="273" spans="3:3" ht="24">
+      <c r="C273" s="1"/>
+    </row>
+    <row r="274" spans="3:3" ht="24">
+      <c r="C274" s="1"/>
+    </row>
+    <row r="275" spans="3:3" ht="24">
+      <c r="C275" s="1"/>
+    </row>
+    <row r="276" spans="3:3" ht="24">
+      <c r="C276" s="1"/>
+    </row>
+    <row r="277" spans="3:3" ht="24">
+      <c r="C277" s="1"/>
+    </row>
+    <row r="278" spans="3:3" ht="24">
+      <c r="C278" s="1"/>
+    </row>
+    <row r="279" spans="3:3" ht="24">
+      <c r="C279" s="1"/>
+    </row>
+    <row r="280" spans="3:3" ht="24">
+      <c r="C280" s="1"/>
+    </row>
+    <row r="281" spans="3:3" ht="24">
+      <c r="C281" s="1"/>
+    </row>
+    <row r="282" spans="3:3" ht="24">
+      <c r="C282" s="1"/>
+    </row>
+    <row r="283" spans="3:3" ht="24">
+      <c r="C283" s="1"/>
+    </row>
+    <row r="284" spans="3:3" ht="24">
+      <c r="C284" s="1"/>
+    </row>
+    <row r="285" spans="3:3" ht="24">
+      <c r="C285" s="1"/>
+    </row>
+    <row r="286" spans="3:3" ht="24">
+      <c r="C286" s="1"/>
+    </row>
+    <row r="287" spans="3:3" ht="24">
+      <c r="C287" s="1"/>
+    </row>
+    <row r="288" spans="3:3" ht="24">
+      <c r="C288" s="1"/>
+    </row>
+    <row r="289" spans="3:3" ht="24">
+      <c r="C289" s="1"/>
+    </row>
+    <row r="290" spans="3:3" ht="24">
+      <c r="C290" s="1"/>
+    </row>
+    <row r="291" spans="3:3" ht="24">
+      <c r="C291" s="1"/>
+    </row>
+    <row r="292" spans="3:3" ht="24">
+      <c r="C292" s="1"/>
+    </row>
+    <row r="293" spans="3:3" ht="24">
+      <c r="C293" s="1"/>
+    </row>
+    <row r="294" spans="3:3" ht="24">
+      <c r="C294" s="1"/>
+    </row>
+    <row r="295" spans="3:3" ht="24">
+      <c r="C295" s="1"/>
+    </row>
+    <row r="296" spans="3:3" ht="24">
+      <c r="C296" s="1"/>
+    </row>
+    <row r="297" spans="3:3" ht="24">
+      <c r="C297" s="1"/>
+    </row>
+    <row r="298" spans="3:3" ht="24">
+      <c r="C298" s="1"/>
+    </row>
+    <row r="299" spans="3:3" ht="24">
+      <c r="C299" s="1"/>
+    </row>
+    <row r="300" spans="3:3" ht="24">
+      <c r="C300" s="1"/>
+    </row>
+    <row r="301" spans="3:3" ht="24">
+      <c r="C301" s="1"/>
+    </row>
+    <row r="302" spans="3:3" ht="24">
+      <c r="C302" s="1"/>
+    </row>
+    <row r="303" spans="3:3" ht="24">
+      <c r="C303" s="1"/>
+    </row>
+    <row r="304" spans="3:3" ht="24">
+      <c r="C304" s="1"/>
+    </row>
+    <row r="305" spans="3:3" ht="24">
+      <c r="C305" s="1"/>
+    </row>
+    <row r="306" spans="3:3" ht="24">
+      <c r="C306" s="1"/>
+    </row>
+    <row r="307" spans="3:3" ht="24">
+      <c r="C307" s="1"/>
+    </row>
+    <row r="308" spans="3:3" ht="24">
+      <c r="C308" s="1"/>
+    </row>
+    <row r="309" spans="3:3" ht="24">
+      <c r="C309" s="1"/>
+    </row>
+    <row r="310" spans="3:3" ht="24">
+      <c r="C310" s="1"/>
+    </row>
+    <row r="311" spans="3:3" ht="24">
+      <c r="C311" s="1"/>
+    </row>
+    <row r="312" spans="3:3" ht="24">
+      <c r="C312" s="1"/>
+    </row>
+    <row r="313" spans="3:3" ht="24">
+      <c r="C313" s="1"/>
+    </row>
+    <row r="314" spans="3:3" ht="24">
+      <c r="C314" s="1"/>
+    </row>
+    <row r="315" spans="3:3" ht="24">
+      <c r="C315" s="1"/>
+    </row>
+    <row r="316" spans="3:3" ht="24">
+      <c r="C316" s="1"/>
+    </row>
+    <row r="317" spans="3:3" ht="24">
+      <c r="C317" s="1"/>
+    </row>
+    <row r="318" spans="3:3" ht="24">
+      <c r="C318" s="1"/>
+    </row>
+    <row r="319" spans="3:3" ht="24">
+      <c r="C319" s="1"/>
+    </row>
+    <row r="320" spans="3:3" ht="24">
+      <c r="C320" s="1"/>
+    </row>
+    <row r="321" spans="3:3" ht="24">
+      <c r="C321" s="1"/>
+    </row>
+    <row r="322" spans="3:3" ht="24">
+      <c r="C322" s="1"/>
+    </row>
+    <row r="323" spans="3:3" ht="24">
+      <c r="C323" s="1"/>
+    </row>
+    <row r="324" spans="3:3" ht="24">
+      <c r="C324" s="1"/>
+    </row>
+    <row r="325" spans="3:3" ht="24">
+      <c r="C325" s="1"/>
+    </row>
+    <row r="326" spans="3:3" ht="24">
+      <c r="C326" s="1"/>
+    </row>
+    <row r="327" spans="3:3" ht="24">
+      <c r="C327" s="1"/>
+    </row>
+    <row r="328" spans="3:3" ht="24">
+      <c r="C328" s="1"/>
+    </row>
+    <row r="329" spans="3:3" ht="24">
+      <c r="C329" s="1"/>
+    </row>
+    <row r="330" spans="3:3" ht="24">
+      <c r="C330" s="1"/>
+    </row>
+    <row r="331" spans="3:3" ht="24">
+      <c r="C331" s="1"/>
+    </row>
+    <row r="332" spans="3:3" ht="24">
+      <c r="C332" s="1"/>
+    </row>
+    <row r="333" spans="3:3" ht="24">
+      <c r="C333" s="1"/>
+    </row>
+    <row r="334" spans="3:3" ht="24">
+      <c r="C334" s="1"/>
+    </row>
+    <row r="335" spans="3:3" ht="24">
+      <c r="C335" s="1"/>
+    </row>
+    <row r="336" spans="3:3" ht="24">
+      <c r="C336" s="1"/>
+    </row>
+    <row r="337" spans="3:3" ht="24">
+      <c r="C337" s="1"/>
+    </row>
+    <row r="338" spans="3:3" ht="24">
+      <c r="C338" s="1"/>
+    </row>
+    <row r="339" spans="3:3" ht="24">
+      <c r="C339" s="1"/>
+    </row>
+    <row r="340" spans="3:3" ht="24">
+      <c r="C340" s="1"/>
+    </row>
+    <row r="341" spans="3:3" ht="24">
+      <c r="C341" s="1"/>
+    </row>
+    <row r="342" spans="3:3" ht="24">
+      <c r="C342" s="1"/>
+    </row>
+    <row r="343" spans="3:3" ht="24">
+      <c r="C343" s="1"/>
+    </row>
+    <row r="344" spans="3:3" ht="24">
+      <c r="C344" s="1"/>
+    </row>
+    <row r="345" spans="3:3" ht="24">
+      <c r="C345" s="1"/>
+    </row>
+    <row r="346" spans="3:3" ht="24">
+      <c r="C346" s="1"/>
+    </row>
+    <row r="347" spans="3:3" ht="24">
+      <c r="C347" s="1"/>
+    </row>
+    <row r="348" spans="3:3" ht="24">
+      <c r="C348" s="1"/>
+    </row>
+    <row r="349" spans="3:3" ht="24">
+      <c r="C349" s="1"/>
+    </row>
+    <row r="350" spans="3:3" ht="24">
+      <c r="C350" s="1"/>
+    </row>
+    <row r="351" spans="3:3" ht="24">
+      <c r="C351" s="1"/>
+    </row>
+    <row r="352" spans="3:3" ht="24">
+      <c r="C352" s="1"/>
+    </row>
+    <row r="353" spans="3:3" ht="24">
+      <c r="C353" s="1"/>
+    </row>
+    <row r="354" spans="3:3" ht="24">
+      <c r="C354" s="1"/>
+    </row>
+    <row r="355" spans="3:3" ht="24">
+      <c r="C355" s="1"/>
+    </row>
+    <row r="356" spans="3:3" ht="24">
+      <c r="C356" s="1"/>
+    </row>
+    <row r="357" spans="3:3" ht="24">
+      <c r="C357" s="1"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J76" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-13 17:42:55
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4243FA-DE93-8546-ABDE-D87CBCA76292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E8D971F-CD3B-AC47-87D2-8DEB8076E149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="81">
   <si>
     <t>证券代码</t>
   </si>
@@ -308,6 +308,10 @@
   <si>
     <t xml:space="preserve">开盘强势 等fomo情绪退潮在下方接了个114的价位但我觉得接的还是太早了 应该在10点后等待均线确认后加仓 这个时候也消除了大部分开盘期间带来的噪音 现在发现在这种市场情况下 顺势而为 浮盈加仓才是一个让我觉得舒服的交易方式 之前一直跌一直补的做法太煎熬了 我感觉自己也不是一个很坚定的人 这套方法貌似不适合现在的我 
 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>华工科技从下午开始就一路走强 这里我并不知道盘后会有什么消息（其实这里应该反省一下）因为今天下午其实就是华工科技一季报发布的时间，我当时居然不知道这个消息 以后绝对不能犯这种错误 对于持仓个股在时间线上的大事应该了如指掌才对 那也就意味着今天加仓的逻辑不是因为一季报的看好 而是发现分数图上华工科技突然的强势 + 量能温和放量 我认为这是一个不错的上升趋势票 + 自己本身盈利中 -&gt; 加仓200股</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3471,7 +3475,7 @@
       <c r="N64" s="4"/>
       <c r="O64" s="1"/>
     </row>
-    <row r="65" spans="1:15" ht="150">
+    <row r="65" spans="1:15" ht="50">
       <c r="A65" s="7" t="s">
         <v>42</v>
       </c>
@@ -3508,7 +3512,7 @@
       </c>
       <c r="O65" s="1"/>
     </row>
-    <row r="66" spans="1:15" ht="150">
+    <row r="66" spans="1:15" ht="75">
       <c r="A66" s="1">
         <v>600584</v>
       </c>
@@ -3921,7 +3925,7 @@
       <c r="N76" s="4"/>
       <c r="O76" s="9"/>
     </row>
-    <row r="77" spans="1:15" ht="400">
+    <row r="77" spans="1:15" ht="325">
       <c r="A77" s="7" t="s">
         <v>66</v>
       </c>
@@ -4106,7 +4110,7 @@
       <c r="N81" s="4"/>
       <c r="O81" s="1"/>
     </row>
-    <row r="82" spans="1:15" ht="409.6">
+    <row r="82" spans="1:15" ht="375">
       <c r="A82" s="7" t="s">
         <v>66</v>
       </c>
@@ -4239,8 +4243,37 @@
         <v>79</v>
       </c>
     </row>
-    <row r="86" spans="1:15" ht="24">
-      <c r="C86" s="1"/>
+    <row r="86" spans="1:15" ht="350">
+      <c r="A86" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D86" s="1">
+        <v>20260413</v>
+      </c>
+      <c r="E86" s="2">
+        <v>0.59583333333333333</v>
+      </c>
+      <c r="F86" s="1">
+        <v>122.5</v>
+      </c>
+      <c r="G86" s="1">
+        <v>200</v>
+      </c>
+      <c r="H86" s="1">
+        <v>24500</v>
+      </c>
+      <c r="J86" s="3">
+        <v>600</v>
+      </c>
+      <c r="K86" s="9" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="87" spans="1:15" ht="24">
       <c r="C87" s="1"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-15 18:54:43
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E8D971F-CD3B-AC47-87D2-8DEB8076E149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C603187A-21DF-904A-9E98-ABCA9B4E1823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="84">
   <si>
     <t>证券代码</t>
   </si>
@@ -312,6 +312,18 @@
   </si>
   <si>
     <t>华工科技从下午开始就一路走强 这里我并不知道盘后会有什么消息（其实这里应该反省一下）因为今天下午其实就是华工科技一季报发布的时间，我当时居然不知道这个消息 以后绝对不能犯这种错误 对于持仓个股在时间线上的大事应该了如指掌才对 那也就意味着今天加仓的逻辑不是因为一季报的看好 而是发现分数图上华工科技突然的强势 + 量能温和放量 我认为这是一个不错的上升趋势票 + 自己本身盈利中 -&gt; 加仓200股</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>华工科技在昨日收盘发布一季报预告 很显然扣非之后不及机构预期 早盘开盘恐慌下杀之后被拉回至接近-轴，午后继续下杀最后-3.62%收盘 清了一半仓位一方面是规避风险落袋为安 因为无论今天是收涨还是如何 光模块近期也可能要到顶了 即使兑现一半的利润，留下了另一半仓位在于昨天的尾盘拉伸 我不认为是散户跟风买入 更可能消息交易者在买入 我不能排除洗盘的可能 同时今天利空出尽的前提下 底部资金有承接 尾盘又出现大量主买 故有吸筹的嫌疑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>光迅科技还没发布季报预告这是一个不确定的点-&gt; 以后我要时刻关注这种时间点 尽量不要在这种公告时间点进行操作 波动太大反而不利于操作 + 今天光迅科技下跌大概率是收到华工科技的恐慌情绪带动的 + 已经有隐约的见顶信号 即使不见顶 都有回踩5日线的可能 +光模块最近涨的太多了+光迅科技最近趋势太好 回调无法避免</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>保本损，确保这一单不是亏损的，这笔交易做的并不好 ，止损不够果断，昨天清半仓的时候抱着防止卖飞的信念留了半仓，可是今天开盘之后一路下杀自己没有做好移动止损的计划 真正到了保本的时候才彻底清仓 这是失败的 我认为不能再用这种到了下跌才开始清仓的策略了 要测试一下在上涨中卖出的表现如何</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -4268,27 +4280,169 @@
       <c r="H86" s="1">
         <v>24500</v>
       </c>
-      <c r="J86" s="3">
+      <c r="J86" s="1">
         <v>600</v>
       </c>
       <c r="K86" s="9" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="87" spans="1:15" ht="24">
-      <c r="C87" s="1"/>
-    </row>
-    <row r="88" spans="1:15" ht="24">
-      <c r="C88" s="1"/>
-    </row>
-    <row r="89" spans="1:15" ht="24">
-      <c r="C89" s="1"/>
+    <row r="87" spans="1:15" ht="409.6">
+      <c r="A87" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D87" s="1">
+        <v>20260414</v>
+      </c>
+      <c r="E87" s="2">
+        <v>0.62291666666666667</v>
+      </c>
+      <c r="F87" s="1">
+        <v>120.55</v>
+      </c>
+      <c r="G87" s="1">
+        <v>300</v>
+      </c>
+      <c r="H87" s="1">
+        <v>36165</v>
+      </c>
+      <c r="J87" s="1">
+        <v>300</v>
+      </c>
+      <c r="O87" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="88" spans="1:15" ht="300">
+      <c r="A88" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D88" s="1">
+        <v>20260414</v>
+      </c>
+      <c r="E88" s="2">
+        <v>0.62291666666666667</v>
+      </c>
+      <c r="F88" s="1">
+        <v>111.35</v>
+      </c>
+      <c r="G88" s="1">
+        <v>300</v>
+      </c>
+      <c r="H88" s="1">
+        <v>33405</v>
+      </c>
+      <c r="J88" s="1">
+        <v>300</v>
+      </c>
+      <c r="O88" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="89" spans="1:15" ht="50">
+      <c r="A89" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D89" s="1">
+        <v>20260415</v>
+      </c>
+      <c r="E89" s="2">
+        <v>0.62291666666666667</v>
+      </c>
+      <c r="F89" s="1">
+        <v>112.26</v>
+      </c>
+      <c r="G89" s="1">
+        <v>300</v>
+      </c>
+      <c r="H89" s="1">
+        <v>33678</v>
+      </c>
+      <c r="I89" s="1">
+        <v>44.23</v>
+      </c>
+      <c r="J89" s="1">
+        <v>0</v>
+      </c>
+      <c r="N89" s="9" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="90" spans="1:15" ht="24">
-      <c r="C90" s="1"/>
+      <c r="A90" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D90" s="1">
+        <v>20260415</v>
+      </c>
+      <c r="E90" s="2">
+        <v>0.42430555555555555</v>
+      </c>
+      <c r="F90" s="1">
+        <v>110.5</v>
+      </c>
+      <c r="G90" s="1">
+        <v>300</v>
+      </c>
+      <c r="H90" s="1">
+        <v>33150</v>
+      </c>
+      <c r="J90" s="1">
+        <v>600</v>
+      </c>
     </row>
     <row r="91" spans="1:15" ht="24">
-      <c r="C91" s="1"/>
+      <c r="A91" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D91" s="1">
+        <v>20260415</v>
+      </c>
+      <c r="E91" s="2">
+        <v>0.60069444444444442</v>
+      </c>
+      <c r="F91" s="1">
+        <v>106.7</v>
+      </c>
+      <c r="G91" s="1">
+        <v>300</v>
+      </c>
+      <c r="H91" s="1">
+        <v>32010</v>
+      </c>
+      <c r="J91" s="1">
+        <v>300</v>
+      </c>
     </row>
     <row r="92" spans="1:15" ht="24">
       <c r="C92" s="1"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-16 20:13:46
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C603187A-21DF-904A-9E98-ABCA9B4E1823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84ABECB2-3AC6-0246-9346-1607A5020452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="90">
   <si>
     <t>证券代码</t>
   </si>
@@ -324,6 +324,31 @@
   </si>
   <si>
     <t>保本损，确保这一单不是亏损的，这笔交易做的并不好 ，止损不够果断，昨天清半仓的时候抱着防止卖飞的信念留了半仓，可是今天开盘之后一路下杀自己没有做好移动止损的计划 真正到了保本的时候才彻底清仓 这是失败的 我认为不能再用这种到了下跌才开始清仓的策略了 要测试一下在上涨中卖出的表现如何</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>601126</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>四方股份</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">四方股份目前处于低位 ， 叠加电网近期有反弹的趋势
+资金不可能一直在光通讯类的板块游动，需要将仓位调至不那么拥挤的赛道，且逻辑也足够硬的赛道，同时电网在这波下跌中已经见底迎来反弹，这时候需要选择一支高弹性的股票，我刻意避开了思源电气 虽然它是龙头股 但是我认为市值太大的情况下弹性不足 不适合短期持仓 四方股份的业绩 显然不如思源电气 增长速度也不行 但市场也没有给出比较大的预期这是一件好事 同时股价正从低位逐步修复 上方筹码也不多 抛压小 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>这里在尾盘加了600股坦白地说是害怕明天行情就启动了的贸然出击，但是总觉得仓位不打到5w块心里不舒服，反而加完仓之后心情好了起来，这个操作确实有点冒失，但我想把它当作感觉的一部分不知道这对不对。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>这几天它可能要去摸48.5这个位置如果价格到了48.5意味着此时仓位浮盈来到5%这个时候加1100股也就是把浮盈摊到2.5%，成本线在47.31，这时候会遇到前期的一个平台位置48.62，如果遇到阻力被打下来了下方会有一个30日线支持（然而这个三十日线在最近一个月并不有效 ）充当的是一个阻力位的作用，同时这个时候下方也会有一个5日线支撑这里的短期支撑作用还在，但是这里直接把仓位double会不会有点太激进了，我能容扔的成本线只能往上继续移动到46.66这个位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>负-7%的时候止损</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -405,7 +430,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -446,6 +471,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4444,11 +4475,75 @@
         <v>300</v>
       </c>
     </row>
-    <row r="92" spans="1:15" ht="24">
-      <c r="C92" s="1"/>
-    </row>
-    <row r="93" spans="1:15" ht="24">
-      <c r="C93" s="1"/>
+    <row r="92" spans="1:15" ht="409.6">
+      <c r="A92" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D92" s="1">
+        <v>20260416</v>
+      </c>
+      <c r="E92" s="2">
+        <v>0.46944444444444444</v>
+      </c>
+      <c r="F92" s="1">
+        <v>45.65</v>
+      </c>
+      <c r="G92" s="1">
+        <v>500</v>
+      </c>
+      <c r="H92" s="1">
+        <v>22825</v>
+      </c>
+      <c r="J92" s="1">
+        <v>500</v>
+      </c>
+      <c r="K92" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L92" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="M92" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="93" spans="1:15" ht="175">
+      <c r="A93" s="15">
+        <v>601126</v>
+      </c>
+      <c r="B93" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D93" s="1">
+        <v>20260416</v>
+      </c>
+      <c r="E93" s="2">
+        <v>0.62152777777777779</v>
+      </c>
+      <c r="F93" s="1">
+        <v>46.43</v>
+      </c>
+      <c r="G93" s="1">
+        <v>600</v>
+      </c>
+      <c r="H93" s="1">
+        <v>27858</v>
+      </c>
+      <c r="J93" s="1">
+        <v>1100</v>
+      </c>
+      <c r="K93" s="5" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="94" spans="1:15" ht="24">
       <c r="C94" s="1"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-20 19:31:57
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84ABECB2-3AC6-0246-9346-1607A5020452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE85E504-703A-1149-A9AC-3075BC68030C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="93">
   <si>
     <t>证券代码</t>
   </si>
@@ -349,6 +349,18 @@
   </si>
   <si>
     <t>负-7%的时候止损</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>看到价格高开并且往上冲 这个时候我没有着急下单 因为不知道是否是短期诱多 等到了9:45 其实不应该在这个时间点买入的 应该在10点等情绪真正平稳的时候才买入的 9:48 涨幅来到7%-8% 这个时候我能够确认昨晚到股权转让是利多消息 这个时候我起了贪念 直接加了3手仓位 也为后来10:13分我卖出1手做了铺垫</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">这个时候以为是真的被哟多了 我选择在这个时候卖出100股以求安稳 自己很显然被股价控制了操作 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">四方股份的价格来到了我的加仓目标价 顺势在这个价格买入6手 </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -964,6 +976,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{2DFF7435-4F95-7449-B724-D5A5EE9FF813}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;9247f0a0-ecd4-46b9-b490-119767bfebf7&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O357"/>
@@ -4517,7 +4551,7 @@
       <c r="A93" s="15">
         <v>601126</v>
       </c>
-      <c r="B93" s="10" t="s">
+      <c r="B93" s="1" t="s">
         <v>85</v>
       </c>
       <c r="C93" s="1" t="s">
@@ -4545,14 +4579,101 @@
         <v>87</v>
       </c>
     </row>
-    <row r="94" spans="1:15" ht="24">
-      <c r="C94" s="1"/>
-    </row>
-    <row r="95" spans="1:15" ht="24">
-      <c r="C95" s="1"/>
-    </row>
-    <row r="96" spans="1:15" ht="24">
-      <c r="C96" s="1"/>
+    <row r="94" spans="1:15" ht="275">
+      <c r="A94" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D94" s="1">
+        <v>20260419</v>
+      </c>
+      <c r="E94" s="2">
+        <v>0.40833333333333333</v>
+      </c>
+      <c r="F94" s="1">
+        <v>115.58</v>
+      </c>
+      <c r="G94" s="1">
+        <v>300</v>
+      </c>
+      <c r="H94" s="1">
+        <v>34674</v>
+      </c>
+      <c r="J94" s="1">
+        <v>600</v>
+      </c>
+      <c r="K94" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="95" spans="1:15" ht="100">
+      <c r="A95" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D95" s="1">
+        <v>20260419</v>
+      </c>
+      <c r="E95" s="2">
+        <v>0.42569444444444443</v>
+      </c>
+      <c r="F95" s="1">
+        <v>112.51</v>
+      </c>
+      <c r="G95" s="1">
+        <v>100</v>
+      </c>
+      <c r="H95" s="1">
+        <v>11251</v>
+      </c>
+      <c r="J95" s="1">
+        <v>500</v>
+      </c>
+      <c r="O95" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="96" spans="1:15" ht="50">
+      <c r="A96" s="15">
+        <v>601126</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D96" s="1">
+        <v>20260419</v>
+      </c>
+      <c r="E96" s="2">
+        <v>0.56319444444444444</v>
+      </c>
+      <c r="F96" s="1">
+        <v>48.54</v>
+      </c>
+      <c r="G96" s="1">
+        <v>600</v>
+      </c>
+      <c r="H96" s="1">
+        <v>29124</v>
+      </c>
+      <c r="J96" s="1">
+        <v>1700</v>
+      </c>
+      <c r="K96" s="5" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="97" spans="3:3" ht="24">
       <c r="C97" s="1"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-21 20:15:39
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE85E504-703A-1149-A9AC-3075BC68030C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D35DAB70-95E8-5A41-BAB9-E4F0EB4436DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="93">
   <si>
     <t>证券代码</t>
   </si>
@@ -4675,52 +4675,110 @@
         <v>92</v>
       </c>
     </row>
-    <row r="97" spans="3:3" ht="24">
-      <c r="C97" s="1"/>
-    </row>
-    <row r="98" spans="3:3" ht="24">
-      <c r="C98" s="1"/>
-    </row>
-    <row r="99" spans="3:3" ht="24">
+    <row r="97" spans="1:10" ht="24">
+      <c r="A97" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D97" s="1">
+        <v>20260420</v>
+      </c>
+      <c r="E97" s="2">
+        <v>0.40138888888888891</v>
+      </c>
+      <c r="F97" s="1">
+        <v>125</v>
+      </c>
+      <c r="G97" s="1">
+        <v>100</v>
+      </c>
+      <c r="H97" s="1">
+        <v>12500</v>
+      </c>
+      <c r="J97" s="1">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" ht="24">
+      <c r="A98" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D98" s="1">
+        <v>20260420</v>
+      </c>
+      <c r="E98" s="2">
+        <v>0.62083333333333335</v>
+      </c>
+      <c r="F98" s="1">
+        <v>120.05</v>
+      </c>
+      <c r="G98" s="1">
+        <v>100</v>
+      </c>
+      <c r="H98" s="1">
+        <v>12005</v>
+      </c>
+      <c r="J98" s="1">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" ht="24">
+      <c r="A99" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>68</v>
+      </c>
       <c r="C99" s="1"/>
     </row>
-    <row r="100" spans="3:3" ht="24">
+    <row r="100" spans="1:10" ht="24">
       <c r="C100" s="1"/>
     </row>
-    <row r="101" spans="3:3" ht="24">
+    <row r="101" spans="1:10" ht="24">
       <c r="C101" s="1"/>
     </row>
-    <row r="102" spans="3:3" ht="24">
+    <row r="102" spans="1:10" ht="24">
       <c r="C102" s="1"/>
     </row>
-    <row r="103" spans="3:3" ht="24">
+    <row r="103" spans="1:10" ht="24">
       <c r="C103" s="1"/>
     </row>
-    <row r="104" spans="3:3" ht="24">
+    <row r="104" spans="1:10" ht="24">
       <c r="C104" s="1"/>
     </row>
-    <row r="105" spans="3:3" ht="24">
+    <row r="105" spans="1:10" ht="24">
       <c r="C105" s="1"/>
     </row>
-    <row r="106" spans="3:3" ht="24">
+    <row r="106" spans="1:10" ht="24">
       <c r="C106" s="1"/>
     </row>
-    <row r="107" spans="3:3" ht="24">
+    <row r="107" spans="1:10" ht="24">
       <c r="C107" s="1"/>
     </row>
-    <row r="108" spans="3:3" ht="24">
+    <row r="108" spans="1:10" ht="24">
       <c r="C108" s="1"/>
     </row>
-    <row r="109" spans="3:3" ht="24">
+    <row r="109" spans="1:10" ht="24">
       <c r="C109" s="1"/>
     </row>
-    <row r="110" spans="3:3" ht="24">
+    <row r="110" spans="1:10" ht="24">
       <c r="C110" s="1"/>
     </row>
-    <row r="111" spans="3:3" ht="24">
+    <row r="111" spans="1:10" ht="24">
       <c r="C111" s="1"/>
     </row>
-    <row r="112" spans="3:3" ht="24">
+    <row r="112" spans="1:10" ht="24">
       <c r="C112" s="1"/>
     </row>
     <row r="113" spans="3:3" ht="24">

</xml_diff>

<commit_message>
vault backup: 2026-04-21 20:18:56
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D35DAB70-95E8-5A41-BAB9-E4F0EB4436DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D77330D3-8B92-6346-B781-EE5C9A1C056F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -36,331 +36,373 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="88">
+  <si>
+    <t>思源电气</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>卖出</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>卖出逻辑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>思源电气在昨天回踩了60日均线且伴随放量但是我并未有发现有什么利空消息在影响股价，一时间难以判断这到底是洗盘还是出货，今天A股全线暴涨思源电气只能说是表现平平，全天仍然缩量为防止踏空+降低风险今天确实应该减仓，这是我从上一次卖飞亨通光电收获的教训，不应该太赌气的清仓留一点悬念和可能性给自己，不要太多的确定性</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>002028</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000988</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>华工科技</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>买入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>长远来看华工科技在三月份连跌之后在短期已经出现明显的底部100作为一个短期支撑，同时今天放量收出阳线有反攻事态，总之这个位置是一个盈亏比例较好的位置，前面有前高141，下方有支撑位100，先小仓试错而后加仓。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>002281</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>光迅科技</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>光迅科技在最近的cpo板块里面是更加强势的股票
+鉴于之前在做亨通光电和长飞光纤的时候我选择了更加处于回调上升的亨通光电而错过了长飞的大涨，这让我觉得更应该选择强势的股票 不是看涨的多了就害怕，所以这里也加了2w仓位 决定在华工科技之间优中选优 去弱留强</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>今天看到光迅科技在早盘冲高，这时候有一个自我的警示就是等待情绪回落开盘从9:30-10:00这段时间是fomo的时间我认为这里存在着大量的交易噪音，一时间可能会被追涨的人群影响，10点之后继续观察 光迅科技价格仍旧坚挺且还有继续上冲的意图 这里可以大概判断出今天的上涨不是单纯的早盘fomo + 最近利空被消化+ 近期在cpo板块里的强势地位（逆势上涨）-&gt; 果断加仓</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">先买入的是光迅科技这里买入华工科技主要有以下考虑：1.作为同板块的个股 光迅科技的可见强势会在一定程度上带动华工科技 2.华工科技从形态上看比光迅科技更加让人安心 因为在3月份的大跌中 它已经铸成了一个显而易见的100作为低点 同时还站稳了5日线 高点明显+低点明显 盈亏比例在这里差不多有2:1 先把目标价格放在130左右 止损放在100元
+</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>思源电气最近的表现疲软虽然今天是4000家个股下跌，但相对于板块来说这几天的表现远远低于整体板块，伴随着缩量可以解读成买盘萎缩，卖盘也不强劲，预计会在这个箱体内横盘一段时间或者沿着60日支撑震荡，但短期出现行情的概率太低了，之前认为可能是洗盘，但现在来看更像是出货，为了规避风险同时尽可能博一点反弹预期 留了1层底仓 若持续低迷跌破60日均线 可以清仓</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>当日思源电气低开高走 一改往日颓势 上午我并没有急于追涨 因为想等大众的
+fomo情绪过去之后再入场 到了13:08的时候思源电气依然走强甚至拉高 这时候我认为前几日的杀跌只是洗盘 果断追涨买入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>开盘之后思源电气大幅杀跌 又回到了前几日的低点 这并不符合之前的假设 如果是洗盘 今天不应该是这样杀跌 当然这依然可能是洗盘 我不能排除这样的可能性 但我想说的是自己没做好的一个点 ，那就是太急于下判断 上仓位了 这里我太鲁莽了 应该等到突破阻力位213进行确认再加仓的 我不知道这里到底是牛回了 还是拉高出货 那这个时候就是等价格确认是最好的 今天清仓的逻辑我也说不清楚 感觉是自己在很快的想要摆脱这种亏损 有种在赌气的感觉 操作不理性了 伴随着自己在cpo板块还有盈利今天总体是正盈利的 所以对割肉没有什么心理上的痛觉 只有对这个股票的失望（好奇怪 我不应该有这样的情绪的 为什么要对它失望 它不清楚我买了它 也没有涨的义务 我是来赚钱的 而不是来产生感情的 我感觉自己确实在一只股票上耗费了太大的感情 或者说精力当他不能为我赚钱或者有理由证明不强势的时候我应该离开 而不是死守着逻辑 或者它曾经给我带来过盈利作为借口而抓着不放</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">开盘强势 等fomo情绪退潮在下方接了个114的价位但我觉得接的还是太早了 应该在10点后等待均线确认后加仓 这个时候也消除了大部分开盘期间带来的噪音 现在发现在这种市场情况下 顺势而为 浮盈加仓才是一个让我觉得舒服的交易方式 之前一直跌一直补的做法太煎熬了 我感觉自己也不是一个很坚定的人 这套方法貌似不适合现在的我 
+</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>华工科技从下午开始就一路走强 这里我并不知道盘后会有什么消息（其实这里应该反省一下）因为今天下午其实就是华工科技一季报发布的时间，我当时居然不知道这个消息 以后绝对不能犯这种错误 对于持仓个股在时间线上的大事应该了如指掌才对 那也就意味着今天加仓的逻辑不是因为一季报的看好 而是发现分数图上华工科技突然的强势 + 量能温和放量 我认为这是一个不错的上升趋势票 + 自己本身盈利中 -&gt; 加仓200股</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>华工科技在昨日收盘发布一季报预告 很显然扣非之后不及机构预期 早盘开盘恐慌下杀之后被拉回至接近-轴，午后继续下杀最后-3.62%收盘 清了一半仓位一方面是规避风险落袋为安 因为无论今天是收涨还是如何 光模块近期也可能要到顶了 即使兑现一半的利润，留下了另一半仓位在于昨天的尾盘拉伸 我不认为是散户跟风买入 更可能消息交易者在买入 我不能排除洗盘的可能 同时今天利空出尽的前提下 底部资金有承接 尾盘又出现大量主买 故有吸筹的嫌疑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>光迅科技还没发布季报预告这是一个不确定的点-&gt; 以后我要时刻关注这种时间点 尽量不要在这种公告时间点进行操作 波动太大反而不利于操作 + 今天光迅科技下跌大概率是收到华工科技的恐慌情绪带动的 + 已经有隐约的见顶信号 即使不见顶 都有回踩5日线的可能 +光模块最近涨的太多了+光迅科技最近趋势太好 回调无法避免</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>保本损，确保这一单不是亏损的，这笔交易做的并不好 ，止损不够果断，昨天清半仓的时候抱着防止卖飞的信念留了半仓，可是今天开盘之后一路下杀自己没有做好移动止损的计划 真正到了保本的时候才彻底清仓 这是失败的 我认为不能再用这种到了下跌才开始清仓的策略了 要测试一下在上涨中卖出的表现如何</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>601126</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>四方股份</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">四方股份目前处于低位 ， 叠加电网近期有反弹的趋势
+资金不可能一直在光通讯类的板块游动，需要将仓位调至不那么拥挤的赛道，且逻辑也足够硬的赛道，同时电网在这波下跌中已经见底迎来反弹，这时候需要选择一支高弹性的股票，我刻意避开了思源电气 虽然它是龙头股 但是我认为市值太大的情况下弹性不足 不适合短期持仓 四方股份的业绩 显然不如思源电气 增长速度也不行 但市场也没有给出比较大的预期这是一件好事 同时股价正从低位逐步修复 上方筹码也不多 抛压小 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>这里在尾盘加了600股坦白地说是害怕明天行情就启动了的贸然出击，但是总觉得仓位不打到5w块心里不舒服，反而加完仓之后心情好了起来，这个操作确实有点冒失，但我想把它当作感觉的一部分不知道这对不对。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>这几天它可能要去摸48.5这个位置如果价格到了48.5意味着此时仓位浮盈来到5%这个时候加1100股也就是把浮盈摊到2.5%，成本线在47.31，这时候会遇到前期的一个平台位置48.62，如果遇到阻力被打下来了下方会有一个30日线支持（然而这个三十日线在最近一个月并不有效 ）充当的是一个阻力位的作用，同时这个时候下方也会有一个5日线支撑这里的短期支撑作用还在，但是这里直接把仓位double会不会有点太激进了，我能容扔的成本线只能往上继续移动到46.66这个位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>负-7%的时候止损</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>看到价格高开并且往上冲 这个时候我没有着急下单 因为不知道是否是短期诱多 等到了9:45 其实不应该在这个时间点买入的 应该在10点等情绪真正平稳的时候才买入的 9:48 涨幅来到7%-8% 这个时候我能够确认昨晚到股权转让是利多消息 这个时候我起了贪念 直接加了3手仓位 也为后来10:13分我卖出1手做了铺垫</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">这个时候以为是真的被哟多了 我选择在这个时候卖出100股以求安稳 自己很显然被股价控制了操作 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">四方股份的价格来到了我的加仓目标价 顺势在这个价格买入6手 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
   <si>
     <t>证券代码</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>证券名称</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>买卖标志</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>成交日期</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>成交时间</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>成交价格</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>成交数量</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>成交金额</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>清仓收益</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>剩余仓位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>买入逻辑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>计划止盈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>计划止损</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>清仓逻辑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>恒瑞医药</t>
-  </si>
-  <si>
-    <t>买入</t>
-  </si>
-  <si>
-    <t>卖出</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>工业富联</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>兆易创新</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>北方稀土</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>立讯精密</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>药明康德</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>北方华创</t>
-  </si>
-  <si>
-    <t>光迅科技</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>市买1（对手方最优价格）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>市卖1（对手方最优价格）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>市卖2（本手方最优价格）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>剑桥科技</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>市买2（本手方最优价格）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>华友钴业</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>长白山</t>
-  </si>
-  <si>
-    <t>思源电气</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>中国西电</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>长电科技</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve"> 1- 长电科技站稳了30日均线  今天下午迎来突破是一个较好追随趋势的机会 
  2 -  nvda财报远超预期 ai硬件炒作尚未停止 还未传导到封测领域 
 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve"> 设置在前高55时止盈半仓</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>放量跌破30日线全仓止损</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">基本面没有改变 思源电气回踩13日线  只是一个短期获利盘的了结  做的不足的地方在于太想抄底了 应该等股价稳稳踩住13日线的时候再进行加仓
 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>止盈依旧设置在250 止盈半仓</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>放量跌破13日均线且没有收复迹象时全仓离场</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">卖出 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">
 止损了600股 主要原因是长电科技有效跌破30日均线且回收的速度不快，温和回收，同时接近尾盘时又下跌了一点 ，对于这种慢慢的温和的回收 我有两个想法 
 一是主力在边打边撤 悄悄出货 二是主力在底部建仓 怕一下子拉飞股价  同时股价是触及到了 短期的支撑位之后回升 留下了长下影 个人主观上我想博一个反弹 客观上破位就走是我定死的纪律 所以中和二者 半苍止损是比较好的选择了</t>
-  </si>
-  <si>
-    <t>002028</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>当时的心态和想法是 博一个反弹 当时思源电气并没有基本面或者重大利空 我不理解为什么这个时候跌破了13日均线 本来13日均线是我的止损价格 可是我没有执行好我的策略 却真的好像在赌博一样依旧加仓 我受到讨论区的影响也有点大 看到大家都觉得没事 回调 这个也一定程度上影响了我的判断 今天是加仓后的第二天我确认我做错了。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>有效跌破210 止盈离场 恢复趋势后才能进场</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>思源电气跌破210支撑位且最终没有有力的回收
 需要适当规避风险，短期走弱，但会持续关注，企稳30日线后可以入场建仓，但现在不是时候</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>尽管今天盘中爆出关于7nm制成工艺的利好
 依旧走势很弱涨幅小，没有回收47块，判定为
 短暂弱势+封测板块本身没什么涨头遂离场</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>思源电气 逻辑还在 今天正式站稳30日线 且上涨幅度达4%强度可延续 今天初步建仓主要为了试仓 最终仓位上限定格在10w</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>跌破30日线离场</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>亨通光电</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>亨通光电作为光纤的人气公司 pe处于低值 同时今天站稳了30日线做一下左侧交易问题应该不大 轻仓试错中</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>有效跌破30日线离场</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>今天在9:57的时候有一波操作 这波操作跟我之前的都不太一样，买点依据当天早上212.8时我看到分时图已经开始反转同时有反弹的趋势，我害怕还像昨天那样错过大反弹+鉴于今天大盘表现不佳 下午拉盘的概率高+思源电气早上反弹的概率大 于是选择买入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>原本设定的限价单放在了210，直到收盘也没有打到210的位置，我认为今天作为一个普跌行情，反弹是最近的大概率事件，尾盘突然的拉伸正想追进去发现尾盘又砸了，既然稳在30日线 逐步布局加仓也是好的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>认为短期是一个加仓的时期 同时早盘
 走的很强势 于是有点贸然加仓了</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>亨通光电早盘高开低走下午探底回升之后十分强势收复前几天大跌的阴线，且当时均价仍低于成本线，短期支撑位40.96已经明晰，寻求一波追涨</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>002208</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>这一波买入跟昨天买入亨通光电的逻辑是一致的在看到思源电气企稳逐步回到趋势后 同时又低于现在仓位均价加仓是看起来很划算的事情 ，电力走的好 一定程度上也带动了电网，但要开始逐步小心风险了</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">今天早盘一波放量下杀之后有效回收了涨幅留下了长下影线 作为一个安全的短期支撑位 同时有隐约上冲的势头 于是我选在在208这个位置买入做一个短t 短期这支票的最大容量为我的50%仓位 已经完全打满 奉高做t降低成本 是现在的主要任务 同时连着两日缩量  股价已经在200-210之间得到了企稳 
 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>3614    （+5.4%）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">1.三天时间亨通光电累计涨幅达到14个点 但是前一天 在上午走出了当日最高点之后一路回落尾盘 收红 留下长下影线 我将这个信号视作滞涨 + 当晚美股对标股票康宁大跌4% 观察了每天亨通光电早上都有冲高回落迹象且都发生在10点左右 于是决定在这个附近清仓 其实一开始都是和预想到差不多 开盘股价一路下杀最后在10点左右开始反弹到开盘价附近 这个时候对我来说是清仓的好时机 因为本来这个仓位就是以短线为主 快进快出才是正解 开仓前我就思考好什么时候做中线什么时候做长线  亨通光电本来就是我想要用来做短线的一个标的 它的热度更好 辨识度更高 弹性也更好 事实证明确实如此 在反弹中我收到大量获利 。 但是如果回看上周五我其实是卖飞了 我认为自己没有做好的点 1. 太把外盘的走势当回事 虽然外盘股价确实与A股对应标的股价有部分相关关系 但不应该就当作全部 它只是参考 不能成为买卖的关键 。 2.昨天的上影线太明显了所有人都知道这是滞涨的信号 我也被这样的表象所迷惑 但或许也不是迷惑因为最近大盘轮转的很快 获利之后快速抽身也并不是错误 这个决定只能等待时间来检验
 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>200是思源电气这几日的短期低点这个地方应当有比较好的支撑，事实证明我做对了 两次探底200之后都得到了回收，但大盘抛压太重今天放量跌了2% 还在努力降低成本 有机会就高卖做t</t>
-  </si>
-  <si>
-    <t>思源电气</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>卖出</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>卖出逻辑</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>思源电气在昨天回踩了60日均线且伴随放量但是我并未有发现有什么利空消息在影响股价，一时间难以判断这到底是洗盘还是出货，今天A股全线暴涨思源电气只能说是表现平平，全天仍然缩量为防止踏空+降低风险今天确实应该减仓，这是我从上一次卖飞亨通光电收获的教训，不应该太赌气的清仓留一点悬念和可能性给自己，不要太多的确定性</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>002028</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>000988</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>华工科技</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>买入</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>长远来看华工科技在三月份连跌之后在短期已经出现明显的底部100作为一个短期支撑，同时今天放量收出阳线有反攻事态，总之这个位置是一个盈亏比例较好的位置，前面有前高141，下方有支撑位100，先小仓试错而后加仓。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>002281</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>光迅科技</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>光迅科技在最近的cpo板块里面是更加强势的股票
-鉴于之前在做亨通光电和长飞光纤的时候我选择了更加处于回调上升的亨通光电而错过了长飞的大涨，这让我觉得更应该选择强势的股票 不是看涨的多了就害怕，所以这里也加了2w仓位 决定在华工科技之间优中选优 去弱留强</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>今天看到光迅科技在早盘冲高，这时候有一个自我的警示就是等待情绪回落开盘从9:30-10:00这段时间是fomo的时间我认为这里存在着大量的交易噪音，一时间可能会被追涨的人群影响，10点之后继续观察 光迅科技价格仍旧坚挺且还有继续上冲的意图 这里可以大概判断出今天的上涨不是单纯的早盘fomo + 最近利空被消化+ 近期在cpo板块里的强势地位（逆势上涨）-&gt; 果断加仓</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">先买入的是光迅科技这里买入华工科技主要有以下考虑：1.作为同板块的个股 光迅科技的可见强势会在一定程度上带动华工科技 2.华工科技从形态上看比光迅科技更加让人安心 因为在3月份的大跌中 它已经铸成了一个显而易见的100作为低点 同时还站稳了5日线 高点明显+低点明显 盈亏比例在这里差不多有2:1 先把目标价格放在130左右 止损放在100元
-</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>思源电气最近的表现疲软虽然今天是4000家个股下跌，但相对于板块来说这几天的表现远远低于整体板块，伴随着缩量可以解读成买盘萎缩，卖盘也不强劲，预计会在这个箱体内横盘一段时间或者沿着60日支撑震荡，但短期出现行情的概率太低了，之前认为可能是洗盘，但现在来看更像是出货，为了规避风险同时尽可能博一点反弹预期 留了1层底仓 若持续低迷跌破60日均线 可以清仓</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>当日思源电气低开高走 一改往日颓势 上午我并没有急于追涨 因为想等大众的
-fomo情绪过去之后再入场 到了13:08的时候思源电气依然走强甚至拉高 这时候我认为前几日的杀跌只是洗盘 果断追涨买入</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>开盘之后思源电气大幅杀跌 又回到了前几日的低点 这并不符合之前的假设 如果是洗盘 今天不应该是这样杀跌 当然这依然可能是洗盘 我不能排除这样的可能性 但我想说的是自己没做好的一个点 ，那就是太急于下判断 上仓位了 这里我太鲁莽了 应该等到突破阻力位213进行确认再加仓的 我不知道这里到底是牛回了 还是拉高出货 那这个时候就是等价格确认是最好的 今天清仓的逻辑我也说不清楚 感觉是自己在很快的想要摆脱这种亏损 有种在赌气的感觉 操作不理性了 伴随着自己在cpo板块还有盈利今天总体是正盈利的 所以对割肉没有什么心理上的痛觉 只有对这个股票的失望（好奇怪 我不应该有这样的情绪的 为什么要对它失望 它不清楚我买了它 也没有涨的义务 我是来赚钱的 而不是来产生感情的 我感觉自己确实在一只股票上耗费了太大的感情 或者说精力当他不能为我赚钱或者有理由证明不强势的时候我应该离开 而不是死守着逻辑 或者它曾经给我带来过盈利作为借口而抓着不放</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">开盘强势 等fomo情绪退潮在下方接了个114的价位但我觉得接的还是太早了 应该在10点后等待均线确认后加仓 这个时候也消除了大部分开盘期间带来的噪音 现在发现在这种市场情况下 顺势而为 浮盈加仓才是一个让我觉得舒服的交易方式 之前一直跌一直补的做法太煎熬了 我感觉自己也不是一个很坚定的人 这套方法貌似不适合现在的我 
-</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>华工科技从下午开始就一路走强 这里我并不知道盘后会有什么消息（其实这里应该反省一下）因为今天下午其实就是华工科技一季报发布的时间，我当时居然不知道这个消息 以后绝对不能犯这种错误 对于持仓个股在时间线上的大事应该了如指掌才对 那也就意味着今天加仓的逻辑不是因为一季报的看好 而是发现分数图上华工科技突然的强势 + 量能温和放量 我认为这是一个不错的上升趋势票 + 自己本身盈利中 -&gt; 加仓200股</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>华工科技在昨日收盘发布一季报预告 很显然扣非之后不及机构预期 早盘开盘恐慌下杀之后被拉回至接近-轴，午后继续下杀最后-3.62%收盘 清了一半仓位一方面是规避风险落袋为安 因为无论今天是收涨还是如何 光模块近期也可能要到顶了 即使兑现一半的利润，留下了另一半仓位在于昨天的尾盘拉伸 我不认为是散户跟风买入 更可能消息交易者在买入 我不能排除洗盘的可能 同时今天利空出尽的前提下 底部资金有承接 尾盘又出现大量主买 故有吸筹的嫌疑</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>光迅科技还没发布季报预告这是一个不确定的点-&gt; 以后我要时刻关注这种时间点 尽量不要在这种公告时间点进行操作 波动太大反而不利于操作 + 今天光迅科技下跌大概率是收到华工科技的恐慌情绪带动的 + 已经有隐约的见顶信号 即使不见顶 都有回踩5日线的可能 +光模块最近涨的太多了+光迅科技最近趋势太好 回调无法避免</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>保本损，确保这一单不是亏损的，这笔交易做的并不好 ，止损不够果断，昨天清半仓的时候抱着防止卖飞的信念留了半仓，可是今天开盘之后一路下杀自己没有做好移动止损的计划 真正到了保本的时候才彻底清仓 这是失败的 我认为不能再用这种到了下跌才开始清仓的策略了 要测试一下在上涨中卖出的表现如何</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>601126</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>四方股份</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">四方股份目前处于低位 ， 叠加电网近期有反弹的趋势
-资金不可能一直在光通讯类的板块游动，需要将仓位调至不那么拥挤的赛道，且逻辑也足够硬的赛道，同时电网在这波下跌中已经见底迎来反弹，这时候需要选择一支高弹性的股票，我刻意避开了思源电气 虽然它是龙头股 但是我认为市值太大的情况下弹性不足 不适合短期持仓 四方股份的业绩 显然不如思源电气 增长速度也不行 但市场也没有给出比较大的预期这是一件好事 同时股价正从低位逐步修复 上方筹码也不多 抛压小 </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>这里在尾盘加了600股坦白地说是害怕明天行情就启动了的贸然出击，但是总觉得仓位不打到5w块心里不舒服，反而加完仓之后心情好了起来，这个操作确实有点冒失，但我想把它当作感觉的一部分不知道这对不对。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>这几天它可能要去摸48.5这个位置如果价格到了48.5意味着此时仓位浮盈来到5%这个时候加1100股也就是把浮盈摊到2.5%，成本线在47.31，这时候会遇到前期的一个平台位置48.62，如果遇到阻力被打下来了下方会有一个30日线支持（然而这个三十日线在最近一个月并不有效 ）充当的是一个阻力位的作用，同时这个时候下方也会有一个5日线支撑这里的短期支撑作用还在，但是这里直接把仓位double会不会有点太激进了，我能容扔的成本线只能往上继续移动到46.66这个位</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>负-7%的时候止损</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>看到价格高开并且往上冲 这个时候我没有着急下单 因为不知道是否是短期诱多 等到了9:45 其实不应该在这个时间点买入的 应该在10点等情绪真正平稳的时候才买入的 9:48 涨幅来到7%-8% 这个时候我能够确认昨晚到股权转让是利多消息 这个时候我起了贪念 直接加了3手仓位 也为后来10:13分我卖出1手做了铺垫</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">这个时候以为是真的被哟多了 我选择在这个时候卖出100股以求安稳 自己很显然被股价控制了操作 </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">四方股份的价格来到了我的加仓目标价 顺势在这个价格买入6手 </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -368,7 +410,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -391,23 +433,7 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="楷体"/>
-      <family val="3"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="楷体"/>
-      <family val="3"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="24"/>
+      <sz val="16"/>
       <color rgb="FFFF0000"/>
       <name val="楷体"/>
       <family val="3"/>
@@ -442,53 +468,15 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="21" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="21" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1000,86 +988,83 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O357"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="17"/>
+  <dimension ref="A1:O99"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="24"/>
   <cols>
-    <col min="1" max="1" width="22.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.1640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.1640625" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="22.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="29.5" style="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="43.83203125" style="10" customWidth="1"/>
-    <col min="12" max="12" width="27.6640625" style="10" customWidth="1"/>
-    <col min="13" max="13" width="49" style="10" customWidth="1"/>
-    <col min="14" max="14" width="255.83203125" style="10" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="39.1640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="10.33203125" style="6"/>
+    <col min="1" max="2" width="22.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="8" width="22.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="43.83203125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="27.6640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="49" style="1" customWidth="1"/>
+    <col min="14" max="14" width="255.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="39.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="10.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="12" customFormat="1" ht="23.25" customHeight="1">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="12" t="s">
+    <row r="1" spans="1:15" s="2" customFormat="1" ht="23.25" customHeight="1">
+      <c r="A1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="12" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="2" spans="1:15" ht="20.5" customHeight="1">
       <c r="A2" s="1">
         <v>600276</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1">
         <v>20250902</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>0.39598379629629599</v>
       </c>
       <c r="F2" s="1">
@@ -1099,26 +1084,21 @@
         <f>SUMIFS($G$2:G2,$A$2:A2,$A2)</f>
         <v>200</v>
       </c>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-    </row>
-    <row r="3" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="3" spans="1:15" ht="20.5" customHeight="1">
       <c r="A3" s="1">
         <v>600276</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D3" s="1">
         <v>20250903</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>0.40028935185185199</v>
       </c>
       <c r="F3" s="1">
@@ -1138,26 +1118,21 @@
         <f>SUMIFS($G$2:G3,$A$2:A3,$A3)</f>
         <v>0</v>
       </c>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-    </row>
-    <row r="4" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="4" spans="1:15" ht="20.5" customHeight="1">
       <c r="A4" s="1">
         <v>601138</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D4" s="1">
         <v>20250912</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>0.40763888888888899</v>
       </c>
       <c r="F4" s="1">
@@ -1177,26 +1152,21 @@
         <f>SUMIFS($G$2:G4,$A$2:A4,$A4)</f>
         <v>400</v>
       </c>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-    </row>
-    <row r="5" spans="1:15" s="3" customFormat="1" ht="20" customHeight="1">
+    </row>
+    <row r="5" spans="1:15" ht="20" customHeight="1">
       <c r="A5" s="1">
         <v>601138</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D5" s="1">
         <v>20250915</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>0.59178240740740695</v>
       </c>
       <c r="F5" s="1">
@@ -1216,26 +1186,21 @@
         <f>SUMIFS($G$2:G5,$A$2:A5,$A5)</f>
         <v>500</v>
       </c>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-    </row>
-    <row r="6" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="6" spans="1:15" ht="20.5" customHeight="1">
       <c r="A6" s="1">
         <v>601138</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D6" s="1">
         <v>20250915</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>0.399363425925926</v>
       </c>
       <c r="F6" s="1">
@@ -1255,26 +1220,21 @@
         <f>SUMIFS($G$2:G6,$A$2:A6,$A6)</f>
         <v>600</v>
       </c>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-    </row>
-    <row r="7" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="7" spans="1:15" ht="20.5" customHeight="1">
       <c r="A7" s="1">
         <v>603986</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D7" s="1">
         <v>20250925</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>0.60934027777777799</v>
       </c>
       <c r="F7" s="1">
@@ -1294,26 +1254,21 @@
         <f>SUMIFS($G$2:G7,$A$2:A7,$A7)</f>
         <v>100</v>
       </c>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-    </row>
-    <row r="8" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="8" spans="1:15" ht="20.5" customHeight="1">
       <c r="A8" s="1">
         <v>601138</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D8" s="1">
         <v>20251009</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>0.446851851851852</v>
       </c>
       <c r="F8" s="1">
@@ -1333,26 +1288,21 @@
         <f>SUMIFS($G$2:G8,$A$2:A8,$A8)</f>
         <v>400</v>
       </c>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-    </row>
-    <row r="9" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="9" spans="1:15" ht="20.5" customHeight="1">
       <c r="A9" s="1">
         <v>600111</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D9" s="1">
         <v>20251010</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>0.41733796296296299</v>
       </c>
       <c r="F9" s="1">
@@ -1372,26 +1322,21 @@
         <f>SUMIFS($G$2:G9,$A$2:A9,$A9)</f>
         <v>200</v>
       </c>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-    </row>
-    <row r="10" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="10" spans="1:15" ht="20.5" customHeight="1">
       <c r="A10" s="1">
         <v>600111</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D10" s="1">
         <v>20251010</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>0.39657407407407402</v>
       </c>
       <c r="F10" s="1">
@@ -1411,26 +1356,21 @@
         <f>SUMIFS($G$2:G10,$A$2:A10,$A10)</f>
         <v>500</v>
       </c>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
-    </row>
-    <row r="11" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="11" spans="1:15" ht="20.5" customHeight="1">
       <c r="A11" s="1">
         <v>601138</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D11" s="1">
         <v>20251015</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>0.45391203703703698</v>
       </c>
       <c r="F11" s="1">
@@ -1450,26 +1390,21 @@
         <f>SUMIFS($G$2:G11,$A$2:A11,$A11)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-    </row>
-    <row r="12" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="12" spans="1:15" ht="20.5" customHeight="1">
       <c r="A12" s="1">
         <v>603986</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D12" s="1">
         <v>20251015</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>0.45378472222222199</v>
       </c>
       <c r="F12" s="1">
@@ -1489,26 +1424,21 @@
         <f>SUMIFS($G$2:G12,$A$2:A12,$A12)</f>
         <v>0</v>
       </c>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-    </row>
-    <row r="13" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="13" spans="1:15" ht="20.5" customHeight="1">
       <c r="A13" s="1">
         <v>600111</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D13" s="1">
         <v>20251015</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>0.42269675925925898</v>
       </c>
       <c r="F13" s="1">
@@ -1528,27 +1458,22 @@
         <f>SUMIFS($G$2:G13,$A$2:A13,$A13)</f>
         <v>0</v>
       </c>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-    </row>
-    <row r="14" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="14" spans="1:15" ht="20.5" customHeight="1">
       <c r="A14" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D14" s="1">
         <v>20251016</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>0.56047453703703698</v>
       </c>
       <c r="F14" s="1">
@@ -1568,26 +1493,21 @@
         <f>SUMIFS($G$2:G14,$A$2:A14,$A14)</f>
         <v>600</v>
       </c>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-    </row>
-    <row r="15" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="15" spans="1:15" ht="20.5" customHeight="1">
       <c r="A15" s="1">
         <v>603259</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D15" s="1">
         <v>20251016</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>0.45853009259259297</v>
       </c>
       <c r="F15" s="1">
@@ -1607,27 +1527,22 @@
         <f>SUMIFS($G$2:G15,$A$2:A15,$A15)</f>
         <v>100</v>
       </c>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-    </row>
-    <row r="16" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="16" spans="1:15" ht="20.5" customHeight="1">
       <c r="A16" s="1" t="str">
         <f>"002371"</f>
         <v>002371</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D16" s="1">
         <v>20251017</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>0.625</v>
       </c>
       <c r="F16" s="1">
@@ -1647,27 +1562,22 @@
         <f>SUMIFS($G$2:G16,$A$2:A16,$A16)</f>
         <v>100</v>
       </c>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-    </row>
-    <row r="17" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="17" spans="1:10" ht="20.5" customHeight="1">
       <c r="A17" s="1" t="str">
         <f>"002281"</f>
         <v>002281</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="D17" s="1">
         <v>20251021</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>0.62155092592592598</v>
       </c>
       <c r="F17" s="1">
@@ -1687,26 +1597,21 @@
         <f>SUMIFS($G$2:G17,$A$2:A17,$A17)</f>
         <v>300</v>
       </c>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-    </row>
-    <row r="18" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="18" spans="1:10" ht="20.5" customHeight="1">
       <c r="A18" s="1">
         <v>603259</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D18" s="1">
         <v>20251021</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>0.46806712962962999</v>
       </c>
       <c r="F18" s="1">
@@ -1726,27 +1631,22 @@
         <f>SUMIFS($G$2:G18,$A$2:A18,$A18)</f>
         <v>0</v>
       </c>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-    </row>
-    <row r="19" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="19" spans="1:10" ht="20.5" customHeight="1">
       <c r="A19" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D19" s="1">
         <v>20251021</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>0.41851851851851901</v>
       </c>
       <c r="F19" s="1">
@@ -1766,26 +1666,21 @@
         <f>SUMIFS($G$2:G19,$A$2:A19,$A19)</f>
         <v>400</v>
       </c>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-    </row>
-    <row r="20" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="20" spans="1:10" ht="20.5" customHeight="1">
       <c r="A20" s="1">
         <v>603986</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D20" s="1">
         <v>20251023</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>0.61777777777777798</v>
       </c>
       <c r="F20" s="1">
@@ -1805,27 +1700,22 @@
         <f>SUMIFS($G$2:G20,$A$2:A20,$A20)</f>
         <v>200</v>
       </c>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-    </row>
-    <row r="21" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="21" spans="1:10" ht="20.5" customHeight="1">
       <c r="A21" s="1" t="str">
         <f>"002371"</f>
         <v>002371</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="D21" s="1">
         <v>20251023</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>0.61611111111111105</v>
       </c>
       <c r="F21" s="1">
@@ -1845,27 +1735,22 @@
         <f>SUMIFS($G$2:G21,$A$2:A21,$A21)</f>
         <v>0</v>
       </c>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-    </row>
-    <row r="22" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="22" spans="1:10" ht="20.5" customHeight="1">
       <c r="A22" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D22" s="1">
         <v>20251024</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>0.60100694444444402</v>
       </c>
       <c r="F22" s="1">
@@ -1885,26 +1770,21 @@
         <f>SUMIFS($G$2:G22,$A$2:A22,$A22)</f>
         <v>300</v>
       </c>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
-    </row>
-    <row r="23" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="23" spans="1:10" ht="20.5" customHeight="1">
       <c r="A23" s="1">
         <v>603986</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D23" s="1">
         <v>20251024</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>0.58921296296296299</v>
       </c>
       <c r="F23" s="1">
@@ -1924,27 +1804,22 @@
         <f>SUMIFS($G$2:G23,$A$2:A23,$A23)</f>
         <v>100</v>
       </c>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-    </row>
-    <row r="24" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="24" spans="1:10" ht="20.5" customHeight="1">
       <c r="A24" s="1" t="str">
         <f>"002281"</f>
         <v>002281</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="D24" s="1">
         <v>20251024</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>0.41842592592592598</v>
       </c>
       <c r="F24" s="1">
@@ -1964,26 +1839,21 @@
         <f>SUMIFS($G$2:G24,$A$2:A24,$A24)</f>
         <v>0</v>
       </c>
-      <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
-    </row>
-    <row r="25" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="25" spans="1:10" ht="20.5" customHeight="1">
       <c r="A25" s="1">
         <v>603083</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="D25" s="1">
         <v>20251027</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>0.39907407407407403</v>
       </c>
       <c r="F25" s="1">
@@ -2003,26 +1873,21 @@
         <f>SUMIFS($G$2:G25,$A$2:A25,$A25)</f>
         <v>200</v>
       </c>
-      <c r="K25" s="1"/>
-      <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
-      <c r="N25" s="1"/>
-      <c r="O25" s="1"/>
-    </row>
-    <row r="26" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="26" spans="1:10" ht="20.5" customHeight="1">
       <c r="A26" s="1">
         <v>603083</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D26" s="1">
         <v>20251028</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>0.625</v>
       </c>
       <c r="F26" s="1">
@@ -2041,26 +1906,21 @@
         <f>SUMIFS($G$2:G26,$A$2:A26,$A26)</f>
         <v>0</v>
       </c>
-      <c r="K26" s="1"/>
-      <c r="L26" s="1"/>
-      <c r="M26" s="1"/>
-      <c r="N26" s="1"/>
-      <c r="O26" s="1"/>
-    </row>
-    <row r="27" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="27" spans="1:10" ht="20.5" customHeight="1">
       <c r="A27" s="1">
         <v>603986</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D27" s="1">
         <v>20251029</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>0.44155092592592599</v>
       </c>
       <c r="F27" s="1">
@@ -2080,26 +1940,21 @@
         <f>SUMIFS($G$2:G27,$A$2:A27,$A27)</f>
         <v>0</v>
       </c>
-      <c r="K27" s="1"/>
-      <c r="L27" s="1"/>
-      <c r="M27" s="1"/>
-      <c r="N27" s="1"/>
-      <c r="O27" s="1"/>
-    </row>
-    <row r="28" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="28" spans="1:10" ht="20.5" customHeight="1">
       <c r="A28" s="1">
         <v>603799</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D28" s="1">
         <v>20251030</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>0.56559027777777804</v>
       </c>
       <c r="F28" s="1">
@@ -2119,26 +1974,21 @@
         <f>SUMIFS($G$2:G28,$A$2:A28,$A28)</f>
         <v>300</v>
       </c>
-      <c r="K28" s="1"/>
-      <c r="L28" s="1"/>
-      <c r="M28" s="1"/>
-      <c r="N28" s="1"/>
-      <c r="O28" s="1"/>
-    </row>
-    <row r="29" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="29" spans="1:10" ht="20.5" customHeight="1">
       <c r="A29" s="1">
         <v>603986</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D29" s="1">
         <v>20251030</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>0.544988425925926</v>
       </c>
       <c r="F29" s="1">
@@ -2158,26 +2008,21 @@
         <f>SUMIFS($G$2:G29,$A$2:A29,$A29)</f>
         <v>100</v>
       </c>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-    </row>
-    <row r="30" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="30" spans="1:10" ht="20.5" customHeight="1">
       <c r="A30" s="1">
         <v>603099</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D30" s="1">
         <v>20251104</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>0.625</v>
       </c>
       <c r="F30" s="1">
@@ -2197,26 +2042,21 @@
         <f>SUMIFS($G$2:G30,$A$2:A30,$A30)</f>
         <v>100</v>
       </c>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-    </row>
-    <row r="31" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="31" spans="1:10" ht="20.5" customHeight="1">
       <c r="A31" s="1">
         <v>603099</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D31" s="1">
         <v>20251104</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>0.625</v>
       </c>
       <c r="F31" s="1">
@@ -2236,26 +2076,21 @@
         <f>SUMIFS($G$2:G31,$A$2:A31,$A31)</f>
         <v>200</v>
       </c>
-      <c r="K31" s="1"/>
-      <c r="L31" s="1"/>
-      <c r="M31" s="1"/>
-      <c r="N31" s="1"/>
-      <c r="O31" s="1"/>
-    </row>
-    <row r="32" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="32" spans="1:10" ht="20.5" customHeight="1">
       <c r="A32" s="1">
         <v>603799</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D32" s="1">
         <v>20251104</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>0.625</v>
       </c>
       <c r="F32" s="1">
@@ -2275,26 +2110,21 @@
         <f>SUMIFS($G$2:G32,$A$2:A32,$A32)</f>
         <v>0</v>
       </c>
-      <c r="K32" s="1"/>
-      <c r="L32" s="1"/>
-      <c r="M32" s="1"/>
-      <c r="N32" s="1"/>
-      <c r="O32" s="1"/>
-    </row>
-    <row r="33" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="33" spans="1:10" ht="20.5" customHeight="1">
       <c r="A33" s="1">
         <v>603099</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="D33" s="1">
         <v>20251105</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>0.41347222222222202</v>
       </c>
       <c r="F33" s="1">
@@ -2314,27 +2144,22 @@
         <f>SUMIFS($G$2:G33,$A$2:A33,$A33)</f>
         <v>0</v>
       </c>
-      <c r="K33" s="1"/>
-      <c r="L33" s="1"/>
-      <c r="M33" s="1"/>
-      <c r="N33" s="1"/>
-      <c r="O33" s="1"/>
-    </row>
-    <row r="34" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="34" spans="1:10" ht="20.5" customHeight="1">
       <c r="A34" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D34" s="1">
         <v>20260119</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>0.42253472222222199</v>
       </c>
       <c r="F34" s="1">
@@ -2354,26 +2179,21 @@
         <f>SUMIFS($G$2:G34,$A$2:A34,$A34)</f>
         <v>100</v>
       </c>
-      <c r="K34" s="1"/>
-      <c r="L34" s="1"/>
-      <c r="M34" s="1"/>
-      <c r="N34" s="1"/>
-      <c r="O34" s="1"/>
-    </row>
-    <row r="35" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="35" spans="1:10" ht="20.5" customHeight="1">
       <c r="A35" s="1">
         <v>601179</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D35" s="1">
         <v>20260119</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>0.40089120370370401</v>
       </c>
       <c r="F35" s="1">
@@ -2393,27 +2213,22 @@
         <f>SUMIFS($G$2:G35,$A$2:A35,$A35)</f>
         <v>1400</v>
       </c>
-      <c r="K35" s="1"/>
-      <c r="L35" s="1"/>
-      <c r="M35" s="1"/>
-      <c r="N35" s="1"/>
-      <c r="O35" s="1"/>
-    </row>
-    <row r="36" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="36" spans="1:10" ht="20.5" customHeight="1">
       <c r="A36" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D36" s="1">
         <v>20260119</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>0.39848379629629599</v>
       </c>
       <c r="F36" s="1">
@@ -2433,26 +2248,21 @@
         <f>SUMIFS($G$2:G36,$A$2:A36,$A36)</f>
         <v>200</v>
       </c>
-      <c r="K36" s="1"/>
-      <c r="L36" s="1"/>
-      <c r="M36" s="1"/>
-      <c r="N36" s="1"/>
-      <c r="O36" s="1"/>
-    </row>
-    <row r="37" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="37" spans="1:10" ht="20.5" customHeight="1">
       <c r="A37" s="1">
         <v>603986</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D37" s="1">
         <v>20260119</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>0.39603009259259297</v>
       </c>
       <c r="F37" s="1">
@@ -2472,27 +2282,22 @@
         <f>SUMIFS($G$2:G37,$A$2:A37,$A37)</f>
         <v>0</v>
       </c>
-      <c r="K37" s="1"/>
-      <c r="L37" s="1"/>
-      <c r="M37" s="1"/>
-      <c r="N37" s="1"/>
-      <c r="O37" s="1"/>
-    </row>
-    <row r="38" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="38" spans="1:10" ht="20.5" customHeight="1">
       <c r="A38" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D38" s="1">
         <v>20260121</v>
       </c>
-      <c r="E38" s="2">
+      <c r="E38" s="1">
         <v>0.39738425925925902</v>
       </c>
       <c r="F38" s="1">
@@ -2512,27 +2317,22 @@
         <f>SUMIFS($G$2:G38,$A$2:A38,$A38)</f>
         <v>300</v>
       </c>
-      <c r="K38" s="1"/>
-      <c r="L38" s="1"/>
-      <c r="M38" s="1"/>
-      <c r="N38" s="1"/>
-      <c r="O38" s="1"/>
-    </row>
-    <row r="39" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="39" spans="1:10" ht="20.5" customHeight="1">
       <c r="A39" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D39" s="1">
         <v>20260122</v>
       </c>
-      <c r="E39" s="2">
+      <c r="E39" s="1">
         <v>0.44486111111111099</v>
       </c>
       <c r="F39" s="1">
@@ -2552,26 +2352,21 @@
         <f>SUMIFS($G$2:G39,$A$2:A39,$A39)</f>
         <v>400</v>
       </c>
-      <c r="K39" s="1"/>
-      <c r="L39" s="1"/>
-      <c r="M39" s="1"/>
-      <c r="N39" s="1"/>
-      <c r="O39" s="1"/>
-    </row>
-    <row r="40" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="40" spans="1:10" ht="20.5" customHeight="1">
       <c r="A40" s="1">
         <v>600584</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D40" s="1">
         <v>20260122</v>
       </c>
-      <c r="E40" s="2">
+      <c r="E40" s="1">
         <v>0.40795138888888899</v>
       </c>
       <c r="F40" s="1">
@@ -2591,26 +2386,21 @@
         <f>SUMIFS($G$2:G40,$A$2:A40,$A40)</f>
         <v>400</v>
       </c>
-      <c r="K40" s="1"/>
-      <c r="L40" s="1"/>
-      <c r="M40" s="1"/>
-      <c r="N40" s="1"/>
-      <c r="O40" s="1"/>
-    </row>
-    <row r="41" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="41" spans="1:10" ht="20.5" customHeight="1">
       <c r="A41" s="1">
         <v>601179</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D41" s="1">
         <v>20260126</v>
       </c>
-      <c r="E41" s="2">
+      <c r="E41" s="1">
         <v>0.62217592592592597</v>
       </c>
       <c r="F41" s="1">
@@ -2630,26 +2420,21 @@
         <f>SUMIFS($G$2:G41,$A$2:A41,$A41)</f>
         <v>700</v>
       </c>
-      <c r="K41" s="1"/>
-      <c r="L41" s="1"/>
-      <c r="M41" s="1"/>
-      <c r="N41" s="1"/>
-      <c r="O41" s="1"/>
-    </row>
-    <row r="42" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="42" spans="1:10" ht="20.5" customHeight="1">
       <c r="A42" s="1">
         <v>600584</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D42" s="1">
         <v>20260127</v>
       </c>
-      <c r="E42" s="2">
+      <c r="E42" s="1">
         <v>0.589479166666667</v>
       </c>
       <c r="F42" s="1">
@@ -2669,27 +2454,22 @@
         <f>SUMIFS($G$2:G42,$A$2:A42,$A42)</f>
         <v>600</v>
       </c>
-      <c r="K42" s="1"/>
-      <c r="L42" s="1"/>
-      <c r="M42" s="1"/>
-      <c r="N42" s="1"/>
-      <c r="O42" s="1"/>
-    </row>
-    <row r="43" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="43" spans="1:10" ht="20.5" customHeight="1">
       <c r="A43" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D43" s="1">
         <v>20260127</v>
       </c>
-      <c r="E43" s="2">
+      <c r="E43" s="1">
         <v>0.41396990740740702</v>
       </c>
       <c r="F43" s="1">
@@ -2709,27 +2489,22 @@
         <f>SUMIFS($G$2:G43,$A$2:A43,$A43)</f>
         <v>500</v>
       </c>
-      <c r="K43" s="1"/>
-      <c r="L43" s="1"/>
-      <c r="M43" s="1"/>
-      <c r="N43" s="1"/>
-      <c r="O43" s="1"/>
-    </row>
-    <row r="44" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="44" spans="1:10" ht="20.5" customHeight="1">
       <c r="A44" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D44" s="1">
         <v>20260129</v>
       </c>
-      <c r="E44" s="2">
+      <c r="E44" s="1">
         <v>0.57781249999999995</v>
       </c>
       <c r="F44" s="1">
@@ -2749,27 +2524,22 @@
         <f>SUMIFS($G$2:G44,$A$2:A44,$A44)</f>
         <v>500</v>
       </c>
-      <c r="K44" s="1"/>
-      <c r="L44" s="1"/>
-      <c r="M44" s="1"/>
-      <c r="N44" s="1"/>
-      <c r="O44" s="1"/>
-    </row>
-    <row r="45" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="45" spans="1:10" ht="20.5" customHeight="1">
       <c r="A45" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D45" s="1">
         <v>20260129</v>
       </c>
-      <c r="E45" s="2">
+      <c r="E45" s="1">
         <v>0.57199074074074097</v>
       </c>
       <c r="F45" s="1">
@@ -2789,26 +2559,21 @@
         <f>SUMIFS($G$2:G45,$A$2:A45,$A45)</f>
         <v>400</v>
       </c>
-      <c r="K45" s="1"/>
-      <c r="L45" s="1"/>
-      <c r="M45" s="1"/>
-      <c r="N45" s="1"/>
-      <c r="O45" s="1"/>
-    </row>
-    <row r="46" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="46" spans="1:10" ht="20.5" customHeight="1">
       <c r="A46" s="1">
         <v>600584</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D46" s="1">
         <v>20260129</v>
       </c>
-      <c r="E46" s="2">
+      <c r="E46" s="1">
         <v>0.57099537037036996</v>
       </c>
       <c r="F46" s="1">
@@ -2828,27 +2593,22 @@
         <f>SUMIFS($G$2:G46,$A$2:A46,$A46)</f>
         <v>400</v>
       </c>
-      <c r="K46" s="1"/>
-      <c r="L46" s="1"/>
-      <c r="M46" s="1"/>
-      <c r="N46" s="1"/>
-      <c r="O46" s="1"/>
-    </row>
-    <row r="47" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="47" spans="1:10" ht="20.5" customHeight="1">
       <c r="A47" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D47" s="1">
         <v>20260129</v>
       </c>
-      <c r="E47" s="2">
+      <c r="E47" s="1">
         <v>0.54546296296296304</v>
       </c>
       <c r="F47" s="1">
@@ -2868,27 +2628,22 @@
         <f>SUMIFS($G$2:G47,$A$2:A47,$A47)</f>
         <v>500</v>
       </c>
-      <c r="K47" s="1"/>
-      <c r="L47" s="1"/>
-      <c r="M47" s="1"/>
-      <c r="N47" s="1"/>
-      <c r="O47" s="1"/>
-    </row>
-    <row r="48" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="48" spans="1:10" ht="20.5" customHeight="1">
       <c r="A48" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D48" s="1">
         <v>20260129</v>
       </c>
-      <c r="E48" s="2">
+      <c r="E48" s="1">
         <v>0.54239583333333297</v>
       </c>
       <c r="F48" s="1">
@@ -2908,26 +2663,21 @@
         <f>SUMIFS($G$2:G48,$A$2:A48,$A48)</f>
         <v>600</v>
       </c>
-      <c r="K48" s="1"/>
-      <c r="L48" s="1"/>
-      <c r="M48" s="1"/>
-      <c r="N48" s="1"/>
-      <c r="O48" s="1"/>
-    </row>
-    <row r="49" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="49" spans="1:14" ht="20.5" customHeight="1">
       <c r="A49" s="1">
         <v>601179</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D49" s="1">
         <v>20260130</v>
       </c>
-      <c r="E49" s="2">
+      <c r="E49" s="1">
         <v>0.44043981481481498</v>
       </c>
       <c r="F49" s="1">
@@ -2947,27 +2697,22 @@
         <f>SUMIFS($G$2:G49,$A$2:A49,$A49)</f>
         <v>1100</v>
       </c>
-      <c r="K49" s="1"/>
-      <c r="L49" s="1"/>
-      <c r="M49" s="1"/>
-      <c r="N49" s="1"/>
-      <c r="O49" s="1"/>
-    </row>
-    <row r="50" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="50" spans="1:14" ht="20.5" customHeight="1">
       <c r="A50" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D50" s="1">
         <v>20260130</v>
       </c>
-      <c r="E50" s="2">
+      <c r="E50" s="1">
         <v>0.43103009259259301</v>
       </c>
       <c r="F50" s="1">
@@ -2987,27 +2732,22 @@
         <f>SUMIFS($G$2:G50,$A$2:A50,$A50)</f>
         <v>700</v>
       </c>
-      <c r="K50" s="1"/>
-      <c r="L50" s="1"/>
-      <c r="M50" s="1"/>
-      <c r="N50" s="1"/>
-      <c r="O50" s="1"/>
-    </row>
-    <row r="51" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="51" spans="1:14" ht="20.5" customHeight="1">
       <c r="A51" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D51" s="1">
         <v>20260202</v>
       </c>
-      <c r="E51" s="2">
+      <c r="E51" s="1">
         <v>0.61899305555555595</v>
       </c>
       <c r="F51" s="1">
@@ -3027,26 +2767,21 @@
         <f>SUMIFS($G$2:G51,$A$2:A51,$A51)</f>
         <v>200</v>
       </c>
-      <c r="K51" s="1"/>
-      <c r="L51" s="1"/>
-      <c r="M51" s="1"/>
-      <c r="N51" s="1"/>
-      <c r="O51" s="1"/>
-    </row>
-    <row r="52" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="52" spans="1:14" ht="20.5" customHeight="1">
       <c r="A52" s="1">
         <v>600584</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D52" s="1">
         <v>20260202</v>
       </c>
-      <c r="E52" s="2">
+      <c r="E52" s="1">
         <v>0.56569444444444394</v>
       </c>
       <c r="F52" s="1">
@@ -3066,26 +2801,21 @@
         <f>SUMIFS($G$2:G52,$A$2:A52,$A52)</f>
         <v>500</v>
       </c>
-      <c r="K52" s="1"/>
-      <c r="L52" s="1"/>
-      <c r="M52" s="1"/>
-      <c r="N52" s="1"/>
-      <c r="O52" s="1"/>
-    </row>
-    <row r="53" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="53" spans="1:14" ht="20.5" customHeight="1">
       <c r="A53" s="1">
         <v>601179</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D53" s="1">
         <v>20260202</v>
       </c>
-      <c r="E53" s="2">
+      <c r="E53" s="1">
         <v>0.55994212962962997</v>
       </c>
       <c r="F53" s="1">
@@ -3105,27 +2835,22 @@
         <f>SUMIFS($G$2:G53,$A$2:A53,$A53)</f>
         <v>0</v>
       </c>
-      <c r="K53" s="1"/>
-      <c r="L53" s="1"/>
-      <c r="M53" s="1"/>
-      <c r="N53" s="1"/>
-      <c r="O53" s="1"/>
-    </row>
-    <row r="54" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="54" spans="1:14" ht="20.5" customHeight="1">
       <c r="A54" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D54" s="1">
         <v>20260202</v>
       </c>
-      <c r="E54" s="2">
+      <c r="E54" s="1">
         <v>0.44674768518518498</v>
       </c>
       <c r="F54" s="1">
@@ -3145,27 +2870,22 @@
         <f>SUMIFS($G$2:G54,$A$2:A54,$A54)</f>
         <v>600</v>
       </c>
-      <c r="K54" s="1"/>
-      <c r="L54" s="1"/>
-      <c r="M54" s="1"/>
-      <c r="N54" s="1"/>
-      <c r="O54" s="1"/>
-    </row>
-    <row r="55" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="55" spans="1:14" ht="20.5" customHeight="1">
       <c r="A55" s="1" t="str">
         <f>"002475"</f>
         <v>002475</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D55" s="1">
         <v>20260202</v>
       </c>
-      <c r="E55" s="2">
+      <c r="E55" s="1">
         <v>0.44067129629629598</v>
       </c>
       <c r="F55" s="1">
@@ -3185,27 +2905,22 @@
         <f>SUMIFS($G$2:G55,$A$2:A55,$A55)</f>
         <v>0</v>
       </c>
-      <c r="K55" s="1"/>
-      <c r="L55" s="1"/>
-      <c r="M55" s="1"/>
-      <c r="N55" s="1"/>
-      <c r="O55" s="1"/>
-    </row>
-    <row r="56" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="56" spans="1:14" ht="20.5" customHeight="1">
       <c r="A56" s="1" t="str">
         <f>"002028"</f>
         <v>002028</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D56" s="1">
         <v>20260203</v>
       </c>
-      <c r="E56" s="2">
+      <c r="E56" s="1">
         <v>0.40917824074074099</v>
       </c>
       <c r="F56" s="1">
@@ -3225,27 +2940,22 @@
         <f>SUMIFS($G$2:G56,$A$2:A56,$A56)</f>
         <v>500</v>
       </c>
-      <c r="K56" s="1"/>
-      <c r="L56" s="1"/>
-      <c r="M56" s="1"/>
-      <c r="N56" s="1"/>
-      <c r="O56" s="1"/>
-    </row>
-    <row r="57" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="57" spans="1:14" ht="20.5" customHeight="1">
       <c r="A57" s="1" t="str">
         <f t="shared" ref="A57:A62" si="0">"002028"</f>
         <v>002028</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D57" s="1">
         <v>20260205</v>
       </c>
-      <c r="E57" s="2">
+      <c r="E57" s="1">
         <v>0.404363425925926</v>
       </c>
       <c r="F57" s="1">
@@ -3265,27 +2975,22 @@
         <f>SUMIFS($G$2:G57,$A$2:A57,$A57)</f>
         <v>600</v>
       </c>
-      <c r="K57" s="1"/>
-      <c r="L57" s="1"/>
-      <c r="M57" s="1"/>
-      <c r="N57" s="1"/>
-      <c r="O57" s="1"/>
-    </row>
-    <row r="58" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="58" spans="1:14" ht="20.5" customHeight="1">
       <c r="A58" s="1" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D58" s="1">
         <v>20260209</v>
       </c>
-      <c r="E58" s="2">
+      <c r="E58" s="1">
         <v>0.44548611111111103</v>
       </c>
       <c r="F58" s="1">
@@ -3305,26 +3010,21 @@
         <f>SUMIFS($G$2:G58,$A$2:A58,$A58)</f>
         <v>700</v>
       </c>
-      <c r="K58" s="1"/>
-      <c r="L58" s="1"/>
-      <c r="M58" s="1"/>
-      <c r="N58" s="1"/>
-      <c r="O58" s="1"/>
-    </row>
-    <row r="59" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="59" spans="1:14" ht="20.5" customHeight="1">
       <c r="A59" s="1">
         <v>600584</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D59" s="1">
         <v>20260209</v>
       </c>
-      <c r="E59" s="2">
+      <c r="E59" s="1">
         <v>0.43886574074074097</v>
       </c>
       <c r="F59" s="1">
@@ -3344,27 +3044,22 @@
         <f>SUMIFS($G$2:G59,$A$2:A59,$A59)</f>
         <v>700</v>
       </c>
-      <c r="K59" s="1"/>
-      <c r="L59" s="1"/>
-      <c r="M59" s="1"/>
-      <c r="N59" s="1"/>
-      <c r="O59" s="1"/>
-    </row>
-    <row r="60" spans="1:15" s="3" customFormat="1" ht="20.5" customHeight="1">
+    </row>
+    <row r="60" spans="1:14" ht="20.5" customHeight="1">
       <c r="A60" s="1" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D60" s="1">
         <v>20260209</v>
       </c>
-      <c r="E60" s="2">
+      <c r="E60" s="1">
         <v>0.41059027777777801</v>
       </c>
       <c r="F60" s="1">
@@ -3384,26 +3079,21 @@
         <f>SUMIFS($G$2:G60,$A$2:A60,$A60)</f>
         <v>500</v>
       </c>
-      <c r="K60" s="1"/>
-      <c r="L60" s="1"/>
-      <c r="M60" s="1"/>
-      <c r="N60" s="1"/>
-      <c r="O60" s="1"/>
-    </row>
-    <row r="61" spans="1:15" ht="16" customHeight="1">
+    </row>
+    <row r="61" spans="1:14" ht="16" customHeight="1">
       <c r="A61" s="1">
         <v>600584</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D61" s="1">
         <v>20260226</v>
       </c>
-      <c r="E61" s="2">
+      <c r="E61" s="1">
         <v>0.54913194444444402</v>
       </c>
       <c r="F61" s="1">
@@ -3415,38 +3105,35 @@
       <c r="H61" s="1">
         <v>19320</v>
       </c>
-      <c r="I61" s="4"/>
       <c r="J61" s="1">
         <f>SUMIFS($G$2:G61,$A$2:A61,$A61)</f>
         <v>1100</v>
       </c>
-      <c r="K61" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="L61" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M61" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="N61" s="4"/>
-      <c r="O61" s="1"/>
-    </row>
-    <row r="62" spans="1:15" ht="150">
+      <c r="K61" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="L61" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="M61" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14">
       <c r="A62" s="1" t="str">
         <f t="shared" si="0"/>
         <v>002028</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D62" s="1">
         <v>20260227</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E62" s="1">
         <v>0.40364583333333298</v>
       </c>
       <c r="F62" s="1">
@@ -3458,37 +3145,34 @@
       <c r="H62" s="1">
         <v>21850</v>
       </c>
-      <c r="I62" s="4"/>
       <c r="J62" s="1">
         <f>SUMIFS($G$2:G62,$A$2:A62,$A62)</f>
         <v>600</v>
       </c>
-      <c r="K62" s="5" t="s">
-        <v>37</v>
+      <c r="K62" s="1" t="s">
+        <v>64</v>
       </c>
       <c r="L62" s="1" t="s">
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="M62" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="N62" s="4"/>
-      <c r="O62" s="1"/>
-    </row>
-    <row r="63" spans="1:15" ht="77" customHeight="1">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" ht="77" customHeight="1">
       <c r="A63" s="1">
         <v>600584</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>40</v>
+        <v>67</v>
       </c>
       <c r="D63" s="1">
         <v>20260309</v>
       </c>
-      <c r="E63" s="2">
+      <c r="E63" s="1">
         <v>0.61805555555555602</v>
       </c>
       <c r="F63" s="1">
@@ -3500,33 +3184,28 @@
       <c r="H63" s="1">
         <v>27018</v>
       </c>
-      <c r="I63" s="4"/>
       <c r="J63" s="1">
         <f>SUMIFS($G$2:G63,$A$2:A63,$A63)</f>
         <v>500</v>
       </c>
-      <c r="K63" s="4"/>
-      <c r="L63" s="4"/>
-      <c r="M63" s="4"/>
-      <c r="N63" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="O63" s="1"/>
-    </row>
-    <row r="64" spans="1:15" ht="300">
-      <c r="A64" s="7" t="s">
-        <v>42</v>
+      <c r="N63" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14">
+      <c r="A64" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D64" s="1">
         <v>22060312</v>
       </c>
-      <c r="E64" s="2">
+      <c r="E64" s="1">
         <v>0.61805555555555602</v>
       </c>
       <c r="F64" s="1">
@@ -3538,34 +3217,30 @@
       <c r="H64" s="1">
         <v>22000</v>
       </c>
-      <c r="I64" s="1"/>
       <c r="J64" s="1">
         <v>700</v>
       </c>
-      <c r="K64" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="L64" s="4"/>
+      <c r="K64" s="1" t="s">
+        <v>69</v>
+      </c>
       <c r="M64" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="N64" s="4"/>
-      <c r="O64" s="1"/>
-    </row>
-    <row r="65" spans="1:15" ht="50">
-      <c r="A65" s="7" t="s">
-        <v>42</v>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15">
+      <c r="A65" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D65" s="1">
         <v>22060316</v>
       </c>
-      <c r="E65" s="2">
+      <c r="E65" s="1">
         <v>0.61805555555555602</v>
       </c>
       <c r="F65" s="1">
@@ -3577,32 +3252,27 @@
       <c r="H65" s="1">
         <v>145698</v>
       </c>
-      <c r="I65" s="4"/>
       <c r="J65" s="1">
         <v>0</v>
       </c>
-      <c r="K65" s="4"/>
-      <c r="L65" s="4"/>
-      <c r="M65" s="4"/>
-      <c r="N65" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="O65" s="1"/>
-    </row>
-    <row r="66" spans="1:15" ht="75">
+      <c r="N65" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15">
       <c r="A66" s="1">
         <v>600584</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D66" s="1">
         <v>22060316</v>
       </c>
-      <c r="E66" s="2">
+      <c r="E66" s="1">
         <v>0.61805555555555602</v>
       </c>
       <c r="F66" s="1">
@@ -3614,32 +3284,27 @@
       <c r="H66" s="1">
         <v>22850</v>
       </c>
-      <c r="I66" s="1"/>
       <c r="J66" s="1">
         <v>0</v>
       </c>
-      <c r="K66" s="4"/>
-      <c r="L66" s="4"/>
-      <c r="M66" s="4"/>
-      <c r="N66" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="O66" s="1"/>
-    </row>
-    <row r="67" spans="1:15" ht="100">
-      <c r="A67" s="7" t="s">
-        <v>42</v>
+      <c r="N66" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15">
+      <c r="A67" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D67" s="1">
         <v>20260318</v>
       </c>
-      <c r="E67" s="2">
+      <c r="E67" s="1">
         <v>0.61805555555555602</v>
       </c>
       <c r="F67" s="1">
@@ -3651,34 +3316,30 @@
       <c r="H67" s="1">
         <v>22018</v>
       </c>
-      <c r="I67" s="1"/>
       <c r="J67" s="1">
         <v>100</v>
       </c>
-      <c r="K67" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="L67" s="4"/>
+      <c r="K67" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="M67" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="N67" s="4"/>
-      <c r="O67" s="1"/>
-    </row>
-    <row r="68" spans="1:15" ht="100">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15">
       <c r="A68" s="1">
         <v>600487</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D68" s="1">
         <v>20260318</v>
       </c>
-      <c r="E68" s="2">
+      <c r="E68" s="1">
         <v>0.61805555555555602</v>
       </c>
       <c r="F68" s="1">
@@ -3690,34 +3351,30 @@
       <c r="H68" s="1">
         <v>26708</v>
       </c>
-      <c r="I68" s="4"/>
       <c r="J68" s="1">
         <v>600</v>
       </c>
-      <c r="K68" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="L68" s="4"/>
-      <c r="M68" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="N68" s="4"/>
-      <c r="O68" s="1"/>
-    </row>
-    <row r="69" spans="1:15" ht="225">
-      <c r="A69" s="7" t="s">
-        <v>42</v>
+      <c r="K68" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="M68" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15">
+      <c r="A69" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D69" s="1">
         <v>20260319</v>
       </c>
-      <c r="E69" s="2">
+      <c r="E69" s="1">
         <v>0.41458333333333303</v>
       </c>
       <c r="F69" s="1">
@@ -3729,32 +3386,27 @@
       <c r="H69" s="1">
         <v>21459</v>
       </c>
-      <c r="I69" s="4"/>
       <c r="J69" s="1">
         <v>200</v>
       </c>
-      <c r="K69" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="L69" s="4"/>
-      <c r="M69" s="4"/>
-      <c r="N69" s="4"/>
-      <c r="O69" s="1"/>
-    </row>
-    <row r="70" spans="1:15" ht="175">
-      <c r="A70" s="7" t="s">
-        <v>42</v>
+      <c r="K69" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15">
+      <c r="A70" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D70" s="1">
         <v>20260319</v>
       </c>
-      <c r="E70" s="2">
+      <c r="E70" s="1">
         <v>0.625</v>
       </c>
       <c r="F70" s="1">
@@ -3766,32 +3418,27 @@
       <c r="H70" s="1">
         <v>21110</v>
       </c>
-      <c r="I70" s="4"/>
       <c r="J70" s="1">
         <v>300</v>
       </c>
-      <c r="K70" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="L70" s="4"/>
-      <c r="M70" s="4"/>
-      <c r="N70" s="4"/>
-      <c r="O70" s="1"/>
-    </row>
-    <row r="71" spans="1:15" ht="100">
+      <c r="K70" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15">
       <c r="A71" s="1">
         <v>600487</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D71" s="1">
         <v>20260320</v>
       </c>
-      <c r="E71" s="2">
+      <c r="E71" s="1">
         <v>0.42499999999999999</v>
       </c>
       <c r="F71" s="1">
@@ -3803,32 +3450,27 @@
       <c r="H71" s="1">
         <v>27042</v>
       </c>
-      <c r="I71" s="4"/>
       <c r="J71" s="1">
         <v>1200</v>
       </c>
-      <c r="K71" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="L71" s="4"/>
-      <c r="M71" s="4"/>
-      <c r="N71" s="4"/>
-      <c r="O71" s="1"/>
-    </row>
-    <row r="72" spans="1:15" ht="125">
+      <c r="K71" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15">
       <c r="A72" s="1">
         <v>600487</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D72" s="1">
         <v>20260324</v>
       </c>
-      <c r="E72" s="2">
+      <c r="E72" s="1">
         <v>0.61666666666666703</v>
       </c>
       <c r="F72" s="1">
@@ -3840,32 +3482,27 @@
       <c r="H72" s="1">
         <v>13200</v>
       </c>
-      <c r="I72" s="4"/>
       <c r="J72" s="1">
         <v>1500</v>
       </c>
-      <c r="K72" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="L72" s="4"/>
-      <c r="M72" s="4"/>
-      <c r="N72" s="4"/>
-      <c r="O72" s="1"/>
-    </row>
-    <row r="73" spans="1:15" ht="175">
-      <c r="A73" s="7" t="s">
-        <v>56</v>
+      <c r="K72" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15">
+      <c r="A73" s="1" t="s">
+        <v>82</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D73" s="1">
         <v>20260325</v>
       </c>
-      <c r="E73" s="2">
+      <c r="E73" s="1">
         <v>0.40902777777777799</v>
       </c>
       <c r="F73" s="1">
@@ -3877,32 +3514,27 @@
       <c r="H73" s="1">
         <v>21377</v>
       </c>
-      <c r="I73" s="4"/>
       <c r="J73" s="1">
         <v>400</v>
       </c>
-      <c r="K73" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="L73" s="4"/>
-      <c r="M73" s="4"/>
-      <c r="N73" s="4"/>
-      <c r="O73" s="1"/>
-    </row>
-    <row r="74" spans="1:15" ht="275">
-      <c r="A74" s="7" t="s">
-        <v>42</v>
+      <c r="K73" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15">
+      <c r="A74" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D74" s="1">
         <v>20260327</v>
       </c>
-      <c r="E74" s="2">
+      <c r="E74" s="1">
         <v>0.44166666666666698</v>
       </c>
       <c r="F74" s="1">
@@ -3914,32 +3546,27 @@
       <c r="H74" s="1">
         <v>20800</v>
       </c>
-      <c r="I74" s="4"/>
       <c r="J74" s="1">
         <v>500</v>
       </c>
-      <c r="K74" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="L74" s="4"/>
-      <c r="M74" s="4"/>
-      <c r="N74" s="4"/>
-      <c r="O74" s="1"/>
-    </row>
-    <row r="75" spans="1:15" ht="409.6">
-      <c r="A75" s="8">
+      <c r="K74" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15">
+      <c r="A75" s="1">
         <v>600487</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D75" s="1">
         <v>20260327</v>
       </c>
-      <c r="E75" s="2">
+      <c r="E75" s="1">
         <v>0.41041666666666698</v>
       </c>
       <c r="F75" s="1">
@@ -3952,33 +3579,29 @@
         <v>70620</v>
       </c>
       <c r="I75" s="1" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
       <c r="J75" s="1">
         <v>0</v>
       </c>
-      <c r="K75" s="4"/>
-      <c r="L75" s="4"/>
-      <c r="M75" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="N75" s="4"/>
-      <c r="O75" s="1"/>
-    </row>
-    <row r="76" spans="1:15" ht="175">
-      <c r="A76" s="7" t="s">
-        <v>42</v>
+      <c r="M75" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15">
+      <c r="A76" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D76" s="1">
         <v>20260331</v>
       </c>
-      <c r="E76" s="2">
+      <c r="E76" s="1">
         <v>0.56597222222222199</v>
       </c>
       <c r="F76" s="1">
@@ -3990,32 +3613,27 @@
       <c r="H76" s="1">
         <v>20050</v>
       </c>
-      <c r="I76" s="4"/>
       <c r="J76" s="1">
         <v>600</v>
       </c>
-      <c r="K76" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="L76" s="4"/>
-      <c r="M76" s="4"/>
-      <c r="N76" s="4"/>
-      <c r="O76" s="9"/>
-    </row>
-    <row r="77" spans="1:15" ht="325">
-      <c r="A77" s="7" t="s">
-        <v>66</v>
+      <c r="K76" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15">
+      <c r="A77" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="D77" s="1">
         <v>20260408</v>
       </c>
-      <c r="E77" s="2">
+      <c r="E77" s="1">
         <v>0.61805555555555558</v>
       </c>
       <c r="F77" s="1">
@@ -4027,32 +3645,27 @@
       <c r="H77" s="1">
         <v>61755</v>
       </c>
-      <c r="I77" s="4"/>
       <c r="J77" s="1">
         <v>300</v>
       </c>
-      <c r="K77" s="4"/>
-      <c r="L77" s="4"/>
-      <c r="M77" s="4"/>
-      <c r="N77" s="4"/>
-      <c r="O77" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="78" spans="1:15" ht="200">
-      <c r="A78" s="7" t="s">
-        <v>67</v>
+      <c r="O77" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15">
+      <c r="A78" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D78" s="1">
         <v>20260408</v>
       </c>
-      <c r="E78" s="2">
+      <c r="E78" s="1">
         <v>0.61805555555555558</v>
       </c>
       <c r="F78" s="1">
@@ -4064,32 +3677,27 @@
       <c r="H78" s="1">
         <v>22030</v>
       </c>
-      <c r="I78" s="4"/>
       <c r="J78" s="1">
         <v>200</v>
       </c>
-      <c r="K78" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="L78" s="4"/>
-      <c r="M78" s="4"/>
-      <c r="N78" s="4"/>
-      <c r="O78" s="1"/>
-    </row>
-    <row r="79" spans="1:15" ht="250">
-      <c r="A79" s="7" t="s">
-        <v>71</v>
+      <c r="K78" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="79" spans="1:15">
+      <c r="A79" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D79" s="1">
         <v>20260408</v>
       </c>
-      <c r="E79" s="2">
+      <c r="E79" s="1">
         <v>0.61805555555555558</v>
       </c>
       <c r="F79" s="1">
@@ -4101,32 +3709,27 @@
       <c r="H79" s="1">
         <v>19652</v>
       </c>
-      <c r="I79" s="4"/>
       <c r="J79" s="1">
         <v>200</v>
       </c>
-      <c r="K79" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="L79" s="4"/>
-      <c r="M79" s="4"/>
-      <c r="N79" s="4"/>
-      <c r="O79" s="1"/>
-    </row>
-    <row r="80" spans="1:15" ht="325">
-      <c r="A80" s="7" t="s">
-        <v>67</v>
+      <c r="K79" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15">
+      <c r="A80" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D80" s="1">
         <v>20260409</v>
       </c>
-      <c r="E80" s="2">
+      <c r="E80" s="1">
         <v>0.42708333333333331</v>
       </c>
       <c r="F80" s="1">
@@ -4138,32 +3741,27 @@
       <c r="H80" s="1">
         <v>23200</v>
       </c>
-      <c r="I80" s="4"/>
       <c r="J80" s="1">
         <v>400</v>
       </c>
-      <c r="K80" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="L80" s="4"/>
-      <c r="M80" s="4"/>
-      <c r="N80" s="4"/>
-      <c r="O80" s="1"/>
-    </row>
-    <row r="81" spans="1:15" ht="325">
-      <c r="A81" s="7" t="s">
-        <v>71</v>
+      <c r="K80" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="81" spans="1:15">
+      <c r="A81" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D81" s="1">
         <v>20260409</v>
       </c>
-      <c r="E81" s="2">
+      <c r="E81" s="1">
         <v>0.4236111111111111</v>
       </c>
       <c r="F81" s="1">
@@ -4175,32 +3773,27 @@
       <c r="H81" s="1">
         <v>21414</v>
       </c>
-      <c r="I81" s="4"/>
       <c r="J81" s="1">
         <v>400</v>
       </c>
-      <c r="K81" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="L81" s="4"/>
-      <c r="M81" s="4"/>
-      <c r="N81" s="4"/>
-      <c r="O81" s="1"/>
-    </row>
-    <row r="82" spans="1:15" ht="375">
-      <c r="A82" s="7" t="s">
-        <v>66</v>
+      <c r="K81" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="82" spans="1:15">
+      <c r="A82" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="D82" s="1">
         <v>20260408</v>
       </c>
-      <c r="E82" s="2">
+      <c r="E82" s="1">
         <v>0.61805555555555558</v>
       </c>
       <c r="F82" s="1">
@@ -4212,32 +3805,27 @@
       <c r="H82" s="1">
         <v>40500</v>
       </c>
-      <c r="I82" s="4"/>
       <c r="J82" s="1">
         <v>100</v>
       </c>
-      <c r="K82" s="4"/>
-      <c r="L82" s="4"/>
-      <c r="M82" s="4"/>
-      <c r="N82" s="4"/>
-      <c r="O82" s="9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="83" spans="1:15" ht="175">
-      <c r="A83" s="7" t="s">
-        <v>66</v>
+      <c r="O82" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="83" spans="1:15">
+      <c r="A83" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D83" s="1">
         <v>20260410</v>
       </c>
-      <c r="E83" s="2">
+      <c r="E83" s="1">
         <v>0.54722222222222228</v>
       </c>
       <c r="F83" s="1">
@@ -4252,24 +3840,24 @@
       <c r="J83" s="1">
         <v>200</v>
       </c>
-      <c r="K83" s="9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="84" spans="1:15" ht="125">
-      <c r="A84" s="7" t="s">
-        <v>66</v>
+      <c r="K83" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15">
+      <c r="A84" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="D84" s="1">
         <v>20260413</v>
       </c>
-      <c r="E84" s="2">
+      <c r="E84" s="1">
         <v>0.40208333333333335</v>
       </c>
       <c r="F84" s="1">
@@ -4284,24 +3872,24 @@
       <c r="J84" s="1">
         <v>0</v>
       </c>
-      <c r="N84" s="14" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="85" spans="1:15" ht="300">
-      <c r="A85" s="7" t="s">
-        <v>71</v>
+      <c r="N84" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="85" spans="1:15">
+      <c r="A85" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D85" s="1">
         <v>202604013</v>
       </c>
-      <c r="E85" s="2">
+      <c r="E85" s="1">
         <v>0.40486111111111112</v>
       </c>
       <c r="F85" s="1">
@@ -4316,24 +3904,24 @@
       <c r="J85" s="1">
         <v>600</v>
       </c>
-      <c r="K85" s="9" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="86" spans="1:15" ht="350">
-      <c r="A86" s="7" t="s">
-        <v>67</v>
+      <c r="K85" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="86" spans="1:15">
+      <c r="A86" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D86" s="1">
         <v>20260413</v>
       </c>
-      <c r="E86" s="2">
+      <c r="E86" s="1">
         <v>0.59583333333333333</v>
       </c>
       <c r="F86" s="1">
@@ -4348,24 +3936,24 @@
       <c r="J86" s="1">
         <v>600</v>
       </c>
-      <c r="K86" s="9" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="87" spans="1:15" ht="409.6">
-      <c r="A87" s="7" t="s">
-        <v>67</v>
+      <c r="K86" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="87" spans="1:15">
+      <c r="A87" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="D87" s="1">
         <v>20260414</v>
       </c>
-      <c r="E87" s="2">
+      <c r="E87" s="1">
         <v>0.62291666666666667</v>
       </c>
       <c r="F87" s="1">
@@ -4380,24 +3968,24 @@
       <c r="J87" s="1">
         <v>300</v>
       </c>
-      <c r="O87" s="9" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="88" spans="1:15" ht="300">
-      <c r="A88" s="7" t="s">
-        <v>71</v>
+      <c r="O87" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="88" spans="1:15">
+      <c r="A88" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="D88" s="1">
         <v>20260414</v>
       </c>
-      <c r="E88" s="2">
+      <c r="E88" s="1">
         <v>0.62291666666666667</v>
       </c>
       <c r="F88" s="1">
@@ -4412,24 +4000,24 @@
       <c r="J88" s="1">
         <v>300</v>
       </c>
-      <c r="O88" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="89" spans="1:15" ht="50">
-      <c r="A89" s="7" t="s">
-        <v>67</v>
+      <c r="O88" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="89" spans="1:15">
+      <c r="A89" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="D89" s="1">
         <v>20260415</v>
       </c>
-      <c r="E89" s="2">
+      <c r="E89" s="1">
         <v>0.62291666666666667</v>
       </c>
       <c r="F89" s="1">
@@ -4447,24 +4035,24 @@
       <c r="J89" s="1">
         <v>0</v>
       </c>
-      <c r="N89" s="9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="90" spans="1:15" ht="24">
-      <c r="A90" s="7" t="s">
-        <v>71</v>
+      <c r="N89" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="90" spans="1:15">
+      <c r="A90" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D90" s="1">
         <v>20260415</v>
       </c>
-      <c r="E90" s="2">
+      <c r="E90" s="1">
         <v>0.42430555555555555</v>
       </c>
       <c r="F90" s="1">
@@ -4480,20 +4068,20 @@
         <v>600</v>
       </c>
     </row>
-    <row r="91" spans="1:15" ht="24">
-      <c r="A91" s="7" t="s">
-        <v>71</v>
+    <row r="91" spans="1:15">
+      <c r="A91" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="D91" s="1">
         <v>20260415</v>
       </c>
-      <c r="E91" s="2">
+      <c r="E91" s="1">
         <v>0.60069444444444442</v>
       </c>
       <c r="F91" s="1">
@@ -4509,20 +4097,20 @@
         <v>300</v>
       </c>
     </row>
-    <row r="92" spans="1:15" ht="409.6">
-      <c r="A92" s="7" t="s">
-        <v>84</v>
+    <row r="92" spans="1:15">
+      <c r="A92" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D92" s="1">
         <v>20260416</v>
       </c>
-      <c r="E92" s="2">
+      <c r="E92" s="1">
         <v>0.46944444444444444</v>
       </c>
       <c r="F92" s="1">
@@ -4537,30 +4125,30 @@
       <c r="J92" s="1">
         <v>500</v>
       </c>
-      <c r="K92" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="L92" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="M92" s="16" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="93" spans="1:15" ht="175">
-      <c r="A93" s="15">
+      <c r="K92" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L92" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M92" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="93" spans="1:15">
+      <c r="A93" s="1">
         <v>601126</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D93" s="1">
         <v>20260416</v>
       </c>
-      <c r="E93" s="2">
+      <c r="E93" s="1">
         <v>0.62152777777777779</v>
       </c>
       <c r="F93" s="1">
@@ -4575,24 +4163,24 @@
       <c r="J93" s="1">
         <v>1100</v>
       </c>
-      <c r="K93" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="94" spans="1:15" ht="275">
-      <c r="A94" s="7" t="s">
-        <v>71</v>
+      <c r="K93" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="94" spans="1:15">
+      <c r="A94" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D94" s="1">
         <v>20260419</v>
       </c>
-      <c r="E94" s="2">
+      <c r="E94" s="1">
         <v>0.40833333333333333</v>
       </c>
       <c r="F94" s="1">
@@ -4607,24 +4195,24 @@
       <c r="J94" s="1">
         <v>600</v>
       </c>
-      <c r="K94" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="95" spans="1:15" ht="100">
-      <c r="A95" s="7" t="s">
-        <v>71</v>
+      <c r="K94" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="95" spans="1:15">
+      <c r="A95" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="D95" s="1">
         <v>20260419</v>
       </c>
-      <c r="E95" s="2">
+      <c r="E95" s="1">
         <v>0.42569444444444443</v>
       </c>
       <c r="F95" s="1">
@@ -4639,24 +4227,24 @@
       <c r="J95" s="1">
         <v>500</v>
       </c>
-      <c r="O95" s="5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="96" spans="1:15" ht="50">
-      <c r="A96" s="15">
+      <c r="O95" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="96" spans="1:15">
+      <c r="A96" s="1">
         <v>601126</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D96" s="1">
         <v>20260419</v>
       </c>
-      <c r="E96" s="2">
+      <c r="E96" s="1">
         <v>0.56319444444444444</v>
       </c>
       <c r="F96" s="1">
@@ -4671,24 +4259,24 @@
       <c r="J96" s="1">
         <v>1700</v>
       </c>
-      <c r="K96" s="5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10" ht="24">
-      <c r="A97" s="7" t="s">
-        <v>71</v>
+      <c r="K96" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10">
+      <c r="A97" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="D97" s="1">
         <v>20260420</v>
       </c>
-      <c r="E97" s="2">
+      <c r="E97" s="1">
         <v>0.40138888888888891</v>
       </c>
       <c r="F97" s="1">
@@ -4704,20 +4292,20 @@
         <v>400</v>
       </c>
     </row>
-    <row r="98" spans="1:10" ht="24">
-      <c r="A98" s="7" t="s">
-        <v>71</v>
+    <row r="98" spans="1:10">
+      <c r="A98" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="D98" s="1">
         <v>20260420</v>
       </c>
-      <c r="E98" s="2">
+      <c r="E98" s="1">
         <v>0.62083333333333335</v>
       </c>
       <c r="F98" s="1">
@@ -4733,792 +4321,21 @@
         <v>300</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="24">
-      <c r="A99" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="B99" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C99" s="1"/>
-    </row>
-    <row r="100" spans="1:10" ht="24">
-      <c r="C100" s="1"/>
-    </row>
-    <row r="101" spans="1:10" ht="24">
-      <c r="C101" s="1"/>
-    </row>
-    <row r="102" spans="1:10" ht="24">
-      <c r="C102" s="1"/>
-    </row>
-    <row r="103" spans="1:10" ht="24">
-      <c r="C103" s="1"/>
-    </row>
-    <row r="104" spans="1:10" ht="24">
-      <c r="C104" s="1"/>
-    </row>
-    <row r="105" spans="1:10" ht="24">
-      <c r="C105" s="1"/>
-    </row>
-    <row r="106" spans="1:10" ht="24">
-      <c r="C106" s="1"/>
-    </row>
-    <row r="107" spans="1:10" ht="24">
-      <c r="C107" s="1"/>
-    </row>
-    <row r="108" spans="1:10" ht="24">
-      <c r="C108" s="1"/>
-    </row>
-    <row r="109" spans="1:10" ht="24">
-      <c r="C109" s="1"/>
-    </row>
-    <row r="110" spans="1:10" ht="24">
-      <c r="C110" s="1"/>
-    </row>
-    <row r="111" spans="1:10" ht="24">
-      <c r="C111" s="1"/>
-    </row>
-    <row r="112" spans="1:10" ht="24">
-      <c r="C112" s="1"/>
-    </row>
-    <row r="113" spans="3:3" ht="24">
-      <c r="C113" s="1"/>
-    </row>
-    <row r="114" spans="3:3" ht="24">
-      <c r="C114" s="1"/>
-    </row>
-    <row r="115" spans="3:3" ht="24">
-      <c r="C115" s="1"/>
-    </row>
-    <row r="116" spans="3:3" ht="24">
-      <c r="C116" s="1"/>
-    </row>
-    <row r="117" spans="3:3" ht="24">
-      <c r="C117" s="1"/>
-    </row>
-    <row r="118" spans="3:3" ht="24">
-      <c r="C118" s="1"/>
-    </row>
-    <row r="119" spans="3:3" ht="24">
-      <c r="C119" s="1"/>
-    </row>
-    <row r="120" spans="3:3" ht="24">
-      <c r="C120" s="1"/>
-    </row>
-    <row r="121" spans="3:3" ht="24">
-      <c r="C121" s="1"/>
-    </row>
-    <row r="122" spans="3:3" ht="24">
-      <c r="C122" s="1"/>
-    </row>
-    <row r="123" spans="3:3" ht="24">
-      <c r="C123" s="1"/>
-    </row>
-    <row r="124" spans="3:3" ht="24">
-      <c r="C124" s="1"/>
-    </row>
-    <row r="125" spans="3:3" ht="24">
-      <c r="C125" s="1"/>
-    </row>
-    <row r="126" spans="3:3" ht="24">
-      <c r="C126" s="1"/>
-    </row>
-    <row r="127" spans="3:3" ht="24">
-      <c r="C127" s="1"/>
-    </row>
-    <row r="128" spans="3:3" ht="24">
-      <c r="C128" s="1"/>
-    </row>
-    <row r="129" spans="3:3" ht="24">
-      <c r="C129" s="1"/>
-    </row>
-    <row r="130" spans="3:3" ht="24">
-      <c r="C130" s="1"/>
-    </row>
-    <row r="131" spans="3:3" ht="24">
-      <c r="C131" s="1"/>
-    </row>
-    <row r="132" spans="3:3" ht="24">
-      <c r="C132" s="1"/>
-    </row>
-    <row r="133" spans="3:3" ht="24">
-      <c r="C133" s="1"/>
-    </row>
-    <row r="134" spans="3:3" ht="24">
-      <c r="C134" s="1"/>
-    </row>
-    <row r="135" spans="3:3" ht="24">
-      <c r="C135" s="1"/>
-    </row>
-    <row r="136" spans="3:3" ht="24">
-      <c r="C136" s="1"/>
-    </row>
-    <row r="137" spans="3:3" ht="24">
-      <c r="C137" s="1"/>
-    </row>
-    <row r="138" spans="3:3" ht="24">
-      <c r="C138" s="1"/>
-    </row>
-    <row r="139" spans="3:3" ht="24">
-      <c r="C139" s="1"/>
-    </row>
-    <row r="140" spans="3:3" ht="24">
-      <c r="C140" s="1"/>
-    </row>
-    <row r="141" spans="3:3" ht="24">
-      <c r="C141" s="1"/>
-    </row>
-    <row r="142" spans="3:3" ht="24">
-      <c r="C142" s="1"/>
-    </row>
-    <row r="143" spans="3:3" ht="24">
-      <c r="C143" s="1"/>
-    </row>
-    <row r="144" spans="3:3" ht="24">
-      <c r="C144" s="1"/>
-    </row>
-    <row r="145" spans="3:3" ht="24">
-      <c r="C145" s="1"/>
-    </row>
-    <row r="146" spans="3:3" ht="24">
-      <c r="C146" s="1"/>
-    </row>
-    <row r="147" spans="3:3" ht="24">
-      <c r="C147" s="1"/>
-    </row>
-    <row r="148" spans="3:3" ht="24">
-      <c r="C148" s="1"/>
-    </row>
-    <row r="149" spans="3:3" ht="24">
-      <c r="C149" s="1"/>
-    </row>
-    <row r="150" spans="3:3" ht="24">
-      <c r="C150" s="1"/>
-    </row>
-    <row r="151" spans="3:3" ht="24">
-      <c r="C151" s="1"/>
-    </row>
-    <row r="152" spans="3:3" ht="24">
-      <c r="C152" s="1"/>
-    </row>
-    <row r="153" spans="3:3" ht="24">
-      <c r="C153" s="1"/>
-    </row>
-    <row r="154" spans="3:3" ht="24">
-      <c r="C154" s="1"/>
-    </row>
-    <row r="155" spans="3:3" ht="24">
-      <c r="C155" s="1"/>
-    </row>
-    <row r="156" spans="3:3" ht="24">
-      <c r="C156" s="1"/>
-    </row>
-    <row r="157" spans="3:3" ht="24">
-      <c r="C157" s="1"/>
-    </row>
-    <row r="158" spans="3:3" ht="24">
-      <c r="C158" s="1"/>
-    </row>
-    <row r="159" spans="3:3" ht="24">
-      <c r="C159" s="1"/>
-    </row>
-    <row r="160" spans="3:3" ht="24">
-      <c r="C160" s="1"/>
-    </row>
-    <row r="161" spans="3:3" ht="24">
-      <c r="C161" s="1"/>
-    </row>
-    <row r="162" spans="3:3" ht="24">
-      <c r="C162" s="1"/>
-    </row>
-    <row r="163" spans="3:3" ht="24">
-      <c r="C163" s="1"/>
-    </row>
-    <row r="164" spans="3:3" ht="24">
-      <c r="C164" s="1"/>
-    </row>
-    <row r="165" spans="3:3" ht="24">
-      <c r="C165" s="1"/>
-    </row>
-    <row r="166" spans="3:3" ht="24">
-      <c r="C166" s="1"/>
-    </row>
-    <row r="167" spans="3:3" ht="24">
-      <c r="C167" s="1"/>
-    </row>
-    <row r="168" spans="3:3" ht="24">
-      <c r="C168" s="1"/>
-    </row>
-    <row r="169" spans="3:3" ht="24">
-      <c r="C169" s="1"/>
-    </row>
-    <row r="170" spans="3:3" ht="24">
-      <c r="C170" s="1"/>
-    </row>
-    <row r="171" spans="3:3" ht="24">
-      <c r="C171" s="1"/>
-    </row>
-    <row r="172" spans="3:3" ht="24">
-      <c r="C172" s="1"/>
-    </row>
-    <row r="173" spans="3:3" ht="24">
-      <c r="C173" s="1"/>
-    </row>
-    <row r="174" spans="3:3" ht="24">
-      <c r="C174" s="1"/>
-    </row>
-    <row r="175" spans="3:3" ht="24">
-      <c r="C175" s="1"/>
-    </row>
-    <row r="176" spans="3:3" ht="24">
-      <c r="C176" s="1"/>
-    </row>
-    <row r="177" spans="3:3" ht="24">
-      <c r="C177" s="1"/>
-    </row>
-    <row r="178" spans="3:3" ht="24">
-      <c r="C178" s="1"/>
-    </row>
-    <row r="179" spans="3:3" ht="24">
-      <c r="C179" s="1"/>
-    </row>
-    <row r="180" spans="3:3" ht="24">
-      <c r="C180" s="1"/>
-    </row>
-    <row r="181" spans="3:3" ht="24">
-      <c r="C181" s="1"/>
-    </row>
-    <row r="182" spans="3:3" ht="24">
-      <c r="C182" s="1"/>
-    </row>
-    <row r="183" spans="3:3" ht="24">
-      <c r="C183" s="1"/>
-    </row>
-    <row r="184" spans="3:3" ht="24">
-      <c r="C184" s="1"/>
-    </row>
-    <row r="185" spans="3:3" ht="24">
-      <c r="C185" s="1"/>
-    </row>
-    <row r="186" spans="3:3" ht="24">
-      <c r="C186" s="1"/>
-    </row>
-    <row r="187" spans="3:3" ht="24">
-      <c r="C187" s="1"/>
-    </row>
-    <row r="188" spans="3:3" ht="24">
-      <c r="C188" s="1"/>
-    </row>
-    <row r="189" spans="3:3" ht="24">
-      <c r="C189" s="1"/>
-    </row>
-    <row r="190" spans="3:3" ht="24">
-      <c r="C190" s="1"/>
-    </row>
-    <row r="191" spans="3:3" ht="24">
-      <c r="C191" s="1"/>
-    </row>
-    <row r="192" spans="3:3" ht="24">
-      <c r="C192" s="1"/>
-    </row>
-    <row r="193" spans="3:3" ht="24">
-      <c r="C193" s="1"/>
-    </row>
-    <row r="194" spans="3:3" ht="24">
-      <c r="C194" s="1"/>
-    </row>
-    <row r="195" spans="3:3" ht="24">
-      <c r="C195" s="1"/>
-    </row>
-    <row r="196" spans="3:3" ht="24">
-      <c r="C196" s="1"/>
-    </row>
-    <row r="197" spans="3:3" ht="24">
-      <c r="C197" s="1"/>
-    </row>
-    <row r="198" spans="3:3" ht="24">
-      <c r="C198" s="1"/>
-    </row>
-    <row r="199" spans="3:3" ht="24">
-      <c r="C199" s="1"/>
-    </row>
-    <row r="200" spans="3:3" ht="24">
-      <c r="C200" s="1"/>
-    </row>
-    <row r="201" spans="3:3" ht="24">
-      <c r="C201" s="1"/>
-    </row>
-    <row r="202" spans="3:3" ht="24">
-      <c r="C202" s="1"/>
-    </row>
-    <row r="203" spans="3:3" ht="24">
-      <c r="C203" s="1"/>
-    </row>
-    <row r="204" spans="3:3" ht="24">
-      <c r="C204" s="1"/>
-    </row>
-    <row r="205" spans="3:3" ht="24">
-      <c r="C205" s="1"/>
-    </row>
-    <row r="206" spans="3:3" ht="24">
-      <c r="C206" s="1"/>
-    </row>
-    <row r="207" spans="3:3" ht="24">
-      <c r="C207" s="1"/>
-    </row>
-    <row r="208" spans="3:3" ht="24">
-      <c r="C208" s="1"/>
-    </row>
-    <row r="209" spans="3:3" ht="24">
-      <c r="C209" s="1"/>
-    </row>
-    <row r="210" spans="3:3" ht="24">
-      <c r="C210" s="1"/>
-    </row>
-    <row r="211" spans="3:3" ht="24">
-      <c r="C211" s="1"/>
-    </row>
-    <row r="212" spans="3:3" ht="24">
-      <c r="C212" s="1"/>
-    </row>
-    <row r="213" spans="3:3" ht="24">
-      <c r="C213" s="1"/>
-    </row>
-    <row r="214" spans="3:3" ht="24">
-      <c r="C214" s="1"/>
-    </row>
-    <row r="215" spans="3:3" ht="24">
-      <c r="C215" s="1"/>
-    </row>
-    <row r="216" spans="3:3" ht="24">
-      <c r="C216" s="1"/>
-    </row>
-    <row r="217" spans="3:3" ht="24">
-      <c r="C217" s="1"/>
-    </row>
-    <row r="218" spans="3:3" ht="24">
-      <c r="C218" s="1"/>
-    </row>
-    <row r="219" spans="3:3" ht="24">
-      <c r="C219" s="1"/>
-    </row>
-    <row r="220" spans="3:3" ht="24">
-      <c r="C220" s="1"/>
-    </row>
-    <row r="221" spans="3:3" ht="24">
-      <c r="C221" s="1"/>
-    </row>
-    <row r="222" spans="3:3" ht="24">
-      <c r="C222" s="1"/>
-    </row>
-    <row r="223" spans="3:3" ht="24">
-      <c r="C223" s="1"/>
-    </row>
-    <row r="224" spans="3:3" ht="24">
-      <c r="C224" s="1"/>
-    </row>
-    <row r="225" spans="3:3" ht="24">
-      <c r="C225" s="1"/>
-    </row>
-    <row r="226" spans="3:3" ht="24">
-      <c r="C226" s="1"/>
-    </row>
-    <row r="227" spans="3:3" ht="24">
-      <c r="C227" s="1"/>
-    </row>
-    <row r="228" spans="3:3" ht="24">
-      <c r="C228" s="1"/>
-    </row>
-    <row r="229" spans="3:3" ht="24">
-      <c r="C229" s="1"/>
-    </row>
-    <row r="230" spans="3:3" ht="24">
-      <c r="C230" s="1"/>
-    </row>
-    <row r="231" spans="3:3" ht="24">
-      <c r="C231" s="1"/>
-    </row>
-    <row r="232" spans="3:3" ht="24">
-      <c r="C232" s="1"/>
-    </row>
-    <row r="233" spans="3:3" ht="24">
-      <c r="C233" s="1"/>
-    </row>
-    <row r="234" spans="3:3" ht="24">
-      <c r="C234" s="1"/>
-    </row>
-    <row r="235" spans="3:3" ht="24">
-      <c r="C235" s="1"/>
-    </row>
-    <row r="236" spans="3:3" ht="24">
-      <c r="C236" s="1"/>
-    </row>
-    <row r="237" spans="3:3" ht="24">
-      <c r="C237" s="1"/>
-    </row>
-    <row r="238" spans="3:3" ht="24">
-      <c r="C238" s="1"/>
-    </row>
-    <row r="239" spans="3:3" ht="24">
-      <c r="C239" s="1"/>
-    </row>
-    <row r="240" spans="3:3" ht="24">
-      <c r="C240" s="1"/>
-    </row>
-    <row r="241" spans="3:3" ht="24">
-      <c r="C241" s="1"/>
-    </row>
-    <row r="242" spans="3:3" ht="24">
-      <c r="C242" s="1"/>
-    </row>
-    <row r="243" spans="3:3" ht="24">
-      <c r="C243" s="1"/>
-    </row>
-    <row r="244" spans="3:3" ht="24">
-      <c r="C244" s="1"/>
-    </row>
-    <row r="245" spans="3:3" ht="24">
-      <c r="C245" s="1"/>
-    </row>
-    <row r="246" spans="3:3" ht="24">
-      <c r="C246" s="1"/>
-    </row>
-    <row r="247" spans="3:3" ht="24">
-      <c r="C247" s="1"/>
-    </row>
-    <row r="248" spans="3:3" ht="24">
-      <c r="C248" s="1"/>
-    </row>
-    <row r="249" spans="3:3" ht="24">
-      <c r="C249" s="1"/>
-    </row>
-    <row r="250" spans="3:3" ht="24">
-      <c r="C250" s="1"/>
-    </row>
-    <row r="251" spans="3:3" ht="24">
-      <c r="C251" s="1"/>
-    </row>
-    <row r="252" spans="3:3" ht="24">
-      <c r="C252" s="1"/>
-    </row>
-    <row r="253" spans="3:3" ht="24">
-      <c r="C253" s="1"/>
-    </row>
-    <row r="254" spans="3:3" ht="24">
-      <c r="C254" s="1"/>
-    </row>
-    <row r="255" spans="3:3" ht="24">
-      <c r="C255" s="1"/>
-    </row>
-    <row r="256" spans="3:3" ht="24">
-      <c r="C256" s="1"/>
-    </row>
-    <row r="257" spans="3:3" ht="24">
-      <c r="C257" s="1"/>
-    </row>
-    <row r="258" spans="3:3" ht="24">
-      <c r="C258" s="1"/>
-    </row>
-    <row r="259" spans="3:3" ht="24">
-      <c r="C259" s="1"/>
-    </row>
-    <row r="260" spans="3:3" ht="24">
-      <c r="C260" s="1"/>
-    </row>
-    <row r="261" spans="3:3" ht="24">
-      <c r="C261" s="1"/>
-    </row>
-    <row r="262" spans="3:3" ht="24">
-      <c r="C262" s="1"/>
-    </row>
-    <row r="263" spans="3:3" ht="24">
-      <c r="C263" s="1"/>
-    </row>
-    <row r="264" spans="3:3" ht="24">
-      <c r="C264" s="1"/>
-    </row>
-    <row r="265" spans="3:3" ht="24">
-      <c r="C265" s="1"/>
-    </row>
-    <row r="266" spans="3:3" ht="24">
-      <c r="C266" s="1"/>
-    </row>
-    <row r="267" spans="3:3" ht="24">
-      <c r="C267" s="1"/>
-    </row>
-    <row r="268" spans="3:3" ht="24">
-      <c r="C268" s="1"/>
-    </row>
-    <row r="269" spans="3:3" ht="24">
-      <c r="C269" s="1"/>
-    </row>
-    <row r="270" spans="3:3" ht="24">
-      <c r="C270" s="1"/>
-    </row>
-    <row r="271" spans="3:3" ht="24">
-      <c r="C271" s="1"/>
-    </row>
-    <row r="272" spans="3:3" ht="24">
-      <c r="C272" s="1"/>
-    </row>
-    <row r="273" spans="3:3" ht="24">
-      <c r="C273" s="1"/>
-    </row>
-    <row r="274" spans="3:3" ht="24">
-      <c r="C274" s="1"/>
-    </row>
-    <row r="275" spans="3:3" ht="24">
-      <c r="C275" s="1"/>
-    </row>
-    <row r="276" spans="3:3" ht="24">
-      <c r="C276" s="1"/>
-    </row>
-    <row r="277" spans="3:3" ht="24">
-      <c r="C277" s="1"/>
-    </row>
-    <row r="278" spans="3:3" ht="24">
-      <c r="C278" s="1"/>
-    </row>
-    <row r="279" spans="3:3" ht="24">
-      <c r="C279" s="1"/>
-    </row>
-    <row r="280" spans="3:3" ht="24">
-      <c r="C280" s="1"/>
-    </row>
-    <row r="281" spans="3:3" ht="24">
-      <c r="C281" s="1"/>
-    </row>
-    <row r="282" spans="3:3" ht="24">
-      <c r="C282" s="1"/>
-    </row>
-    <row r="283" spans="3:3" ht="24">
-      <c r="C283" s="1"/>
-    </row>
-    <row r="284" spans="3:3" ht="24">
-      <c r="C284" s="1"/>
-    </row>
-    <row r="285" spans="3:3" ht="24">
-      <c r="C285" s="1"/>
-    </row>
-    <row r="286" spans="3:3" ht="24">
-      <c r="C286" s="1"/>
-    </row>
-    <row r="287" spans="3:3" ht="24">
-      <c r="C287" s="1"/>
-    </row>
-    <row r="288" spans="3:3" ht="24">
-      <c r="C288" s="1"/>
-    </row>
-    <row r="289" spans="3:3" ht="24">
-      <c r="C289" s="1"/>
-    </row>
-    <row r="290" spans="3:3" ht="24">
-      <c r="C290" s="1"/>
-    </row>
-    <row r="291" spans="3:3" ht="24">
-      <c r="C291" s="1"/>
-    </row>
-    <row r="292" spans="3:3" ht="24">
-      <c r="C292" s="1"/>
-    </row>
-    <row r="293" spans="3:3" ht="24">
-      <c r="C293" s="1"/>
-    </row>
-    <row r="294" spans="3:3" ht="24">
-      <c r="C294" s="1"/>
-    </row>
-    <row r="295" spans="3:3" ht="24">
-      <c r="C295" s="1"/>
-    </row>
-    <row r="296" spans="3:3" ht="24">
-      <c r="C296" s="1"/>
-    </row>
-    <row r="297" spans="3:3" ht="24">
-      <c r="C297" s="1"/>
-    </row>
-    <row r="298" spans="3:3" ht="24">
-      <c r="C298" s="1"/>
-    </row>
-    <row r="299" spans="3:3" ht="24">
-      <c r="C299" s="1"/>
-    </row>
-    <row r="300" spans="3:3" ht="24">
-      <c r="C300" s="1"/>
-    </row>
-    <row r="301" spans="3:3" ht="24">
-      <c r="C301" s="1"/>
-    </row>
-    <row r="302" spans="3:3" ht="24">
-      <c r="C302" s="1"/>
-    </row>
-    <row r="303" spans="3:3" ht="24">
-      <c r="C303" s="1"/>
-    </row>
-    <row r="304" spans="3:3" ht="24">
-      <c r="C304" s="1"/>
-    </row>
-    <row r="305" spans="3:3" ht="24">
-      <c r="C305" s="1"/>
-    </row>
-    <row r="306" spans="3:3" ht="24">
-      <c r="C306" s="1"/>
-    </row>
-    <row r="307" spans="3:3" ht="24">
-      <c r="C307" s="1"/>
-    </row>
-    <row r="308" spans="3:3" ht="24">
-      <c r="C308" s="1"/>
-    </row>
-    <row r="309" spans="3:3" ht="24">
-      <c r="C309" s="1"/>
-    </row>
-    <row r="310" spans="3:3" ht="24">
-      <c r="C310" s="1"/>
-    </row>
-    <row r="311" spans="3:3" ht="24">
-      <c r="C311" s="1"/>
-    </row>
-    <row r="312" spans="3:3" ht="24">
-      <c r="C312" s="1"/>
-    </row>
-    <row r="313" spans="3:3" ht="24">
-      <c r="C313" s="1"/>
-    </row>
-    <row r="314" spans="3:3" ht="24">
-      <c r="C314" s="1"/>
-    </row>
-    <row r="315" spans="3:3" ht="24">
-      <c r="C315" s="1"/>
-    </row>
-    <row r="316" spans="3:3" ht="24">
-      <c r="C316" s="1"/>
-    </row>
-    <row r="317" spans="3:3" ht="24">
-      <c r="C317" s="1"/>
-    </row>
-    <row r="318" spans="3:3" ht="24">
-      <c r="C318" s="1"/>
-    </row>
-    <row r="319" spans="3:3" ht="24">
-      <c r="C319" s="1"/>
-    </row>
-    <row r="320" spans="3:3" ht="24">
-      <c r="C320" s="1"/>
-    </row>
-    <row r="321" spans="3:3" ht="24">
-      <c r="C321" s="1"/>
-    </row>
-    <row r="322" spans="3:3" ht="24">
-      <c r="C322" s="1"/>
-    </row>
-    <row r="323" spans="3:3" ht="24">
-      <c r="C323" s="1"/>
-    </row>
-    <row r="324" spans="3:3" ht="24">
-      <c r="C324" s="1"/>
-    </row>
-    <row r="325" spans="3:3" ht="24">
-      <c r="C325" s="1"/>
-    </row>
-    <row r="326" spans="3:3" ht="24">
-      <c r="C326" s="1"/>
-    </row>
-    <row r="327" spans="3:3" ht="24">
-      <c r="C327" s="1"/>
-    </row>
-    <row r="328" spans="3:3" ht="24">
-      <c r="C328" s="1"/>
-    </row>
-    <row r="329" spans="3:3" ht="24">
-      <c r="C329" s="1"/>
-    </row>
-    <row r="330" spans="3:3" ht="24">
-      <c r="C330" s="1"/>
-    </row>
-    <row r="331" spans="3:3" ht="24">
-      <c r="C331" s="1"/>
-    </row>
-    <row r="332" spans="3:3" ht="24">
-      <c r="C332" s="1"/>
-    </row>
-    <row r="333" spans="3:3" ht="24">
-      <c r="C333" s="1"/>
-    </row>
-    <row r="334" spans="3:3" ht="24">
-      <c r="C334" s="1"/>
-    </row>
-    <row r="335" spans="3:3" ht="24">
-      <c r="C335" s="1"/>
-    </row>
-    <row r="336" spans="3:3" ht="24">
-      <c r="C336" s="1"/>
-    </row>
-    <row r="337" spans="3:3" ht="24">
-      <c r="C337" s="1"/>
-    </row>
-    <row r="338" spans="3:3" ht="24">
-      <c r="C338" s="1"/>
-    </row>
-    <row r="339" spans="3:3" ht="24">
-      <c r="C339" s="1"/>
-    </row>
-    <row r="340" spans="3:3" ht="24">
-      <c r="C340" s="1"/>
-    </row>
-    <row r="341" spans="3:3" ht="24">
-      <c r="C341" s="1"/>
-    </row>
-    <row r="342" spans="3:3" ht="24">
-      <c r="C342" s="1"/>
-    </row>
-    <row r="343" spans="3:3" ht="24">
-      <c r="C343" s="1"/>
-    </row>
-    <row r="344" spans="3:3" ht="24">
-      <c r="C344" s="1"/>
-    </row>
-    <row r="345" spans="3:3" ht="24">
-      <c r="C345" s="1"/>
-    </row>
-    <row r="346" spans="3:3" ht="24">
-      <c r="C346" s="1"/>
-    </row>
-    <row r="347" spans="3:3" ht="24">
-      <c r="C347" s="1"/>
-    </row>
-    <row r="348" spans="3:3" ht="24">
-      <c r="C348" s="1"/>
-    </row>
-    <row r="349" spans="3:3" ht="24">
-      <c r="C349" s="1"/>
-    </row>
-    <row r="350" spans="3:3" ht="24">
-      <c r="C350" s="1"/>
-    </row>
-    <row r="351" spans="3:3" ht="24">
-      <c r="C351" s="1"/>
-    </row>
-    <row r="352" spans="3:3" ht="24">
-      <c r="C352" s="1"/>
-    </row>
-    <row r="353" spans="3:3" ht="24">
-      <c r="C353" s="1"/>
-    </row>
-    <row r="354" spans="3:3" ht="24">
-      <c r="C354" s="1"/>
-    </row>
-    <row r="355" spans="3:3" ht="24">
-      <c r="C355" s="1"/>
-    </row>
-    <row r="356" spans="3:3" ht="24">
-      <c r="C356" s="1"/>
-    </row>
-    <row r="357" spans="3:3" ht="24">
-      <c r="C357" s="1"/>
+    <row r="99" spans="1:10">
+      <c r="A99" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J76" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-04-25 20:28:30
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3C78122-6710-7D4F-8865-67EF03928CF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC27E31D-9E92-CA4C-BE68-0EE8646A0D47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="111">
   <si>
     <t>证券代码</t>
   </si>
@@ -374,6 +374,30 @@
   </si>
   <si>
     <t>cpo光模块这波拉升过程中 华工科技几乎没有受益 同时一季度报并不理想 扣费后增长缓慢 不如光迅科技 +这波涨幅可能已经接近尾声当全场下杀华工科技也难以幸免</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>603019</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>中科曙光</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>中午收盘时看到deepseekv4发布的消息+11:14分已经有资金抢跑股价明显上v，博弈一个deepseekv4的消息能在短时间内发酵，于是选择开盘后直接以市价单成交</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>002261</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>拓维信息</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>依旧是博弈deepseekv4适配华为升腾芯片+deepseekv4后续直接发酵大爆的消息，拓维信息是公司继续强调基于“鲲鹏+昇腾AI”算力底座，打造覆盖中心侧、边端侧、终端侧的全栈式智能计算产品体系，并推出兆瀚 DeepSeek 一体机、AI 工作站等产品，与华为升腾概念强相关叠加从筹码峰上看上方套牢盘不重，于是决定市价买入，然而现在复盘我发现了一个错误，dsv4的消息和传言已经在前些日子有了预期或者预防 这个不是一个突发的事件，因此早就有埋伏资金在里面了，这是我当时考虑不周的事情，当利好落地了就是迎面而来的利空，而周末dsv4的消息也没有持续发酵，因为性能其实真的不如顶尖模型，因此我的买入逻辑也不存在了 周一无论什么价格都要先止损离场</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -5148,29 +5172,71 @@
         <v>104</v>
       </c>
     </row>
-    <row r="112" spans="1:15" ht="25" customHeight="1">
-      <c r="A112" s="6"/>
-      <c r="B112" s="6"/>
-      <c r="C112" s="6"/>
-      <c r="D112" s="6"/>
-      <c r="E112" s="8"/>
-      <c r="F112" s="6"/>
-      <c r="G112" s="6"/>
-      <c r="H112" s="6"/>
-      <c r="J112" s="6"/>
-    </row>
-    <row r="113" spans="1:10" ht="25" customHeight="1">
-      <c r="A113" s="6"/>
-      <c r="B113" s="6"/>
-      <c r="C113" s="6"/>
-      <c r="D113" s="6"/>
-      <c r="E113" s="8"/>
-      <c r="F113" s="6"/>
-      <c r="G113" s="6"/>
-      <c r="H113" s="6"/>
-      <c r="J113" s="6"/>
-    </row>
-    <row r="114" spans="1:10" ht="25" customHeight="1">
+    <row r="112" spans="1:15" ht="100">
+      <c r="A112" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="B112" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C112" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D112" s="6">
+        <v>20260424</v>
+      </c>
+      <c r="E112" s="8">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="F112" s="6">
+        <v>93.89</v>
+      </c>
+      <c r="G112" s="6">
+        <v>500</v>
+      </c>
+      <c r="H112" s="6">
+        <v>46945</v>
+      </c>
+      <c r="J112" s="6">
+        <v>500</v>
+      </c>
+      <c r="K112" s="12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" ht="375">
+      <c r="A113" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B113" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C113" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D113" s="6">
+        <v>20260424</v>
+      </c>
+      <c r="E113" s="8">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="F113" s="6">
+        <v>39.479999999999997</v>
+      </c>
+      <c r="G113" s="6">
+        <v>1600</v>
+      </c>
+      <c r="H113" s="6">
+        <v>64128</v>
+      </c>
+      <c r="J113" s="6">
+        <v>1600</v>
+      </c>
+      <c r="K113" s="12" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" ht="25" customHeight="1">
       <c r="A114" s="6"/>
       <c r="B114" s="6"/>
       <c r="C114" s="6"/>
@@ -5181,7 +5247,7 @@
       <c r="H114" s="6"/>
       <c r="J114" s="6"/>
     </row>
-    <row r="115" spans="1:10" ht="25" customHeight="1">
+    <row r="115" spans="1:11" ht="25" customHeight="1">
       <c r="A115" s="6"/>
       <c r="B115" s="6"/>
       <c r="C115" s="6"/>
@@ -5192,7 +5258,7 @@
       <c r="H115" s="6"/>
       <c r="J115" s="6"/>
     </row>
-    <row r="116" spans="1:10" ht="25" customHeight="1">
+    <row r="116" spans="1:11" ht="25" customHeight="1">
       <c r="A116" s="6"/>
       <c r="B116" s="6"/>
       <c r="C116" s="6"/>
@@ -5203,7 +5269,7 @@
       <c r="H116" s="6"/>
       <c r="J116" s="6"/>
     </row>
-    <row r="117" spans="1:10" ht="25" customHeight="1">
+    <row r="117" spans="1:11" ht="25" customHeight="1">
       <c r="A117" s="6"/>
       <c r="B117" s="6"/>
       <c r="C117" s="6"/>
@@ -5214,7 +5280,7 @@
       <c r="H117" s="6"/>
       <c r="J117" s="6"/>
     </row>
-    <row r="118" spans="1:10" ht="25" customHeight="1">
+    <row r="118" spans="1:11" ht="25" customHeight="1">
       <c r="A118" s="6"/>
       <c r="B118" s="6"/>
       <c r="C118" s="6"/>
@@ -5225,7 +5291,7 @@
       <c r="H118" s="6"/>
       <c r="J118" s="6"/>
     </row>
-    <row r="119" spans="1:10" ht="25" customHeight="1">
+    <row r="119" spans="1:11" ht="25" customHeight="1">
       <c r="A119" s="6"/>
       <c r="B119" s="6"/>
       <c r="C119" s="6"/>
@@ -5236,7 +5302,7 @@
       <c r="H119" s="6"/>
       <c r="J119" s="6"/>
     </row>
-    <row r="120" spans="1:10" ht="25" customHeight="1">
+    <row r="120" spans="1:11" ht="25" customHeight="1">
       <c r="A120" s="6"/>
       <c r="B120" s="6"/>
       <c r="C120" s="6"/>
@@ -5247,7 +5313,7 @@
       <c r="H120" s="6"/>
       <c r="J120" s="6"/>
     </row>
-    <row r="121" spans="1:10" ht="25" customHeight="1">
+    <row r="121" spans="1:11" ht="25" customHeight="1">
       <c r="A121" s="6"/>
       <c r="B121" s="6"/>
       <c r="C121" s="6"/>
@@ -5258,7 +5324,7 @@
       <c r="H121" s="6"/>
       <c r="J121" s="6"/>
     </row>
-    <row r="122" spans="1:10" ht="25" customHeight="1">
+    <row r="122" spans="1:11" ht="25" customHeight="1">
       <c r="A122" s="6"/>
       <c r="B122" s="6"/>
       <c r="C122" s="6"/>
@@ -5269,7 +5335,7 @@
       <c r="H122" s="6"/>
       <c r="J122" s="6"/>
     </row>
-    <row r="123" spans="1:10" ht="25" customHeight="1">
+    <row r="123" spans="1:11" ht="25" customHeight="1">
       <c r="A123" s="6"/>
       <c r="B123" s="6"/>
       <c r="C123" s="6"/>
@@ -5280,7 +5346,7 @@
       <c r="H123" s="6"/>
       <c r="J123" s="6"/>
     </row>
-    <row r="124" spans="1:10" ht="25" customHeight="1">
+    <row r="124" spans="1:11" ht="25" customHeight="1">
       <c r="A124" s="6"/>
       <c r="B124" s="6"/>
       <c r="C124" s="6"/>
@@ -5291,7 +5357,7 @@
       <c r="H124" s="6"/>
       <c r="J124" s="6"/>
     </row>
-    <row r="125" spans="1:10" ht="25" customHeight="1">
+    <row r="125" spans="1:11" ht="25" customHeight="1">
       <c r="A125" s="6"/>
       <c r="B125" s="6"/>
       <c r="C125" s="6"/>
@@ -5302,7 +5368,7 @@
       <c r="H125" s="6"/>
       <c r="J125" s="6"/>
     </row>
-    <row r="126" spans="1:10" ht="25" customHeight="1">
+    <row r="126" spans="1:11" ht="25" customHeight="1">
       <c r="A126" s="6"/>
       <c r="B126" s="6"/>
       <c r="C126" s="6"/>
@@ -5313,7 +5379,7 @@
       <c r="H126" s="6"/>
       <c r="J126" s="6"/>
     </row>
-    <row r="127" spans="1:10" ht="25" customHeight="1">
+    <row r="127" spans="1:11" ht="25" customHeight="1">
       <c r="A127" s="6"/>
       <c r="B127" s="6"/>
       <c r="C127" s="6"/>
@@ -5324,7 +5390,7 @@
       <c r="H127" s="6"/>
       <c r="J127" s="6"/>
     </row>
-    <row r="128" spans="1:10" ht="25" customHeight="1">
+    <row r="128" spans="1:11" ht="25" customHeight="1">
       <c r="A128" s="6"/>
       <c r="B128" s="6"/>
       <c r="C128" s="6"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-28 22:01:01
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51EB2D72-546C-C947-BECD-E6507A62F50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF255EC6-1570-3443-8D55-692DFC4EF810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="123">
   <si>
     <t>证券代码</t>
   </si>
@@ -397,14 +397,39 @@
     <t>首先看好pcb的长期发展导向，pcb相对于光模块还没有进入全民炒作的狂热，资金也在选择方向，最后还是要集中于ai基建无论是怎样pcb背板都是主要的存在+ccl一季度涨价的消息可以博弈第一季度财报</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>反思</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
     <t>对这两笔失败的交易进行反思：1.首先我觉得自己最近的操作有点太散户思维或者说对于价格太敏感了，容易在分时上被价格的波动所牵动，而这又会导致我在盘中作出一些低卖高买的操作，这一来一回之间反而损耗了应该有的利润 2.我太急了 太想开仓了 开仓太草率了 草率到明明原因还不明朗就冲进去 其实对于今天的生益科技我也有这样的感觉 但我似乎又有一个声音在劝自己如果不上车那就再也上不去了3，看问题抓不到主要矛盾 为什么ds一发就要去追最近最想关的和华为有关的板块呢 为什么不发散思维 或者说聪明一点 明明拓维信息不算纯血的科技股还要往里面跳，以后交易应该考虑保守和激进的结合 选择沾边的但又同时提供了一定安全边际的股票反而会让我感到舒服 且更应该抓住主要矛盾 这是对国产制造国产半导体的利好 不能一叶障目去追那些垃圾票</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>002028</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>思源电气</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>买入</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>短线资金恐慌砸盘离场 思源电气一季报基本符合预期 但资金同样在寻找瑕疵 如毛利率恶化 这主要是销售费用以及开发费用所造成的影响 无论是净利润还是营收都在同比高增速增长 +高存或 负现金流 可以理解为扩产快 需求大 我认为在这里思源电气的基本面并没有改变只是一部分想要博弈交易季报的资金认为不及预期 于是离场形成的踩踏</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>600183</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>生益科技</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>这里当做一个5日线确认 生益科技价格一直徘徊在5日线附近 给我的信号是：这里是有人在做多的 + 长期看好ccl涨价 今天的季报符合预期或者超预期都有可能 -&gt; 加仓 但只加了200股-&gt;原因在于即便业绩达到预期明天兑现的概率也存在 没必要打满仓位</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1086,7 +1111,7 @@
         <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:16" s="2" customFormat="1" ht="20.5" customHeight="1">
@@ -5281,7 +5306,7 @@
         <v>109</v>
       </c>
       <c r="P114" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="115" spans="1:16" ht="50">
@@ -5349,30 +5374,69 @@
         <v>113</v>
       </c>
     </row>
-    <row r="117" spans="1:16" ht="25" customHeight="1">
-      <c r="A117" s="6"/>
-      <c r="B117" s="6"/>
-      <c r="C117" s="6"/>
-      <c r="D117" s="6"/>
-      <c r="E117" s="8"/>
-      <c r="F117" s="6"/>
-      <c r="G117" s="6"/>
-      <c r="H117" s="6"/>
-      <c r="J117" s="6"/>
-      <c r="K117" s="3" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="118" spans="1:16" ht="25" customHeight="1">
-      <c r="A118" s="6"/>
-      <c r="B118" s="6"/>
-      <c r="C118" s="6"/>
-      <c r="D118" s="6"/>
-      <c r="E118" s="8"/>
-      <c r="F118" s="6"/>
-      <c r="G118" s="6"/>
-      <c r="H118" s="6"/>
-      <c r="J118" s="6"/>
+    <row r="117" spans="1:16" ht="200">
+      <c r="A117" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="B117" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C117" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D117" s="6">
+        <v>20260428</v>
+      </c>
+      <c r="E117" s="8">
+        <v>0.40069444444444446</v>
+      </c>
+      <c r="F117" s="6">
+        <v>198</v>
+      </c>
+      <c r="G117" s="6">
+        <v>100</v>
+      </c>
+      <c r="H117" s="6">
+        <v>19800</v>
+      </c>
+      <c r="J117" s="6">
+        <v>100</v>
+      </c>
+      <c r="K117" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="118" spans="1:16" ht="150">
+      <c r="A118" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C118" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D118" s="6">
+        <v>20260428</v>
+      </c>
+      <c r="E118" s="8">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="F118" s="6">
+        <v>75.400000000000006</v>
+      </c>
+      <c r="G118" s="6">
+        <v>200</v>
+      </c>
+      <c r="H118" s="6">
+        <v>15080</v>
+      </c>
+      <c r="J118" s="6">
+        <v>500</v>
+      </c>
+      <c r="K118" s="12" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="119" spans="1:16" ht="25" customHeight="1">
       <c r="A119" s="6"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-29 17:43:34
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuguan1/Documents/github/Trading_assess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF255EC6-1570-3443-8D55-692DFC4EF810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E77B1FE-0B66-9746-9205-B8724906C00B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="127">
   <si>
     <t>证券代码</t>
   </si>
@@ -430,6 +430,22 @@
   </si>
   <si>
     <t>这里当做一个5日线确认 生益科技价格一直徘徊在5日线附近 给我的信号是：这里是有人在做多的 + 长期看好ccl涨价 今天的季报符合预期或者超预期都有可能 -&gt; 加仓 但只加了200股-&gt;原因在于即便业绩达到预期明天兑现的概率也存在 没必要打满仓位</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>看到接近中午盘前上涨的热潮仍然还在没有褪去，于是决定在回调的低点选择买入加仓确认</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>卖出</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>中午盘后价格走势一路向下，且并没有反弹的意思越到尾盘价格越是走低，伴随着放量 我可以认为是一部分前期获利盘在离场了，外加明天最后出金日是时候规避一下风险，我认为我今天其实没有做好不应该在形式还不明朗的时候就确认加仓，至少应该等到接近尾盘确认的时候才上车 而不是匆匆忙忙的想要追涨 简直就是一波韭菜操作</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>是时候好好反思一下自己的操作了 买入中科曙光的逻辑本身就是不正确的 如果当时周末ds没发酵 周一就应该割掉走人 但是我当时却寄希望于新的概念 例如它的云计算啊 cpu啊但这根本就不是我当初买入的原因 我持有的原因已经和当时不一样了 我不该拖着不放手的 这是个最大的错误 改变持仓原因 坚决不能再有这种问题出现</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -5438,38 +5454,103 @@
         <v>122</v>
       </c>
     </row>
-    <row r="119" spans="1:16" ht="25" customHeight="1">
-      <c r="A119" s="6"/>
-      <c r="B119" s="6"/>
-      <c r="C119" s="6"/>
-      <c r="D119" s="6"/>
-      <c r="E119" s="8"/>
-      <c r="F119" s="6"/>
-      <c r="G119" s="6"/>
-      <c r="H119" s="6"/>
-      <c r="J119" s="6"/>
-    </row>
-    <row r="120" spans="1:16" ht="25" customHeight="1">
-      <c r="A120" s="6"/>
-      <c r="B120" s="6"/>
-      <c r="C120" s="6"/>
-      <c r="D120" s="6"/>
-      <c r="E120" s="8"/>
-      <c r="F120" s="6"/>
-      <c r="G120" s="6"/>
-      <c r="H120" s="6"/>
-      <c r="J120" s="6"/>
-    </row>
-    <row r="121" spans="1:16" ht="25" customHeight="1">
-      <c r="A121" s="6"/>
-      <c r="B121" s="6"/>
-      <c r="C121" s="6"/>
-      <c r="D121" s="6"/>
-      <c r="E121" s="8"/>
-      <c r="F121" s="6"/>
-      <c r="G121" s="6"/>
-      <c r="H121" s="6"/>
-      <c r="J121" s="6"/>
+    <row r="119" spans="1:16" ht="50">
+      <c r="A119" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B119" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C119" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D119" s="6">
+        <v>20260429</v>
+      </c>
+      <c r="E119" s="8">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="F119" s="6">
+        <v>79.97</v>
+      </c>
+      <c r="G119" s="6">
+        <v>300</v>
+      </c>
+      <c r="H119" s="6">
+        <v>23991</v>
+      </c>
+      <c r="J119" s="6">
+        <v>800</v>
+      </c>
+      <c r="K119" s="12" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="120" spans="1:16" ht="325">
+      <c r="A120" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B120" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C120" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D120" s="6">
+        <v>20260429</v>
+      </c>
+      <c r="E120" s="8">
+        <v>0.62152777777777779</v>
+      </c>
+      <c r="F120" s="6">
+        <v>77.87</v>
+      </c>
+      <c r="G120" s="6">
+        <v>300</v>
+      </c>
+      <c r="H120" s="6">
+        <v>23361</v>
+      </c>
+      <c r="J120" s="6">
+        <v>500</v>
+      </c>
+      <c r="K120" s="12"/>
+      <c r="O120" s="12" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="121" spans="1:16" ht="50">
+      <c r="A121" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="B121" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C121" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D121" s="6">
+        <v>20260429</v>
+      </c>
+      <c r="E121" s="8">
+        <v>0.62152777777777779</v>
+      </c>
+      <c r="F121" s="6">
+        <v>90.41</v>
+      </c>
+      <c r="G121" s="6">
+        <v>500</v>
+      </c>
+      <c r="H121" s="6">
+        <v>45200</v>
+      </c>
+      <c r="J121" s="6">
+        <v>0</v>
+      </c>
+      <c r="K121" s="12"/>
+      <c r="N121" s="12" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="122" spans="1:16" ht="25" customHeight="1">
       <c r="A122" s="6"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-23 15:41:00
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="13060"/>
+    <workbookView windowHeight="24460"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="153">
   <si>
     <t>证券代码</t>
   </si>
@@ -489,18 +489,34 @@
   </si>
   <si>
     <t>底仓清空：6-15起分批减，6-17在107.12反弹中清完，本轮(5-27建仓)全平</t>
+  </si>
+  <si>
+    <t>首先：我不认为当前存在任何的利空 从解读研报和nvda最近传出的压价方面都证明 这都是传言且不真实 ，股价在这个地方下跌的原因我更倾向于归结为整体涨多了的回调 把生益科技和其他同类型股票 如 沪电股份 深南电路放一起确实他是跌的最多的 但前期也是涨的最多的 所以我认为这只是短期的一种回调罢了  接着：减仓原因在于 今天对于五日线来说是一个明显的破位 下方缺口为价格提供了一点的支撑 但是我不愿意在这个地方继续押注了 短期继续下跌可能就会到10日线附近 前几个交易日也有类似的破位 最终第二日收回 这也是我没有全部清仓的原因  还想再次博弈明天的反弹 最后：资金问题 今天下跌后出现了部分我想要初步减仓的标的 如mlcc 的风华高科 这里只是初步的试仓阶段 同时东山精密今天在五日线并没有明显的破位 不做减仓 只能卖掉部分生益科技 获得换仓资金</t>
+  </si>
+  <si>
+    <t>000636</t>
+  </si>
+  <si>
+    <t>风华高科</t>
+  </si>
+  <si>
+    <t xml:space="preserve">首先 风华高科的多头上升现在看来是好的 （趋势正确）其次：分时图里 在66.64位置存在抄底的资金 短期这个位置有支撑的 同时今天大环境不好的情况下 比同行更加抗跌这里我认为是强的表现 行业层面：mlcc不断上修预期 行业的风向在 </t>
+  </si>
+  <si>
+    <t>66.64（前一日的最低点附近）</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="0.000"/>
+    <numFmt numFmtId="177" formatCode="0.00_ "/>
   </numFmts>
   <fonts count="25">
     <font>
@@ -542,7 +558,7 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="18"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -1121,7 +1137,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1185,8 +1201,17 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -6766,9 +6791,6 @@
         <v>1100</v>
       </c>
       <c r="K147" s="23"/>
-      <c r="L147"/>
-      <c r="M147"/>
-      <c r="N147"/>
       <c r="O147" t="s">
         <v>145</v>
       </c>
@@ -7053,8 +7075,6 @@
         <v>0</v>
       </c>
       <c r="K156" s="23"/>
-      <c r="L156"/>
-      <c r="M156"/>
       <c r="N156" t="s">
         <v>147</v>
       </c>
@@ -7183,15 +7203,76 @@
       </c>
       <c r="K160" s="23"/>
     </row>
-    <row r="161" ht="24" customHeight="1" spans="3:5">
-      <c r="C161" s="6"/>
-      <c r="D161" s="6"/>
-      <c r="E161" s="8"/>
-    </row>
-    <row r="162" ht="24" customHeight="1" spans="3:5">
-      <c r="C162" s="6"/>
-      <c r="D162" s="6"/>
-      <c r="E162" s="8"/>
+    <row r="161" customFormat="1" ht="388" spans="1:16">
+      <c r="A161" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="B161" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C161" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D161" s="17">
+        <v>20260623</v>
+      </c>
+      <c r="E161" s="19">
+        <v>0.622407407407407</v>
+      </c>
+      <c r="F161" s="20">
+        <v>168.4</v>
+      </c>
+      <c r="G161" s="17">
+        <v>300</v>
+      </c>
+      <c r="H161" s="20">
+        <v>50520</v>
+      </c>
+      <c r="I161" s="22"/>
+      <c r="J161" s="17">
+        <v>400</v>
+      </c>
+      <c r="K161" s="23"/>
+      <c r="P161" s="24" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="162" customFormat="1" ht="156" spans="1:16">
+      <c r="A162" s="26" t="s">
+        <v>149</v>
+      </c>
+      <c r="B162" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="C162" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D162" s="17">
+        <v>20260623</v>
+      </c>
+      <c r="E162" s="19">
+        <v>0.622407407407407</v>
+      </c>
+      <c r="F162" s="20">
+        <v>70.25</v>
+      </c>
+      <c r="G162" s="17">
+        <v>600</v>
+      </c>
+      <c r="H162" s="20">
+        <v>42126</v>
+      </c>
+      <c r="I162" s="22"/>
+      <c r="J162" s="17">
+        <v>600</v>
+      </c>
+      <c r="K162" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="M162" s="25" t="s">
+        <v>152</v>
+      </c>
+      <c r="P162" s="24"/>
     </row>
     <row r="163" ht="24" customHeight="1" spans="3:5">
       <c r="C163" s="6"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-24 15:38:49
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="24460"/>
+    <workbookView windowWidth="26860" windowHeight="14500"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="157">
   <si>
     <t>证券代码</t>
   </si>
@@ -504,6 +504,18 @@
   </si>
   <si>
     <t>66.64（前一日的最低点附近）</t>
+  </si>
+  <si>
+    <t>这里加仓我认为我加急了 还是应该等到尾盘买入的 这种直线的分时图拉伸还是不能这么武断的去追涨 风险存在 还好昨天尾盘尚且有一定的利润作为保护</t>
+  </si>
+  <si>
+    <t>今天的修复太弱了 总是在0轴徘徊 但不能这么简单的归咎到个股问题 因为今天光模块整体的表现都很差 缺乏有效的修复 今天减仓的主要原因是价格已经开始逼近我的成本线 同时下方10日线的支撑还有一定距离 减仓或许 能规避一定程度的风险 同时 这个股票在我组合中的占比还是太大了 这是我担忧的问题</t>
+  </si>
+  <si>
+    <t>生益科技在10日线出现了有效的修复 虽然没有完全回收昨日的跌幅 但我认为这个10日线位置短期是安全的 且 现在对于完全推出生益科技还是过早 市值虽然已经大 但是估值还不算过高 临近中期报 把资金重新聚焦pcb这一主线</t>
+  </si>
+  <si>
+    <t>我认为昨天我的操作是做错了的 首先我没有看到生益科技在10日线这里是有支撑的 其次我之前该弱不弱就是强的理论在这里似乎失效了 同时我觉得自己最该反思的是昨天尾盘的减仓 既然基本面没有变化 而同时有这么大的跌幅 更应该判定成是一次假摔 或者主力在换筹码 叠加放出天量 我应该深入思考一下到底是谁在卖谁在买 如果单单看五日线破位 是否太武断了？？</t>
   </si>
 </sst>
 </file>
@@ -1137,7 +1149,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1209,6 +1221,9 @@
     </xf>
     <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center"/>
@@ -7238,7 +7253,7 @@
       </c>
     </row>
     <row r="162" customFormat="1" ht="156" spans="1:16">
-      <c r="A162" s="26" t="s">
+      <c r="A162" s="27" t="s">
         <v>149</v>
       </c>
       <c r="B162" s="16" t="s">
@@ -7274,20 +7289,110 @@
       </c>
       <c r="P162" s="24"/>
     </row>
-    <row r="163" ht="24" customHeight="1" spans="3:5">
-      <c r="C163" s="6"/>
-      <c r="D163" s="6"/>
-      <c r="E163" s="8"/>
-    </row>
-    <row r="164" ht="24" customHeight="1" spans="3:5">
-      <c r="C164" s="6"/>
-      <c r="D164" s="6"/>
-      <c r="E164" s="8"/>
-    </row>
-    <row r="165" ht="24" customHeight="1" spans="3:5">
-      <c r="C165" s="6"/>
-      <c r="D165" s="6"/>
-      <c r="E165" s="8"/>
+    <row r="163" customFormat="1" ht="104" spans="1:16">
+      <c r="A163" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="B163" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="C163" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D163" s="17">
+        <v>20260624</v>
+      </c>
+      <c r="E163" s="19">
+        <v>0.560416666666667</v>
+      </c>
+      <c r="F163" s="20">
+        <v>73.49</v>
+      </c>
+      <c r="G163" s="17">
+        <v>100</v>
+      </c>
+      <c r="H163" s="20">
+        <v>7349</v>
+      </c>
+      <c r="I163" s="22"/>
+      <c r="J163" s="17">
+        <v>700</v>
+      </c>
+      <c r="K163" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="M163" s="25" t="s">
+        <v>152</v>
+      </c>
+      <c r="P163" s="24"/>
+    </row>
+    <row r="164" customFormat="1" ht="150" customHeight="1" spans="1:15">
+      <c r="A164" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="B164" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="C164" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D164" s="17">
+        <v>20260624</v>
+      </c>
+      <c r="E164" s="19">
+        <v>0.622511574074074</v>
+      </c>
+      <c r="F164" s="20">
+        <v>256.24</v>
+      </c>
+      <c r="G164" s="17">
+        <v>200</v>
+      </c>
+      <c r="H164" s="20">
+        <v>52148</v>
+      </c>
+      <c r="I164" s="22"/>
+      <c r="J164" s="17"/>
+      <c r="K164" s="23"/>
+      <c r="O164" s="26" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="165" customFormat="1" ht="184" spans="1:16">
+      <c r="A165" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="B165" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C165" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D165" s="17">
+        <v>20260624</v>
+      </c>
+      <c r="E165" s="19">
+        <v>0.622407407407407</v>
+      </c>
+      <c r="F165" s="20">
+        <v>177.75</v>
+      </c>
+      <c r="G165" s="17">
+        <v>300</v>
+      </c>
+      <c r="H165" s="20">
+        <v>53325</v>
+      </c>
+      <c r="I165" s="22"/>
+      <c r="J165" s="17">
+        <v>700</v>
+      </c>
+      <c r="K165" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="P165" s="24" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="166" ht="24" customHeight="1" spans="3:5">
       <c r="C166" s="6"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-26 21:08:27
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26860" windowHeight="14500"/>
+    <workbookView windowWidth="29100" windowHeight="14640"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="161">
   <si>
     <t>证券代码</t>
   </si>
@@ -516,6 +516,18 @@
   </si>
   <si>
     <t>我认为昨天我的操作是做错了的 首先我没有看到生益科技在10日线这里是有支撑的 其次我之前该弱不弱就是强的理论在这里似乎失效了 同时我觉得自己最该反思的是昨天尾盘的减仓 既然基本面没有变化 而同时有这么大的跌幅 更应该判定成是一次假摔 或者主力在换筹码 叠加放出天量 我应该深入思考一下到底是谁在卖谁在买 如果单单看五日线破位 是否太武断了？？</t>
+  </si>
+  <si>
+    <t>当时的想法是被市场上那些超跌的标的吸引 想去博一下中天科技下一周的修复 鉴于一直在东山精密这只股票上耗费了太多的时间也没赚什么钱 决定逐步抽离</t>
+  </si>
+  <si>
+    <t>600522</t>
+  </si>
+  <si>
+    <t>中天科技</t>
+  </si>
+  <si>
+    <t>今天光纤这条线因为康宁的小作文而大跌 虽然当时我还没有真正的去了解整一个技术链 但是直觉上来讲这次恐慌下跌是不合理的 光纤这条线仍然是长期的主线剧情之一 利空并没有很大的出现 我更愿意相信是错杀 于是买入 等待周一的修复 最大亏损为5%外加本身在参与光纤这个主线的时候就一直想找机会入手中天科技 今天说不定是个上车的机会</t>
   </si>
 </sst>
 </file>
@@ -1438,7 +1450,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:P1006"/>
+  <dimension ref="A1:AC1006"/>
   <sheetFormatPr defaultColWidth="10.3365384615385" defaultRowHeight="20.4"/>
   <cols>
     <col min="1" max="1" width="22.1634615384615" style="2" customWidth="1"/>
@@ -7394,20 +7406,143 @@
         <v>156</v>
       </c>
     </row>
-    <row r="166" ht="24" customHeight="1" spans="3:5">
-      <c r="C166" s="6"/>
-      <c r="D166" s="6"/>
-      <c r="E166" s="8"/>
-    </row>
-    <row r="167" ht="24" customHeight="1" spans="3:5">
-      <c r="C167" s="6"/>
-      <c r="D167" s="6"/>
-      <c r="E167" s="8"/>
-    </row>
-    <row r="168" ht="24" customHeight="1" spans="3:5">
-      <c r="C168" s="6"/>
-      <c r="D168" s="6"/>
-      <c r="E168" s="8"/>
+    <row r="166" ht="182" spans="1:29">
+      <c r="A166" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="B166" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="C166" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D166" s="17">
+        <v>20260626</v>
+      </c>
+      <c r="E166" s="19">
+        <v>0.554861111111111</v>
+      </c>
+      <c r="F166" s="20">
+        <v>262.09</v>
+      </c>
+      <c r="G166" s="17">
+        <v>100</v>
+      </c>
+      <c r="H166" s="20">
+        <v>26209</v>
+      </c>
+      <c r="I166" s="22"/>
+      <c r="J166" s="17">
+        <v>300</v>
+      </c>
+      <c r="K166" s="23"/>
+      <c r="L166"/>
+      <c r="M166"/>
+      <c r="N166"/>
+      <c r="O166" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="P166"/>
+      <c r="Q166"/>
+      <c r="R166"/>
+      <c r="S166"/>
+      <c r="T166"/>
+      <c r="U166"/>
+      <c r="V166"/>
+      <c r="W166"/>
+      <c r="X166"/>
+      <c r="Y166"/>
+      <c r="Z166"/>
+      <c r="AA166"/>
+      <c r="AB166"/>
+      <c r="AC166"/>
+    </row>
+    <row r="167" ht="24" customHeight="1" spans="1:29">
+      <c r="A167" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="B167" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C167" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D167" s="17">
+        <v>20260626</v>
+      </c>
+      <c r="E167" s="19">
+        <v>0.554861111111111</v>
+      </c>
+      <c r="F167" s="20">
+        <v>176.45</v>
+      </c>
+      <c r="G167" s="17">
+        <v>100</v>
+      </c>
+      <c r="H167" s="20">
+        <v>17645</v>
+      </c>
+      <c r="I167" s="22"/>
+      <c r="J167" s="17">
+        <v>600</v>
+      </c>
+      <c r="K167" s="23"/>
+      <c r="L167"/>
+      <c r="M167"/>
+      <c r="N167"/>
+      <c r="O167"/>
+      <c r="P167" s="24"/>
+      <c r="Q167"/>
+      <c r="R167"/>
+      <c r="S167"/>
+      <c r="T167"/>
+      <c r="U167"/>
+      <c r="V167"/>
+      <c r="W167"/>
+      <c r="X167"/>
+      <c r="Y167"/>
+      <c r="Z167"/>
+      <c r="AA167"/>
+      <c r="AB167"/>
+      <c r="AC167"/>
+    </row>
+    <row r="168" customFormat="1" ht="234" spans="1:16">
+      <c r="A168" s="27" t="s">
+        <v>158</v>
+      </c>
+      <c r="B168" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="C168" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D168" s="17">
+        <v>20260626</v>
+      </c>
+      <c r="E168" s="19">
+        <v>0.554861111111111</v>
+      </c>
+      <c r="F168" s="20">
+        <v>61.93</v>
+      </c>
+      <c r="G168" s="17">
+        <v>700</v>
+      </c>
+      <c r="H168" s="20">
+        <v>42903</v>
+      </c>
+      <c r="I168" s="22"/>
+      <c r="J168" s="17">
+        <v>700</v>
+      </c>
+      <c r="K168" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="L168"/>
+      <c r="M168"/>
+      <c r="N168"/>
+      <c r="O168"/>
+      <c r="P168" s="24"/>
     </row>
     <row r="169" ht="24" customHeight="1" spans="3:5">
       <c r="C169" s="6"/>

</xml_diff>

<commit_message>
vault backup: 2026-06-30 16:23:13
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="14640"/>
+    <workbookView windowHeight="24460"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="178">
   <si>
     <t>证券代码</t>
   </si>
@@ -528,6 +528,63 @@
   </si>
   <si>
     <t>今天光纤这条线因为康宁的小作文而大跌 虽然当时我还没有真正的去了解整一个技术链 但是直觉上来讲这次恐慌下跌是不合理的 光纤这条线仍然是长期的主线剧情之一 利空并没有很大的出现 我更愿意相信是错杀 于是买入 等待周一的修复 最大亏损为5%外加本身在参与光纤这个主线的时候就一直想找机会入手中天科技 今天说不定是个上车的机会</t>
+  </si>
+  <si>
+    <t>然而问题在于 上一个交易日我做了许多的研究 但都是关于中国巨石和中材科技的 今天要交易的话也应该是交易这两个标的 但是我看到这部分中天科技的超跌反而去做了我不熟悉的股票 这需要认真反思了 我觉得我这样的决定 太过于草率 同时自己应该尽可能对所有观察中的标的都有一定的了解再下手</t>
+  </si>
+  <si>
+    <t xml:space="preserve">当天风华高科需要控制异动 但是今天早盘高开之后一路高走到6%的位置 盘中必须下杀第二天才能有更高涨幅 所以这一波下杀是确定的 于是卖出400股 等待控制异动 而如果这种强势涨幅一直保持到最后 绝对触发异动 第二天风险较大 更早的获利了解也没问题
+</t>
+  </si>
+  <si>
+    <t>600584</t>
+  </si>
+  <si>
+    <t>首先长电科技作为近期炒作热度高的票 叠加了 hbm封测概念 以及近期突破了前期高点 估值还处于低位 所以是指的买入的 接着今天早盘我没有想到居然是这么快速的下杀 同时为了能让自己买到 把买单挂到了五日线上方一点 但是早晨恐慌性的抛盘实在太大 几乎整个上午都处于浮亏状态 这里是需要反思的 如果下午没有v起来怎么办？如果一直下杀怎么办 ？最好的方法似乎不是挂单而是更耐心一点 尾盘等待局势明朗些再进或许更好</t>
+  </si>
+  <si>
+    <t>首先 我并不是因为这场恐慌性下跌才因为恐惧而卖出东山精密
+真正的原因是近期很显然光模块板块正在处于一个调整震荡阶段已经不是市场的主线
+卖出东山精密是为了更好的将资金聚焦于主线 同时 东山精密向上的空间已经不是很大 我在这个地方浪费了太多的时间 
+以后给自己的提示就是在突破后没有更进一步的股票可以选择离场了 因为这场调整不知道要持续多久
+但主要原因 还是保本损 加上 时间成本 以及向上空间 优势已经不在我这边</t>
+  </si>
+  <si>
+    <t>600176</t>
+  </si>
+  <si>
+    <t>中国巨石</t>
+  </si>
+  <si>
+    <t>中国巨石是我一直研究且具备业绩的企业 最近也是走出了明显的多头趋势 今天的恐慌性下跌里面我认为自己是接早了 从分时图上来说 我看到底部五日线v起来已经说明短期5日线的支撑够强 于是贸然追涨 整个上午依旧是浮亏状态 但是做的好的一点是 这里的我敢于调仓 追逐那些真正处在优势的公司 从当日来看我的买点并不是很好 甚至有点草率 以后更应该警惕一波抛物线的上涨 不应该无脑追入 但五日线v起说明趋势仍在且还强势 可以继续持有</t>
+  </si>
+  <si>
+    <t>没控制住异动范围 清仓</t>
+  </si>
+  <si>
+    <t>尾盘全部收回跌幅 太强势了 加仓100股</t>
+  </si>
+  <si>
+    <t xml:space="preserve">这里主要是想对pcb这个板块的持仓进行调仓 将资金用于加仓涨势更好的中国巨石 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">这一次我没有在直线拉升中买入 而是选择一段时间后的冲高回落后再买入 这是我相比以往做对了的地方 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">中天科技从日线图上来看是在10日线企稳了
+又同时距离我的回本线更近一步 这里我违背了自己的交易规则 就是在亏损的时候加仓 这个时候我的想法是 既然都是在往上而且企稳 加仓能拉低成本同时增大收益 何乐不为 但是这里我却买在了几乎当日最高点 问题在于 我不认为这笔交易或许存在什么问题 我太心急了 怕在小仓位的时候踏空 太想重新创造账户的新高  </t>
+  </si>
+  <si>
+    <t>这里看到一个巨大买单 直冲云霄 之后小幅度的回落 这里其实我算比以往有点耐心 轻轻v起来 我就认为 应该是反弹了 这一波要涨停 生怕踏空 但我忽略了一点 午后的开盘总伴随着噪音 这是不真实的价格 我需要更耐心 至少在尾盘才能看出来谁的涨幅更可持续</t>
+  </si>
+  <si>
+    <t>买入之后中国巨石的价格一路下跌 底部并没有强烈的脱单 而我因为多次加仓使得价格已经逐步逼近成本线附近 这是很危险的举动 将至少1/3的仓位暴露在这个票上 且我没有很大的利润垫 只能割掉一半仓位 降低风险 等待趋势最终确认再加仓</t>
+  </si>
+  <si>
+    <t>'002281</t>
+  </si>
+  <si>
+    <t>初步进行减仓 理由是光迅科技的业绩确定性更高 + 今天量能相对健康 以及昨日回踩30日线得到支撑 这一波我看探底回升走出三浪</t>
   </si>
 </sst>
 </file>
@@ -1301,6 +1358,236 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>742315</xdr:colOff>
+      <xdr:row>176</xdr:row>
+      <xdr:rowOff>2582545</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>3491230</xdr:colOff>
+      <xdr:row>179</xdr:row>
+      <xdr:rowOff>614045</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="图片 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21521420" y="246295545"/>
+          <a:ext cx="7811770" cy="4102100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1031875</xdr:colOff>
+      <xdr:row>179</xdr:row>
+      <xdr:rowOff>1469390</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>2893695</xdr:colOff>
+      <xdr:row>187</xdr:row>
+      <xdr:rowOff>49530</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="图片 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21810980" y="251252990"/>
+          <a:ext cx="6924675" cy="3710940"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>4110990</xdr:colOff>
+      <xdr:row>180</xdr:row>
+      <xdr:rowOff>580390</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>801370</xdr:colOff>
+      <xdr:row>180</xdr:row>
+      <xdr:rowOff>580390</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp>
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="4" name="直接箭头连接符 3"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="20476210" y="252345190"/>
+          <a:ext cx="1104265" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="arrow"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:srgbClr val="FFFFFF"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:srgbClr val="FFFFFF"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>93345</xdr:colOff>
+      <xdr:row>178</xdr:row>
+      <xdr:rowOff>1016635</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>568325</xdr:colOff>
+      <xdr:row>178</xdr:row>
+      <xdr:rowOff>1423670</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp>
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="5" name="直接箭头连接符 4"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="20872450" y="248488835"/>
+          <a:ext cx="474980" cy="407035"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="arrow"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:srgbClr val="FFFFFF"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:srgbClr val="FFFFFF"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>4313555</xdr:colOff>
+      <xdr:row>178</xdr:row>
+      <xdr:rowOff>1342390</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>608965</xdr:colOff>
+      <xdr:row>179</xdr:row>
+      <xdr:rowOff>1125220</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp>
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="6" name="直接箭头连接符 5"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="20678775" y="248814590"/>
+          <a:ext cx="709295" cy="2094230"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="arrow"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:srgbClr val="FFFFFF"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:srgbClr val="FFFFFF"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -7538,76 +7825,485 @@
       <c r="K168" s="23" t="s">
         <v>160</v>
       </c>
-      <c r="L168"/>
-      <c r="M168"/>
-      <c r="N168"/>
-      <c r="O168"/>
-      <c r="P168" s="24"/>
-    </row>
-    <row r="169" ht="24" customHeight="1" spans="3:5">
-      <c r="C169" s="6"/>
-      <c r="D169" s="6"/>
-      <c r="E169" s="8"/>
-    </row>
-    <row r="170" ht="24" customHeight="1" spans="3:5">
-      <c r="C170" s="6"/>
-      <c r="D170" s="6"/>
-      <c r="E170" s="8"/>
-    </row>
-    <row r="171" ht="24" customHeight="1" spans="3:5">
-      <c r="C171" s="6"/>
-      <c r="D171" s="6"/>
-      <c r="E171" s="8"/>
-    </row>
-    <row r="172" ht="24" customHeight="1" spans="3:5">
-      <c r="C172" s="6"/>
-      <c r="D172" s="6"/>
-      <c r="E172" s="8"/>
-    </row>
-    <row r="173" ht="24" customHeight="1" spans="3:5">
-      <c r="C173" s="6"/>
-      <c r="D173" s="6"/>
-      <c r="E173" s="8"/>
-    </row>
-    <row r="174" ht="24" customHeight="1" spans="3:5">
-      <c r="C174" s="6"/>
-      <c r="D174" s="6"/>
-      <c r="E174" s="8"/>
-    </row>
-    <row r="175" ht="24" customHeight="1" spans="3:5">
-      <c r="C175" s="6"/>
-      <c r="D175" s="6"/>
-      <c r="E175" s="8"/>
-    </row>
-    <row r="176" ht="24" customHeight="1" spans="3:5">
-      <c r="C176" s="6"/>
-      <c r="D176" s="6"/>
-      <c r="E176" s="8"/>
-    </row>
-    <row r="177" ht="24" customHeight="1" spans="3:5">
-      <c r="C177" s="6"/>
-      <c r="D177" s="6"/>
-      <c r="E177" s="8"/>
-    </row>
-    <row r="178" ht="24" customHeight="1" spans="3:5">
-      <c r="C178" s="6"/>
-      <c r="D178" s="6"/>
-      <c r="E178" s="8"/>
-    </row>
-    <row r="179" ht="24" customHeight="1" spans="3:5">
-      <c r="C179" s="6"/>
-      <c r="D179" s="6"/>
-      <c r="E179" s="8"/>
-    </row>
-    <row r="180" ht="24" customHeight="1" spans="3:5">
-      <c r="C180" s="6"/>
-      <c r="D180" s="6"/>
-      <c r="E180" s="8"/>
-    </row>
-    <row r="181" ht="24" customHeight="1" spans="3:5">
-      <c r="C181" s="6"/>
-      <c r="D181" s="6"/>
-      <c r="E181" s="8"/>
+      <c r="O168" s="24"/>
+      <c r="P168" s="24" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="169" customFormat="1" ht="204" spans="1:16">
+      <c r="A169" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="B169" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="C169" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D169" s="17">
+        <v>20260629</v>
+      </c>
+      <c r="E169" s="19">
+        <v>0.405555555555556</v>
+      </c>
+      <c r="F169" s="20">
+        <v>83.21</v>
+      </c>
+      <c r="G169" s="17">
+        <v>500</v>
+      </c>
+      <c r="H169" s="20">
+        <v>41600</v>
+      </c>
+      <c r="I169" s="22"/>
+      <c r="J169" s="17">
+        <v>200</v>
+      </c>
+      <c r="K169" s="23"/>
+      <c r="M169" s="25"/>
+      <c r="O169" s="24" t="s">
+        <v>162</v>
+      </c>
+      <c r="P169" s="24"/>
+    </row>
+    <row r="170" customFormat="1" ht="286" spans="1:16">
+      <c r="A170" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="B170" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C170" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D170" s="17">
+        <v>20260629</v>
+      </c>
+      <c r="E170" s="19">
+        <v>0.419444444444444</v>
+      </c>
+      <c r="F170" s="20">
+        <v>97.77</v>
+      </c>
+      <c r="G170" s="17">
+        <v>400</v>
+      </c>
+      <c r="H170" s="20">
+        <v>39108</v>
+      </c>
+      <c r="I170" s="22"/>
+      <c r="J170" s="17">
+        <v>400</v>
+      </c>
+      <c r="K170" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="O170" s="24"/>
+      <c r="P170" s="24"/>
+    </row>
+    <row r="171" customFormat="1" ht="130" spans="1:16">
+      <c r="A171" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="B171" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="C171" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D171" s="17">
+        <v>20260629</v>
+      </c>
+      <c r="E171" s="19">
+        <v>0.428472222222222</v>
+      </c>
+      <c r="F171" s="20">
+        <v>244.53</v>
+      </c>
+      <c r="G171" s="17">
+        <v>300</v>
+      </c>
+      <c r="H171" s="20">
+        <v>73359</v>
+      </c>
+      <c r="I171" s="22"/>
+      <c r="J171" s="17">
+        <v>0</v>
+      </c>
+      <c r="K171" s="23"/>
+      <c r="N171" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="O171" s="24"/>
+      <c r="P171" s="24"/>
+    </row>
+    <row r="172" customFormat="1" ht="286" spans="1:16">
+      <c r="A172" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="B172" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="C172" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D172" s="17">
+        <v>20260629</v>
+      </c>
+      <c r="E172" s="19">
+        <v>0.434722222222222</v>
+      </c>
+      <c r="F172" s="20">
+        <v>69.187</v>
+      </c>
+      <c r="G172" s="17">
+        <v>700</v>
+      </c>
+      <c r="H172" s="20">
+        <v>49686</v>
+      </c>
+      <c r="I172" s="22"/>
+      <c r="J172" s="17">
+        <v>700</v>
+      </c>
+      <c r="K172" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="N172" s="23"/>
+      <c r="O172" s="24"/>
+      <c r="P172" s="24"/>
+    </row>
+    <row r="173" customFormat="1" ht="204" spans="1:16">
+      <c r="A173" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="B173" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="C173" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D173" s="17">
+        <v>20260629</v>
+      </c>
+      <c r="E173" s="19">
+        <v>0.620833333333333</v>
+      </c>
+      <c r="F173" s="20">
+        <v>80.04</v>
+      </c>
+      <c r="G173" s="17">
+        <v>200</v>
+      </c>
+      <c r="H173" s="20">
+        <v>16080</v>
+      </c>
+      <c r="I173" s="22"/>
+      <c r="J173" s="17">
+        <v>0</v>
+      </c>
+      <c r="K173" s="23"/>
+      <c r="M173" s="25"/>
+      <c r="N173" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="O173" s="24" t="s">
+        <v>162</v>
+      </c>
+      <c r="P173" s="24"/>
+    </row>
+    <row r="174" customFormat="1" ht="26" spans="1:16">
+      <c r="A174" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="B174" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C174" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D174" s="17">
+        <v>20260629</v>
+      </c>
+      <c r="E174" s="19">
+        <v>0.620833333333333</v>
+      </c>
+      <c r="F174" s="20">
+        <v>103.26</v>
+      </c>
+      <c r="G174" s="17">
+        <v>100</v>
+      </c>
+      <c r="H174" s="20">
+        <v>10326</v>
+      </c>
+      <c r="I174" s="22"/>
+      <c r="J174" s="17">
+        <v>500</v>
+      </c>
+      <c r="K174" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="O174" s="24"/>
+      <c r="P174" s="24"/>
+    </row>
+    <row r="175" customFormat="1" ht="62" spans="1:16">
+      <c r="A175" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="B175" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C175" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D175" s="17">
+        <v>20260630</v>
+      </c>
+      <c r="E175" s="19">
+        <v>0.452777777777778</v>
+      </c>
+      <c r="F175" s="20">
+        <v>175.01</v>
+      </c>
+      <c r="G175" s="17">
+        <v>100</v>
+      </c>
+      <c r="H175" s="20">
+        <v>17501</v>
+      </c>
+      <c r="I175" s="22"/>
+      <c r="J175" s="17">
+        <v>500</v>
+      </c>
+      <c r="K175" s="23"/>
+      <c r="L175"/>
+      <c r="M175"/>
+      <c r="N175"/>
+      <c r="O175" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="P175" s="24"/>
+    </row>
+    <row r="176" customFormat="1" ht="78" spans="1:16">
+      <c r="A176" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="B176" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="C176" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D176" s="17">
+        <v>20260630</v>
+      </c>
+      <c r="E176" s="19">
+        <v>0.45625</v>
+      </c>
+      <c r="F176" s="20">
+        <v>74.49</v>
+      </c>
+      <c r="G176" s="17">
+        <v>400</v>
+      </c>
+      <c r="H176" s="20">
+        <f t="shared" ref="H176:H179" si="0">F176*G176</f>
+        <v>29796</v>
+      </c>
+      <c r="I176" s="22"/>
+      <c r="J176" s="17">
+        <v>1100</v>
+      </c>
+      <c r="K176" s="23" t="s">
+        <v>172</v>
+      </c>
+      <c r="N176" s="23"/>
+      <c r="O176" s="24"/>
+      <c r="P176" s="24"/>
+    </row>
+    <row r="177" customFormat="1" ht="234" spans="1:16">
+      <c r="A177" s="27" t="s">
+        <v>158</v>
+      </c>
+      <c r="B177" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="C177" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D177" s="17">
+        <v>20260630</v>
+      </c>
+      <c r="E177" s="19">
+        <v>0.478472222222222</v>
+      </c>
+      <c r="F177" s="20">
+        <v>61.23</v>
+      </c>
+      <c r="G177" s="17">
+        <v>300</v>
+      </c>
+      <c r="H177" s="20">
+        <f t="shared" si="0"/>
+        <v>18369</v>
+      </c>
+      <c r="I177" s="22"/>
+      <c r="J177" s="17">
+        <v>1000</v>
+      </c>
+      <c r="K177" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="N177" s="23"/>
+      <c r="O177" s="24"/>
+      <c r="P177" s="24"/>
+    </row>
+    <row r="178" customFormat="1" ht="62" spans="1:16">
+      <c r="A178" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="B178" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C178" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D178" s="17">
+        <v>20260630</v>
+      </c>
+      <c r="E178" s="19">
+        <v>0.543055555555556</v>
+      </c>
+      <c r="F178" s="20">
+        <v>175.5</v>
+      </c>
+      <c r="G178" s="17">
+        <v>100</v>
+      </c>
+      <c r="H178" s="20">
+        <v>17550</v>
+      </c>
+      <c r="I178" s="22"/>
+      <c r="J178" s="17">
+        <v>400</v>
+      </c>
+      <c r="K178" s="23"/>
+      <c r="O178" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="P178" s="24"/>
+    </row>
+    <row r="179" customFormat="1" ht="182" spans="1:16">
+      <c r="A179" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="B179" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="C179" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D179" s="17">
+        <v>20260630</v>
+      </c>
+      <c r="E179" s="19">
+        <v>0.544444444444444</v>
+      </c>
+      <c r="F179" s="20">
+        <v>76.79</v>
+      </c>
+      <c r="G179" s="17">
+        <v>200</v>
+      </c>
+      <c r="H179" s="20">
+        <f>F179*G179</f>
+        <v>15358</v>
+      </c>
+      <c r="I179" s="22"/>
+      <c r="J179" s="17">
+        <v>1300</v>
+      </c>
+      <c r="K179" s="23" t="s">
+        <v>174</v>
+      </c>
+      <c r="N179" s="23"/>
+      <c r="O179" s="24"/>
+      <c r="P179" s="24"/>
+    </row>
+    <row r="180" customFormat="1" ht="156" spans="1:16">
+      <c r="A180" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="B180" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="C180" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D180" s="17">
+        <v>20260630</v>
+      </c>
+      <c r="E180" s="19">
+        <v>0.561805555555556</v>
+      </c>
+      <c r="F180" s="20">
+        <v>72.16</v>
+      </c>
+      <c r="G180" s="17">
+        <v>700</v>
+      </c>
+      <c r="H180" s="20">
+        <f>F180*G180</f>
+        <v>50512</v>
+      </c>
+      <c r="I180" s="22"/>
+      <c r="J180" s="17">
+        <v>600</v>
+      </c>
+      <c r="K180" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="N180" s="23"/>
+      <c r="O180" s="24"/>
+      <c r="P180" s="24"/>
+    </row>
+    <row r="181" customFormat="1" ht="104" spans="1:16">
+      <c r="A181" s="27" t="s">
+        <v>176</v>
+      </c>
+      <c r="B181" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C181" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D181" s="17">
+        <v>20260630</v>
+      </c>
+      <c r="E181" s="19">
+        <v>0.619444444444444</v>
+      </c>
+      <c r="F181" s="20">
+        <v>257.3</v>
+      </c>
+      <c r="G181" s="17">
+        <v>200</v>
+      </c>
+      <c r="H181" s="20">
+        <f>F181*G181</f>
+        <v>51460</v>
+      </c>
+      <c r="I181" s="22"/>
+      <c r="J181" s="17">
+        <v>200</v>
+      </c>
+      <c r="K181" s="23" t="s">
+        <v>177</v>
+      </c>
+      <c r="N181" s="23"/>
+      <c r="O181" s="24"/>
+      <c r="P181" s="24"/>
     </row>
     <row r="182" ht="24" customHeight="1" spans="3:5">
       <c r="C182" s="6"/>
@@ -10293,5 +10989,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-07-02 19:11:39
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="180">
   <si>
     <t>证券代码</t>
   </si>
@@ -585,6 +585,13 @@
   </si>
   <si>
     <t>初步进行减仓 理由是光迅科技的业绩确定性更高 + 今天量能相对健康 以及昨日回踩30日线得到支撑 这一波我看探底回升走出三浪</t>
+  </si>
+  <si>
+    <t>中天科技已经跌破了我预示的止损位 甚至超了许多 我也在思考自己的止损是不是设置的太过谨慎了 于是在这笔交易里我试着放宽止损 但我忘记了一个关键的点 当初买入的逻辑是
+认为这是一次错杀 我应该等待修复 但是两天下来并没有有效的修复 这个时候我应该保持警惕了 今天又是一波大下杀 且下面一个支撑位要到51块 虽然我认为这只票的行情并没那么快终结 但短期来看 确实很难 我选择了割肉离场</t>
+  </si>
+  <si>
+    <t xml:space="preserve">首先第一点买入的时候是跌停板 我在接飞刀 以后坚决不能接飞刀 即使错过行情也不能在一个票是跌停板的时候去接 第二点 浮亏加仓 在接近回本的时候 我尝试浮亏加仓 最终却扩大了自己的亏损 当时我安慰自己说 既然我看涨就应该在上涨中去加仓降低成本 一举两得 这样看来是错的 第三 心急 我太心急了 总是在当日buy到最高点 我当时在想什么？这是一个突破 我要跟上？但看到突然的红柱拉升跟上是错误的 基本上都是抛物线 很容易把自己挂在高处 第四 我刚刚想了一下为什么每次在当日买入的时候我都是在最高点 原因出在 如果这只股票在日内波动较小 这个时候我不会选择买入 反而是动量突然的上涨 诱使我买入 这也就意味着 该加仓或者该买入的时候 不是突然拉升后的那一波 而是在震荡中吸收筹码 在自己的节奏中买入 我一直都是在别人的节奏中买入 有人拉涨 我也跟风买入 这是我每日买在最高点的原因 </t>
   </si>
 </sst>
 </file>
@@ -1218,7 +1225,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1292,6 +1299,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
@@ -1405,15 +1415,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>1031875</xdr:colOff>
+      <xdr:colOff>1030605</xdr:colOff>
       <xdr:row>179</xdr:row>
       <xdr:rowOff>1469390</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>2893695</xdr:colOff>
-      <xdr:row>187</xdr:row>
-      <xdr:rowOff>49530</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>2692400</xdr:colOff>
+      <xdr:row>181</xdr:row>
+      <xdr:rowOff>34925</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1430,8 +1440,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="21810980" y="251252990"/>
-          <a:ext cx="6924675" cy="3710940"/>
+          <a:off x="21809710" y="251252990"/>
+          <a:ext cx="3488690" cy="1867535"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1737,7 +1747,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AC1006"/>
+  <dimension ref="A1:AC1005"/>
   <sheetFormatPr defaultColWidth="10.3365384615385" defaultRowHeight="20.4"/>
   <cols>
     <col min="1" max="1" width="22.1634615384615" style="2" customWidth="1"/>
@@ -7552,7 +7562,7 @@
       </c>
     </row>
     <row r="162" customFormat="1" ht="156" spans="1:16">
-      <c r="A162" s="27" t="s">
+      <c r="A162" s="28" t="s">
         <v>149</v>
       </c>
       <c r="B162" s="16" t="s">
@@ -7589,7 +7599,7 @@
       <c r="P162" s="24"/>
     </row>
     <row r="163" customFormat="1" ht="104" spans="1:16">
-      <c r="A163" s="27" t="s">
+      <c r="A163" s="28" t="s">
         <v>149</v>
       </c>
       <c r="B163" s="16" t="s">
@@ -7794,7 +7804,7 @@
       <c r="AC167"/>
     </row>
     <row r="168" customFormat="1" ht="234" spans="1:16">
-      <c r="A168" s="27" t="s">
+      <c r="A168" s="28" t="s">
         <v>158</v>
       </c>
       <c r="B168" s="16" t="s">
@@ -7831,7 +7841,7 @@
       </c>
     </row>
     <row r="169" customFormat="1" ht="204" spans="1:16">
-      <c r="A169" s="27" t="s">
+      <c r="A169" s="28" t="s">
         <v>149</v>
       </c>
       <c r="B169" s="16" t="s">
@@ -7867,7 +7877,7 @@
       <c r="P169" s="24"/>
     </row>
     <row r="170" customFormat="1" ht="286" spans="1:16">
-      <c r="A170" s="27" t="s">
+      <c r="A170" s="28" t="s">
         <v>163</v>
       </c>
       <c r="B170" s="16" t="s">
@@ -7902,7 +7912,7 @@
       <c r="P170" s="24"/>
     </row>
     <row r="171" customFormat="1" ht="130" spans="1:16">
-      <c r="A171" s="27" t="s">
+      <c r="A171" s="28" t="s">
         <v>126</v>
       </c>
       <c r="B171" s="16" t="s">
@@ -7938,7 +7948,7 @@
       <c r="P171" s="24"/>
     </row>
     <row r="172" customFormat="1" ht="286" spans="1:16">
-      <c r="A172" s="27" t="s">
+      <c r="A172" s="28" t="s">
         <v>166</v>
       </c>
       <c r="B172" s="16" t="s">
@@ -7974,7 +7984,7 @@
       <c r="P172" s="24"/>
     </row>
     <row r="173" customFormat="1" ht="204" spans="1:16">
-      <c r="A173" s="27" t="s">
+      <c r="A173" s="28" t="s">
         <v>149</v>
       </c>
       <c r="B173" s="16" t="s">
@@ -8013,7 +8023,7 @@
       <c r="P173" s="24"/>
     </row>
     <row r="174" customFormat="1" ht="26" spans="1:16">
-      <c r="A174" s="27" t="s">
+      <c r="A174" s="28" t="s">
         <v>163</v>
       </c>
       <c r="B174" s="16" t="s">
@@ -8086,7 +8096,7 @@
       <c r="P175" s="24"/>
     </row>
     <row r="176" customFormat="1" ht="78" spans="1:16">
-      <c r="A176" s="27" t="s">
+      <c r="A176" s="28" t="s">
         <v>166</v>
       </c>
       <c r="B176" s="16" t="s">
@@ -8123,7 +8133,7 @@
       <c r="P176" s="24"/>
     </row>
     <row r="177" customFormat="1" ht="234" spans="1:16">
-      <c r="A177" s="27" t="s">
+      <c r="A177" s="28" t="s">
         <v>158</v>
       </c>
       <c r="B177" s="16" t="s">
@@ -8195,7 +8205,7 @@
       <c r="P178" s="24"/>
     </row>
     <row r="179" customFormat="1" ht="182" spans="1:16">
-      <c r="A179" s="27" t="s">
+      <c r="A179" s="28" t="s">
         <v>166</v>
       </c>
       <c r="B179" s="16" t="s">
@@ -8232,7 +8242,7 @@
       <c r="P179" s="24"/>
     </row>
     <row r="180" customFormat="1" ht="156" spans="1:16">
-      <c r="A180" s="27" t="s">
+      <c r="A180" s="28" t="s">
         <v>166</v>
       </c>
       <c r="B180" s="16" t="s">
@@ -8269,7 +8279,7 @@
       <c r="P180" s="24"/>
     </row>
     <row r="181" customFormat="1" ht="104" spans="1:16">
-      <c r="A181" s="27" t="s">
+      <c r="A181" s="28" t="s">
         <v>176</v>
       </c>
       <c r="B181" s="16" t="s">
@@ -8305,10 +8315,43 @@
       <c r="O181" s="24"/>
       <c r="P181" s="24"/>
     </row>
-    <row r="182" ht="24" customHeight="1" spans="3:5">
-      <c r="C182" s="6"/>
-      <c r="D182" s="6"/>
-      <c r="E182" s="8"/>
+    <row r="182" customFormat="1" ht="388" spans="1:16">
+      <c r="A182" s="28" t="s">
+        <v>158</v>
+      </c>
+      <c r="B182" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="C182" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D182" s="17">
+        <v>20260701</v>
+      </c>
+      <c r="E182" s="19">
+        <v>0.618055555555556</v>
+      </c>
+      <c r="F182" s="20">
+        <v>54.82</v>
+      </c>
+      <c r="G182" s="17">
+        <v>1000</v>
+      </c>
+      <c r="H182" s="20">
+        <v>54820</v>
+      </c>
+      <c r="I182" s="22"/>
+      <c r="J182" s="17">
+        <v>0</v>
+      </c>
+      <c r="K182" s="23"/>
+      <c r="N182" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="O182" s="24"/>
+      <c r="P182" s="27" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="183" ht="24" customHeight="1" spans="3:5">
       <c r="C183" s="6"/>
@@ -8445,10 +8488,9 @@
       <c r="D209" s="6"/>
       <c r="E209" s="8"/>
     </row>
-    <row r="210" ht="24" customHeight="1" spans="3:5">
+    <row r="210" ht="24" customHeight="1" spans="3:4">
       <c r="C210" s="6"/>
       <c r="D210" s="6"/>
-      <c r="E210" s="8"/>
     </row>
     <row r="211" ht="24" customHeight="1" spans="3:4">
       <c r="C211" s="6"/>
@@ -9038,8 +9080,7 @@
       <c r="C357" s="6"/>
       <c r="D357" s="6"/>
     </row>
-    <row r="358" ht="24" customHeight="1" spans="3:4">
-      <c r="C358" s="6"/>
+    <row r="358" ht="24" customHeight="1" spans="4:4">
       <c r="D358" s="6"/>
     </row>
     <row r="359" ht="24" customHeight="1" spans="4:4">
@@ -10982,9 +11023,6 @@
     </row>
     <row r="1005" ht="24" customHeight="1" spans="4:4">
       <c r="D1005" s="6"/>
-    </row>
-    <row r="1006" ht="24" customHeight="1" spans="4:4">
-      <c r="D1006" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-06 23:34:31
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="13020"/>
+    <workbookView windowHeight="22240"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="185">
   <si>
     <t>证券代码</t>
   </si>
@@ -592,6 +592,21 @@
   </si>
   <si>
     <t xml:space="preserve">首先第一点买入的时候是跌停板 我在接飞刀 以后坚决不能接飞刀 即使错过行情也不能在一个票是跌停板的时候去接 第二点 浮亏加仓 在接近回本的时候 我尝试浮亏加仓 最终却扩大了自己的亏损 当时我安慰自己说 既然我看涨就应该在上涨中去加仓降低成本 一举两得 这样看来是错的 第三 心急 我太心急了 总是在当日buy到最高点 我当时在想什么？这是一个突破 我要跟上？但看到突然的红柱拉升跟上是错误的 基本上都是抛物线 很容易把自己挂在高处 第四 我刚刚想了一下为什么每次在当日买入的时候我都是在最高点 原因出在 如果这只股票在日内波动较小 这个时候我不会选择买入 反而是动量突然的上涨 诱使我买入 这也就意味着 该加仓或者该买入的时候 不是突然拉升后的那一波 而是在震荡中吸收筹码 在自己的节奏中买入 我一直都是在别人的节奏中买入 有人拉涨 我也跟风买入 这是我每日买在最高点的原因 </t>
+  </si>
+  <si>
+    <t>清仓的动作 发生在早上 清仓的主要原因 ： 1临近中报发布 长电科技的财报显然不如存储正股来的要炸裂 此乃颓势1 2. 10日线趋势跌破 下跌往下还有继续下跌的空间  同时认为兆易创新在这个价位要优于长电科技更占主线优势 于是清仓换股</t>
+  </si>
+  <si>
+    <t>603986</t>
+  </si>
+  <si>
+    <t>首先 ： 在这次大跌里我认为我应该去选择那些基本面更好 更占据主线的板块 当光模块陷入长时间盘整时 主要收到市场热烈讨论的还是存储 因为这是最出业绩 也是业绩最确定的方向 2.兆易创新作为存储芯片研发厂更区别于了其他如江波龙这种的组装厂 护城河也更深 更受益 3. 两天20%的下跌至少是一个相对便宜的价格 只买入100股是为了在后续还可以继续补仓</t>
+  </si>
+  <si>
+    <t>追涨买入 30日线有止跌迹象</t>
+  </si>
+  <si>
+    <t>这是一个延迟许多的止损 也是我应该反思的地方 在看到6.30时一根大阳线让我以后这只是一次简单的调整 于是试图去追涨 第二天出现了一定调整 这也在意料之内 于是我没有进行止损 但突然起来的新闻使得第三天低开跌停 第四天也没有像样的修复  价格重新回到测试6.11日的低点 多头的走势现在开来要逐步逆转 当日冲高强度也不高最后尾盘回落 最终清仓离场</t>
   </si>
 </sst>
 </file>
@@ -1398,7 +1413,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="21521420" y="246295545"/>
+          <a:off x="21521420" y="246282845"/>
           <a:ext cx="7811770" cy="4102100"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1440,7 +1455,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="21809710" y="251252990"/>
+          <a:off x="21809710" y="251240290"/>
           <a:ext cx="3488690" cy="1867535"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1474,7 +1489,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="20476210" y="252345190"/>
+          <a:off x="20476210" y="252332490"/>
           <a:ext cx="1104265" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -1521,7 +1536,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="20872450" y="248488835"/>
+          <a:off x="20872450" y="248476135"/>
           <a:ext cx="474980" cy="407035"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -1568,7 +1583,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="20678775" y="248814590"/>
+          <a:off x="20678775" y="248801890"/>
           <a:ext cx="709295" cy="2094230"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -8022,7 +8037,7 @@
       </c>
       <c r="P173" s="24"/>
     </row>
-    <row r="174" customFormat="1" ht="26" spans="1:16">
+    <row r="174" customFormat="1" ht="25" customHeight="1" spans="1:16">
       <c r="A174" s="28" t="s">
         <v>163</v>
       </c>
@@ -8087,9 +8102,6 @@
         <v>500</v>
       </c>
       <c r="K175" s="23"/>
-      <c r="L175"/>
-      <c r="M175"/>
-      <c r="N175"/>
       <c r="O175" s="24" t="s">
         <v>171</v>
       </c>
@@ -8353,25 +8365,149 @@
         <v>179</v>
       </c>
     </row>
-    <row r="183" ht="24" customHeight="1" spans="3:5">
-      <c r="C183" s="6"/>
-      <c r="D183" s="6"/>
-      <c r="E183" s="8"/>
-    </row>
-    <row r="184" ht="24" customHeight="1" spans="3:5">
-      <c r="C184" s="6"/>
-      <c r="D184" s="6"/>
-      <c r="E184" s="8"/>
-    </row>
-    <row r="185" ht="24" customHeight="1" spans="3:5">
-      <c r="C185" s="6"/>
-      <c r="D185" s="6"/>
-      <c r="E185" s="8"/>
-    </row>
-    <row r="186" ht="24" customHeight="1" spans="3:5">
-      <c r="C186" s="6"/>
-      <c r="D186" s="6"/>
-      <c r="E186" s="8"/>
+    <row r="183" customFormat="1" ht="52" spans="1:16">
+      <c r="A183" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="B183" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C183" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D183" s="17">
+        <v>20260703</v>
+      </c>
+      <c r="E183" s="19">
+        <v>0.415277777777778</v>
+      </c>
+      <c r="F183" s="20">
+        <v>90.56</v>
+      </c>
+      <c r="G183" s="17">
+        <v>700</v>
+      </c>
+      <c r="H183" s="20">
+        <v>63392</v>
+      </c>
+      <c r="I183" s="22"/>
+      <c r="J183" s="17">
+        <v>0</v>
+      </c>
+      <c r="K183" s="23"/>
+      <c r="N183" s="23" t="s">
+        <v>180</v>
+      </c>
+      <c r="O183" s="24"/>
+      <c r="P183" s="24"/>
+    </row>
+    <row r="184" customFormat="1" ht="234" spans="1:16">
+      <c r="A184" s="28" t="s">
+        <v>181</v>
+      </c>
+      <c r="B184" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C184" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D184" s="17">
+        <v>20260703</v>
+      </c>
+      <c r="E184" s="19">
+        <v>0.426388888888889</v>
+      </c>
+      <c r="F184" s="20">
+        <v>680</v>
+      </c>
+      <c r="G184" s="17">
+        <v>100</v>
+      </c>
+      <c r="H184" s="20">
+        <v>68000</v>
+      </c>
+      <c r="I184" s="22"/>
+      <c r="J184" s="17">
+        <v>100</v>
+      </c>
+      <c r="K184" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="N184" s="23"/>
+      <c r="O184" s="24"/>
+      <c r="P184" s="24"/>
+    </row>
+    <row r="185" customFormat="1" ht="184" spans="1:16">
+      <c r="A185" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="B185" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C185" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D185" s="17">
+        <v>20260703</v>
+      </c>
+      <c r="E185" s="19">
+        <v>0.446527777777778</v>
+      </c>
+      <c r="F185" s="20">
+        <v>164.23</v>
+      </c>
+      <c r="G185" s="17">
+        <v>200</v>
+      </c>
+      <c r="H185" s="20">
+        <v>32846</v>
+      </c>
+      <c r="I185" s="22"/>
+      <c r="J185" s="17">
+        <v>600</v>
+      </c>
+      <c r="K185" s="23" t="s">
+        <v>183</v>
+      </c>
+      <c r="N185" s="23"/>
+      <c r="O185" s="24"/>
+      <c r="P185" s="24" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="186" customFormat="1" ht="26" spans="1:16">
+      <c r="A186" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="B186" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C186" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D186" s="17">
+        <v>20260703</v>
+      </c>
+      <c r="E186" s="19">
+        <v>0.625</v>
+      </c>
+      <c r="F186" s="20">
+        <v>217.33</v>
+      </c>
+      <c r="G186" s="17">
+        <v>200</v>
+      </c>
+      <c r="H186" s="20">
+        <v>43466</v>
+      </c>
+      <c r="I186" s="22"/>
+      <c r="J186" s="17">
+        <v>0</v>
+      </c>
+      <c r="K186" s="23"/>
+      <c r="N186" s="23"/>
+      <c r="O186" s="24"/>
+      <c r="P186" s="24"/>
     </row>
     <row r="187" ht="24" customHeight="1" spans="3:5">
       <c r="C187" s="6"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-13 15:10:45
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="22240"/>
+    <workbookView windowWidth="29100" windowHeight="14640"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="189">
   <si>
     <t>证券代码</t>
   </si>
@@ -607,6 +607,18 @@
   </si>
   <si>
     <t>这是一个延迟许多的止损 也是我应该反思的地方 在看到6.30时一根大阳线让我以后这只是一次简单的调整 于是试图去追涨 第二天出现了一定调整 这也在意料之内 于是我没有进行止损 但突然起来的新闻使得第三天低开跌停 第四天也没有像样的修复  价格重新回到测试6.11日的低点 多头的走势现在开来要逐步逆转 当日冲高强度也不高最后尾盘回落 最终清仓离场</t>
+  </si>
+  <si>
+    <t>以为当时存储股已经接近止跌 看到韩股上涨太冒进了 于是在中午挂了单  但是来不及撤走了 被迫以当天最高价格成交 这里看来是十分错误的 最近的科技行情基本都是以冲高回落为主 很少有能一直冲高往上最后收盘的 还是没管住手</t>
+  </si>
+  <si>
+    <t>前一天强势反弹涨停之后 第二天高开低走 一路下杀到-7 同时放出天量 短时间来看 这根本不是洗盘而是出货 下跌的势头太过猛烈 但自己也不想就此错过周一的反弹 于是先卖了半仓 后来我承认自己错了 这里完全就是趋势结束的意味 割肉应该离场</t>
+  </si>
+  <si>
+    <t xml:space="preserve">兆易创新是我没做好的交易 反思的点有以下几点： 1. 浮亏加仓 这里我以为自己拿到了很好的价格 于是选择浮亏加仓 虽然在大反弹那天终于回本 但因为贪婪而没有及时减仓 2.止盈止损不够果断 大涨之后第二天的下杀 到了成本线的时候我就应该有预警需要离场 或者2%的保本损 而不是硬抗 让利润消失了  3. 我感觉我太想赢了 太想赚钱了 因此忽略了大环境的作用 完全还是在以之前的市场环境思考问题 现在似乎不是追高的时刻 </t>
+  </si>
+  <si>
+    <t>这里我主要铆钉的是它和通微富电的关系 早盘同为复电冲高的时候 我承认自己fomo了 认为封测可能会是这场下跌后的又一个主线 心急了 在早盘情绪最高时买入 相比于其他股票诚然封测更加抗跌 同时叠加 市场这么差的情况 会出现一定的资金抱团 我在这里堵了长电科技 今天的下杀太过严重 明天可能会有一定程度的修复</t>
   </si>
 </sst>
 </file>
@@ -1610,6 +1622,95 @@
     </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>8946515</xdr:colOff>
+      <xdr:row>190</xdr:row>
+      <xdr:rowOff>499745</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>15420340</xdr:colOff>
+      <xdr:row>192</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="图片 8"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34788475" y="270133445"/>
+          <a:ext cx="6473825" cy="3919855"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>15819120</xdr:colOff>
+      <xdr:row>191</xdr:row>
+      <xdr:rowOff>500380</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>16741775</xdr:colOff>
+      <xdr:row>191</xdr:row>
+      <xdr:rowOff>1029970</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp>
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="11" name="直接箭头连接符 10"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="41661080" y="272115280"/>
+          <a:ext cx="922655" cy="529590"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="arrow"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:srgbClr val="FFFFFF"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:srgbClr val="FFFFFF"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -8509,45 +8610,291 @@
       <c r="O186" s="24"/>
       <c r="P186" s="24"/>
     </row>
-    <row r="187" ht="24" customHeight="1" spans="3:5">
-      <c r="C187" s="6"/>
-      <c r="D187" s="6"/>
-      <c r="E187" s="8"/>
-    </row>
-    <row r="188" ht="24" customHeight="1" spans="3:5">
-      <c r="C188" s="6"/>
-      <c r="D188" s="6"/>
-      <c r="E188" s="8"/>
-    </row>
-    <row r="189" ht="24" customHeight="1" spans="3:5">
-      <c r="C189" s="6"/>
-      <c r="D189" s="6"/>
-      <c r="E189" s="8"/>
-    </row>
-    <row r="190" ht="24" customHeight="1" spans="3:5">
-      <c r="C190" s="6"/>
-      <c r="D190" s="6"/>
-      <c r="E190" s="8"/>
-    </row>
-    <row r="191" ht="24" customHeight="1" spans="3:5">
-      <c r="C191" s="6"/>
-      <c r="D191" s="6"/>
-      <c r="E191" s="8"/>
-    </row>
-    <row r="192" ht="24" customHeight="1" spans="3:5">
-      <c r="C192" s="6"/>
-      <c r="D192" s="6"/>
-      <c r="E192" s="8"/>
-    </row>
-    <row r="193" ht="24" customHeight="1" spans="3:5">
-      <c r="C193" s="6"/>
-      <c r="D193" s="6"/>
-      <c r="E193" s="8"/>
-    </row>
-    <row r="194" ht="24" customHeight="1" spans="3:5">
-      <c r="C194" s="6"/>
-      <c r="D194" s="6"/>
-      <c r="E194" s="8"/>
+    <row r="187" customFormat="1" ht="26" spans="1:16">
+      <c r="A187" s="28" t="s">
+        <v>166</v>
+      </c>
+      <c r="B187" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="C187" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D187" s="17">
+        <v>20260706</v>
+      </c>
+      <c r="E187" s="19">
+        <v>0.542361111111111</v>
+      </c>
+      <c r="F187" s="20">
+        <v>65.177</v>
+      </c>
+      <c r="G187" s="17">
+        <v>300</v>
+      </c>
+      <c r="H187" s="20">
+        <f>F187*G187</f>
+        <v>19553.1</v>
+      </c>
+      <c r="I187" s="22"/>
+      <c r="J187" s="17">
+        <v>300</v>
+      </c>
+      <c r="K187" s="23"/>
+      <c r="N187" s="23"/>
+      <c r="O187" s="24"/>
+      <c r="P187" s="24"/>
+    </row>
+    <row r="188" customFormat="1" ht="184" spans="1:16">
+      <c r="A188" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="B188" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C188" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D188" s="17">
+        <v>20260707</v>
+      </c>
+      <c r="E188" s="19">
+        <v>0.403472222222222</v>
+      </c>
+      <c r="F188" s="20">
+        <v>154.43</v>
+      </c>
+      <c r="G188" s="17">
+        <v>100</v>
+      </c>
+      <c r="H188" s="20">
+        <v>15443</v>
+      </c>
+      <c r="I188" s="22"/>
+      <c r="J188" s="17">
+        <v>500</v>
+      </c>
+      <c r="K188" s="23"/>
+      <c r="N188" s="23"/>
+      <c r="O188" s="24"/>
+      <c r="P188" s="24" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="189" customFormat="1" ht="184" spans="1:16">
+      <c r="A189" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="B189" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C189" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D189" s="17">
+        <v>20260707</v>
+      </c>
+      <c r="E189" s="19">
+        <v>0.40625</v>
+      </c>
+      <c r="F189" s="20">
+        <v>155.9</v>
+      </c>
+      <c r="G189" s="17">
+        <v>100</v>
+      </c>
+      <c r="H189" s="20">
+        <v>15590</v>
+      </c>
+      <c r="I189" s="22"/>
+      <c r="J189" s="17">
+        <v>400</v>
+      </c>
+      <c r="K189" s="23"/>
+      <c r="N189" s="23"/>
+      <c r="O189" s="24"/>
+      <c r="P189" s="24" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="190" customFormat="1" ht="26" spans="1:16">
+      <c r="A190" s="28" t="s">
+        <v>166</v>
+      </c>
+      <c r="B190" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="C190" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D190" s="17">
+        <v>20260707</v>
+      </c>
+      <c r="E190" s="19">
+        <v>0.411111111111111</v>
+      </c>
+      <c r="F190" s="20">
+        <v>62.76</v>
+      </c>
+      <c r="G190" s="17">
+        <v>300</v>
+      </c>
+      <c r="H190" s="20">
+        <f>F190*G190</f>
+        <v>18828</v>
+      </c>
+      <c r="I190" s="22"/>
+      <c r="J190" s="17">
+        <v>0</v>
+      </c>
+      <c r="K190" s="23"/>
+      <c r="N190" s="23"/>
+      <c r="O190" s="24"/>
+      <c r="P190" s="24"/>
+    </row>
+    <row r="191" customFormat="1" ht="156" spans="1:16">
+      <c r="A191" s="28" t="s">
+        <v>181</v>
+      </c>
+      <c r="B191" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C191" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D191" s="17">
+        <v>20260708</v>
+      </c>
+      <c r="E191" s="19">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="F191" s="20">
+        <v>634.66</v>
+      </c>
+      <c r="G191" s="17">
+        <v>100</v>
+      </c>
+      <c r="H191" s="20">
+        <v>63466</v>
+      </c>
+      <c r="I191" s="22"/>
+      <c r="J191" s="17">
+        <v>200</v>
+      </c>
+      <c r="K191" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="N191" s="23"/>
+      <c r="O191" s="24"/>
+      <c r="P191" s="24"/>
+    </row>
+    <row r="192" customFormat="1" ht="184" spans="1:16">
+      <c r="A192" s="28" t="s">
+        <v>181</v>
+      </c>
+      <c r="B192" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C192" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D192" s="17">
+        <v>20260710</v>
+      </c>
+      <c r="E192" s="19">
+        <v>0.619444444444444</v>
+      </c>
+      <c r="F192" s="20">
+        <v>616.9</v>
+      </c>
+      <c r="G192" s="17">
+        <v>100</v>
+      </c>
+      <c r="H192" s="20">
+        <v>61690</v>
+      </c>
+      <c r="I192" s="22"/>
+      <c r="J192" s="17">
+        <v>100</v>
+      </c>
+      <c r="K192" s="23"/>
+      <c r="N192" s="23"/>
+      <c r="O192" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="P192" s="24"/>
+    </row>
+    <row r="193" customFormat="1" ht="204" spans="1:16">
+      <c r="A193" s="28" t="s">
+        <v>181</v>
+      </c>
+      <c r="B193" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C193" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D193" s="17">
+        <v>20260713</v>
+      </c>
+      <c r="E193" s="19">
+        <v>0.400694444444444</v>
+      </c>
+      <c r="F193" s="20">
+        <v>577.4</v>
+      </c>
+      <c r="G193" s="17">
+        <v>100</v>
+      </c>
+      <c r="H193" s="20">
+        <v>57740</v>
+      </c>
+      <c r="I193" s="22"/>
+      <c r="J193" s="17">
+        <v>0</v>
+      </c>
+      <c r="K193" s="23"/>
+      <c r="N193" s="23"/>
+      <c r="O193" s="24"/>
+      <c r="P193" s="24" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="194" customFormat="1" ht="208" spans="1:16">
+      <c r="A194" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="B194" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C194" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D194" s="17">
+        <v>20260713</v>
+      </c>
+      <c r="E194" s="19">
+        <v>0.405555555555556</v>
+      </c>
+      <c r="F194" s="20">
+        <v>104.13</v>
+      </c>
+      <c r="G194" s="17">
+        <v>400</v>
+      </c>
+      <c r="H194" s="20">
+        <v>41652</v>
+      </c>
+      <c r="I194" s="22"/>
+      <c r="J194" s="17">
+        <v>400</v>
+      </c>
+      <c r="K194" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="N194" s="23"/>
+      <c r="O194" s="24"/>
+      <c r="P194" s="24"/>
     </row>
     <row r="195" ht="24" customHeight="1" spans="3:5">
       <c r="C195" s="6"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-15 18:42:03
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="190">
   <si>
     <t>证券代码</t>
   </si>
@@ -619,6 +619,9 @@
   </si>
   <si>
     <t>这里我主要铆钉的是它和通微富电的关系 早盘同为复电冲高的时候 我承认自己fomo了 认为封测可能会是这场下跌后的又一个主线 心急了 在早盘情绪最高时买入 相比于其他股票诚然封测更加抗跌 同时叠加 市场这么差的情况 会出现一定的资金抱团 我在这里堵了长电科技 今天的下杀太过严重 明天可能会有一定程度的修复</t>
+  </si>
+  <si>
+    <t>早盘下杀 想着的是 不断向下加仓摊平成本博取明天修复的机会离场 但是这里需要反思的是 这个月亏的太多 其实有点慌乱了 不知道自己在干嘛 无论做出什么决策都是亏损的结局 十分懊恼 但又舍不得狠下心来空仓 为什么这样</t>
   </si>
 </sst>
 </file>
@@ -1252,7 +1255,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1330,6 +1333,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center"/>
@@ -7678,7 +7684,7 @@
       </c>
     </row>
     <row r="162" customFormat="1" ht="156" spans="1:16">
-      <c r="A162" s="28" t="s">
+      <c r="A162" s="29" t="s">
         <v>149</v>
       </c>
       <c r="B162" s="16" t="s">
@@ -7715,7 +7721,7 @@
       <c r="P162" s="24"/>
     </row>
     <row r="163" customFormat="1" ht="104" spans="1:16">
-      <c r="A163" s="28" t="s">
+      <c r="A163" s="29" t="s">
         <v>149</v>
       </c>
       <c r="B163" s="16" t="s">
@@ -7920,7 +7926,7 @@
       <c r="AC167"/>
     </row>
     <row r="168" customFormat="1" ht="234" spans="1:16">
-      <c r="A168" s="28" t="s">
+      <c r="A168" s="29" t="s">
         <v>158</v>
       </c>
       <c r="B168" s="16" t="s">
@@ -7957,7 +7963,7 @@
       </c>
     </row>
     <row r="169" customFormat="1" ht="204" spans="1:16">
-      <c r="A169" s="28" t="s">
+      <c r="A169" s="29" t="s">
         <v>149</v>
       </c>
       <c r="B169" s="16" t="s">
@@ -7993,7 +7999,7 @@
       <c r="P169" s="24"/>
     </row>
     <row r="170" customFormat="1" ht="286" spans="1:16">
-      <c r="A170" s="28" t="s">
+      <c r="A170" s="29" t="s">
         <v>163</v>
       </c>
       <c r="B170" s="16" t="s">
@@ -8028,7 +8034,7 @@
       <c r="P170" s="24"/>
     </row>
     <row r="171" customFormat="1" ht="130" spans="1:16">
-      <c r="A171" s="28" t="s">
+      <c r="A171" s="29" t="s">
         <v>126</v>
       </c>
       <c r="B171" s="16" t="s">
@@ -8064,7 +8070,7 @@
       <c r="P171" s="24"/>
     </row>
     <row r="172" customFormat="1" ht="286" spans="1:16">
-      <c r="A172" s="28" t="s">
+      <c r="A172" s="29" t="s">
         <v>166</v>
       </c>
       <c r="B172" s="16" t="s">
@@ -8100,7 +8106,7 @@
       <c r="P172" s="24"/>
     </row>
     <row r="173" customFormat="1" ht="204" spans="1:16">
-      <c r="A173" s="28" t="s">
+      <c r="A173" s="29" t="s">
         <v>149</v>
       </c>
       <c r="B173" s="16" t="s">
@@ -8139,7 +8145,7 @@
       <c r="P173" s="24"/>
     </row>
     <row r="174" customFormat="1" ht="25" customHeight="1" spans="1:16">
-      <c r="A174" s="28" t="s">
+      <c r="A174" s="29" t="s">
         <v>163</v>
       </c>
       <c r="B174" s="16" t="s">
@@ -8209,7 +8215,7 @@
       <c r="P175" s="24"/>
     </row>
     <row r="176" customFormat="1" ht="78" spans="1:16">
-      <c r="A176" s="28" t="s">
+      <c r="A176" s="29" t="s">
         <v>166</v>
       </c>
       <c r="B176" s="16" t="s">
@@ -8246,7 +8252,7 @@
       <c r="P176" s="24"/>
     </row>
     <row r="177" customFormat="1" ht="234" spans="1:16">
-      <c r="A177" s="28" t="s">
+      <c r="A177" s="29" t="s">
         <v>158</v>
       </c>
       <c r="B177" s="16" t="s">
@@ -8318,7 +8324,7 @@
       <c r="P178" s="24"/>
     </row>
     <row r="179" customFormat="1" ht="182" spans="1:16">
-      <c r="A179" s="28" t="s">
+      <c r="A179" s="29" t="s">
         <v>166</v>
       </c>
       <c r="B179" s="16" t="s">
@@ -8355,7 +8361,7 @@
       <c r="P179" s="24"/>
     </row>
     <row r="180" customFormat="1" ht="156" spans="1:16">
-      <c r="A180" s="28" t="s">
+      <c r="A180" s="29" t="s">
         <v>166</v>
       </c>
       <c r="B180" s="16" t="s">
@@ -8392,7 +8398,7 @@
       <c r="P180" s="24"/>
     </row>
     <row r="181" customFormat="1" ht="104" spans="1:16">
-      <c r="A181" s="28" t="s">
+      <c r="A181" s="29" t="s">
         <v>176</v>
       </c>
       <c r="B181" s="16" t="s">
@@ -8429,7 +8435,7 @@
       <c r="P181" s="24"/>
     </row>
     <row r="182" customFormat="1" ht="388" spans="1:16">
-      <c r="A182" s="28" t="s">
+      <c r="A182" s="29" t="s">
         <v>158</v>
       </c>
       <c r="B182" s="16" t="s">
@@ -8467,7 +8473,7 @@
       </c>
     </row>
     <row r="183" customFormat="1" ht="52" spans="1:16">
-      <c r="A183" s="28" t="s">
+      <c r="A183" s="29" t="s">
         <v>163</v>
       </c>
       <c r="B183" s="16" t="s">
@@ -8503,7 +8509,7 @@
       <c r="P183" s="24"/>
     </row>
     <row r="184" customFormat="1" ht="234" spans="1:16">
-      <c r="A184" s="28" t="s">
+      <c r="A184" s="29" t="s">
         <v>181</v>
       </c>
       <c r="B184" s="16" t="s">
@@ -8539,7 +8545,7 @@
       <c r="P184" s="24"/>
     </row>
     <row r="185" customFormat="1" ht="184" spans="1:16">
-      <c r="A185" s="28" t="s">
+      <c r="A185" s="29" t="s">
         <v>113</v>
       </c>
       <c r="B185" s="16" t="s">
@@ -8577,7 +8583,7 @@
       </c>
     </row>
     <row r="186" customFormat="1" ht="26" spans="1:16">
-      <c r="A186" s="28" t="s">
+      <c r="A186" s="29" t="s">
         <v>68</v>
       </c>
       <c r="B186" s="16" t="s">
@@ -8611,7 +8617,7 @@
       <c r="P186" s="24"/>
     </row>
     <row r="187" customFormat="1" ht="26" spans="1:16">
-      <c r="A187" s="28" t="s">
+      <c r="A187" s="29" t="s">
         <v>166</v>
       </c>
       <c r="B187" s="16" t="s">
@@ -8646,7 +8652,7 @@
       <c r="P187" s="24"/>
     </row>
     <row r="188" customFormat="1" ht="184" spans="1:16">
-      <c r="A188" s="28" t="s">
+      <c r="A188" s="29" t="s">
         <v>113</v>
       </c>
       <c r="B188" s="16" t="s">
@@ -8682,7 +8688,7 @@
       </c>
     </row>
     <row r="189" customFormat="1" ht="184" spans="1:16">
-      <c r="A189" s="28" t="s">
+      <c r="A189" s="29" t="s">
         <v>113</v>
       </c>
       <c r="B189" s="16" t="s">
@@ -8718,7 +8724,7 @@
       </c>
     </row>
     <row r="190" customFormat="1" ht="26" spans="1:16">
-      <c r="A190" s="28" t="s">
+      <c r="A190" s="29" t="s">
         <v>166</v>
       </c>
       <c r="B190" s="16" t="s">
@@ -8753,7 +8759,7 @@
       <c r="P190" s="24"/>
     </row>
     <row r="191" customFormat="1" ht="156" spans="1:16">
-      <c r="A191" s="28" t="s">
+      <c r="A191" s="29" t="s">
         <v>181</v>
       </c>
       <c r="B191" s="16" t="s">
@@ -8789,7 +8795,7 @@
       <c r="P191" s="24"/>
     </row>
     <row r="192" customFormat="1" ht="184" spans="1:16">
-      <c r="A192" s="28" t="s">
+      <c r="A192" s="29" t="s">
         <v>181</v>
       </c>
       <c r="B192" s="16" t="s">
@@ -8825,7 +8831,7 @@
       <c r="P192" s="24"/>
     </row>
     <row r="193" customFormat="1" ht="204" spans="1:16">
-      <c r="A193" s="28" t="s">
+      <c r="A193" s="29" t="s">
         <v>181</v>
       </c>
       <c r="B193" s="16" t="s">
@@ -8861,7 +8867,7 @@
       </c>
     </row>
     <row r="194" customFormat="1" ht="208" spans="1:16">
-      <c r="A194" s="28" t="s">
+      <c r="A194" s="29" t="s">
         <v>163</v>
       </c>
       <c r="B194" s="16" t="s">
@@ -8896,25 +8902,143 @@
       <c r="O194" s="24"/>
       <c r="P194" s="24"/>
     </row>
-    <row r="195" ht="24" customHeight="1" spans="3:5">
-      <c r="C195" s="6"/>
-      <c r="D195" s="6"/>
-      <c r="E195" s="8"/>
-    </row>
-    <row r="196" ht="24" customHeight="1" spans="3:5">
-      <c r="C196" s="6"/>
-      <c r="D196" s="6"/>
-      <c r="E196" s="8"/>
-    </row>
-    <row r="197" ht="24" customHeight="1" spans="3:5">
-      <c r="C197" s="6"/>
-      <c r="D197" s="6"/>
-      <c r="E197" s="8"/>
-    </row>
-    <row r="198" ht="24" customHeight="1" spans="3:5">
-      <c r="C198" s="6"/>
-      <c r="D198" s="6"/>
-      <c r="E198" s="8"/>
+    <row r="195" customFormat="1" ht="26" spans="1:16">
+      <c r="A195" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="B195" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C195" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D195" s="17">
+        <v>20260715</v>
+      </c>
+      <c r="E195" s="19">
+        <v>0.400694444444444</v>
+      </c>
+      <c r="F195" s="20">
+        <v>97.97</v>
+      </c>
+      <c r="G195" s="17">
+        <v>200</v>
+      </c>
+      <c r="H195" s="20">
+        <v>19594</v>
+      </c>
+      <c r="I195" s="22"/>
+      <c r="J195" s="17">
+        <v>600</v>
+      </c>
+      <c r="K195" s="28" t="s">
+        <v>189</v>
+      </c>
+      <c r="N195" s="23"/>
+      <c r="O195" s="24"/>
+      <c r="P195" s="24"/>
+    </row>
+    <row r="196" customFormat="1" ht="26" spans="1:16">
+      <c r="A196" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="B196" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C196" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D196" s="17">
+        <v>20260715</v>
+      </c>
+      <c r="E196" s="19">
+        <v>0.401388888888889</v>
+      </c>
+      <c r="F196" s="20">
+        <v>96</v>
+      </c>
+      <c r="G196" s="17">
+        <v>100</v>
+      </c>
+      <c r="H196" s="20">
+        <v>9600</v>
+      </c>
+      <c r="I196" s="22"/>
+      <c r="J196" s="17">
+        <v>700</v>
+      </c>
+      <c r="K196" s="28"/>
+      <c r="N196" s="23"/>
+      <c r="O196" s="24"/>
+      <c r="P196" s="24"/>
+    </row>
+    <row r="197" customFormat="1" ht="26" spans="1:16">
+      <c r="A197" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="B197" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C197" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D197" s="17">
+        <v>20260715</v>
+      </c>
+      <c r="E197" s="19">
+        <v>0.408333333333333</v>
+      </c>
+      <c r="F197" s="20">
+        <v>97.23</v>
+      </c>
+      <c r="G197" s="17">
+        <v>100</v>
+      </c>
+      <c r="H197" s="20">
+        <v>9723</v>
+      </c>
+      <c r="I197" s="22"/>
+      <c r="J197" s="17">
+        <v>800</v>
+      </c>
+      <c r="K197" s="28"/>
+      <c r="N197" s="23"/>
+      <c r="O197" s="24"/>
+      <c r="P197" s="24"/>
+    </row>
+    <row r="198" customFormat="1" ht="26" spans="1:16">
+      <c r="A198" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="B198" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C198" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D198" s="17">
+        <v>20260715</v>
+      </c>
+      <c r="E198" s="19">
+        <v>0.620833333333333</v>
+      </c>
+      <c r="F198" s="20">
+        <v>93</v>
+      </c>
+      <c r="G198" s="17">
+        <v>100</v>
+      </c>
+      <c r="H198" s="20">
+        <v>9300</v>
+      </c>
+      <c r="I198" s="22"/>
+      <c r="J198" s="17">
+        <v>900</v>
+      </c>
+      <c r="K198" s="28"/>
+      <c r="N198" s="23"/>
+      <c r="O198" s="24"/>
+      <c r="P198" s="24"/>
     </row>
     <row r="199" ht="24" customHeight="1" spans="3:5">
       <c r="C199" s="6"/>
@@ -11508,6 +11632,9 @@
       <c r="D1005" s="6"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="K195:K198"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-18 14:20:56
</commit_message>
<xml_diff>
--- a/交易记录.xlsx
+++ b/交易记录.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="191">
   <si>
     <t>证券代码</t>
   </si>
@@ -622,6 +622,9 @@
   </si>
   <si>
     <t>早盘下杀 想着的是 不断向下加仓摊平成本博取明天修复的机会离场 但是这里需要反思的是 这个月亏的太多 其实有点慌乱了 不知道自己在干嘛 无论做出什么决策都是亏损的结局 十分懊恼 但又舍不得狠下心来空仓 为什么这样</t>
+  </si>
+  <si>
+    <t xml:space="preserve">底部长电科技已经初步探底 今天大盘整体走势很差 接近千股跌停 长电科技逆势收红 基本面一路向好 大盘距离反弹不远 于是选择加仓 </t>
   </si>
 </sst>
 </file>
@@ -9040,10 +9043,42 @@
       <c r="O198" s="24"/>
       <c r="P198" s="24"/>
     </row>
-    <row r="199" ht="24" customHeight="1" spans="3:5">
-      <c r="C199" s="6"/>
-      <c r="D199" s="6"/>
-      <c r="E199" s="8"/>
+    <row r="199" customFormat="1" ht="104" spans="1:16">
+      <c r="A199" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="B199" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C199" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D199" s="17">
+        <v>20260717</v>
+      </c>
+      <c r="E199" s="19">
+        <v>0.620833333333333</v>
+      </c>
+      <c r="F199" s="20">
+        <v>85.21</v>
+      </c>
+      <c r="G199" s="17">
+        <v>200</v>
+      </c>
+      <c r="H199" s="20">
+        <f>G199*F199</f>
+        <v>17042</v>
+      </c>
+      <c r="I199" s="22"/>
+      <c r="J199" s="17">
+        <v>1100</v>
+      </c>
+      <c r="K199" s="28" t="s">
+        <v>190</v>
+      </c>
+      <c r="N199" s="23"/>
+      <c r="O199" s="24"/>
+      <c r="P199" s="24"/>
     </row>
     <row r="200" ht="24" customHeight="1" spans="3:5">
       <c r="C200" s="6"/>

</xml_diff>